<commit_message>
Expand 组合管理 functions (Slide 44) + add detail sheet
- Module 7 functions: 6 placeholders → 17 detailed functions across
  6 domains (组合分析/风险计量/绩效归因/组合优化/流动性/量化底座)
- Module 7 estimate updated: 9m/10p/76pm → 12m/12p/120pm
- New sheet 详情_组合管理: full function detail with acceptance
  criteria, integration dependencies, priority (P1/P2), dev days
- Source: 基于国内外FICC平台发展经验规划FICC平台建设路径0417.pptx Slide 44

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Feasibility_analysis/FICC_Gap_Analysis.xlsx
+++ b/Feasibility_analysis/FICC_Gap_Analysis.xlsx
@@ -11,6 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="关键功能清单" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="资源规划" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="P1优先启动计划" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="详情_组合管理" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Area" localSheetId="0">'差距分析总表'!$A$1:$P$19</definedName>
@@ -22,7 +23,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="13">
+  <fonts count="15">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -95,6 +96,18 @@
     <font>
       <name val="Arial"/>
       <color rgb="00E53935"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="13"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <i val="1"/>
+      <color rgb="001B3275"/>
       <sz val="10"/>
     </font>
   </fonts>
@@ -215,7 +228,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="39">
+  <cellXfs count="46">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -328,6 +341,27 @@
     </xf>
     <xf numFmtId="0" fontId="10" fillId="3" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="3" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1315,17 +1349,17 @@
         </is>
       </c>
       <c r="M9" s="3" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="N9" s="3" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="O9" s="8" t="n">
-        <v>76</v>
+        <v>120</v>
       </c>
       <c r="P9" s="5" t="inlineStr">
         <is>
-          <t>Brinson归因+固收久期优化</t>
+          <t>17项功能含量化底座集成；Slide44全景展开</t>
         </is>
       </c>
     </row>
@@ -2035,7 +2069,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H104"/>
+  <dimension ref="A1:H115"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -3484,12 +3518,12 @@
       </c>
       <c r="D43" s="4" t="inlineStr">
         <is>
-          <t>多维度组合构建</t>
+          <t>债券横截面与时序分析</t>
         </is>
       </c>
       <c r="E43" s="5" t="inlineStr">
         <is>
-          <t>因子约束/跟踪误差/久期目标等多目标组合优化</t>
+          <t>跨品种横截面信号挖掘（利差、久期偏差），历史时序趋势/均值回归分析</t>
         </is>
       </c>
       <c r="F43" s="5" t="inlineStr">
@@ -3503,7 +3537,7 @@
         </is>
       </c>
       <c r="H43" s="8" t="n">
-        <v>40</v>
+        <v>35</v>
       </c>
     </row>
     <row r="44" ht="28" customHeight="1">
@@ -3524,12 +3558,12 @@
       </c>
       <c r="D44" s="4" t="inlineStr">
         <is>
-          <t>再平衡引擎</t>
+          <t>相对价值分析</t>
         </is>
       </c>
       <c r="E44" s="5" t="inlineStr">
         <is>
-          <t>基于信号/规则自动生成调仓指令，考虑交易成本与冲击</t>
+          <t>利差/Z-spread/OAS相对价值，历史分位数定位，套利信号识别</t>
         </is>
       </c>
       <c r="F44" s="5" t="inlineStr">
@@ -3564,26 +3598,26 @@
       </c>
       <c r="D45" s="4" t="inlineStr">
         <is>
-          <t>Brinson绩效归因</t>
+          <t>组合相关度分析</t>
         </is>
       </c>
       <c r="E45" s="5" t="inlineStr">
         <is>
-          <t>Brinson-Hood-Beebower模型，资产配置/个券选择/交互效应</t>
+          <t>资产间收益相关矩阵计算，组合集中度风险识别，分散化系数监控</t>
         </is>
       </c>
       <c r="F45" s="5" t="inlineStr">
         <is>
-          <t>功能完整/边界测试/集成冒烟/性能基线</t>
-        </is>
-      </c>
-      <c r="G45" s="24" t="inlineStr">
-        <is>
-          <t>高</t>
+          <t>功能测试通过/正确率100%</t>
+        </is>
+      </c>
+      <c r="G45" s="25" t="inlineStr">
+        <is>
+          <t>中</t>
         </is>
       </c>
       <c r="H45" s="8" t="n">
-        <v>35</v>
+        <v>25</v>
       </c>
     </row>
     <row r="46" ht="28" customHeight="1">
@@ -3604,26 +3638,26 @@
       </c>
       <c r="D46" s="4" t="inlineStr">
         <is>
-          <t>固收久期/凸度管理</t>
+          <t>情景分析</t>
         </is>
       </c>
       <c r="E46" s="5" t="inlineStr">
         <is>
-          <t>组合DV01/凸度实时监控，与风险计量平台对接</t>
+          <t>利率/信用/流动性三类自定义情景，组合P&amp;L影响量化，多情景并行对比</t>
         </is>
       </c>
       <c r="F46" s="5" t="inlineStr">
         <is>
-          <t>功能测试通过/正确率100%</t>
-        </is>
-      </c>
-      <c r="G46" s="25" t="inlineStr">
-        <is>
-          <t>中</t>
+          <t>功能完整/边界测试/集成冒烟/性能基线</t>
+        </is>
+      </c>
+      <c r="G46" s="24" t="inlineStr">
+        <is>
+          <t>高</t>
         </is>
       </c>
       <c r="H46" s="8" t="n">
-        <v>20</v>
+        <v>35</v>
       </c>
     </row>
     <row r="47" ht="28" customHeight="1">
@@ -3644,26 +3678,26 @@
       </c>
       <c r="D47" s="4" t="inlineStr">
         <is>
-          <t>基准指数对比</t>
+          <t>敏感度分析</t>
         </is>
       </c>
       <c r="E47" s="5" t="inlineStr">
         <is>
-          <t>跟踪误差计算，超额收益（Alpha）归因，信息比率监控</t>
+          <t>久期/DV01/凸度/利差敏感度多因子并行计算，组合对冲比率建议</t>
         </is>
       </c>
       <c r="F47" s="5" t="inlineStr">
         <is>
-          <t>功能测试通过/正确率100%</t>
-        </is>
-      </c>
-      <c r="G47" s="25" t="inlineStr">
-        <is>
-          <t>中</t>
+          <t>功能完整/边界测试/集成冒烟/性能基线</t>
+        </is>
+      </c>
+      <c r="G47" s="24" t="inlineStr">
+        <is>
+          <t>高</t>
         </is>
       </c>
       <c r="H47" s="8" t="n">
-        <v>20</v>
+        <v>25</v>
       </c>
     </row>
     <row r="48" ht="28" customHeight="1">
@@ -3684,12 +3718,12 @@
       </c>
       <c r="D48" s="4" t="inlineStr">
         <is>
-          <t>实时PnL归因</t>
+          <t>极端事件分析</t>
         </is>
       </c>
       <c r="E48" s="5" t="inlineStr">
         <is>
-          <t>已实现/未实现PnL按因子/资产/策略三维归因</t>
+          <t>历史极端情景（924行情/2015股灾/2020疫情）组合压测，尾部损失分布</t>
         </is>
       </c>
       <c r="F48" s="5" t="inlineStr">
@@ -3706,17 +3740,50 @@
         <v>30</v>
       </c>
     </row>
-    <row r="49" ht="20" customHeight="1">
-      <c r="A49" s="23" t="inlineStr">
-        <is>
-          <t>【P1】 策略投资/量化  (Quant Strategy)</t>
-        </is>
+    <row r="49" ht="28" customHeight="1">
+      <c r="A49" s="5" t="inlineStr">
+        <is>
+          <t>组合管理+绩效归因</t>
+        </is>
+      </c>
+      <c r="B49" s="3" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="C49" s="3" t="inlineStr">
+        <is>
+          <t>F07-07</t>
+        </is>
+      </c>
+      <c r="D49" s="4" t="inlineStr">
+        <is>
+          <t>指数比较分析</t>
+        </is>
+      </c>
+      <c r="E49" s="5" t="inlineStr">
+        <is>
+          <t>对标中债综合/信用/政策行等指数，跟踪误差（TE）实时监控，超额Alpha分解</t>
+        </is>
+      </c>
+      <c r="F49" s="5" t="inlineStr">
+        <is>
+          <t>功能测试通过/正确率100%</t>
+        </is>
+      </c>
+      <c r="G49" s="25" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="H49" s="8" t="n">
+        <v>25</v>
       </c>
     </row>
     <row r="50" ht="28" customHeight="1">
       <c r="A50" s="5" t="inlineStr">
         <is>
-          <t>策略投资/量化</t>
+          <t>组合管理+绩效归因</t>
         </is>
       </c>
       <c r="B50" s="3" t="inlineStr">
@@ -3726,17 +3793,17 @@
       </c>
       <c r="C50" s="3" t="inlineStr">
         <is>
-          <t>F08-01</t>
+          <t>F07-08</t>
         </is>
       </c>
       <c r="D50" s="4" t="inlineStr">
         <is>
-          <t>因子模型框架</t>
+          <t>绩效归因（Brinson）</t>
         </is>
       </c>
       <c r="E50" s="5" t="inlineStr">
         <is>
-          <t>多因子Alpha模型+风险因子，支持自定义因子上传与测试</t>
+          <t>BHB模型三效应：资产配置/个券选择/交互效应，日频计算，周/月/季报自动生成</t>
         </is>
       </c>
       <c r="F50" s="5" t="inlineStr">
@@ -3756,7 +3823,7 @@
     <row r="51" ht="28" customHeight="1">
       <c r="A51" s="5" t="inlineStr">
         <is>
-          <t>策略投资/量化</t>
+          <t>组合管理+绩效归因</t>
         </is>
       </c>
       <c r="B51" s="3" t="inlineStr">
@@ -3766,37 +3833,37 @@
       </c>
       <c r="C51" s="3" t="inlineStr">
         <is>
-          <t>F08-02</t>
+          <t>F07-09</t>
         </is>
       </c>
       <c r="D51" s="4" t="inlineStr">
         <is>
-          <t>Tick级回测引擎</t>
+          <t>虚拟组合分析</t>
         </is>
       </c>
       <c r="E51" s="5" t="inlineStr">
         <is>
-          <t>Tick数据驱动回测，真实滑点/冲击模型，批量参数优化</t>
+          <t>组合调整前后效果模拟（净值/风险/收益），交易冲击成本预估，方案比较</t>
         </is>
       </c>
       <c r="F51" s="5" t="inlineStr">
         <is>
-          <t>p99延迟/误差率/精度验证/压测10k TPS</t>
-        </is>
-      </c>
-      <c r="G51" s="27" t="inlineStr">
-        <is>
-          <t>极高</t>
+          <t>功能完整/边界测试/集成冒烟/性能基线</t>
+        </is>
+      </c>
+      <c r="G51" s="24" t="inlineStr">
+        <is>
+          <t>高</t>
         </is>
       </c>
       <c r="H51" s="8" t="n">
-        <v>60</v>
+        <v>20</v>
       </c>
     </row>
     <row r="52" ht="28" customHeight="1">
       <c r="A52" s="5" t="inlineStr">
         <is>
-          <t>策略投资/量化</t>
+          <t>组合管理+绩效归因</t>
         </is>
       </c>
       <c r="B52" s="3" t="inlineStr">
@@ -3806,17 +3873,17 @@
       </c>
       <c r="C52" s="3" t="inlineStr">
         <is>
-          <t>F08-03</t>
+          <t>F07-10</t>
         </is>
       </c>
       <c r="D52" s="4" t="inlineStr">
         <is>
-          <t>信号生成与调度</t>
+          <t>再平衡方案试算与比较</t>
         </is>
       </c>
       <c r="E52" s="5" t="inlineStr">
         <is>
-          <t>策略信号实时计算，支持Python/C++策略脚本沙箱运行</t>
+          <t>久期/集中度/流动性约束联合优化，多方案并行试算，最优路径推荐</t>
         </is>
       </c>
       <c r="F52" s="5" t="inlineStr">
@@ -3830,13 +3897,13 @@
         </is>
       </c>
       <c r="H52" s="8" t="n">
-        <v>40</v>
+        <v>35</v>
       </c>
     </row>
     <row r="53" ht="28" customHeight="1">
       <c r="A53" s="5" t="inlineStr">
         <is>
-          <t>策略投资/量化</t>
+          <t>组合管理+绩效归因</t>
         </is>
       </c>
       <c r="B53" s="3" t="inlineStr">
@@ -3846,491 +3913,491 @@
       </c>
       <c r="C53" s="3" t="inlineStr">
         <is>
-          <t>F08-04</t>
+          <t>F07-11</t>
         </is>
       </c>
       <c r="D53" s="4" t="inlineStr">
         <is>
-          <t>低延迟执行接口</t>
+          <t>资产配置策略分析</t>
         </is>
       </c>
       <c r="E53" s="5" t="inlineStr">
         <is>
-          <t>与ATP超低延迟执行层对接，算法拆单（TWAP/VWAP/IS）</t>
+          <t>宏观因子驱动大类资产配置模型（利率/信用/权益），动态权重优化建议</t>
         </is>
       </c>
       <c r="F53" s="5" t="inlineStr">
         <is>
-          <t>p99延迟/误差率/精度验证/压测10k TPS</t>
-        </is>
-      </c>
-      <c r="G53" s="27" t="inlineStr">
-        <is>
-          <t>极高</t>
+          <t>功能完整/边界测试/集成冒烟/性能基线</t>
+        </is>
+      </c>
+      <c r="G53" s="24" t="inlineStr">
+        <is>
+          <t>高</t>
         </is>
       </c>
       <c r="H53" s="8" t="n">
-        <v>45</v>
+        <v>40</v>
       </c>
     </row>
     <row r="54" ht="28" customHeight="1">
       <c r="A54" s="5" t="inlineStr">
         <is>
+          <t>组合管理+绩效归因</t>
+        </is>
+      </c>
+      <c r="B54" s="3" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="C54" s="3" t="inlineStr">
+        <is>
+          <t>F07-12</t>
+        </is>
+      </c>
+      <c r="D54" s="4" t="inlineStr">
+        <is>
+          <t>固收+策略分析</t>
+        </is>
+      </c>
+      <c r="E54" s="5" t="inlineStr">
+        <is>
+          <t>债券底仓+衍生品增强策略P&amp;L归因，风险分解，固收+产品净值模拟</t>
+        </is>
+      </c>
+      <c r="F54" s="5" t="inlineStr">
+        <is>
+          <t>功能完整/边界测试/集成冒烟/性能基线</t>
+        </is>
+      </c>
+      <c r="G54" s="24" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="H54" s="8" t="n">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="55" ht="28" customHeight="1">
+      <c r="A55" s="5" t="inlineStr">
+        <is>
+          <t>组合管理+绩效归因</t>
+        </is>
+      </c>
+      <c r="B55" s="3" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="C55" s="3" t="inlineStr">
+        <is>
+          <t>F07-13</t>
+        </is>
+      </c>
+      <c r="D55" s="4" t="inlineStr">
+        <is>
+          <t>量化策略组合分析</t>
+        </is>
+      </c>
+      <c r="E55" s="5" t="inlineStr">
+        <is>
+          <t>多策略组合叠加容量约束，策略相关性管理，Sharpe/最大回撤监控</t>
+        </is>
+      </c>
+      <c r="F55" s="5" t="inlineStr">
+        <is>
+          <t>功能完整/边界测试/集成冒烟/性能基线</t>
+        </is>
+      </c>
+      <c r="G55" s="24" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="H55" s="8" t="n">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="56" ht="28" customHeight="1">
+      <c r="A56" s="5" t="inlineStr">
+        <is>
+          <t>组合管理+绩效归因</t>
+        </is>
+      </c>
+      <c r="B56" s="3" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="C56" s="3" t="inlineStr">
+        <is>
+          <t>F07-14</t>
+        </is>
+      </c>
+      <c r="D56" s="4" t="inlineStr">
+        <is>
+          <t>流动性分析</t>
+        </is>
+      </c>
+      <c r="E56" s="5" t="inlineStr">
+        <is>
+          <t>逐券换手率/市场深度评估，组合变现能力分析，流动性压力下变现损失估算</t>
+        </is>
+      </c>
+      <c r="F56" s="5" t="inlineStr">
+        <is>
+          <t>功能测试通过/正确率100%</t>
+        </is>
+      </c>
+      <c r="G56" s="25" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="H56" s="8" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="57" ht="28" customHeight="1">
+      <c r="A57" s="5" t="inlineStr">
+        <is>
+          <t>组合管理+绩效归因</t>
+        </is>
+      </c>
+      <c r="B57" s="3" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="C57" s="3" t="inlineStr">
+        <is>
+          <t>F07-15</t>
+        </is>
+      </c>
+      <c r="D57" s="4" t="inlineStr">
+        <is>
+          <t>定价计算集成</t>
+        </is>
+      </c>
+      <c r="E57" s="5" t="inlineStr">
+        <is>
+          <t>调用量化定价引擎实时估值与Greeks，支持含权债/可转债，结果缓存与推送</t>
+        </is>
+      </c>
+      <c r="F57" s="5" t="inlineStr">
+        <is>
+          <t>功能完整/边界测试/集成冒烟/性能基线</t>
+        </is>
+      </c>
+      <c r="G57" s="24" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="H57" s="8" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="58" ht="28" customHeight="1">
+      <c r="A58" s="5" t="inlineStr">
+        <is>
+          <t>组合管理+绩效归因</t>
+        </is>
+      </c>
+      <c r="B58" s="3" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="C58" s="3" t="inlineStr">
+        <is>
+          <t>F07-16</t>
+        </is>
+      </c>
+      <c r="D58" s="4" t="inlineStr">
+        <is>
+          <t>利率曲线集成</t>
+        </is>
+      </c>
+      <c r="E58" s="5" t="inlineStr">
+        <is>
+          <t>多曲线实时消费（国债/政策行/信用），曲线因子提取（水平/斜率/曲率），敏感度映射</t>
+        </is>
+      </c>
+      <c r="F58" s="5" t="inlineStr">
+        <is>
+          <t>功能测试通过/正确率100%</t>
+        </is>
+      </c>
+      <c r="G58" s="25" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="H58" s="8" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="59" ht="28" customHeight="1">
+      <c r="A59" s="5" t="inlineStr">
+        <is>
+          <t>组合管理+绩效归因</t>
+        </is>
+      </c>
+      <c r="B59" s="3" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="C59" s="3" t="inlineStr">
+        <is>
+          <t>F07-17</t>
+        </is>
+      </c>
+      <c r="D59" s="4" t="inlineStr">
+        <is>
+          <t>因子模型</t>
+        </is>
+      </c>
+      <c r="E59" s="5" t="inlineStr">
+        <is>
+          <t>多因子风险模型（利率/信用/流动性/行业因子），Alpha因子库，因子暴露实时计算</t>
+        </is>
+      </c>
+      <c r="F59" s="5" t="inlineStr">
+        <is>
+          <t>功能完整/边界测试/集成冒烟/性能基线</t>
+        </is>
+      </c>
+      <c r="G59" s="24" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="H59" s="8" t="n">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="60" ht="20" customHeight="1">
+      <c r="A60" s="23" t="inlineStr">
+        <is>
+          <t>【P1】 策略投资/量化  (Quant Strategy)</t>
+        </is>
+      </c>
+    </row>
+    <row r="61" ht="28" customHeight="1">
+      <c r="A61" s="5" t="inlineStr">
+        <is>
           <t>策略投资/量化</t>
         </is>
       </c>
-      <c r="B54" s="3" t="inlineStr">
+      <c r="B61" s="3" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="C54" s="3" t="inlineStr">
+      <c r="C61" s="3" t="inlineStr">
+        <is>
+          <t>F08-01</t>
+        </is>
+      </c>
+      <c r="D61" s="4" t="inlineStr">
+        <is>
+          <t>因子模型框架</t>
+        </is>
+      </c>
+      <c r="E61" s="5" t="inlineStr">
+        <is>
+          <t>多因子Alpha模型+风险因子，支持自定义因子上传与测试</t>
+        </is>
+      </c>
+      <c r="F61" s="5" t="inlineStr">
+        <is>
+          <t>功能完整/边界测试/集成冒烟/性能基线</t>
+        </is>
+      </c>
+      <c r="G61" s="24" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="H61" s="8" t="n">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="62" ht="28" customHeight="1">
+      <c r="A62" s="5" t="inlineStr">
+        <is>
+          <t>策略投资/量化</t>
+        </is>
+      </c>
+      <c r="B62" s="3" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="C62" s="3" t="inlineStr">
+        <is>
+          <t>F08-02</t>
+        </is>
+      </c>
+      <c r="D62" s="4" t="inlineStr">
+        <is>
+          <t>Tick级回测引擎</t>
+        </is>
+      </c>
+      <c r="E62" s="5" t="inlineStr">
+        <is>
+          <t>Tick数据驱动回测，真实滑点/冲击模型，批量参数优化</t>
+        </is>
+      </c>
+      <c r="F62" s="5" t="inlineStr">
+        <is>
+          <t>p99延迟/误差率/精度验证/压测10k TPS</t>
+        </is>
+      </c>
+      <c r="G62" s="27" t="inlineStr">
+        <is>
+          <t>极高</t>
+        </is>
+      </c>
+      <c r="H62" s="8" t="n">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="63" ht="28" customHeight="1">
+      <c r="A63" s="5" t="inlineStr">
+        <is>
+          <t>策略投资/量化</t>
+        </is>
+      </c>
+      <c r="B63" s="3" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="C63" s="3" t="inlineStr">
+        <is>
+          <t>F08-03</t>
+        </is>
+      </c>
+      <c r="D63" s="4" t="inlineStr">
+        <is>
+          <t>信号生成与调度</t>
+        </is>
+      </c>
+      <c r="E63" s="5" t="inlineStr">
+        <is>
+          <t>策略信号实时计算，支持Python/C++策略脚本沙箱运行</t>
+        </is>
+      </c>
+      <c r="F63" s="5" t="inlineStr">
+        <is>
+          <t>功能完整/边界测试/集成冒烟/性能基线</t>
+        </is>
+      </c>
+      <c r="G63" s="24" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="H63" s="8" t="n">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="64" ht="28" customHeight="1">
+      <c r="A64" s="5" t="inlineStr">
+        <is>
+          <t>策略投资/量化</t>
+        </is>
+      </c>
+      <c r="B64" s="3" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="C64" s="3" t="inlineStr">
+        <is>
+          <t>F08-04</t>
+        </is>
+      </c>
+      <c r="D64" s="4" t="inlineStr">
+        <is>
+          <t>低延迟执行接口</t>
+        </is>
+      </c>
+      <c r="E64" s="5" t="inlineStr">
+        <is>
+          <t>与ATP超低延迟执行层对接，算法拆单（TWAP/VWAP/IS）</t>
+        </is>
+      </c>
+      <c r="F64" s="5" t="inlineStr">
+        <is>
+          <t>p99延迟/误差率/精度验证/压测10k TPS</t>
+        </is>
+      </c>
+      <c r="G64" s="27" t="inlineStr">
+        <is>
+          <t>极高</t>
+        </is>
+      </c>
+      <c r="H64" s="8" t="n">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="65" ht="28" customHeight="1">
+      <c r="A65" s="5" t="inlineStr">
+        <is>
+          <t>策略投资/量化</t>
+        </is>
+      </c>
+      <c r="B65" s="3" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="C65" s="3" t="inlineStr">
         <is>
           <t>F08-05</t>
         </is>
       </c>
-      <c r="D54" s="4" t="inlineStr">
+      <c r="D65" s="4" t="inlineStr">
         <is>
           <t>实时策略监控</t>
         </is>
       </c>
-      <c r="E54" s="5" t="inlineStr">
+      <c r="E65" s="5" t="inlineStr">
         <is>
           <t>持仓/PnL/回撤/Sharpe实时看板，风险触发自动平仓</t>
         </is>
       </c>
-      <c r="F54" s="5" t="inlineStr">
+      <c r="F65" s="5" t="inlineStr">
         <is>
           <t>功能测试通过/正确率100%</t>
         </is>
       </c>
-      <c r="G54" s="25" t="inlineStr">
+      <c r="G65" s="25" t="inlineStr">
         <is>
           <t>中</t>
         </is>
       </c>
-      <c r="H54" s="8" t="n">
+      <c r="H65" s="8" t="n">
         <v>20</v>
       </c>
     </row>
-    <row r="55" ht="20" customHeight="1">
-      <c r="A55" s="28" t="inlineStr">
+    <row r="66" ht="20" customHeight="1">
+      <c r="A66" s="28" t="inlineStr">
         <is>
           <t>【P2】 量化定价引擎  (Quant Pricing Engine)</t>
         </is>
-      </c>
-    </row>
-    <row r="56" ht="28" customHeight="1">
-      <c r="A56" s="11" t="inlineStr">
-        <is>
-          <t>量化定价引擎</t>
-        </is>
-      </c>
-      <c r="B56" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
-        </is>
-      </c>
-      <c r="C56" s="10" t="inlineStr">
-        <is>
-          <t>F09-01</t>
-        </is>
-      </c>
-      <c r="D56" s="29" t="inlineStr">
-        <is>
-          <t>期限结构模型</t>
-        </is>
-      </c>
-      <c r="E56" s="11" t="inlineStr">
-        <is>
-          <t>Nelson-Siegel/Svensson/HJM等多模型参数拟合，实时曲线</t>
-        </is>
-      </c>
-      <c r="F56" s="11" t="inlineStr">
-        <is>
-          <t>p99延迟/误差率/精度验证/压测10k TPS</t>
-        </is>
-      </c>
-      <c r="G56" s="27" t="inlineStr">
-        <is>
-          <t>极高</t>
-        </is>
-      </c>
-      <c r="H56" s="14" t="n">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="57" ht="28" customHeight="1">
-      <c r="A57" s="11" t="inlineStr">
-        <is>
-          <t>量化定价引擎</t>
-        </is>
-      </c>
-      <c r="B57" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
-        </is>
-      </c>
-      <c r="C57" s="10" t="inlineStr">
-        <is>
-          <t>F09-02</t>
-        </is>
-      </c>
-      <c r="D57" s="29" t="inlineStr">
-        <is>
-          <t>蒙特卡洛求解器</t>
-        </is>
-      </c>
-      <c r="E57" s="11" t="inlineStr">
-        <is>
-          <t>GPU加速MC，QMC低差异序列，支持路径相关期权定价</t>
-        </is>
-      </c>
-      <c r="F57" s="11" t="inlineStr">
-        <is>
-          <t>p99延迟/误差率/精度验证/压测10k TPS</t>
-        </is>
-      </c>
-      <c r="G57" s="27" t="inlineStr">
-        <is>
-          <t>极高</t>
-        </is>
-      </c>
-      <c r="H57" s="14" t="n">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="58" ht="28" customHeight="1">
-      <c r="A58" s="11" t="inlineStr">
-        <is>
-          <t>量化定价引擎</t>
-        </is>
-      </c>
-      <c r="B58" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
-        </is>
-      </c>
-      <c r="C58" s="10" t="inlineStr">
-        <is>
-          <t>F09-03</t>
-        </is>
-      </c>
-      <c r="D58" s="29" t="inlineStr">
-        <is>
-          <t>有限差分（PDE）</t>
-        </is>
-      </c>
-      <c r="E58" s="11" t="inlineStr">
-        <is>
-          <t>Crank-Nicolson/ADI方法，含权债/可转债精确定价</t>
-        </is>
-      </c>
-      <c r="F58" s="11" t="inlineStr">
-        <is>
-          <t>p99延迟/误差率/精度验证/压测10k TPS</t>
-        </is>
-      </c>
-      <c r="G58" s="27" t="inlineStr">
-        <is>
-          <t>极高</t>
-        </is>
-      </c>
-      <c r="H58" s="14" t="n">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="59" ht="28" customHeight="1">
-      <c r="A59" s="11" t="inlineStr">
-        <is>
-          <t>量化定价引擎</t>
-        </is>
-      </c>
-      <c r="B59" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
-        </is>
-      </c>
-      <c r="C59" s="10" t="inlineStr">
-        <is>
-          <t>F09-04</t>
-        </is>
-      </c>
-      <c r="D59" s="29" t="inlineStr">
-        <is>
-          <t>实时Greeks</t>
-        </is>
-      </c>
-      <c r="E59" s="11" t="inlineStr">
-        <is>
-          <t>Delta/Gamma/Vega/Theta/Rho分布式实时计算</t>
-        </is>
-      </c>
-      <c r="F59" s="11" t="inlineStr">
-        <is>
-          <t>功能完整/边界测试/集成冒烟/性能基线</t>
-        </is>
-      </c>
-      <c r="G59" s="24" t="inlineStr">
-        <is>
-          <t>高</t>
-        </is>
-      </c>
-      <c r="H59" s="14" t="n">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="60" ht="28" customHeight="1">
-      <c r="A60" s="11" t="inlineStr">
-        <is>
-          <t>量化定价引擎</t>
-        </is>
-      </c>
-      <c r="B60" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
-        </is>
-      </c>
-      <c r="C60" s="10" t="inlineStr">
-        <is>
-          <t>F09-05</t>
-        </is>
-      </c>
-      <c r="D60" s="29" t="inlineStr">
-        <is>
-          <t>定价服务微服务架构</t>
-        </is>
-      </c>
-      <c r="E60" s="11" t="inlineStr">
-        <is>
-          <t>REST/gRPC定价API，支持横向扩展，p99&lt;100ms</t>
-        </is>
-      </c>
-      <c r="F60" s="11" t="inlineStr">
-        <is>
-          <t>功能完整/边界测试/集成冒烟/性能基线</t>
-        </is>
-      </c>
-      <c r="G60" s="24" t="inlineStr">
-        <is>
-          <t>高</t>
-        </is>
-      </c>
-      <c r="H60" s="14" t="n">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="61" ht="28" customHeight="1">
-      <c r="A61" s="11" t="inlineStr">
-        <is>
-          <t>量化定价引擎</t>
-        </is>
-      </c>
-      <c r="B61" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
-        </is>
-      </c>
-      <c r="C61" s="10" t="inlineStr">
-        <is>
-          <t>F09-06</t>
-        </is>
-      </c>
-      <c r="D61" s="29" t="inlineStr">
-        <is>
-          <t>历史估值回测</t>
-        </is>
-      </c>
-      <c r="E61" s="11" t="inlineStr">
-        <is>
-          <t>基于历史行情重放定价误差分析，模型验证框架</t>
-        </is>
-      </c>
-      <c r="F61" s="11" t="inlineStr">
-        <is>
-          <t>功能完整/边界测试/集成冒烟/性能基线</t>
-        </is>
-      </c>
-      <c r="G61" s="24" t="inlineStr">
-        <is>
-          <t>高</t>
-        </is>
-      </c>
-      <c r="H61" s="14" t="n">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="62" ht="20" customHeight="1">
-      <c r="A62" s="28" t="inlineStr">
-        <is>
-          <t>【P2】 利率衍生品  (Interest Rate Derivatives)</t>
-        </is>
-      </c>
-    </row>
-    <row r="63" ht="28" customHeight="1">
-      <c r="A63" s="11" t="inlineStr">
-        <is>
-          <t>利率衍生品</t>
-        </is>
-      </c>
-      <c r="B63" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
-        </is>
-      </c>
-      <c r="C63" s="10" t="inlineStr">
-        <is>
-          <t>F10-01</t>
-        </is>
-      </c>
-      <c r="D63" s="29" t="inlineStr">
-        <is>
-          <t>IRS/OIS/CCS定价</t>
-        </is>
-      </c>
-      <c r="E63" s="11" t="inlineStr">
-        <is>
-          <t>利率互换标准与非标结构定价，折现曲线OIS</t>
-        </is>
-      </c>
-      <c r="F63" s="11" t="inlineStr">
-        <is>
-          <t>p99延迟/误差率/精度验证/压测10k TPS</t>
-        </is>
-      </c>
-      <c r="G63" s="27" t="inlineStr">
-        <is>
-          <t>极高</t>
-        </is>
-      </c>
-      <c r="H63" s="14" t="n">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="64" ht="28" customHeight="1">
-      <c r="A64" s="11" t="inlineStr">
-        <is>
-          <t>利率衍生品</t>
-        </is>
-      </c>
-      <c r="B64" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
-        </is>
-      </c>
-      <c r="C64" s="10" t="inlineStr">
-        <is>
-          <t>F10-02</t>
-        </is>
-      </c>
-      <c r="D64" s="29" t="inlineStr">
-        <is>
-          <t>久期/DV01/凸度</t>
-        </is>
-      </c>
-      <c r="E64" s="11" t="inlineStr">
-        <is>
-          <t>利率衍生品Greeks实时计算，组合对冲比率</t>
-        </is>
-      </c>
-      <c r="F64" s="11" t="inlineStr">
-        <is>
-          <t>功能完整/边界测试/集成冒烟/性能基线</t>
-        </is>
-      </c>
-      <c r="G64" s="24" t="inlineStr">
-        <is>
-          <t>高</t>
-        </is>
-      </c>
-      <c r="H64" s="14" t="n">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="65" ht="28" customHeight="1">
-      <c r="A65" s="11" t="inlineStr">
-        <is>
-          <t>利率衍生品</t>
-        </is>
-      </c>
-      <c r="B65" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
-        </is>
-      </c>
-      <c r="C65" s="10" t="inlineStr">
-        <is>
-          <t>F10-03</t>
-        </is>
-      </c>
-      <c r="D65" s="29" t="inlineStr">
-        <is>
-          <t>LCH/上清所CCP接口</t>
-        </is>
-      </c>
-      <c r="E65" s="11" t="inlineStr">
-        <is>
-          <t>标准化IRS中央清算，保证金（IM/VM）计算</t>
-        </is>
-      </c>
-      <c r="F65" s="11" t="inlineStr">
-        <is>
-          <t>功能完整/边界测试/集成冒烟/性能基线</t>
-        </is>
-      </c>
-      <c r="G65" s="24" t="inlineStr">
-        <is>
-          <t>高</t>
-        </is>
-      </c>
-      <c r="H65" s="14" t="n">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="66" ht="28" customHeight="1">
-      <c r="A66" s="11" t="inlineStr">
-        <is>
-          <t>利率衍生品</t>
-        </is>
-      </c>
-      <c r="B66" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
-        </is>
-      </c>
-      <c r="C66" s="10" t="inlineStr">
-        <is>
-          <t>F10-04</t>
-        </is>
-      </c>
-      <c r="D66" s="29" t="inlineStr">
-        <is>
-          <t>压力测试/情景分析</t>
-        </is>
-      </c>
-      <c r="E66" s="11" t="inlineStr">
-        <is>
-          <t>利率曲线平移/扭转/蝶式情景，组合P&amp;L影响</t>
-        </is>
-      </c>
-      <c r="F66" s="11" t="inlineStr">
-        <is>
-          <t>功能完整/边界测试/集成冒烟/性能基线</t>
-        </is>
-      </c>
-      <c r="G66" s="24" t="inlineStr">
-        <is>
-          <t>高</t>
-        </is>
-      </c>
-      <c r="H66" s="14" t="n">
-        <v>30</v>
       </c>
     </row>
     <row r="67" ht="28" customHeight="1">
       <c r="A67" s="11" t="inlineStr">
         <is>
-          <t>利率衍生品</t>
+          <t>量化定价引擎</t>
         </is>
       </c>
       <c r="B67" s="10" t="inlineStr">
@@ -4340,44 +4407,77 @@
       </c>
       <c r="C67" s="10" t="inlineStr">
         <is>
-          <t>F10-05</t>
+          <t>F09-01</t>
         </is>
       </c>
       <c r="D67" s="29" t="inlineStr">
         <is>
-          <t>利率曲线发布</t>
+          <t>期限结构模型</t>
         </is>
       </c>
       <c r="E67" s="11" t="inlineStr">
         <is>
-          <t>多曲线框架（OIS/Libor过渡/中债曲线）实时发布</t>
+          <t>Nelson-Siegel/Svensson/HJM等多模型参数拟合，实时曲线</t>
         </is>
       </c>
       <c r="F67" s="11" t="inlineStr">
         <is>
-          <t>功能完整/边界测试/集成冒烟/性能基线</t>
-        </is>
-      </c>
-      <c r="G67" s="24" t="inlineStr">
-        <is>
-          <t>高</t>
+          <t>p99延迟/误差率/精度验证/压测10k TPS</t>
+        </is>
+      </c>
+      <c r="G67" s="27" t="inlineStr">
+        <is>
+          <t>极高</t>
         </is>
       </c>
       <c r="H67" s="14" t="n">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="68" ht="20" customHeight="1">
-      <c r="A68" s="28" t="inlineStr">
-        <is>
-          <t>【P2】 信用债/信用衍生品  (Credit &amp; CDS)</t>
-        </is>
+        <v>60</v>
+      </c>
+    </row>
+    <row r="68" ht="28" customHeight="1">
+      <c r="A68" s="11" t="inlineStr">
+        <is>
+          <t>量化定价引擎</t>
+        </is>
+      </c>
+      <c r="B68" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="C68" s="10" t="inlineStr">
+        <is>
+          <t>F09-02</t>
+        </is>
+      </c>
+      <c r="D68" s="29" t="inlineStr">
+        <is>
+          <t>蒙特卡洛求解器</t>
+        </is>
+      </c>
+      <c r="E68" s="11" t="inlineStr">
+        <is>
+          <t>GPU加速MC，QMC低差异序列，支持路径相关期权定价</t>
+        </is>
+      </c>
+      <c r="F68" s="11" t="inlineStr">
+        <is>
+          <t>p99延迟/误差率/精度验证/压测10k TPS</t>
+        </is>
+      </c>
+      <c r="G68" s="27" t="inlineStr">
+        <is>
+          <t>极高</t>
+        </is>
+      </c>
+      <c r="H68" s="14" t="n">
+        <v>70</v>
       </c>
     </row>
     <row r="69" ht="28" customHeight="1">
       <c r="A69" s="11" t="inlineStr">
         <is>
-          <t>信用债/信用衍生品</t>
+          <t>量化定价引擎</t>
         </is>
       </c>
       <c r="B69" s="10" t="inlineStr">
@@ -4387,37 +4487,37 @@
       </c>
       <c r="C69" s="10" t="inlineStr">
         <is>
-          <t>F11-01</t>
+          <t>F09-03</t>
         </is>
       </c>
       <c r="D69" s="29" t="inlineStr">
         <is>
-          <t>信用利差分析</t>
+          <t>有限差分（PDE）</t>
         </is>
       </c>
       <c r="E69" s="11" t="inlineStr">
         <is>
-          <t>行业/评级/期限信用利差曲线实时计算，历史分位数分析</t>
+          <t>Crank-Nicolson/ADI方法，含权债/可转债精确定价</t>
         </is>
       </c>
       <c r="F69" s="11" t="inlineStr">
         <is>
-          <t>功能完整/边界测试/集成冒烟/性能基线</t>
-        </is>
-      </c>
-      <c r="G69" s="24" t="inlineStr">
-        <is>
-          <t>高</t>
+          <t>p99延迟/误差率/精度验证/压测10k TPS</t>
+        </is>
+      </c>
+      <c r="G69" s="27" t="inlineStr">
+        <is>
+          <t>极高</t>
         </is>
       </c>
       <c r="H69" s="14" t="n">
-        <v>30</v>
+        <v>60</v>
       </c>
     </row>
     <row r="70" ht="28" customHeight="1">
       <c r="A70" s="11" t="inlineStr">
         <is>
-          <t>信用债/信用衍生品</t>
+          <t>量化定价引擎</t>
         </is>
       </c>
       <c r="B70" s="10" t="inlineStr">
@@ -4427,37 +4527,37 @@
       </c>
       <c r="C70" s="10" t="inlineStr">
         <is>
-          <t>F11-02</t>
+          <t>F09-04</t>
         </is>
       </c>
       <c r="D70" s="29" t="inlineStr">
         <is>
-          <t>CDS/CLN定价</t>
+          <t>实时Greeks</t>
         </is>
       </c>
       <c r="E70" s="11" t="inlineStr">
         <is>
-          <t>信用违约互换定价，ISDA标准，生存概率曲线校准</t>
+          <t>Delta/Gamma/Vega/Theta/Rho分布式实时计算</t>
         </is>
       </c>
       <c r="F70" s="11" t="inlineStr">
         <is>
-          <t>p99延迟/误差率/精度验证/压测10k TPS</t>
-        </is>
-      </c>
-      <c r="G70" s="27" t="inlineStr">
-        <is>
-          <t>极高</t>
+          <t>功能完整/边界测试/集成冒烟/性能基线</t>
+        </is>
+      </c>
+      <c r="G70" s="24" t="inlineStr">
+        <is>
+          <t>高</t>
         </is>
       </c>
       <c r="H70" s="14" t="n">
-        <v>50</v>
+        <v>40</v>
       </c>
     </row>
     <row r="71" ht="28" customHeight="1">
       <c r="A71" s="11" t="inlineStr">
         <is>
-          <t>信用债/信用衍生品</t>
+          <t>量化定价引擎</t>
         </is>
       </c>
       <c r="B71" s="10" t="inlineStr">
@@ -4467,37 +4567,37 @@
       </c>
       <c r="C71" s="10" t="inlineStr">
         <is>
-          <t>F11-03</t>
+          <t>F09-05</t>
         </is>
       </c>
       <c r="D71" s="29" t="inlineStr">
         <is>
-          <t>信用评级动态监控</t>
+          <t>定价服务微服务架构</t>
         </is>
       </c>
       <c r="E71" s="11" t="inlineStr">
         <is>
-          <t>对接外部评级机构（中诚信/联合/大公），评级下调预警</t>
+          <t>REST/gRPC定价API，支持横向扩展，p99&lt;100ms</t>
         </is>
       </c>
       <c r="F71" s="11" t="inlineStr">
         <is>
-          <t>功能测试通过/正确率100%</t>
-        </is>
-      </c>
-      <c r="G71" s="25" t="inlineStr">
-        <is>
-          <t>中</t>
+          <t>功能完整/边界测试/集成冒烟/性能基线</t>
+        </is>
+      </c>
+      <c r="G71" s="24" t="inlineStr">
+        <is>
+          <t>高</t>
         </is>
       </c>
       <c r="H71" s="14" t="n">
-        <v>20</v>
+        <v>40</v>
       </c>
     </row>
     <row r="72" ht="28" customHeight="1">
       <c r="A72" s="11" t="inlineStr">
         <is>
-          <t>信用债/信用衍生品</t>
+          <t>量化定价引擎</t>
         </is>
       </c>
       <c r="B72" s="10" t="inlineStr">
@@ -4507,17 +4607,17 @@
       </c>
       <c r="C72" s="10" t="inlineStr">
         <is>
-          <t>F11-04</t>
+          <t>F09-06</t>
         </is>
       </c>
       <c r="D72" s="29" t="inlineStr">
         <is>
-          <t>违约概率（PD）建模</t>
+          <t>历史估值回测</t>
         </is>
       </c>
       <c r="E72" s="11" t="inlineStr">
         <is>
-          <t>结构化Merton模型+市场隐含PD，信用风险计量</t>
+          <t>基于历史行情重放定价误差分析，模型验证框架</t>
         </is>
       </c>
       <c r="F72" s="11" t="inlineStr">
@@ -4531,60 +4631,60 @@
         </is>
       </c>
       <c r="H72" s="14" t="n">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="73" ht="28" customHeight="1">
-      <c r="A73" s="11" t="inlineStr">
-        <is>
-          <t>信用债/信用衍生品</t>
-        </is>
-      </c>
-      <c r="B73" s="10" t="inlineStr">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="73" ht="20" customHeight="1">
+      <c r="A73" s="28" t="inlineStr">
+        <is>
+          <t>【P2】 利率衍生品  (Interest Rate Derivatives)</t>
+        </is>
+      </c>
+    </row>
+    <row r="74" ht="28" customHeight="1">
+      <c r="A74" s="11" t="inlineStr">
+        <is>
+          <t>利率衍生品</t>
+        </is>
+      </c>
+      <c r="B74" s="10" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
       </c>
-      <c r="C73" s="10" t="inlineStr">
-        <is>
-          <t>F11-05</t>
-        </is>
-      </c>
-      <c r="D73" s="29" t="inlineStr">
-        <is>
-          <t>集中度限额管理</t>
-        </is>
-      </c>
-      <c r="E73" s="11" t="inlineStr">
-        <is>
-          <t>行业/发行人/评级集中度多维限额，超限预警</t>
-        </is>
-      </c>
-      <c r="F73" s="11" t="inlineStr">
-        <is>
-          <t>功能测试通过/正确率100%</t>
-        </is>
-      </c>
-      <c r="G73" s="25" t="inlineStr">
-        <is>
-          <t>中</t>
-        </is>
-      </c>
-      <c r="H73" s="14" t="n">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="74" ht="20" customHeight="1">
-      <c r="A74" s="28" t="inlineStr">
-        <is>
-          <t>【P2】 数据管理/行情平台  (Market Data Platform)</t>
-        </is>
+      <c r="C74" s="10" t="inlineStr">
+        <is>
+          <t>F10-01</t>
+        </is>
+      </c>
+      <c r="D74" s="29" t="inlineStr">
+        <is>
+          <t>IRS/OIS/CCS定价</t>
+        </is>
+      </c>
+      <c r="E74" s="11" t="inlineStr">
+        <is>
+          <t>利率互换标准与非标结构定价，折现曲线OIS</t>
+        </is>
+      </c>
+      <c r="F74" s="11" t="inlineStr">
+        <is>
+          <t>p99延迟/误差率/精度验证/压测10k TPS</t>
+        </is>
+      </c>
+      <c r="G74" s="27" t="inlineStr">
+        <is>
+          <t>极高</t>
+        </is>
+      </c>
+      <c r="H74" s="14" t="n">
+        <v>60</v>
       </c>
     </row>
     <row r="75" ht="28" customHeight="1">
       <c r="A75" s="11" t="inlineStr">
         <is>
-          <t>数据管理/行情平台</t>
+          <t>利率衍生品</t>
         </is>
       </c>
       <c r="B75" s="10" t="inlineStr">
@@ -4594,17 +4694,17 @@
       </c>
       <c r="C75" s="10" t="inlineStr">
         <is>
-          <t>F12-01</t>
+          <t>F10-02</t>
         </is>
       </c>
       <c r="D75" s="29" t="inlineStr">
         <is>
-          <t>多源行情聚合</t>
+          <t>久期/DV01/凸度</t>
         </is>
       </c>
       <c r="E75" s="11" t="inlineStr">
         <is>
-          <t>Bloomberg/Wind/中汇信/Refinitiv多源融合，冲突解析</t>
+          <t>利率衍生品Greeks实时计算，组合对冲比率</t>
         </is>
       </c>
       <c r="F75" s="11" t="inlineStr">
@@ -4618,13 +4718,13 @@
         </is>
       </c>
       <c r="H75" s="14" t="n">
-        <v>25</v>
+        <v>30</v>
       </c>
     </row>
     <row r="76" ht="28" customHeight="1">
       <c r="A76" s="11" t="inlineStr">
         <is>
-          <t>数据管理/行情平台</t>
+          <t>利率衍生品</t>
         </is>
       </c>
       <c r="B76" s="10" t="inlineStr">
@@ -4634,37 +4734,37 @@
       </c>
       <c r="C76" s="10" t="inlineStr">
         <is>
-          <t>F12-02</t>
+          <t>F10-03</t>
         </is>
       </c>
       <c r="D76" s="29" t="inlineStr">
         <is>
-          <t>数据质量校验</t>
+          <t>LCH/上清所CCP接口</t>
         </is>
       </c>
       <c r="E76" s="11" t="inlineStr">
         <is>
-          <t>异常值/缺失值/跳价自动检测，修复建议与人工审核</t>
+          <t>标准化IRS中央清算，保证金（IM/VM）计算</t>
         </is>
       </c>
       <c r="F76" s="11" t="inlineStr">
         <is>
-          <t>功能测试通过/正确率100%</t>
-        </is>
-      </c>
-      <c r="G76" s="25" t="inlineStr">
-        <is>
-          <t>中</t>
+          <t>功能完整/边界测试/集成冒烟/性能基线</t>
+        </is>
+      </c>
+      <c r="G76" s="24" t="inlineStr">
+        <is>
+          <t>高</t>
         </is>
       </c>
       <c r="H76" s="14" t="n">
-        <v>15</v>
+        <v>35</v>
       </c>
     </row>
     <row r="77" ht="28" customHeight="1">
       <c r="A77" s="11" t="inlineStr">
         <is>
-          <t>数据管理/行情平台</t>
+          <t>利率衍生品</t>
         </is>
       </c>
       <c r="B77" s="10" t="inlineStr">
@@ -4674,17 +4774,17 @@
       </c>
       <c r="C77" s="10" t="inlineStr">
         <is>
-          <t>F12-03</t>
+          <t>F10-04</t>
         </is>
       </c>
       <c r="D77" s="29" t="inlineStr">
         <is>
-          <t>历史数据仓库</t>
+          <t>压力测试/情景分析</t>
         </is>
       </c>
       <c r="E77" s="11" t="inlineStr">
         <is>
-          <t>Tick/日频历史行情存储，高效查询（ClickHouse/TimescaleDB）</t>
+          <t>利率曲线平移/扭转/蝶式情景，组合P&amp;L影响</t>
         </is>
       </c>
       <c r="F77" s="11" t="inlineStr">
@@ -4698,13 +4798,13 @@
         </is>
       </c>
       <c r="H77" s="14" t="n">
-        <v>25</v>
+        <v>30</v>
       </c>
     </row>
     <row r="78" ht="28" customHeight="1">
       <c r="A78" s="11" t="inlineStr">
         <is>
-          <t>数据管理/行情平台</t>
+          <t>利率衍生品</t>
         </is>
       </c>
       <c r="B78" s="10" t="inlineStr">
@@ -4714,17 +4814,17 @@
       </c>
       <c r="C78" s="10" t="inlineStr">
         <is>
-          <t>F12-04</t>
+          <t>F10-05</t>
         </is>
       </c>
       <c r="D78" s="29" t="inlineStr">
         <is>
-          <t>收益率曲线发布</t>
+          <t>利率曲线发布</t>
         </is>
       </c>
       <c r="E78" s="11" t="inlineStr">
         <is>
-          <t>国债/政策行/高等级信用曲线实时发布，Kafka广播</t>
+          <t>多曲线框架（OIS/Libor过渡/中债曲线）实时发布</t>
         </is>
       </c>
       <c r="F78" s="11" t="inlineStr">
@@ -4738,60 +4838,60 @@
         </is>
       </c>
       <c r="H78" s="14" t="n">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="79" ht="28" customHeight="1">
-      <c r="A79" s="11" t="inlineStr">
-        <is>
-          <t>数据管理/行情平台</t>
-        </is>
-      </c>
-      <c r="B79" s="10" t="inlineStr">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="79" ht="20" customHeight="1">
+      <c r="A79" s="28" t="inlineStr">
+        <is>
+          <t>【P2】 信用债/信用衍生品  (Credit &amp; CDS)</t>
+        </is>
+      </c>
+    </row>
+    <row r="80" ht="28" customHeight="1">
+      <c r="A80" s="11" t="inlineStr">
+        <is>
+          <t>信用债/信用衍生品</t>
+        </is>
+      </c>
+      <c r="B80" s="10" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
       </c>
-      <c r="C79" s="10" t="inlineStr">
-        <is>
-          <t>F12-05</t>
-        </is>
-      </c>
-      <c r="D79" s="29" t="inlineStr">
-        <is>
-          <t>估值价格服务</t>
-        </is>
-      </c>
-      <c r="E79" s="11" t="inlineStr">
-        <is>
-          <t>非活跃债券估值价格（中债估值基准），API接口提供</t>
-        </is>
-      </c>
-      <c r="F79" s="11" t="inlineStr">
-        <is>
-          <t>功能测试通过/正确率100%</t>
-        </is>
-      </c>
-      <c r="G79" s="25" t="inlineStr">
-        <is>
-          <t>中</t>
-        </is>
-      </c>
-      <c r="H79" s="14" t="n">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="80" ht="20" customHeight="1">
-      <c r="A80" s="28" t="inlineStr">
-        <is>
-          <t>【P2】 交易对手管理  (Counterparty Management)</t>
-        </is>
+      <c r="C80" s="10" t="inlineStr">
+        <is>
+          <t>F11-01</t>
+        </is>
+      </c>
+      <c r="D80" s="29" t="inlineStr">
+        <is>
+          <t>信用利差分析</t>
+        </is>
+      </c>
+      <c r="E80" s="11" t="inlineStr">
+        <is>
+          <t>行业/评级/期限信用利差曲线实时计算，历史分位数分析</t>
+        </is>
+      </c>
+      <c r="F80" s="11" t="inlineStr">
+        <is>
+          <t>功能完整/边界测试/集成冒烟/性能基线</t>
+        </is>
+      </c>
+      <c r="G80" s="24" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="H80" s="14" t="n">
+        <v>30</v>
       </c>
     </row>
     <row r="81" ht="28" customHeight="1">
       <c r="A81" s="11" t="inlineStr">
         <is>
-          <t>交易对手管理</t>
+          <t>信用债/信用衍生品</t>
         </is>
       </c>
       <c r="B81" s="10" t="inlineStr">
@@ -4801,37 +4901,37 @@
       </c>
       <c r="C81" s="10" t="inlineStr">
         <is>
-          <t>F13-01</t>
+          <t>F11-02</t>
         </is>
       </c>
       <c r="D81" s="29" t="inlineStr">
         <is>
-          <t>对手方评级与审批</t>
+          <t>CDS/CLN定价</t>
         </is>
       </c>
       <c r="E81" s="11" t="inlineStr">
         <is>
-          <t>内部信用评级模型，新增/变更交易对手审批流</t>
+          <t>信用违约互换定价，ISDA标准，生存概率曲线校准</t>
         </is>
       </c>
       <c r="F81" s="11" t="inlineStr">
         <is>
-          <t>功能测试通过/正确率100%</t>
-        </is>
-      </c>
-      <c r="G81" s="25" t="inlineStr">
-        <is>
-          <t>中</t>
+          <t>p99延迟/误差率/精度验证/压测10k TPS</t>
+        </is>
+      </c>
+      <c r="G81" s="27" t="inlineStr">
+        <is>
+          <t>极高</t>
         </is>
       </c>
       <c r="H81" s="14" t="n">
-        <v>20</v>
+        <v>50</v>
       </c>
     </row>
     <row r="82" ht="28" customHeight="1">
       <c r="A82" s="11" t="inlineStr">
         <is>
-          <t>交易对手管理</t>
+          <t>信用债/信用衍生品</t>
         </is>
       </c>
       <c r="B82" s="10" t="inlineStr">
@@ -4841,37 +4941,37 @@
       </c>
       <c r="C82" s="10" t="inlineStr">
         <is>
-          <t>F13-02</t>
+          <t>F11-03</t>
         </is>
       </c>
       <c r="D82" s="29" t="inlineStr">
         <is>
-          <t>实时敞口聚合</t>
+          <t>信用评级动态监控</t>
         </is>
       </c>
       <c r="E82" s="11" t="inlineStr">
         <is>
-          <t>跨产品交易对手名义/MtM敞口实时聚合，压力敞口（EPE）</t>
+          <t>对接外部评级机构（中诚信/联合/大公），评级下调预警</t>
         </is>
       </c>
       <c r="F82" s="11" t="inlineStr">
         <is>
-          <t>功能完整/边界测试/集成冒烟/性能基线</t>
-        </is>
-      </c>
-      <c r="G82" s="24" t="inlineStr">
-        <is>
-          <t>高</t>
+          <t>功能测试通过/正确率100%</t>
+        </is>
+      </c>
+      <c r="G82" s="25" t="inlineStr">
+        <is>
+          <t>中</t>
         </is>
       </c>
       <c r="H82" s="14" t="n">
-        <v>35</v>
+        <v>20</v>
       </c>
     </row>
     <row r="83" ht="28" customHeight="1">
       <c r="A83" s="11" t="inlineStr">
         <is>
-          <t>交易对手管理</t>
+          <t>信用债/信用衍生品</t>
         </is>
       </c>
       <c r="B83" s="10" t="inlineStr">
@@ -4881,17 +4981,17 @@
       </c>
       <c r="C83" s="10" t="inlineStr">
         <is>
-          <t>F13-03</t>
+          <t>F11-04</t>
         </is>
       </c>
       <c r="D83" s="29" t="inlineStr">
         <is>
-          <t>ISDA/CSA协议管理</t>
+          <t>违约概率（PD）建模</t>
         </is>
       </c>
       <c r="E83" s="11" t="inlineStr">
         <is>
-          <t>主协议文档管理，净额结算协议（Netting Set）配置</t>
+          <t>结构化Merton模型+市场隐含PD，信用风险计量</t>
         </is>
       </c>
       <c r="F83" s="11" t="inlineStr">
@@ -4905,13 +5005,13 @@
         </is>
       </c>
       <c r="H83" s="14" t="n">
-        <v>25</v>
+        <v>40</v>
       </c>
     </row>
     <row r="84" ht="28" customHeight="1">
       <c r="A84" s="11" t="inlineStr">
         <is>
-          <t>交易对手管理</t>
+          <t>信用债/信用衍生品</t>
         </is>
       </c>
       <c r="B84" s="10" t="inlineStr">
@@ -4921,84 +5021,84 @@
       </c>
       <c r="C84" s="10" t="inlineStr">
         <is>
-          <t>F13-04</t>
+          <t>F11-05</t>
         </is>
       </c>
       <c r="D84" s="29" t="inlineStr">
         <is>
-          <t>CVA/DVA/FVA计算</t>
+          <t>集中度限额管理</t>
         </is>
       </c>
       <c r="E84" s="11" t="inlineStr">
         <is>
-          <t>信用/债务/资金估值调整实时估算，敞口报告</t>
+          <t>行业/发行人/评级集中度多维限额，超限预警</t>
         </is>
       </c>
       <c r="F84" s="11" t="inlineStr">
         <is>
-          <t>p99延迟/误差率/精度验证/压测10k TPS</t>
-        </is>
-      </c>
-      <c r="G84" s="27" t="inlineStr">
-        <is>
-          <t>极高</t>
+          <t>功能测试通过/正确率100%</t>
+        </is>
+      </c>
+      <c r="G84" s="25" t="inlineStr">
+        <is>
+          <t>中</t>
         </is>
       </c>
       <c r="H84" s="14" t="n">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="85" ht="28" customHeight="1">
-      <c r="A85" s="11" t="inlineStr">
-        <is>
-          <t>交易对手管理</t>
-        </is>
-      </c>
-      <c r="B85" s="10" t="inlineStr">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="85" ht="20" customHeight="1">
+      <c r="A85" s="28" t="inlineStr">
+        <is>
+          <t>【P2】 数据管理/行情平台  (Market Data Platform)</t>
+        </is>
+      </c>
+    </row>
+    <row r="86" ht="28" customHeight="1">
+      <c r="A86" s="11" t="inlineStr">
+        <is>
+          <t>数据管理/行情平台</t>
+        </is>
+      </c>
+      <c r="B86" s="10" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
       </c>
-      <c r="C85" s="10" t="inlineStr">
-        <is>
-          <t>F13-05</t>
-        </is>
-      </c>
-      <c r="D85" s="29" t="inlineStr">
-        <is>
-          <t>集中度与限额</t>
-        </is>
-      </c>
-      <c r="E85" s="11" t="inlineStr">
-        <is>
-          <t>对手方/集团合并敞口限额，超限审批与记录</t>
-        </is>
-      </c>
-      <c r="F85" s="11" t="inlineStr">
-        <is>
-          <t>功能测试通过/正确率100%</t>
-        </is>
-      </c>
-      <c r="G85" s="25" t="inlineStr">
-        <is>
-          <t>中</t>
-        </is>
-      </c>
-      <c r="H85" s="14" t="n">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="86" ht="20" customHeight="1">
-      <c r="A86" s="28" t="inlineStr">
-        <is>
-          <t>【P2】 清算结算后台  (Clearing &amp; Settlement)</t>
-        </is>
+      <c r="C86" s="10" t="inlineStr">
+        <is>
+          <t>F12-01</t>
+        </is>
+      </c>
+      <c r="D86" s="29" t="inlineStr">
+        <is>
+          <t>多源行情聚合</t>
+        </is>
+      </c>
+      <c r="E86" s="11" t="inlineStr">
+        <is>
+          <t>Bloomberg/Wind/中汇信/Refinitiv多源融合，冲突解析</t>
+        </is>
+      </c>
+      <c r="F86" s="11" t="inlineStr">
+        <is>
+          <t>功能完整/边界测试/集成冒烟/性能基线</t>
+        </is>
+      </c>
+      <c r="G86" s="24" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="H86" s="14" t="n">
+        <v>25</v>
       </c>
     </row>
     <row r="87" ht="28" customHeight="1">
       <c r="A87" s="11" t="inlineStr">
         <is>
-          <t>清算结算后台</t>
+          <t>数据管理/行情平台</t>
         </is>
       </c>
       <c r="B87" s="10" t="inlineStr">
@@ -5008,37 +5108,37 @@
       </c>
       <c r="C87" s="10" t="inlineStr">
         <is>
-          <t>F14-01</t>
+          <t>F12-02</t>
         </is>
       </c>
       <c r="D87" s="29" t="inlineStr">
         <is>
-          <t>DVP/FOP指令生成</t>
+          <t>数据质量校验</t>
         </is>
       </c>
       <c r="E87" s="11" t="inlineStr">
         <is>
-          <t>成交后自动生成交割指令，批量/单笔支持</t>
+          <t>异常值/缺失值/跳价自动检测，修复建议与人工审核</t>
         </is>
       </c>
       <c r="F87" s="11" t="inlineStr">
         <is>
-          <t>功能完整/边界测试/集成冒烟/性能基线</t>
-        </is>
-      </c>
-      <c r="G87" s="24" t="inlineStr">
-        <is>
-          <t>高</t>
+          <t>功能测试通过/正确率100%</t>
+        </is>
+      </c>
+      <c r="G87" s="25" t="inlineStr">
+        <is>
+          <t>中</t>
         </is>
       </c>
       <c r="H87" s="14" t="n">
-        <v>25</v>
+        <v>15</v>
       </c>
     </row>
     <row r="88" ht="28" customHeight="1">
       <c r="A88" s="11" t="inlineStr">
         <is>
-          <t>清算结算后台</t>
+          <t>数据管理/行情平台</t>
         </is>
       </c>
       <c r="B88" s="10" t="inlineStr">
@@ -5048,37 +5148,37 @@
       </c>
       <c r="C88" s="10" t="inlineStr">
         <is>
-          <t>F14-02</t>
+          <t>F12-03</t>
         </is>
       </c>
       <c r="D88" s="29" t="inlineStr">
         <is>
-          <t>中登/中债登接口</t>
+          <t>历史数据仓库</t>
         </is>
       </c>
       <c r="E88" s="11" t="inlineStr">
         <is>
-          <t>银行间债券（中债登）和交易所债券（中登）接口对接</t>
+          <t>Tick/日频历史行情存储，高效查询（ClickHouse/TimescaleDB）</t>
         </is>
       </c>
       <c r="F88" s="11" t="inlineStr">
         <is>
-          <t>p99延迟/误差率/精度验证/压测10k TPS</t>
-        </is>
-      </c>
-      <c r="G88" s="27" t="inlineStr">
-        <is>
-          <t>极高</t>
+          <t>功能完整/边界测试/集成冒烟/性能基线</t>
+        </is>
+      </c>
+      <c r="G88" s="24" t="inlineStr">
+        <is>
+          <t>高</t>
         </is>
       </c>
       <c r="H88" s="14" t="n">
-        <v>40</v>
+        <v>25</v>
       </c>
     </row>
     <row r="89" ht="28" customHeight="1">
       <c r="A89" s="11" t="inlineStr">
         <is>
-          <t>清算结算后台</t>
+          <t>数据管理/行情平台</t>
         </is>
       </c>
       <c r="B89" s="10" t="inlineStr">
@@ -5088,17 +5188,17 @@
       </c>
       <c r="C89" s="10" t="inlineStr">
         <is>
-          <t>F14-03</t>
+          <t>F12-04</t>
         </is>
       </c>
       <c r="D89" s="29" t="inlineStr">
         <is>
-          <t>待交割明细管理</t>
+          <t>收益率曲线发布</t>
         </is>
       </c>
       <c r="E89" s="11" t="inlineStr">
         <is>
-          <t>T+0/T+1待交割跟踪，提前预警可能失败交割</t>
+          <t>国债/政策行/高等级信用曲线实时发布，Kafka广播</t>
         </is>
       </c>
       <c r="F89" s="11" t="inlineStr">
@@ -5112,533 +5212,907 @@
         </is>
       </c>
       <c r="H89" s="14" t="n">
-        <v>25</v>
+        <v>20</v>
       </c>
     </row>
     <row r="90" ht="28" customHeight="1">
       <c r="A90" s="11" t="inlineStr">
         <is>
+          <t>数据管理/行情平台</t>
+        </is>
+      </c>
+      <c r="B90" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="C90" s="10" t="inlineStr">
+        <is>
+          <t>F12-05</t>
+        </is>
+      </c>
+      <c r="D90" s="29" t="inlineStr">
+        <is>
+          <t>估值价格服务</t>
+        </is>
+      </c>
+      <c r="E90" s="11" t="inlineStr">
+        <is>
+          <t>非活跃债券估值价格（中债估值基准），API接口提供</t>
+        </is>
+      </c>
+      <c r="F90" s="11" t="inlineStr">
+        <is>
+          <t>功能测试通过/正确率100%</t>
+        </is>
+      </c>
+      <c r="G90" s="25" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="H90" s="14" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="91" ht="20" customHeight="1">
+      <c r="A91" s="28" t="inlineStr">
+        <is>
+          <t>【P2】 交易对手管理  (Counterparty Management)</t>
+        </is>
+      </c>
+    </row>
+    <row r="92" ht="28" customHeight="1">
+      <c r="A92" s="11" t="inlineStr">
+        <is>
+          <t>交易对手管理</t>
+        </is>
+      </c>
+      <c r="B92" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="C92" s="10" t="inlineStr">
+        <is>
+          <t>F13-01</t>
+        </is>
+      </c>
+      <c r="D92" s="29" t="inlineStr">
+        <is>
+          <t>对手方评级与审批</t>
+        </is>
+      </c>
+      <c r="E92" s="11" t="inlineStr">
+        <is>
+          <t>内部信用评级模型，新增/变更交易对手审批流</t>
+        </is>
+      </c>
+      <c r="F92" s="11" t="inlineStr">
+        <is>
+          <t>功能测试通过/正确率100%</t>
+        </is>
+      </c>
+      <c r="G92" s="25" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="H92" s="14" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="93" ht="28" customHeight="1">
+      <c r="A93" s="11" t="inlineStr">
+        <is>
+          <t>交易对手管理</t>
+        </is>
+      </c>
+      <c r="B93" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="C93" s="10" t="inlineStr">
+        <is>
+          <t>F13-02</t>
+        </is>
+      </c>
+      <c r="D93" s="29" t="inlineStr">
+        <is>
+          <t>实时敞口聚合</t>
+        </is>
+      </c>
+      <c r="E93" s="11" t="inlineStr">
+        <is>
+          <t>跨产品交易对手名义/MtM敞口实时聚合，压力敞口（EPE）</t>
+        </is>
+      </c>
+      <c r="F93" s="11" t="inlineStr">
+        <is>
+          <t>功能完整/边界测试/集成冒烟/性能基线</t>
+        </is>
+      </c>
+      <c r="G93" s="24" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="H93" s="14" t="n">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="94" ht="28" customHeight="1">
+      <c r="A94" s="11" t="inlineStr">
+        <is>
+          <t>交易对手管理</t>
+        </is>
+      </c>
+      <c r="B94" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="C94" s="10" t="inlineStr">
+        <is>
+          <t>F13-03</t>
+        </is>
+      </c>
+      <c r="D94" s="29" t="inlineStr">
+        <is>
+          <t>ISDA/CSA协议管理</t>
+        </is>
+      </c>
+      <c r="E94" s="11" t="inlineStr">
+        <is>
+          <t>主协议文档管理，净额结算协议（Netting Set）配置</t>
+        </is>
+      </c>
+      <c r="F94" s="11" t="inlineStr">
+        <is>
+          <t>功能完整/边界测试/集成冒烟/性能基线</t>
+        </is>
+      </c>
+      <c r="G94" s="24" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="H94" s="14" t="n">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="95" ht="28" customHeight="1">
+      <c r="A95" s="11" t="inlineStr">
+        <is>
+          <t>交易对手管理</t>
+        </is>
+      </c>
+      <c r="B95" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="C95" s="10" t="inlineStr">
+        <is>
+          <t>F13-04</t>
+        </is>
+      </c>
+      <c r="D95" s="29" t="inlineStr">
+        <is>
+          <t>CVA/DVA/FVA计算</t>
+        </is>
+      </c>
+      <c r="E95" s="11" t="inlineStr">
+        <is>
+          <t>信用/债务/资金估值调整实时估算，敞口报告</t>
+        </is>
+      </c>
+      <c r="F95" s="11" t="inlineStr">
+        <is>
+          <t>p99延迟/误差率/精度验证/压测10k TPS</t>
+        </is>
+      </c>
+      <c r="G95" s="27" t="inlineStr">
+        <is>
+          <t>极高</t>
+        </is>
+      </c>
+      <c r="H95" s="14" t="n">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="96" ht="28" customHeight="1">
+      <c r="A96" s="11" t="inlineStr">
+        <is>
+          <t>交易对手管理</t>
+        </is>
+      </c>
+      <c r="B96" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="C96" s="10" t="inlineStr">
+        <is>
+          <t>F13-05</t>
+        </is>
+      </c>
+      <c r="D96" s="29" t="inlineStr">
+        <is>
+          <t>集中度与限额</t>
+        </is>
+      </c>
+      <c r="E96" s="11" t="inlineStr">
+        <is>
+          <t>对手方/集团合并敞口限额，超限审批与记录</t>
+        </is>
+      </c>
+      <c r="F96" s="11" t="inlineStr">
+        <is>
+          <t>功能测试通过/正确率100%</t>
+        </is>
+      </c>
+      <c r="G96" s="25" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="H96" s="14" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="97" ht="20" customHeight="1">
+      <c r="A97" s="28" t="inlineStr">
+        <is>
+          <t>【P2】 清算结算后台  (Clearing &amp; Settlement)</t>
+        </is>
+      </c>
+    </row>
+    <row r="98" ht="28" customHeight="1">
+      <c r="A98" s="11" t="inlineStr">
+        <is>
           <t>清算结算后台</t>
         </is>
       </c>
-      <c r="B90" s="10" t="inlineStr">
+      <c r="B98" s="10" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
       </c>
-      <c r="C90" s="10" t="inlineStr">
+      <c r="C98" s="10" t="inlineStr">
+        <is>
+          <t>F14-01</t>
+        </is>
+      </c>
+      <c r="D98" s="29" t="inlineStr">
+        <is>
+          <t>DVP/FOP指令生成</t>
+        </is>
+      </c>
+      <c r="E98" s="11" t="inlineStr">
+        <is>
+          <t>成交后自动生成交割指令，批量/单笔支持</t>
+        </is>
+      </c>
+      <c r="F98" s="11" t="inlineStr">
+        <is>
+          <t>功能完整/边界测试/集成冒烟/性能基线</t>
+        </is>
+      </c>
+      <c r="G98" s="24" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="H98" s="14" t="n">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="99" ht="28" customHeight="1">
+      <c r="A99" s="11" t="inlineStr">
+        <is>
+          <t>清算结算后台</t>
+        </is>
+      </c>
+      <c r="B99" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="C99" s="10" t="inlineStr">
+        <is>
+          <t>F14-02</t>
+        </is>
+      </c>
+      <c r="D99" s="29" t="inlineStr">
+        <is>
+          <t>中登/中债登接口</t>
+        </is>
+      </c>
+      <c r="E99" s="11" t="inlineStr">
+        <is>
+          <t>银行间债券（中债登）和交易所债券（中登）接口对接</t>
+        </is>
+      </c>
+      <c r="F99" s="11" t="inlineStr">
+        <is>
+          <t>p99延迟/误差率/精度验证/压测10k TPS</t>
+        </is>
+      </c>
+      <c r="G99" s="27" t="inlineStr">
+        <is>
+          <t>极高</t>
+        </is>
+      </c>
+      <c r="H99" s="14" t="n">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="100" ht="28" customHeight="1">
+      <c r="A100" s="11" t="inlineStr">
+        <is>
+          <t>清算结算后台</t>
+        </is>
+      </c>
+      <c r="B100" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="C100" s="10" t="inlineStr">
+        <is>
+          <t>F14-03</t>
+        </is>
+      </c>
+      <c r="D100" s="29" t="inlineStr">
+        <is>
+          <t>待交割明细管理</t>
+        </is>
+      </c>
+      <c r="E100" s="11" t="inlineStr">
+        <is>
+          <t>T+0/T+1待交割跟踪，提前预警可能失败交割</t>
+        </is>
+      </c>
+      <c r="F100" s="11" t="inlineStr">
+        <is>
+          <t>功能完整/边界测试/集成冒烟/性能基线</t>
+        </is>
+      </c>
+      <c r="G100" s="24" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="H100" s="14" t="n">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="101" ht="28" customHeight="1">
+      <c r="A101" s="11" t="inlineStr">
+        <is>
+          <t>清算结算后台</t>
+        </is>
+      </c>
+      <c r="B101" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="C101" s="10" t="inlineStr">
         <is>
           <t>F14-04</t>
         </is>
       </c>
-      <c r="D90" s="29" t="inlineStr">
+      <c r="D101" s="29" t="inlineStr">
         <is>
           <t>资金调拨确认</t>
         </is>
       </c>
-      <c r="E90" s="11" t="inlineStr">
+      <c r="E101" s="11" t="inlineStr">
         <is>
           <t>资金划拨指令生成，银行资金头寸确认，轧差净额</t>
         </is>
       </c>
-      <c r="F90" s="11" t="inlineStr">
+      <c r="F101" s="11" t="inlineStr">
         <is>
           <t>功能完整/边界测试/集成冒烟/性能基线</t>
         </is>
       </c>
-      <c r="G90" s="24" t="inlineStr">
+      <c r="G101" s="24" t="inlineStr">
         <is>
           <t>高</t>
         </is>
       </c>
-      <c r="H90" s="14" t="n">
+      <c r="H101" s="14" t="n">
         <v>25</v>
       </c>
     </row>
-    <row r="91" ht="28" customHeight="1">
-      <c r="A91" s="11" t="inlineStr">
+    <row r="102" ht="28" customHeight="1">
+      <c r="A102" s="11" t="inlineStr">
         <is>
           <t>清算结算后台</t>
         </is>
       </c>
-      <c r="B91" s="10" t="inlineStr">
+      <c r="B102" s="10" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
       </c>
-      <c r="C91" s="10" t="inlineStr">
+      <c r="C102" s="10" t="inlineStr">
         <is>
           <t>F14-05</t>
         </is>
       </c>
-      <c r="D91" s="29" t="inlineStr">
+      <c r="D102" s="29" t="inlineStr">
         <is>
           <t>交割失败处理</t>
         </is>
       </c>
-      <c r="E91" s="11" t="inlineStr">
+      <c r="E102" s="11" t="inlineStr">
         <is>
           <t>失败交割自动识别，补交割流程，罚息计算</t>
         </is>
       </c>
-      <c r="F91" s="11" t="inlineStr">
+      <c r="F102" s="11" t="inlineStr">
         <is>
           <t>功能测试通过/正确率100%</t>
         </is>
       </c>
-      <c r="G91" s="25" t="inlineStr">
+      <c r="G102" s="25" t="inlineStr">
         <is>
           <t>中</t>
         </is>
       </c>
-      <c r="H91" s="14" t="n">
+      <c r="H102" s="14" t="n">
         <v>20</v>
       </c>
     </row>
-    <row r="92" ht="20" customHeight="1">
-      <c r="A92" s="30" t="inlineStr">
+    <row r="103" ht="20" customHeight="1">
+      <c r="A103" s="30" t="inlineStr">
         <is>
           <t>【P3】 做市商系统  (Market Making)</t>
         </is>
       </c>
     </row>
-    <row r="93" ht="28" customHeight="1">
-      <c r="A93" s="17" t="inlineStr">
+    <row r="104" ht="28" customHeight="1">
+      <c r="A104" s="17" t="inlineStr">
         <is>
           <t>做市商系统</t>
         </is>
       </c>
-      <c r="B93" s="16" t="inlineStr">
+      <c r="B104" s="16" t="inlineStr">
         <is>
           <t>P3</t>
         </is>
       </c>
-      <c r="C93" s="16" t="inlineStr">
+      <c r="C104" s="16" t="inlineStr">
         <is>
           <t>F15-01</t>
         </is>
       </c>
-      <c r="D93" s="31" t="inlineStr">
+      <c r="D104" s="31" t="inlineStr">
         <is>
           <t>双边报价引擎</t>
         </is>
       </c>
-      <c r="E93" s="17" t="inlineStr">
+      <c r="E104" s="17" t="inlineStr">
         <is>
           <t>多品种同时双边报价，延迟&lt;5ms，报价宽度动态优化</t>
         </is>
       </c>
-      <c r="F93" s="17" t="inlineStr">
+      <c r="F104" s="17" t="inlineStr">
         <is>
           <t>p99延迟/误差率/精度验证/压测10k TPS</t>
         </is>
       </c>
-      <c r="G93" s="27" t="inlineStr">
+      <c r="G104" s="27" t="inlineStr">
         <is>
           <t>极高</t>
         </is>
       </c>
-      <c r="H93" s="19" t="n">
+      <c r="H104" s="19" t="n">
         <v>70</v>
       </c>
     </row>
-    <row r="94" ht="28" customHeight="1">
-      <c r="A94" s="17" t="inlineStr">
+    <row r="105" ht="28" customHeight="1">
+      <c r="A105" s="17" t="inlineStr">
         <is>
           <t>做市商系统</t>
         </is>
       </c>
-      <c r="B94" s="16" t="inlineStr">
+      <c r="B105" s="16" t="inlineStr">
         <is>
           <t>P3</t>
         </is>
       </c>
-      <c r="C94" s="16" t="inlineStr">
+      <c r="C105" s="16" t="inlineStr">
         <is>
           <t>F15-02</t>
         </is>
       </c>
-      <c r="D94" s="31" t="inlineStr">
+      <c r="D105" s="31" t="inlineStr">
         <is>
           <t>库存风险实时管理</t>
         </is>
       </c>
-      <c r="E94" s="17" t="inlineStr">
+      <c r="E105" s="17" t="inlineStr">
         <is>
           <t>做市库存PnL实时监控，Delta对冲自动触发</t>
         </is>
       </c>
-      <c r="F94" s="17" t="inlineStr">
+      <c r="F105" s="17" t="inlineStr">
         <is>
           <t>p99延迟/误差率/精度验证/压测10k TPS</t>
         </is>
       </c>
-      <c r="G94" s="27" t="inlineStr">
+      <c r="G105" s="27" t="inlineStr">
         <is>
           <t>极高</t>
         </is>
       </c>
-      <c r="H94" s="19" t="n">
+      <c r="H105" s="19" t="n">
         <v>60</v>
       </c>
     </row>
-    <row r="95" ht="28" customHeight="1">
-      <c r="A95" s="17" t="inlineStr">
+    <row r="106" ht="28" customHeight="1">
+      <c r="A106" s="17" t="inlineStr">
         <is>
           <t>做市商系统</t>
         </is>
       </c>
-      <c r="B95" s="16" t="inlineStr">
+      <c r="B106" s="16" t="inlineStr">
         <is>
           <t>P3</t>
         </is>
       </c>
-      <c r="C95" s="16" t="inlineStr">
+      <c r="C106" s="16" t="inlineStr">
         <is>
           <t>F15-03</t>
         </is>
       </c>
-      <c r="D95" s="31" t="inlineStr">
+      <c r="D106" s="31" t="inlineStr">
         <is>
           <t>报价优化算法</t>
         </is>
       </c>
-      <c r="E95" s="17" t="inlineStr">
+      <c r="E106" s="17" t="inlineStr">
         <is>
           <t>基于市场微结构理论动态调整bid-ask spread</t>
         </is>
       </c>
-      <c r="F95" s="17" t="inlineStr">
+      <c r="F106" s="17" t="inlineStr">
         <is>
           <t>p99延迟/误差率/精度验证/压测10k TPS</t>
         </is>
       </c>
-      <c r="G95" s="27" t="inlineStr">
+      <c r="G106" s="27" t="inlineStr">
         <is>
           <t>极高</t>
         </is>
       </c>
-      <c r="H95" s="19" t="n">
+      <c r="H106" s="19" t="n">
         <v>50</v>
       </c>
     </row>
-    <row r="96" ht="28" customHeight="1">
-      <c r="A96" s="17" t="inlineStr">
+    <row r="107" ht="28" customHeight="1">
+      <c r="A107" s="17" t="inlineStr">
         <is>
           <t>做市商系统</t>
         </is>
       </c>
-      <c r="B96" s="16" t="inlineStr">
+      <c r="B107" s="16" t="inlineStr">
         <is>
           <t>P3</t>
         </is>
       </c>
-      <c r="C96" s="16" t="inlineStr">
+      <c r="C107" s="16" t="inlineStr">
         <is>
           <t>F15-04</t>
         </is>
       </c>
-      <c r="D96" s="31" t="inlineStr">
+      <c r="D107" s="31" t="inlineStr">
         <is>
           <t>竞争力分析</t>
         </is>
       </c>
-      <c r="E96" s="17" t="inlineStr">
+      <c r="E107" s="17" t="inlineStr">
         <is>
           <t>与市场最优报价对比，中签率分析，策略调优</t>
         </is>
       </c>
-      <c r="F96" s="17" t="inlineStr">
+      <c r="F107" s="17" t="inlineStr">
         <is>
           <t>功能完整/边界测试/集成冒烟/性能基线</t>
         </is>
       </c>
-      <c r="G96" s="24" t="inlineStr">
+      <c r="G107" s="24" t="inlineStr">
         <is>
           <t>高</t>
         </is>
       </c>
-      <c r="H96" s="19" t="n">
+      <c r="H107" s="19" t="n">
         <v>25</v>
       </c>
     </row>
-    <row r="97" ht="28" customHeight="1">
-      <c r="A97" s="17" t="inlineStr">
+    <row r="108" ht="28" customHeight="1">
+      <c r="A108" s="17" t="inlineStr">
         <is>
           <t>做市商系统</t>
         </is>
       </c>
-      <c r="B97" s="16" t="inlineStr">
+      <c r="B108" s="16" t="inlineStr">
         <is>
           <t>P3</t>
         </is>
       </c>
-      <c r="C97" s="16" t="inlineStr">
+      <c r="C108" s="16" t="inlineStr">
         <is>
           <t>F15-05</t>
         </is>
       </c>
-      <c r="D97" s="31" t="inlineStr">
+      <c r="D108" s="31" t="inlineStr">
         <is>
           <t>交易对手管理集成</t>
         </is>
       </c>
-      <c r="E97" s="17" t="inlineStr">
+      <c r="E108" s="17" t="inlineStr">
         <is>
           <t>做市交易对手信用实时检查，额度占用同步更新</t>
         </is>
       </c>
-      <c r="F97" s="17" t="inlineStr">
+      <c r="F108" s="17" t="inlineStr">
         <is>
           <t>功能测试通过/正确率100%</t>
         </is>
       </c>
-      <c r="G97" s="25" t="inlineStr">
+      <c r="G108" s="25" t="inlineStr">
         <is>
           <t>中</t>
         </is>
       </c>
-      <c r="H97" s="19" t="n">
+      <c r="H108" s="19" t="n">
         <v>20</v>
       </c>
     </row>
-    <row r="98" ht="20" customHeight="1">
-      <c r="A98" s="30" t="inlineStr">
+    <row r="109" ht="20" customHeight="1">
+      <c r="A109" s="30" t="inlineStr">
         <is>
           <t>【P3】 外汇/外汇衍生品  (FX &amp; FX Derivatives)</t>
         </is>
       </c>
     </row>
-    <row r="99" ht="28" customHeight="1">
-      <c r="A99" s="17" t="inlineStr">
+    <row r="110" ht="28" customHeight="1">
+      <c r="A110" s="17" t="inlineStr">
         <is>
           <t>外汇/外汇衍生品</t>
         </is>
       </c>
-      <c r="B99" s="16" t="inlineStr">
+      <c r="B110" s="16" t="inlineStr">
         <is>
           <t>P3</t>
         </is>
       </c>
-      <c r="C99" s="16" t="inlineStr">
+      <c r="C110" s="16" t="inlineStr">
         <is>
           <t>F16-01</t>
         </is>
       </c>
-      <c r="D99" s="31" t="inlineStr">
+      <c r="D110" s="31" t="inlineStr">
         <is>
           <t>即期/远期报价</t>
         </is>
       </c>
-      <c r="E99" s="17" t="inlineStr">
+      <c r="E110" s="17" t="inlineStr">
         <is>
           <t>USD/CNY等主要货币对即期汇率+远期点数报价</t>
         </is>
       </c>
-      <c r="F99" s="17" t="inlineStr">
+      <c r="F110" s="17" t="inlineStr">
         <is>
           <t>功能完整/边界测试/集成冒烟/性能基线</t>
         </is>
       </c>
-      <c r="G99" s="24" t="inlineStr">
+      <c r="G110" s="24" t="inlineStr">
         <is>
           <t>高</t>
         </is>
       </c>
-      <c r="H99" s="19" t="n">
+      <c r="H110" s="19" t="n">
         <v>40</v>
       </c>
     </row>
-    <row r="100" ht="28" customHeight="1">
-      <c r="A100" s="17" t="inlineStr">
+    <row r="111" ht="28" customHeight="1">
+      <c r="A111" s="17" t="inlineStr">
         <is>
           <t>外汇/外汇衍生品</t>
         </is>
       </c>
-      <c r="B100" s="16" t="inlineStr">
+      <c r="B111" s="16" t="inlineStr">
         <is>
           <t>P3</t>
         </is>
       </c>
-      <c r="C100" s="16" t="inlineStr">
+      <c r="C111" s="16" t="inlineStr">
         <is>
           <t>F16-02</t>
         </is>
       </c>
-      <c r="D100" s="31" t="inlineStr">
+      <c r="D111" s="31" t="inlineStr">
         <is>
           <t>外汇期权（FXO）</t>
         </is>
       </c>
-      <c r="E100" s="17" t="inlineStr">
+      <c r="E111" s="17" t="inlineStr">
         <is>
           <t>欧式/美式FXO定价（Garman-Kohlhagen），Greeks</t>
         </is>
       </c>
-      <c r="F100" s="17" t="inlineStr">
+      <c r="F111" s="17" t="inlineStr">
         <is>
           <t>p99延迟/误差率/精度验证/压测10k TPS</t>
         </is>
       </c>
-      <c r="G100" s="27" t="inlineStr">
+      <c r="G111" s="27" t="inlineStr">
         <is>
           <t>极高</t>
         </is>
       </c>
-      <c r="H100" s="19" t="n">
+      <c r="H111" s="19" t="n">
         <v>60</v>
       </c>
     </row>
-    <row r="101" ht="28" customHeight="1">
-      <c r="A101" s="17" t="inlineStr">
+    <row r="112" ht="28" customHeight="1">
+      <c r="A112" s="17" t="inlineStr">
         <is>
           <t>外汇/外汇衍生品</t>
         </is>
       </c>
-      <c r="B101" s="16" t="inlineStr">
+      <c r="B112" s="16" t="inlineStr">
         <is>
           <t>P3</t>
         </is>
       </c>
-      <c r="C101" s="16" t="inlineStr">
+      <c r="C112" s="16" t="inlineStr">
         <is>
           <t>F16-03</t>
         </is>
       </c>
-      <c r="D101" s="31" t="inlineStr">
+      <c r="D112" s="31" t="inlineStr">
         <is>
           <t>NDF/NDO定价</t>
         </is>
       </c>
-      <c r="E101" s="17" t="inlineStr">
+      <c r="E112" s="17" t="inlineStr">
         <is>
           <t>不可交割远期/期权定价，境外对手对接</t>
         </is>
       </c>
-      <c r="F101" s="17" t="inlineStr">
+      <c r="F112" s="17" t="inlineStr">
         <is>
           <t>p99延迟/误差率/精度验证/压测10k TPS</t>
         </is>
       </c>
-      <c r="G101" s="27" t="inlineStr">
+      <c r="G112" s="27" t="inlineStr">
         <is>
           <t>极高</t>
         </is>
       </c>
-      <c r="H101" s="19" t="n">
+      <c r="H112" s="19" t="n">
         <v>50</v>
       </c>
     </row>
-    <row r="102" ht="28" customHeight="1">
-      <c r="A102" s="17" t="inlineStr">
+    <row r="113" ht="28" customHeight="1">
+      <c r="A113" s="17" t="inlineStr">
         <is>
           <t>外汇/外汇衍生品</t>
         </is>
       </c>
-      <c r="B102" s="16" t="inlineStr">
+      <c r="B113" s="16" t="inlineStr">
         <is>
           <t>P3</t>
         </is>
       </c>
-      <c r="C102" s="16" t="inlineStr">
+      <c r="C113" s="16" t="inlineStr">
         <is>
           <t>F16-04</t>
         </is>
       </c>
-      <c r="D102" s="31" t="inlineStr">
+      <c r="D113" s="31" t="inlineStr">
         <is>
           <t>跨货币敞口汇总</t>
         </is>
       </c>
-      <c r="E102" s="17" t="inlineStr">
+      <c r="E113" s="17" t="inlineStr">
         <is>
           <t>多币种资产折算人民币敞口，汇率风险VaR</t>
         </is>
       </c>
-      <c r="F102" s="17" t="inlineStr">
+      <c r="F113" s="17" t="inlineStr">
         <is>
           <t>功能完整/边界测试/集成冒烟/性能基线</t>
         </is>
       </c>
-      <c r="G102" s="24" t="inlineStr">
+      <c r="G113" s="24" t="inlineStr">
         <is>
           <t>高</t>
         </is>
       </c>
-      <c r="H102" s="19" t="n">
+      <c r="H113" s="19" t="n">
         <v>30</v>
       </c>
     </row>
-    <row r="103" ht="28" customHeight="1">
-      <c r="A103" s="17" t="inlineStr">
+    <row r="114" ht="28" customHeight="1">
+      <c r="A114" s="17" t="inlineStr">
         <is>
           <t>外汇/外汇衍生品</t>
         </is>
       </c>
-      <c r="B103" s="16" t="inlineStr">
+      <c r="B114" s="16" t="inlineStr">
         <is>
           <t>P3</t>
         </is>
       </c>
-      <c r="C103" s="16" t="inlineStr">
+      <c r="C114" s="16" t="inlineStr">
         <is>
           <t>F16-05</t>
         </is>
       </c>
-      <c r="D103" s="31" t="inlineStr">
+      <c r="D114" s="31" t="inlineStr">
         <is>
           <t>CFETS/外汇局接口</t>
         </is>
       </c>
-      <c r="E103" s="17" t="inlineStr">
+      <c r="E114" s="17" t="inlineStr">
         <is>
           <t>银行间外汇市场CFETS接口，外汇局合规报送</t>
         </is>
       </c>
-      <c r="F103" s="17" t="inlineStr">
+      <c r="F114" s="17" t="inlineStr">
         <is>
           <t>功能完整/边界测试/集成冒烟/性能基线</t>
         </is>
       </c>
-      <c r="G103" s="24" t="inlineStr">
+      <c r="G114" s="24" t="inlineStr">
         <is>
           <t>高</t>
         </is>
       </c>
-      <c r="H103" s="19" t="n">
+      <c r="H114" s="19" t="n">
         <v>35</v>
       </c>
     </row>
-    <row r="104">
-      <c r="A104" s="20" t="inlineStr">
+    <row r="115">
+      <c r="A115" s="20" t="inlineStr">
         <is>
           <t>总计功能数 / Total Function Points</t>
         </is>
       </c>
-      <c r="H104" s="21">
-        <f>SUM(H3:H103)</f>
+      <c r="H115" s="21">
+        <f>SUM(H3:H114)</f>
         <v/>
       </c>
     </row>
   </sheetData>
   <mergeCells count="18">
-    <mergeCell ref="A80:H80"/>
-    <mergeCell ref="A62:H62"/>
     <mergeCell ref="A3:H3"/>
     <mergeCell ref="A30:H30"/>
-    <mergeCell ref="A92:H92"/>
-    <mergeCell ref="A55:H55"/>
-    <mergeCell ref="A86:H86"/>
+    <mergeCell ref="A91:H91"/>
+    <mergeCell ref="A109:H109"/>
+    <mergeCell ref="A73:H73"/>
+    <mergeCell ref="A115:G115"/>
     <mergeCell ref="A10:H10"/>
     <mergeCell ref="A42:H42"/>
-    <mergeCell ref="A98:H98"/>
+    <mergeCell ref="A60:H60"/>
+    <mergeCell ref="A85:H85"/>
     <mergeCell ref="A36:H36"/>
-    <mergeCell ref="A49:H49"/>
-    <mergeCell ref="A68:H68"/>
-    <mergeCell ref="A104:G104"/>
+    <mergeCell ref="A66:H66"/>
+    <mergeCell ref="A103:H103"/>
     <mergeCell ref="A1:H1"/>
     <mergeCell ref="A23:H23"/>
-    <mergeCell ref="A74:H74"/>
+    <mergeCell ref="A79:H79"/>
+    <mergeCell ref="A97:H97"/>
     <mergeCell ref="A17:H17"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -6711,4 +7185,1005 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J28"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="48" customWidth="1" min="4" max="4"/>
+    <col width="26" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="6" max="6"/>
+    <col width="8" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="8" max="8"/>
+    <col width="7" customWidth="1" min="9" max="9"/>
+    <col width="18" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="24" customHeight="1">
+      <c r="A1" s="39" t="inlineStr">
+        <is>
+          <t>系统详情：组合管理+绩效归因  |  Portfolio Management &amp; Performance Attribution</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="36" customHeight="1">
+      <c r="A2" s="40" t="inlineStr">
+        <is>
+          <t>核心目标（Slide 44）：为FICC投资组合管理提供全面解决方案，通过分析投资组合头寸、风险计量、绩效归因，为投资经理在资产管理、组合构建、组合再平衡、指数投资等方面赋能。</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="28" customHeight="1">
+      <c r="A3" s="41" t="inlineStr">
+        <is>
+          <t>架构层次：  【数据层】交易数据 / 头寸数据 / 行情数据 / 估值数据  →  【量化底座】定价计算 · 利率曲线 · 因子模型  →  【组合分析平台】6大功能域（见下表）</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="28" customHeight="1">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>功能域</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>编号</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>功能名称</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>功能描述（来源Slide44）</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>验收标准</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>集成依赖</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>复杂度</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>预估(人天)</t>
+        </is>
+      </c>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t>优先级</t>
+        </is>
+      </c>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>备注</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="18" customHeight="1">
+      <c r="A5" s="23" t="inlineStr">
+        <is>
+          <t>A. 组合分析</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="48" customHeight="1">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>A. 组合分析</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>F07-01</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>债券横截面与时序分析</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>跨品种横截面信号挖掘（利差/久期偏差），历史时序趋势与均值回归分析，支持日/周/月时间窗口</t>
+        </is>
+      </c>
+      <c r="E6" s="5" t="inlineStr">
+        <is>
+          <t>横截面信号与实际收益相关性&gt;0.3；时序模型回测夏普&gt;0.5</t>
+        </is>
+      </c>
+      <c r="F6" s="5" t="inlineStr">
+        <is>
+          <t>AMD行情平台 / 估值数据</t>
+        </is>
+      </c>
+      <c r="G6" s="42" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="H6" s="8" t="n">
+        <v>35</v>
+      </c>
+      <c r="I6" s="6" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="J6" s="5" t="inlineStr">
+        <is>
+          <t>Slide44首项分析能力</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="48" customHeight="1">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>A. 组合分析</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>F07-02</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>相对价值分析</t>
+        </is>
+      </c>
+      <c r="D7" s="5" t="inlineStr">
+        <is>
+          <t>利差/Z-spread/OAS相对价值计算，历史分位数定位，跨品种套利信号识别，个券评分</t>
+        </is>
+      </c>
+      <c r="E7" s="5" t="inlineStr">
+        <is>
+          <t>OAS计算误差&lt;1bps；分位数计算覆盖5年历史</t>
+        </is>
+      </c>
+      <c r="F7" s="5" t="inlineStr">
+        <is>
+          <t>量化定价引擎 / AMD行情</t>
+        </is>
+      </c>
+      <c r="G7" s="42" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="H7" s="8" t="n">
+        <v>30</v>
+      </c>
+      <c r="I7" s="6" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="J7" s="5" t="inlineStr">
+        <is>
+          <t>投资经理最常用分析工具</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="48" customHeight="1">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>A. 组合分析</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>F07-03</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="inlineStr">
+        <is>
+          <t>组合相关度分析</t>
+        </is>
+      </c>
+      <c r="D8" s="5" t="inlineStr">
+        <is>
+          <t>资产间收益相关矩阵计算（滚动窗口60/120/250日），组合集中度风险识别，分散化系数监控</t>
+        </is>
+      </c>
+      <c r="E8" s="5" t="inlineStr">
+        <is>
+          <t>相关矩阵计算耗时&lt;30s（500券组合）</t>
+        </is>
+      </c>
+      <c r="F8" s="5" t="inlineStr">
+        <is>
+          <t>IBOR头寸 / AMD历史行情</t>
+        </is>
+      </c>
+      <c r="G8" s="43" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="H8" s="8" t="n">
+        <v>25</v>
+      </c>
+      <c r="I8" s="6" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="J8" s="5" t="inlineStr"/>
+    </row>
+    <row r="9" ht="18" customHeight="1">
+      <c r="A9" s="41" t="inlineStr">
+        <is>
+          <t>B. 风险计量</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="48" customHeight="1">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>B. 风险计量</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>F07-04</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="inlineStr">
+        <is>
+          <t>情景分析</t>
+        </is>
+      </c>
+      <c r="D10" s="5" t="inlineStr">
+        <is>
+          <t>利率平移/扭转/蝶式、信用利差扩大、流动性冲击三类情景；自定义情景编辑器；多情景P&amp;L并行对比</t>
+        </is>
+      </c>
+      <c r="E10" s="5" t="inlineStr">
+        <is>
+          <t>情景P&amp;L计算与手工核算误差&lt;0.5%；支持≥20个情景并行</t>
+        </is>
+      </c>
+      <c r="F10" s="5" t="inlineStr">
+        <is>
+          <t>FICC风险计量平台 / 量化定价引擎</t>
+        </is>
+      </c>
+      <c r="G10" s="42" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="H10" s="8" t="n">
+        <v>35</v>
+      </c>
+      <c r="I10" s="6" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="J10" s="5" t="inlineStr">
+        <is>
+          <t>复用风险计量模块情景库</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="48" customHeight="1">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>B. 风险计量</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>F07-05</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="inlineStr">
+        <is>
+          <t>敏感度分析</t>
+        </is>
+      </c>
+      <c r="D11" s="5" t="inlineStr">
+        <is>
+          <t>久期/DV01/凸度/利差/Vega敏感度多因子并行计算，组合层面聚合，对冲比率建议输出</t>
+        </is>
+      </c>
+      <c r="E11" s="5" t="inlineStr">
+        <is>
+          <t>DV01与Bloomberg基准误差&lt;0.5bps</t>
+        </is>
+      </c>
+      <c r="F11" s="5" t="inlineStr">
+        <is>
+          <t>量化定价引擎Greeks接口</t>
+        </is>
+      </c>
+      <c r="G11" s="42" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="H11" s="8" t="n">
+        <v>25</v>
+      </c>
+      <c r="I11" s="6" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="J11" s="5" t="inlineStr"/>
+    </row>
+    <row r="12" ht="48" customHeight="1">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>B. 风险计量</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>F07-06</t>
+        </is>
+      </c>
+      <c r="C12" s="4" t="inlineStr">
+        <is>
+          <t>极端事件分析</t>
+        </is>
+      </c>
+      <c r="D12" s="5" t="inlineStr">
+        <is>
+          <t>内置924行情/2015股灾/2020疫情等8+极端情景，组合尾部损失分布，ES(99%)计算</t>
+        </is>
+      </c>
+      <c r="E12" s="5" t="inlineStr">
+        <is>
+          <t>历史情景复现误差&lt;1%；与风险计量平台情景库共享</t>
+        </is>
+      </c>
+      <c r="F12" s="5" t="inlineStr">
+        <is>
+          <t>FICC风险计量平台</t>
+        </is>
+      </c>
+      <c r="G12" s="42" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="H12" s="8" t="n">
+        <v>30</v>
+      </c>
+      <c r="I12" s="6" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="J12" s="5" t="inlineStr">
+        <is>
+          <t>与风险计量平台共享情景库</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="18" customHeight="1">
+      <c r="A13" s="44" t="inlineStr">
+        <is>
+          <t>C. 绩效归因</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="48" customHeight="1">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>C. 绩效归因</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>F07-07</t>
+        </is>
+      </c>
+      <c r="C14" s="4" t="inlineStr">
+        <is>
+          <t>指数比较分析</t>
+        </is>
+      </c>
+      <c r="D14" s="5" t="inlineStr">
+        <is>
+          <t>对标中债综合/信用/政策行/定制基准指数；跟踪误差（TE）日频实时监控；超额Alpha三因子分解</t>
+        </is>
+      </c>
+      <c r="E14" s="5" t="inlineStr">
+        <is>
+          <t>TE计算误差&lt;1bps；支持≥10个基准指数同时跟踪</t>
+        </is>
+      </c>
+      <c r="F14" s="5" t="inlineStr">
+        <is>
+          <t>AMD中债估值 / IBOR持仓</t>
+        </is>
+      </c>
+      <c r="G14" s="43" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="H14" s="8" t="n">
+        <v>25</v>
+      </c>
+      <c r="I14" s="6" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="J14" s="5" t="inlineStr">
+        <is>
+          <t>中债指数数据接入为前提</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="48" customHeight="1">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>C. 绩效归因</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>F07-08</t>
+        </is>
+      </c>
+      <c r="C15" s="4" t="inlineStr">
+        <is>
+          <t>绩效归因（Brinson模型）</t>
+        </is>
+      </c>
+      <c r="D15" s="5" t="inlineStr">
+        <is>
+          <t>BHB三效应：资产配置/个券选择/交互效应；日/周/月/季多时间维度；报告PDF自动生成</t>
+        </is>
+      </c>
+      <c r="E15" s="5" t="inlineStr">
+        <is>
+          <t>Brinson归因结果与Bloomberg AIM误差&lt;0.1%；报告T+1 9:00前自动生成</t>
+        </is>
+      </c>
+      <c r="F15" s="5" t="inlineStr">
+        <is>
+          <t>IBOR持仓 / AMD行情 / 指数数据</t>
+        </is>
+      </c>
+      <c r="G15" s="42" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="H15" s="8" t="n">
+        <v>40</v>
+      </c>
+      <c r="I15" s="6" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="J15" s="5" t="inlineStr">
+        <is>
+          <t>核心差异化功能，对标SimCorp/Aladdin</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="18" customHeight="1">
+      <c r="A16" s="44" t="inlineStr">
+        <is>
+          <t>D. 组合优化与再平衡</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="48" customHeight="1">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>D. 组合优化与再平衡</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>F07-09</t>
+        </is>
+      </c>
+      <c r="C17" s="4" t="inlineStr">
+        <is>
+          <t>虚拟组合分析</t>
+        </is>
+      </c>
+      <c r="D17" s="5" t="inlineStr">
+        <is>
+          <t>组合调整前后净值/风险/收益效果模拟（纸面交易）；市场冲击成本预估；多方案结果对比展示</t>
+        </is>
+      </c>
+      <c r="E17" s="5" t="inlineStr">
+        <is>
+          <t>虚拟组合模拟结果与真实执行偏差&lt;0.3%</t>
+        </is>
+      </c>
+      <c r="F17" s="5" t="inlineStr">
+        <is>
+          <t>IBOR / 现券交易系统（冲击模型）</t>
+        </is>
+      </c>
+      <c r="G17" s="42" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="H17" s="8" t="n">
+        <v>20</v>
+      </c>
+      <c r="I17" s="6" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="J17" s="5" t="inlineStr"/>
+    </row>
+    <row r="18" ht="48" customHeight="1">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>D. 组合优化与再平衡</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>F07-10</t>
+        </is>
+      </c>
+      <c r="C18" s="4" t="inlineStr">
+        <is>
+          <t>再平衡方案试算与比较</t>
+        </is>
+      </c>
+      <c r="D18" s="5" t="inlineStr">
+        <is>
+          <t>久期/集中度/流动性/合规约束联合优化（二次规划QP），多方案并行试算，最优路径推荐</t>
+        </is>
+      </c>
+      <c r="E18" s="5" t="inlineStr">
+        <is>
+          <t>QP求解100券组合&lt;5s；约束满足率100%</t>
+        </is>
+      </c>
+      <c r="F18" s="5" t="inlineStr">
+        <is>
+          <t>事前风控/合规 / IBOR / 现券系统</t>
+        </is>
+      </c>
+      <c r="G18" s="42" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="H18" s="8" t="n">
+        <v>35</v>
+      </c>
+      <c r="I18" s="6" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="J18" s="5" t="inlineStr">
+        <is>
+          <t>QP求解器选型：CVXPY/Gurobi</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="48" customHeight="1">
+      <c r="A19" s="11" t="inlineStr">
+        <is>
+          <t>D. 组合优化与再平衡</t>
+        </is>
+      </c>
+      <c r="B19" s="10" t="inlineStr">
+        <is>
+          <t>F07-11</t>
+        </is>
+      </c>
+      <c r="C19" s="29" t="inlineStr">
+        <is>
+          <t>资产配置策略分析</t>
+        </is>
+      </c>
+      <c r="D19" s="11" t="inlineStr">
+        <is>
+          <t>宏观因子（利率周期/信用周期/流动性）驱动大类资产配置模型；动态权重优化建议；历史回测验证</t>
+        </is>
+      </c>
+      <c r="E19" s="11" t="inlineStr">
+        <is>
+          <t>回测期≥5年；模型收益预测方向胜率&gt;55%</t>
+        </is>
+      </c>
+      <c r="F19" s="11" t="inlineStr">
+        <is>
+          <t>AMD宏观数据 / 因子模型</t>
+        </is>
+      </c>
+      <c r="G19" s="42" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="H19" s="14" t="n">
+        <v>40</v>
+      </c>
+      <c r="I19" s="12" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="J19" s="11" t="inlineStr">
+        <is>
+          <t>Phase 1后期或Phase 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="48" customHeight="1">
+      <c r="A20" s="11" t="inlineStr">
+        <is>
+          <t>D. 组合优化与再平衡</t>
+        </is>
+      </c>
+      <c r="B20" s="10" t="inlineStr">
+        <is>
+          <t>F07-12</t>
+        </is>
+      </c>
+      <c r="C20" s="29" t="inlineStr">
+        <is>
+          <t>固收+策略分析</t>
+        </is>
+      </c>
+      <c r="D20" s="11" t="inlineStr">
+        <is>
+          <t>债券底仓+衍生品增强策略P&amp;L归因，风险分解（利率/信用/期权贡献），固收+产品净值模拟</t>
+        </is>
+      </c>
+      <c r="E20" s="11" t="inlineStr">
+        <is>
+          <t>固收+净值模拟与实际偏差&lt;0.5%</t>
+        </is>
+      </c>
+      <c r="F20" s="11" t="inlineStr">
+        <is>
+          <t>IBOR / 利率衍生品系统（Phase 2）</t>
+        </is>
+      </c>
+      <c r="G20" s="42" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="H20" s="14" t="n">
+        <v>30</v>
+      </c>
+      <c r="I20" s="12" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="J20" s="11" t="inlineStr">
+        <is>
+          <t>依赖利率衍生品模块</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="48" customHeight="1">
+      <c r="A21" s="11" t="inlineStr">
+        <is>
+          <t>D. 组合优化与再平衡</t>
+        </is>
+      </c>
+      <c r="B21" s="10" t="inlineStr">
+        <is>
+          <t>F07-13</t>
+        </is>
+      </c>
+      <c r="C21" s="29" t="inlineStr">
+        <is>
+          <t>量化策略组合分析</t>
+        </is>
+      </c>
+      <c r="D21" s="11" t="inlineStr">
+        <is>
+          <t>多策略组合叠加容量约束，策略相关性管理，Sharpe/最大回撤/Calmar实时监控，策略权重优化</t>
+        </is>
+      </c>
+      <c r="E21" s="11" t="inlineStr">
+        <is>
+          <t>策略容量计算误差&lt;5%；组合Sharpe≥1.2（回测）</t>
+        </is>
+      </c>
+      <c r="F21" s="11" t="inlineStr">
+        <is>
+          <t>策略投资/量化系统</t>
+        </is>
+      </c>
+      <c r="G21" s="42" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="H21" s="14" t="n">
+        <v>35</v>
+      </c>
+      <c r="I21" s="12" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="J21" s="11" t="inlineStr">
+        <is>
+          <t>与策略投资模块深度整合</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="18" customHeight="1">
+      <c r="A22" s="30" t="inlineStr">
+        <is>
+          <t>E. 流动性管理</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="48" customHeight="1">
+      <c r="A23" s="5" t="inlineStr">
+        <is>
+          <t>E. 流动性管理</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t>F07-14</t>
+        </is>
+      </c>
+      <c r="C23" s="4" t="inlineStr">
+        <is>
+          <t>流动性分析</t>
+        </is>
+      </c>
+      <c r="D23" s="5" t="inlineStr">
+        <is>
+          <t>逐券换手率/市场深度评估（日均成交量法），组合变现能力分析，流动性压力下变现损失（LVaR）估算</t>
+        </is>
+      </c>
+      <c r="E23" s="5" t="inlineStr">
+        <is>
+          <t>LVaR计算与市场基准误差&lt;5%；日均成交量数据覆盖≥95%持仓</t>
+        </is>
+      </c>
+      <c r="F23" s="5" t="inlineStr">
+        <is>
+          <t>AMD行情（成交量） / IBOR持仓</t>
+        </is>
+      </c>
+      <c r="G23" s="43" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="H23" s="8" t="n">
+        <v>20</v>
+      </c>
+      <c r="I23" s="6" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="J23" s="5" t="inlineStr">
+        <is>
+          <t>监管流动性要求驱动</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="18" customHeight="1">
+      <c r="A24" s="45" t="inlineStr">
+        <is>
+          <t>F. 量化底座集成</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="48" customHeight="1">
+      <c r="A25" s="11" t="inlineStr">
+        <is>
+          <t>F. 量化底座集成</t>
+        </is>
+      </c>
+      <c r="B25" s="10" t="inlineStr">
+        <is>
+          <t>F07-15</t>
+        </is>
+      </c>
+      <c r="C25" s="29" t="inlineStr">
+        <is>
+          <t>定价计算集成</t>
+        </is>
+      </c>
+      <c r="D25" s="11" t="inlineStr">
+        <is>
+          <t>调用量化定价引擎实时估值与Greeks；支持含权债/可转债/IRS；结果缓存（Redis）与Kafka推送</t>
+        </is>
+      </c>
+      <c r="E25" s="11" t="inlineStr">
+        <is>
+          <t>定价API p99&lt;200ms；日终全量估值&lt;30min（10万券）</t>
+        </is>
+      </c>
+      <c r="F25" s="11" t="inlineStr">
+        <is>
+          <t>量化定价引擎（P2模块）</t>
+        </is>
+      </c>
+      <c r="G25" s="42" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="H25" s="14" t="n">
+        <v>20</v>
+      </c>
+      <c r="I25" s="12" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="J25" s="11" t="inlineStr">
+        <is>
+          <t>Phase 1用AMD估值代替，Phase 2升级</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="48" customHeight="1">
+      <c r="A26" s="5" t="inlineStr">
+        <is>
+          <t>F. 量化底座集成</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="inlineStr">
+        <is>
+          <t>F07-16</t>
+        </is>
+      </c>
+      <c r="C26" s="4" t="inlineStr">
+        <is>
+          <t>利率曲线集成</t>
+        </is>
+      </c>
+      <c r="D26" s="5" t="inlineStr">
+        <is>
+          <t>多曲线实时消费（国债/政策行/AAA信用/OIS）；Nelson-Siegel参数提取（水平/斜率/曲率）；敏感度映射</t>
+        </is>
+      </c>
+      <c r="E26" s="5" t="inlineStr">
+        <is>
+          <t>曲线更新延迟&lt;1s；NS参数拟合R²&gt;0.999</t>
+        </is>
+      </c>
+      <c r="F26" s="5" t="inlineStr">
+        <is>
+          <t>AMD行情平台 / 量化定价引擎</t>
+        </is>
+      </c>
+      <c r="G26" s="43" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="H26" s="8" t="n">
+        <v>15</v>
+      </c>
+      <c r="I26" s="6" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="J26" s="5" t="inlineStr"/>
+    </row>
+    <row r="27" ht="48" customHeight="1">
+      <c r="A27" s="5" t="inlineStr">
+        <is>
+          <t>F. 量化底座集成</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="inlineStr">
+        <is>
+          <t>F07-17</t>
+        </is>
+      </c>
+      <c r="C27" s="4" t="inlineStr">
+        <is>
+          <t>因子模型</t>
+        </is>
+      </c>
+      <c r="D27" s="5" t="inlineStr">
+        <is>
+          <t>多因子风险模型（利率/信用/流动性/行业因子）；Alpha因子库（≥20个因子）；因子暴露实时计算与归因</t>
+        </is>
+      </c>
+      <c r="E27" s="5" t="inlineStr">
+        <is>
+          <t>因子模型解释方差&gt;80%；Alpha IC均值&gt;0.05</t>
+        </is>
+      </c>
+      <c r="F27" s="5" t="inlineStr">
+        <is>
+          <t>AMD历史行情 / IBOR持仓</t>
+        </is>
+      </c>
+      <c r="G27" s="42" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="H27" s="8" t="n">
+        <v>40</v>
+      </c>
+      <c r="I27" s="6" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="J27" s="5" t="inlineStr">
+        <is>
+          <t>复用策略投资模块因子库</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="41" t="inlineStr">
+        <is>
+          <t>合计 17项功能  |  P1: 12项  |  P2: 5项  |  来源：Slide 44 + 扩展</t>
+        </is>
+      </c>
+      <c r="H28" s="21">
+        <f>SUM(H5:H27)</f>
+        <v/>
+      </c>
+      <c r="I28" s="35" t="inlineStr"/>
+      <c r="J28" s="35" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <mergeCells count="10">
+    <mergeCell ref="A1:J1"/>
+    <mergeCell ref="A5:J5"/>
+    <mergeCell ref="A22:J22"/>
+    <mergeCell ref="A16:J16"/>
+    <mergeCell ref="A9:J9"/>
+    <mergeCell ref="A28:G28"/>
+    <mergeCell ref="A3:J3"/>
+    <mergeCell ref="A24:J24"/>
+    <mergeCell ref="A2:J2"/>
+    <mergeCell ref="A13:J13"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" fitToWidth="1"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Expand module 05 异常交易风控 from Slide 50
12 functions across 3 domains: AI智能引擎 (LLM/RAG/Agent/MCP),
异常识别引擎 (9 specific trade anomaly types), 运营与报告.
Adds LLM+RAG+Agent stack as key differentiator. Duration 6→8m, 42→55pm.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Feasibility_analysis/FICC_Gap_Analysis.xlsx
+++ b/Feasibility_analysis/FICC_Gap_Analysis.xlsx
@@ -14,7 +14,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="详情_IBOR投资账薄管理" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="详情_现券交易系统" sheetId="6" state="visible" r:id="rId6"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="详情_FICC风险计量平台" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="详情_组合管理+绩效归因" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="详情_异常交易风控" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="详情_组合管理+绩效归因" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Area" localSheetId="0">'差距分析总表'!$A$1:$P$17</definedName>
@@ -1201,17 +1202,17 @@
         </is>
       </c>
       <c r="M7" s="3" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="N7" s="3" t="n">
         <v>8</v>
       </c>
       <c r="O7" s="8" t="n">
-        <v>42</v>
+        <v>55</v>
       </c>
       <c r="P7" s="5" t="inlineStr">
         <is>
-          <t>监管驱动，AI差异化，快速商业化</t>
+          <t>监管驱动，AI差异化（LLM+RAG+Agent+MCP），快速商业化；对应PPT Slide 50</t>
         </is>
       </c>
     </row>
@@ -1921,7 +1922,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H163"/>
+  <dimension ref="A1:H170"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -5236,12 +5237,12 @@
       </c>
       <c r="D88" s="4" t="inlineStr">
         <is>
-          <t>实时CEP监控引擎</t>
+          <t>LLM大语言模型应用</t>
         </is>
       </c>
       <c r="E88" s="5" t="inlineStr">
         <is>
-          <t>基于复杂事件处理（CEP），毫秒级事件流检测，滑动窗口聚合</t>
+          <t>客户意图识别，自然语言处理交易描述，智能报告自动生成，新规合规解读</t>
         </is>
       </c>
       <c r="F88" s="5" t="inlineStr">
@@ -5255,7 +5256,7 @@
         </is>
       </c>
       <c r="H88" s="8" t="n">
-        <v>50</v>
+        <v>40</v>
       </c>
     </row>
     <row r="89" ht="28" customHeight="1">
@@ -5276,12 +5277,12 @@
       </c>
       <c r="D89" s="4" t="inlineStr">
         <is>
-          <t>异常价格检测</t>
+          <t>RAG检索增强生成</t>
         </is>
       </c>
       <c r="E89" s="5" t="inlineStr">
         <is>
-          <t>基于历史分位数/实时行情计算价格偏离度，动态阈值自适应</t>
+          <t>监管规则知识库构建，新规则智能固化，合规智能问答，上下文理解与规则推理</t>
         </is>
       </c>
       <c r="F89" s="5" t="inlineStr">
@@ -5295,7 +5296,7 @@
         </is>
       </c>
       <c r="H89" s="8" t="n">
-        <v>25</v>
+        <v>30</v>
       </c>
     </row>
     <row r="90" ht="28" customHeight="1">
@@ -5316,12 +5317,12 @@
       </c>
       <c r="D90" s="4" t="inlineStr">
         <is>
-          <t>AI异常识别模型</t>
+          <t>Agent智能体</t>
         </is>
       </c>
       <c r="E90" s="5" t="inlineStr">
         <is>
-          <t>机器学习（XGBoost/LSTM）训练异常交易识别模型，在线推理</t>
+          <t>异常处置任务自动化，决策支持工作流，多步骤异常核查流程优化，自动推送处置建议</t>
         </is>
       </c>
       <c r="F90" s="5" t="inlineStr">
@@ -5335,7 +5336,7 @@
         </is>
       </c>
       <c r="H90" s="8" t="n">
-        <v>40</v>
+        <v>30</v>
       </c>
     </row>
     <row r="91" ht="28" customHeight="1">
@@ -5356,12 +5357,12 @@
       </c>
       <c r="D91" s="4" t="inlineStr">
         <is>
-          <t>规则引擎（可配置）</t>
+          <t>MCP外部服务集成</t>
         </is>
       </c>
       <c r="E91" s="5" t="inlineStr">
         <is>
-          <t>No-Code规则配置界面，合规人员自助维护检测规则</t>
+          <t>外部数据源调用接口，固化规则调用标准协议，与行情/持仓/交易系统数据对接</t>
         </is>
       </c>
       <c r="F91" s="5" t="inlineStr">
@@ -5396,39 +5397,72 @@
       </c>
       <c r="D92" s="4" t="inlineStr">
         <is>
-          <t>监管报送自动化</t>
+          <t>代持与反向交易识别</t>
         </is>
       </c>
       <c r="E92" s="5" t="inlineStr">
         <is>
-          <t>一键生成证监会/人行格式异常交易报告，历史追溯查询</t>
+          <t>代持相关交易检测，同券同额反向识别，多日反向低频交易模式识别</t>
         </is>
       </c>
       <c r="F92" s="5" t="inlineStr">
         <is>
-          <t>功能测试通过/正确率100%</t>
-        </is>
-      </c>
-      <c r="G92" s="24" t="inlineStr">
-        <is>
-          <t>中</t>
+          <t>功能完整/边界测试/集成冒烟/性能基线</t>
+        </is>
+      </c>
+      <c r="G92" s="23" t="inlineStr">
+        <is>
+          <t>高</t>
         </is>
       </c>
       <c r="H92" s="8" t="n">
         <v>25</v>
       </c>
     </row>
-    <row r="93" ht="20" customHeight="1">
-      <c r="A93" s="22" t="inlineStr">
-        <is>
-          <t>【P1】 事前风控/合规  (Pre-trade Risk)</t>
-        </is>
+    <row r="93" ht="28" customHeight="1">
+      <c r="A93" s="5" t="inlineStr">
+        <is>
+          <t>异常交易风控</t>
+        </is>
+      </c>
+      <c r="B93" s="3" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="C93" s="3" t="inlineStr">
+        <is>
+          <t>F05-06</t>
+        </is>
+      </c>
+      <c r="D93" s="4" t="inlineStr">
+        <is>
+          <t>价格行为异常检测</t>
+        </is>
+      </c>
+      <c r="E93" s="5" t="inlineStr">
+        <is>
+          <t>高买低卖行为识别，信用债价格异常检测，基于历史分位数与实时行情动态偏离度计算</t>
+        </is>
+      </c>
+      <c r="F93" s="5" t="inlineStr">
+        <is>
+          <t>功能完整/边界测试/集成冒烟/性能基线</t>
+        </is>
+      </c>
+      <c r="G93" s="23" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="H93" s="8" t="n">
+        <v>25</v>
       </c>
     </row>
     <row r="94" ht="28" customHeight="1">
       <c r="A94" s="5" t="inlineStr">
         <is>
-          <t>事前风控/合规</t>
+          <t>异常交易风控</t>
         </is>
       </c>
       <c r="B94" s="3" t="inlineStr">
@@ -5438,17 +5472,17 @@
       </c>
       <c r="C94" s="3" t="inlineStr">
         <is>
-          <t>F06-01</t>
+          <t>F05-07</t>
         </is>
       </c>
       <c r="D94" s="4" t="inlineStr">
         <is>
-          <t>投资策略合规规则库</t>
+          <t>交易对手异常监控</t>
         </is>
       </c>
       <c r="E94" s="5" t="inlineStr">
         <is>
-          <t>内置1000+条监管规则（投资指引/证监会规定），支持新增</t>
+          <t>同一交易对手频繁交易预警，多次修改交易对手行为识别，持仓结构异常检测</t>
         </is>
       </c>
       <c r="F94" s="5" t="inlineStr">
@@ -5462,13 +5496,13 @@
         </is>
       </c>
       <c r="H94" s="8" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
     </row>
     <row r="95" ht="28" customHeight="1">
       <c r="A95" s="5" t="inlineStr">
         <is>
-          <t>事前风控/合规</t>
+          <t>异常交易风控</t>
         </is>
       </c>
       <c r="B95" s="3" t="inlineStr">
@@ -5478,37 +5512,37 @@
       </c>
       <c r="C95" s="3" t="inlineStr">
         <is>
-          <t>F06-02</t>
+          <t>F05-08</t>
         </is>
       </c>
       <c r="D95" s="4" t="inlineStr">
         <is>
-          <t>实时订单拦截</t>
+          <t>交易量异常检测</t>
         </is>
       </c>
       <c r="E95" s="5" t="inlineStr">
         <is>
-          <t>在交易指令提交前同步校验，不满足规则则拦截+原因告知</t>
+          <t>交易量统计异常识别，集中度异常告警，与历史基准对比的量级偏离检测</t>
         </is>
       </c>
       <c r="F95" s="5" t="inlineStr">
         <is>
-          <t>p99延迟/误差率/精度验证/压测10k TPS</t>
-        </is>
-      </c>
-      <c r="G95" s="28" t="inlineStr">
-        <is>
-          <t>极高</t>
+          <t>功能测试通过/正确率100%</t>
+        </is>
+      </c>
+      <c r="G95" s="24" t="inlineStr">
+        <is>
+          <t>中</t>
         </is>
       </c>
       <c r="H95" s="8" t="n">
-        <v>25</v>
+        <v>15</v>
       </c>
     </row>
     <row r="96" ht="28" customHeight="1">
       <c r="A96" s="5" t="inlineStr">
         <is>
-          <t>事前风控/合规</t>
+          <t>异常交易风控</t>
         </is>
       </c>
       <c r="B96" s="3" t="inlineStr">
@@ -5518,37 +5552,37 @@
       </c>
       <c r="C96" s="3" t="inlineStr">
         <is>
-          <t>F06-03</t>
+          <t>F05-09</t>
         </is>
       </c>
       <c r="D96" s="4" t="inlineStr">
         <is>
-          <t>限额多维度检查</t>
+          <t>动态规则管理</t>
         </is>
       </c>
       <c r="E96" s="5" t="inlineStr">
         <is>
-          <t>单笔名义/资产类别/集中度/净敞口/利率敏感度多维并行检查</t>
+          <t>异常模式智能探索与规则固化，No-Code规则配置界面，合规人员自助维护，规则版本管理</t>
         </is>
       </c>
       <c r="F96" s="5" t="inlineStr">
         <is>
-          <t>功能完整/边界测试/集成冒烟/性能基线</t>
-        </is>
-      </c>
-      <c r="G96" s="23" t="inlineStr">
-        <is>
-          <t>高</t>
+          <t>功能测试通过/正确率100%</t>
+        </is>
+      </c>
+      <c r="G96" s="24" t="inlineStr">
+        <is>
+          <t>中</t>
         </is>
       </c>
       <c r="H96" s="8" t="n">
-        <v>25</v>
+        <v>20</v>
       </c>
     </row>
     <row r="97" ht="28" customHeight="1">
       <c r="A97" s="5" t="inlineStr">
         <is>
-          <t>事前风控/合规</t>
+          <t>异常交易风控</t>
         </is>
       </c>
       <c r="B97" s="3" t="inlineStr">
@@ -5558,17 +5592,17 @@
       </c>
       <c r="C97" s="3" t="inlineStr">
         <is>
-          <t>F06-04</t>
+          <t>F05-10</t>
         </is>
       </c>
       <c r="D97" s="4" t="inlineStr">
         <is>
-          <t>合规审批工作流</t>
+          <t>异常交易定位</t>
         </is>
       </c>
       <c r="E97" s="5" t="inlineStr">
         <is>
-          <t>超限申请→审批→记录全流程，支持移动端审批</t>
+          <t>按时间范围快速查找历史异常交易，标记异常类型，可视化展示异常分布与趋势</t>
         </is>
       </c>
       <c r="F97" s="5" t="inlineStr">
@@ -5588,7 +5622,7 @@
     <row r="98" ht="28" customHeight="1">
       <c r="A98" s="5" t="inlineStr">
         <is>
-          <t>事前风控/合规</t>
+          <t>异常交易风控</t>
         </is>
       </c>
       <c r="B98" s="3" t="inlineStr">
@@ -5598,17 +5632,17 @@
       </c>
       <c r="C98" s="3" t="inlineStr">
         <is>
-          <t>F06-05</t>
+          <t>F05-11</t>
         </is>
       </c>
       <c r="D98" s="4" t="inlineStr">
         <is>
-          <t>监管白/黑名单</t>
+          <t>数据上传校验</t>
         </is>
       </c>
       <c r="E98" s="5" t="inlineStr">
         <is>
-          <t>证券/交易对手监管限制名单实时同步，拦截违规交易</t>
+          <t>支持用户上传交易数据文件，瞬时完成异常交易校验并输出校验结果报告</t>
         </is>
       </c>
       <c r="F98" s="5" t="inlineStr">
@@ -5625,57 +5659,57 @@
         <v>15</v>
       </c>
     </row>
-    <row r="99" ht="20" customHeight="1">
-      <c r="A99" s="22" t="inlineStr">
-        <is>
-          <t>【P1】 组合管理+绩效归因  (Portfolio Mgmt &amp; Perf)</t>
-        </is>
-      </c>
-    </row>
-    <row r="100" ht="28" customHeight="1">
-      <c r="A100" s="5" t="inlineStr">
-        <is>
-          <t>组合管理+绩效归因</t>
-        </is>
-      </c>
-      <c r="B100" s="3" t="inlineStr">
-        <is>
-          <t>P1</t>
-        </is>
-      </c>
-      <c r="C100" s="3" t="inlineStr">
-        <is>
-          <t>F07-01</t>
-        </is>
-      </c>
-      <c r="D100" s="4" t="inlineStr">
-        <is>
-          <t>债券横截面与时序分析</t>
-        </is>
-      </c>
-      <c r="E100" s="5" t="inlineStr">
-        <is>
-          <t>跨品种横截面信号挖掘（利差/久期偏差），历史时序趋势与均值回归分析</t>
-        </is>
-      </c>
-      <c r="F100" s="5" t="inlineStr">
-        <is>
-          <t>横截面信号与实际收益相关性&gt;0.3</t>
-        </is>
-      </c>
-      <c r="G100" s="23" t="inlineStr">
-        <is>
-          <t>高</t>
-        </is>
-      </c>
-      <c r="H100" s="8" t="n">
-        <v>35</v>
+    <row r="99" ht="28" customHeight="1">
+      <c r="A99" s="5" t="inlineStr">
+        <is>
+          <t>异常交易风控</t>
+        </is>
+      </c>
+      <c r="B99" s="3" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="C99" s="3" t="inlineStr">
+        <is>
+          <t>F05-12</t>
+        </is>
+      </c>
+      <c r="D99" s="4" t="inlineStr">
+        <is>
+          <t>智能报告生成</t>
+        </is>
+      </c>
+      <c r="E99" s="5" t="inlineStr">
+        <is>
+          <t>模板自定义与场景数据一键应用，监管报送格式（证监会/人行），新业务过会合规分析报告</t>
+        </is>
+      </c>
+      <c r="F99" s="5" t="inlineStr">
+        <is>
+          <t>功能测试通过/正确率100%</t>
+        </is>
+      </c>
+      <c r="G99" s="24" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="H99" s="8" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="100" ht="20" customHeight="1">
+      <c r="A100" s="22" t="inlineStr">
+        <is>
+          <t>【P1】 事前风控/合规  (Pre-trade Risk)</t>
+        </is>
       </c>
     </row>
     <row r="101" ht="28" customHeight="1">
       <c r="A101" s="5" t="inlineStr">
         <is>
-          <t>组合管理+绩效归因</t>
+          <t>事前风控/合规</t>
         </is>
       </c>
       <c r="B101" s="3" t="inlineStr">
@@ -5685,22 +5719,22 @@
       </c>
       <c r="C101" s="3" t="inlineStr">
         <is>
-          <t>F07-02</t>
+          <t>F06-01</t>
         </is>
       </c>
       <c r="D101" s="4" t="inlineStr">
         <is>
-          <t>相对价值分析</t>
+          <t>投资策略合规规则库</t>
         </is>
       </c>
       <c r="E101" s="5" t="inlineStr">
         <is>
-          <t>利差/Z-spread/OAS相对价值计算，历史分位数定位，跨品种套利信号识别</t>
+          <t>内置1000+条监管规则（投资指引/证监会规定），支持新增</t>
         </is>
       </c>
       <c r="F101" s="5" t="inlineStr">
         <is>
-          <t>OAS计算误差&lt;1bps，分位数覆盖5年历史</t>
+          <t>功能完整/边界测试/集成冒烟/性能基线</t>
         </is>
       </c>
       <c r="G101" s="23" t="inlineStr">
@@ -5715,7 +5749,7 @@
     <row r="102" ht="28" customHeight="1">
       <c r="A102" s="5" t="inlineStr">
         <is>
-          <t>组合管理+绩效归因</t>
+          <t>事前风控/合规</t>
         </is>
       </c>
       <c r="B102" s="3" t="inlineStr">
@@ -5725,27 +5759,27 @@
       </c>
       <c r="C102" s="3" t="inlineStr">
         <is>
-          <t>F07-03</t>
+          <t>F06-02</t>
         </is>
       </c>
       <c r="D102" s="4" t="inlineStr">
         <is>
-          <t>组合相关度分析</t>
+          <t>实时订单拦截</t>
         </is>
       </c>
       <c r="E102" s="5" t="inlineStr">
         <is>
-          <t>资产间收益相关矩阵计算（滚动60/120/250日），组合集中度风险识别，分散化系数监控</t>
+          <t>在交易指令提交前同步校验，不满足规则则拦截+原因告知</t>
         </is>
       </c>
       <c r="F102" s="5" t="inlineStr">
         <is>
-          <t>相关矩阵计算&lt;30s（500券组合）</t>
-        </is>
-      </c>
-      <c r="G102" s="24" t="inlineStr">
-        <is>
-          <t>中</t>
+          <t>p99延迟/误差率/精度验证/压测10k TPS</t>
+        </is>
+      </c>
+      <c r="G102" s="28" t="inlineStr">
+        <is>
+          <t>极高</t>
         </is>
       </c>
       <c r="H102" s="8" t="n">
@@ -5755,7 +5789,7 @@
     <row r="103" ht="28" customHeight="1">
       <c r="A103" s="5" t="inlineStr">
         <is>
-          <t>组合管理+绩效归因</t>
+          <t>事前风控/合规</t>
         </is>
       </c>
       <c r="B103" s="3" t="inlineStr">
@@ -5765,22 +5799,22 @@
       </c>
       <c r="C103" s="3" t="inlineStr">
         <is>
-          <t>F07-04</t>
+          <t>F06-03</t>
         </is>
       </c>
       <c r="D103" s="4" t="inlineStr">
         <is>
-          <t>情景分析</t>
+          <t>限额多维度检查</t>
         </is>
       </c>
       <c r="E103" s="5" t="inlineStr">
         <is>
-          <t>利率/信用/流动性三类自定义情景，组合P&amp;L影响量化，多情景并行对比</t>
+          <t>单笔名义/资产类别/集中度/净敞口/利率敏感度多维并行检查</t>
         </is>
       </c>
       <c r="F103" s="5" t="inlineStr">
         <is>
-          <t>情景P&amp;L与手工核算误差&lt;0.5%，支持≥20情景并行</t>
+          <t>功能完整/边界测试/集成冒烟/性能基线</t>
         </is>
       </c>
       <c r="G103" s="23" t="inlineStr">
@@ -5789,13 +5823,13 @@
         </is>
       </c>
       <c r="H103" s="8" t="n">
-        <v>35</v>
+        <v>25</v>
       </c>
     </row>
     <row r="104" ht="28" customHeight="1">
       <c r="A104" s="5" t="inlineStr">
         <is>
-          <t>组合管理+绩效归因</t>
+          <t>事前风控/合规</t>
         </is>
       </c>
       <c r="B104" s="3" t="inlineStr">
@@ -5805,37 +5839,37 @@
       </c>
       <c r="C104" s="3" t="inlineStr">
         <is>
-          <t>F07-05</t>
+          <t>F06-04</t>
         </is>
       </c>
       <c r="D104" s="4" t="inlineStr">
         <is>
-          <t>敏感度分析</t>
+          <t>合规审批工作流</t>
         </is>
       </c>
       <c r="E104" s="5" t="inlineStr">
         <is>
-          <t>久期/DV01/凸度/利差/Vega敏感度多因子并行计算，组合对冲比率建议</t>
+          <t>超限申请→审批→记录全流程，支持移动端审批</t>
         </is>
       </c>
       <c r="F104" s="5" t="inlineStr">
         <is>
-          <t>DV01与Bloomberg基准误差&lt;0.5bps</t>
-        </is>
-      </c>
-      <c r="G104" s="23" t="inlineStr">
-        <is>
-          <t>高</t>
+          <t>功能测试通过/正确率100%</t>
+        </is>
+      </c>
+      <c r="G104" s="24" t="inlineStr">
+        <is>
+          <t>中</t>
         </is>
       </c>
       <c r="H104" s="8" t="n">
-        <v>25</v>
+        <v>15</v>
       </c>
     </row>
     <row r="105" ht="28" customHeight="1">
       <c r="A105" s="5" t="inlineStr">
         <is>
-          <t>组合管理+绩效归因</t>
+          <t>事前风控/合规</t>
         </is>
       </c>
       <c r="B105" s="3" t="inlineStr">
@@ -5845,71 +5879,38 @@
       </c>
       <c r="C105" s="3" t="inlineStr">
         <is>
-          <t>F07-06</t>
+          <t>F06-05</t>
         </is>
       </c>
       <c r="D105" s="4" t="inlineStr">
         <is>
-          <t>极端事件分析</t>
+          <t>监管白/黑名单</t>
         </is>
       </c>
       <c r="E105" s="5" t="inlineStr">
         <is>
-          <t>历史极端情景（924行情/2015股灾/2020疫情等8+情景），组合尾部损失分布，ES(99%)计算</t>
+          <t>证券/交易对手监管限制名单实时同步，拦截违规交易</t>
         </is>
       </c>
       <c r="F105" s="5" t="inlineStr">
         <is>
-          <t>历史情景复现误差&lt;1%</t>
-        </is>
-      </c>
-      <c r="G105" s="23" t="inlineStr">
-        <is>
-          <t>高</t>
+          <t>功能测试通过/正确率100%</t>
+        </is>
+      </c>
+      <c r="G105" s="24" t="inlineStr">
+        <is>
+          <t>中</t>
         </is>
       </c>
       <c r="H105" s="8" t="n">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="106" ht="28" customHeight="1">
-      <c r="A106" s="5" t="inlineStr">
-        <is>
-          <t>组合管理+绩效归因</t>
-        </is>
-      </c>
-      <c r="B106" s="3" t="inlineStr">
-        <is>
-          <t>P1</t>
-        </is>
-      </c>
-      <c r="C106" s="3" t="inlineStr">
-        <is>
-          <t>F07-07</t>
-        </is>
-      </c>
-      <c r="D106" s="4" t="inlineStr">
-        <is>
-          <t>指数比较分析</t>
-        </is>
-      </c>
-      <c r="E106" s="5" t="inlineStr">
-        <is>
-          <t>对标中债综合/信用/政策行等指数，跟踪误差（TE）日频监控，超额Alpha三因子分解</t>
-        </is>
-      </c>
-      <c r="F106" s="5" t="inlineStr">
-        <is>
-          <t>TE计算误差&lt;1bps，支持≥10基准指数</t>
-        </is>
-      </c>
-      <c r="G106" s="24" t="inlineStr">
-        <is>
-          <t>中</t>
-        </is>
-      </c>
-      <c r="H106" s="8" t="n">
-        <v>25</v>
+        <v>15</v>
+      </c>
+    </row>
+    <row r="106" ht="20" customHeight="1">
+      <c r="A106" s="22" t="inlineStr">
+        <is>
+          <t>【P1】 组合管理+绩效归因  (Portfolio Mgmt &amp; Perf)</t>
+        </is>
       </c>
     </row>
     <row r="107" ht="28" customHeight="1">
@@ -5925,22 +5926,22 @@
       </c>
       <c r="C107" s="3" t="inlineStr">
         <is>
-          <t>F07-08</t>
+          <t>F07-01</t>
         </is>
       </c>
       <c r="D107" s="4" t="inlineStr">
         <is>
-          <t>绩效归因（Brinson）</t>
+          <t>债券横截面与时序分析</t>
         </is>
       </c>
       <c r="E107" s="5" t="inlineStr">
         <is>
-          <t>BHB三效应：资产配置/个券选择/交互效应，日/周/月/季多维度，报告PDF自动生成</t>
+          <t>跨品种横截面信号挖掘（利差/久期偏差），历史时序趋势与均值回归分析</t>
         </is>
       </c>
       <c r="F107" s="5" t="inlineStr">
         <is>
-          <t>Brinson结果与Bloomberg AIM误差&lt;0.1%，T+1 9:00前自动报告</t>
+          <t>横截面信号与实际收益相关性&gt;0.3</t>
         </is>
       </c>
       <c r="G107" s="23" t="inlineStr">
@@ -5949,7 +5950,7 @@
         </is>
       </c>
       <c r="H107" s="8" t="n">
-        <v>40</v>
+        <v>35</v>
       </c>
     </row>
     <row r="108" ht="28" customHeight="1">
@@ -5965,22 +5966,22 @@
       </c>
       <c r="C108" s="3" t="inlineStr">
         <is>
-          <t>F07-09</t>
+          <t>F07-02</t>
         </is>
       </c>
       <c r="D108" s="4" t="inlineStr">
         <is>
-          <t>虚拟组合分析</t>
+          <t>相对价值分析</t>
         </is>
       </c>
       <c r="E108" s="5" t="inlineStr">
         <is>
-          <t>组合调整前后净值/风险/收益效果模拟（纸面交易），冲击成本预估，多方案对比</t>
+          <t>利差/Z-spread/OAS相对价值计算，历史分位数定位，跨品种套利信号识别</t>
         </is>
       </c>
       <c r="F108" s="5" t="inlineStr">
         <is>
-          <t>虚拟组合模拟与真实执行偏差&lt;0.3%</t>
+          <t>OAS计算误差&lt;1bps，分位数覆盖5年历史</t>
         </is>
       </c>
       <c r="G108" s="23" t="inlineStr">
@@ -5989,7 +5990,7 @@
         </is>
       </c>
       <c r="H108" s="8" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
     </row>
     <row r="109" ht="28" customHeight="1">
@@ -6005,31 +6006,31 @@
       </c>
       <c r="C109" s="3" t="inlineStr">
         <is>
-          <t>F07-10</t>
+          <t>F07-03</t>
         </is>
       </c>
       <c r="D109" s="4" t="inlineStr">
         <is>
-          <t>再平衡方案试算与比较</t>
+          <t>组合相关度分析</t>
         </is>
       </c>
       <c r="E109" s="5" t="inlineStr">
         <is>
-          <t>久期/集中度/流动性/合规约束联合优化（二次规划QP），多方案并行试算，最优路径推荐</t>
+          <t>资产间收益相关矩阵计算（滚动60/120/250日），组合集中度风险识别，分散化系数监控</t>
         </is>
       </c>
       <c r="F109" s="5" t="inlineStr">
         <is>
-          <t>QP求解100券组合&lt;5s，约束满足率100%</t>
-        </is>
-      </c>
-      <c r="G109" s="23" t="inlineStr">
-        <is>
-          <t>高</t>
+          <t>相关矩阵计算&lt;30s（500券组合）</t>
+        </is>
+      </c>
+      <c r="G109" s="24" t="inlineStr">
+        <is>
+          <t>中</t>
         </is>
       </c>
       <c r="H109" s="8" t="n">
-        <v>35</v>
+        <v>25</v>
       </c>
     </row>
     <row r="110" ht="28" customHeight="1">
@@ -6045,22 +6046,22 @@
       </c>
       <c r="C110" s="3" t="inlineStr">
         <is>
-          <t>F07-11</t>
+          <t>F07-04</t>
         </is>
       </c>
       <c r="D110" s="4" t="inlineStr">
         <is>
-          <t>资产配置策略分析</t>
+          <t>情景分析</t>
         </is>
       </c>
       <c r="E110" s="5" t="inlineStr">
         <is>
-          <t>宏观因子（利率/信用/流动性周期）驱动大类资产配置模型，动态权重优化，历史回测验证</t>
+          <t>利率/信用/流动性三类自定义情景，组合P&amp;L影响量化，多情景并行对比</t>
         </is>
       </c>
       <c r="F110" s="5" t="inlineStr">
         <is>
-          <t>回测期≥5年，预测方向胜率&gt;55%</t>
+          <t>情景P&amp;L与手工核算误差&lt;0.5%，支持≥20情景并行</t>
         </is>
       </c>
       <c r="G110" s="23" t="inlineStr">
@@ -6069,7 +6070,7 @@
         </is>
       </c>
       <c r="H110" s="8" t="n">
-        <v>40</v>
+        <v>35</v>
       </c>
     </row>
     <row r="111" ht="28" customHeight="1">
@@ -6085,22 +6086,22 @@
       </c>
       <c r="C111" s="3" t="inlineStr">
         <is>
-          <t>F07-12</t>
+          <t>F07-05</t>
         </is>
       </c>
       <c r="D111" s="4" t="inlineStr">
         <is>
-          <t>固收+策略分析</t>
+          <t>敏感度分析</t>
         </is>
       </c>
       <c r="E111" s="5" t="inlineStr">
         <is>
-          <t>债券底仓+衍生品增强策略P&amp;L归因，风险分解（利率/信用/期权贡献），固收+净值模拟</t>
+          <t>久期/DV01/凸度/利差/Vega敏感度多因子并行计算，组合对冲比率建议</t>
         </is>
       </c>
       <c r="F111" s="5" t="inlineStr">
         <is>
-          <t>固收+净值模拟与实际偏差&lt;0.5%</t>
+          <t>DV01与Bloomberg基准误差&lt;0.5bps</t>
         </is>
       </c>
       <c r="G111" s="23" t="inlineStr">
@@ -6109,7 +6110,7 @@
         </is>
       </c>
       <c r="H111" s="8" t="n">
-        <v>30</v>
+        <v>25</v>
       </c>
     </row>
     <row r="112" ht="28" customHeight="1">
@@ -6125,22 +6126,22 @@
       </c>
       <c r="C112" s="3" t="inlineStr">
         <is>
-          <t>F07-13</t>
+          <t>F07-06</t>
         </is>
       </c>
       <c r="D112" s="4" t="inlineStr">
         <is>
-          <t>量化策略组合分析</t>
+          <t>极端事件分析</t>
         </is>
       </c>
       <c r="E112" s="5" t="inlineStr">
         <is>
-          <t>多策略组合叠加容量约束，策略相关性管理，Sharpe/最大回撤/Calmar实时监控</t>
+          <t>历史极端情景（924行情/2015股灾/2020疫情等8+情景），组合尾部损失分布，ES(99%)计算</t>
         </is>
       </c>
       <c r="F112" s="5" t="inlineStr">
         <is>
-          <t>策略容量计算误差&lt;5%</t>
+          <t>历史情景复现误差&lt;1%</t>
         </is>
       </c>
       <c r="G112" s="23" t="inlineStr">
@@ -6149,7 +6150,7 @@
         </is>
       </c>
       <c r="H112" s="8" t="n">
-        <v>35</v>
+        <v>30</v>
       </c>
     </row>
     <row r="113" ht="28" customHeight="1">
@@ -6165,22 +6166,22 @@
       </c>
       <c r="C113" s="3" t="inlineStr">
         <is>
-          <t>F07-14</t>
+          <t>F07-07</t>
         </is>
       </c>
       <c r="D113" s="4" t="inlineStr">
         <is>
-          <t>流动性分析</t>
+          <t>指数比较分析</t>
         </is>
       </c>
       <c r="E113" s="5" t="inlineStr">
         <is>
-          <t>逐券换手率/市场深度评估，组合变现能力分析，流动性压力下变现损失（LVaR）估算</t>
+          <t>对标中债综合/信用/政策行等指数，跟踪误差（TE）日频监控，超额Alpha三因子分解</t>
         </is>
       </c>
       <c r="F113" s="5" t="inlineStr">
         <is>
-          <t>LVaR与市场基准误差&lt;5%，日均成交量覆盖≥95%持仓</t>
+          <t>TE计算误差&lt;1bps，支持≥10基准指数</t>
         </is>
       </c>
       <c r="G113" s="24" t="inlineStr">
@@ -6189,7 +6190,7 @@
         </is>
       </c>
       <c r="H113" s="8" t="n">
-        <v>20</v>
+        <v>25</v>
       </c>
     </row>
     <row r="114" ht="28" customHeight="1">
@@ -6205,22 +6206,22 @@
       </c>
       <c r="C114" s="3" t="inlineStr">
         <is>
-          <t>F07-15</t>
+          <t>F07-08</t>
         </is>
       </c>
       <c r="D114" s="4" t="inlineStr">
         <is>
-          <t>定价计算集成</t>
+          <t>绩效归因（Brinson）</t>
         </is>
       </c>
       <c r="E114" s="5" t="inlineStr">
         <is>
-          <t>调用量化定价引擎实时估值与Greeks，含权债/可转债/IRS，结果缓存（Redis）与Kafka推送</t>
+          <t>BHB三效应：资产配置/个券选择/交互效应，日/周/月/季多维度，报告PDF自动生成</t>
         </is>
       </c>
       <c r="F114" s="5" t="inlineStr">
         <is>
-          <t>定价API p99&lt;200ms，日终全量估值&lt;30min（10万券）</t>
+          <t>Brinson结果与Bloomberg AIM误差&lt;0.1%，T+1 9:00前自动报告</t>
         </is>
       </c>
       <c r="G114" s="23" t="inlineStr">
@@ -6229,7 +6230,7 @@
         </is>
       </c>
       <c r="H114" s="8" t="n">
-        <v>20</v>
+        <v>40</v>
       </c>
     </row>
     <row r="115" ht="28" customHeight="1">
@@ -6245,31 +6246,31 @@
       </c>
       <c r="C115" s="3" t="inlineStr">
         <is>
-          <t>F07-16</t>
+          <t>F07-09</t>
         </is>
       </c>
       <c r="D115" s="4" t="inlineStr">
         <is>
-          <t>利率曲线集成</t>
+          <t>虚拟组合分析</t>
         </is>
       </c>
       <c r="E115" s="5" t="inlineStr">
         <is>
-          <t>多曲线实时消费（国债/政策行/AAA信用/OIS），NS参数提取（水平/斜率/曲率），敏感度映射</t>
+          <t>组合调整前后净值/风险/收益效果模拟（纸面交易），冲击成本预估，多方案对比</t>
         </is>
       </c>
       <c r="F115" s="5" t="inlineStr">
         <is>
-          <t>曲线更新延迟&lt;1s，NS拟合R²&gt;0.999</t>
-        </is>
-      </c>
-      <c r="G115" s="24" t="inlineStr">
-        <is>
-          <t>中</t>
+          <t>虚拟组合模拟与真实执行偏差&lt;0.3%</t>
+        </is>
+      </c>
+      <c r="G115" s="23" t="inlineStr">
+        <is>
+          <t>高</t>
         </is>
       </c>
       <c r="H115" s="8" t="n">
-        <v>15</v>
+        <v>20</v>
       </c>
     </row>
     <row r="116" ht="28" customHeight="1">
@@ -6285,22 +6286,22 @@
       </c>
       <c r="C116" s="3" t="inlineStr">
         <is>
-          <t>F07-17</t>
+          <t>F07-10</t>
         </is>
       </c>
       <c r="D116" s="4" t="inlineStr">
         <is>
-          <t>因子模型</t>
+          <t>再平衡方案试算与比较</t>
         </is>
       </c>
       <c r="E116" s="5" t="inlineStr">
         <is>
-          <t>多因子风险模型（利率/信用/流动性/行业因子），Alpha因子库（≥20因子），因子暴露实时计算</t>
+          <t>久期/集中度/流动性/合规约束联合优化（二次规划QP），多方案并行试算，最优路径推荐</t>
         </is>
       </c>
       <c r="F116" s="5" t="inlineStr">
         <is>
-          <t>因子模型解释方差&gt;80%，Alpha IC均值&gt;0.05</t>
+          <t>QP求解100券组合&lt;5s，约束满足率100%</t>
         </is>
       </c>
       <c r="G116" s="23" t="inlineStr">
@@ -6309,20 +6310,53 @@
         </is>
       </c>
       <c r="H116" s="8" t="n">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="117" ht="28" customHeight="1">
+      <c r="A117" s="5" t="inlineStr">
+        <is>
+          <t>组合管理+绩效归因</t>
+        </is>
+      </c>
+      <c r="B117" s="3" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="C117" s="3" t="inlineStr">
+        <is>
+          <t>F07-11</t>
+        </is>
+      </c>
+      <c r="D117" s="4" t="inlineStr">
+        <is>
+          <t>资产配置策略分析</t>
+        </is>
+      </c>
+      <c r="E117" s="5" t="inlineStr">
+        <is>
+          <t>宏观因子（利率/信用/流动性周期）驱动大类资产配置模型，动态权重优化，历史回测验证</t>
+        </is>
+      </c>
+      <c r="F117" s="5" t="inlineStr">
+        <is>
+          <t>回测期≥5年，预测方向胜率&gt;55%</t>
+        </is>
+      </c>
+      <c r="G117" s="23" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="H117" s="8" t="n">
         <v>40</v>
-      </c>
-    </row>
-    <row r="117" ht="20" customHeight="1">
-      <c r="A117" s="22" t="inlineStr">
-        <is>
-          <t>【P1】 策略投资/量化  (Quant Strategy)</t>
-        </is>
       </c>
     </row>
     <row r="118" ht="28" customHeight="1">
       <c r="A118" s="5" t="inlineStr">
         <is>
-          <t>策略投资/量化</t>
+          <t>组合管理+绩效归因</t>
         </is>
       </c>
       <c r="B118" s="3" t="inlineStr">
@@ -6332,22 +6366,22 @@
       </c>
       <c r="C118" s="3" t="inlineStr">
         <is>
-          <t>F08-01</t>
+          <t>F07-12</t>
         </is>
       </c>
       <c r="D118" s="4" t="inlineStr">
         <is>
-          <t>因子模型框架</t>
+          <t>固收+策略分析</t>
         </is>
       </c>
       <c r="E118" s="5" t="inlineStr">
         <is>
-          <t>多因子Alpha模型+风险因子，支持自定义因子上传与测试</t>
+          <t>债券底仓+衍生品增强策略P&amp;L归因，风险分解（利率/信用/期权贡献），固收+净值模拟</t>
         </is>
       </c>
       <c r="F118" s="5" t="inlineStr">
         <is>
-          <t>功能完整/边界测试/集成冒烟/性能基线</t>
+          <t>固收+净值模拟与实际偏差&lt;0.5%</t>
         </is>
       </c>
       <c r="G118" s="23" t="inlineStr">
@@ -6356,13 +6390,13 @@
         </is>
       </c>
       <c r="H118" s="8" t="n">
-        <v>40</v>
+        <v>30</v>
       </c>
     </row>
     <row r="119" ht="28" customHeight="1">
       <c r="A119" s="5" t="inlineStr">
         <is>
-          <t>策略投资/量化</t>
+          <t>组合管理+绩效归因</t>
         </is>
       </c>
       <c r="B119" s="3" t="inlineStr">
@@ -6372,37 +6406,37 @@
       </c>
       <c r="C119" s="3" t="inlineStr">
         <is>
-          <t>F08-02</t>
+          <t>F07-13</t>
         </is>
       </c>
       <c r="D119" s="4" t="inlineStr">
         <is>
-          <t>Tick级回测引擎</t>
+          <t>量化策略组合分析</t>
         </is>
       </c>
       <c r="E119" s="5" t="inlineStr">
         <is>
-          <t>Tick数据驱动回测，真实滑点/冲击模型，批量参数优化</t>
+          <t>多策略组合叠加容量约束，策略相关性管理，Sharpe/最大回撤/Calmar实时监控</t>
         </is>
       </c>
       <c r="F119" s="5" t="inlineStr">
         <is>
-          <t>p99延迟/误差率/精度验证/压测10k TPS</t>
-        </is>
-      </c>
-      <c r="G119" s="28" t="inlineStr">
-        <is>
-          <t>极高</t>
+          <t>策略容量计算误差&lt;5%</t>
+        </is>
+      </c>
+      <c r="G119" s="23" t="inlineStr">
+        <is>
+          <t>高</t>
         </is>
       </c>
       <c r="H119" s="8" t="n">
-        <v>60</v>
+        <v>35</v>
       </c>
     </row>
     <row r="120" ht="28" customHeight="1">
       <c r="A120" s="5" t="inlineStr">
         <is>
-          <t>策略投资/量化</t>
+          <t>组合管理+绩效归因</t>
         </is>
       </c>
       <c r="B120" s="3" t="inlineStr">
@@ -6412,37 +6446,37 @@
       </c>
       <c r="C120" s="3" t="inlineStr">
         <is>
-          <t>F08-03</t>
+          <t>F07-14</t>
         </is>
       </c>
       <c r="D120" s="4" t="inlineStr">
         <is>
-          <t>信号生成与调度</t>
+          <t>流动性分析</t>
         </is>
       </c>
       <c r="E120" s="5" t="inlineStr">
         <is>
-          <t>策略信号实时计算，支持Python/C++策略脚本沙箱运行</t>
+          <t>逐券换手率/市场深度评估，组合变现能力分析，流动性压力下变现损失（LVaR）估算</t>
         </is>
       </c>
       <c r="F120" s="5" t="inlineStr">
         <is>
-          <t>功能完整/边界测试/集成冒烟/性能基线</t>
-        </is>
-      </c>
-      <c r="G120" s="23" t="inlineStr">
-        <is>
-          <t>高</t>
+          <t>LVaR与市场基准误差&lt;5%，日均成交量覆盖≥95%持仓</t>
+        </is>
+      </c>
+      <c r="G120" s="24" t="inlineStr">
+        <is>
+          <t>中</t>
         </is>
       </c>
       <c r="H120" s="8" t="n">
-        <v>40</v>
+        <v>20</v>
       </c>
     </row>
     <row r="121" ht="28" customHeight="1">
       <c r="A121" s="5" t="inlineStr">
         <is>
-          <t>策略投资/量化</t>
+          <t>组合管理+绩效归因</t>
         </is>
       </c>
       <c r="B121" s="3" t="inlineStr">
@@ -6452,331 +6486,331 @@
       </c>
       <c r="C121" s="3" t="inlineStr">
         <is>
-          <t>F08-04</t>
+          <t>F07-15</t>
         </is>
       </c>
       <c r="D121" s="4" t="inlineStr">
         <is>
-          <t>低延迟执行接口</t>
+          <t>定价计算集成</t>
         </is>
       </c>
       <c r="E121" s="5" t="inlineStr">
         <is>
-          <t>与ATP超低延迟执行层对接，算法拆单（TWAP/VWAP/IS）</t>
+          <t>调用量化定价引擎实时估值与Greeks，含权债/可转债/IRS，结果缓存（Redis）与Kafka推送</t>
         </is>
       </c>
       <c r="F121" s="5" t="inlineStr">
         <is>
-          <t>p99延迟/误差率/精度验证/压测10k TPS</t>
-        </is>
-      </c>
-      <c r="G121" s="28" t="inlineStr">
-        <is>
-          <t>极高</t>
+          <t>定价API p99&lt;200ms，日终全量估值&lt;30min（10万券）</t>
+        </is>
+      </c>
+      <c r="G121" s="23" t="inlineStr">
+        <is>
+          <t>高</t>
         </is>
       </c>
       <c r="H121" s="8" t="n">
-        <v>45</v>
+        <v>20</v>
       </c>
     </row>
     <row r="122" ht="28" customHeight="1">
       <c r="A122" s="5" t="inlineStr">
         <is>
+          <t>组合管理+绩效归因</t>
+        </is>
+      </c>
+      <c r="B122" s="3" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="C122" s="3" t="inlineStr">
+        <is>
+          <t>F07-16</t>
+        </is>
+      </c>
+      <c r="D122" s="4" t="inlineStr">
+        <is>
+          <t>利率曲线集成</t>
+        </is>
+      </c>
+      <c r="E122" s="5" t="inlineStr">
+        <is>
+          <t>多曲线实时消费（国债/政策行/AAA信用/OIS），NS参数提取（水平/斜率/曲率），敏感度映射</t>
+        </is>
+      </c>
+      <c r="F122" s="5" t="inlineStr">
+        <is>
+          <t>曲线更新延迟&lt;1s，NS拟合R²&gt;0.999</t>
+        </is>
+      </c>
+      <c r="G122" s="24" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="H122" s="8" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="123" ht="28" customHeight="1">
+      <c r="A123" s="5" t="inlineStr">
+        <is>
+          <t>组合管理+绩效归因</t>
+        </is>
+      </c>
+      <c r="B123" s="3" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="C123" s="3" t="inlineStr">
+        <is>
+          <t>F07-17</t>
+        </is>
+      </c>
+      <c r="D123" s="4" t="inlineStr">
+        <is>
+          <t>因子模型</t>
+        </is>
+      </c>
+      <c r="E123" s="5" t="inlineStr">
+        <is>
+          <t>多因子风险模型（利率/信用/流动性/行业因子），Alpha因子库（≥20因子），因子暴露实时计算</t>
+        </is>
+      </c>
+      <c r="F123" s="5" t="inlineStr">
+        <is>
+          <t>因子模型解释方差&gt;80%，Alpha IC均值&gt;0.05</t>
+        </is>
+      </c>
+      <c r="G123" s="23" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="H123" s="8" t="n">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="124" ht="20" customHeight="1">
+      <c r="A124" s="22" t="inlineStr">
+        <is>
+          <t>【P1】 策略投资/量化  (Quant Strategy)</t>
+        </is>
+      </c>
+    </row>
+    <row r="125" ht="28" customHeight="1">
+      <c r="A125" s="5" t="inlineStr">
+        <is>
           <t>策略投资/量化</t>
         </is>
       </c>
-      <c r="B122" s="3" t="inlineStr">
-        <is>
-          <t>P1</t>
-        </is>
-      </c>
-      <c r="C122" s="3" t="inlineStr">
+      <c r="B125" s="3" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="C125" s="3" t="inlineStr">
+        <is>
+          <t>F08-01</t>
+        </is>
+      </c>
+      <c r="D125" s="4" t="inlineStr">
+        <is>
+          <t>因子模型框架</t>
+        </is>
+      </c>
+      <c r="E125" s="5" t="inlineStr">
+        <is>
+          <t>多因子Alpha模型+风险因子，支持自定义因子上传与测试</t>
+        </is>
+      </c>
+      <c r="F125" s="5" t="inlineStr">
+        <is>
+          <t>功能完整/边界测试/集成冒烟/性能基线</t>
+        </is>
+      </c>
+      <c r="G125" s="23" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="H125" s="8" t="n">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="126" ht="28" customHeight="1">
+      <c r="A126" s="5" t="inlineStr">
+        <is>
+          <t>策略投资/量化</t>
+        </is>
+      </c>
+      <c r="B126" s="3" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="C126" s="3" t="inlineStr">
+        <is>
+          <t>F08-02</t>
+        </is>
+      </c>
+      <c r="D126" s="4" t="inlineStr">
+        <is>
+          <t>Tick级回测引擎</t>
+        </is>
+      </c>
+      <c r="E126" s="5" t="inlineStr">
+        <is>
+          <t>Tick数据驱动回测，真实滑点/冲击模型，批量参数优化</t>
+        </is>
+      </c>
+      <c r="F126" s="5" t="inlineStr">
+        <is>
+          <t>p99延迟/误差率/精度验证/压测10k TPS</t>
+        </is>
+      </c>
+      <c r="G126" s="28" t="inlineStr">
+        <is>
+          <t>极高</t>
+        </is>
+      </c>
+      <c r="H126" s="8" t="n">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="127" ht="28" customHeight="1">
+      <c r="A127" s="5" t="inlineStr">
+        <is>
+          <t>策略投资/量化</t>
+        </is>
+      </c>
+      <c r="B127" s="3" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="C127" s="3" t="inlineStr">
+        <is>
+          <t>F08-03</t>
+        </is>
+      </c>
+      <c r="D127" s="4" t="inlineStr">
+        <is>
+          <t>信号生成与调度</t>
+        </is>
+      </c>
+      <c r="E127" s="5" t="inlineStr">
+        <is>
+          <t>策略信号实时计算，支持Python/C++策略脚本沙箱运行</t>
+        </is>
+      </c>
+      <c r="F127" s="5" t="inlineStr">
+        <is>
+          <t>功能完整/边界测试/集成冒烟/性能基线</t>
+        </is>
+      </c>
+      <c r="G127" s="23" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="H127" s="8" t="n">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="128" ht="28" customHeight="1">
+      <c r="A128" s="5" t="inlineStr">
+        <is>
+          <t>策略投资/量化</t>
+        </is>
+      </c>
+      <c r="B128" s="3" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="C128" s="3" t="inlineStr">
+        <is>
+          <t>F08-04</t>
+        </is>
+      </c>
+      <c r="D128" s="4" t="inlineStr">
+        <is>
+          <t>低延迟执行接口</t>
+        </is>
+      </c>
+      <c r="E128" s="5" t="inlineStr">
+        <is>
+          <t>与ATP超低延迟执行层对接，算法拆单（TWAP/VWAP/IS）</t>
+        </is>
+      </c>
+      <c r="F128" s="5" t="inlineStr">
+        <is>
+          <t>p99延迟/误差率/精度验证/压测10k TPS</t>
+        </is>
+      </c>
+      <c r="G128" s="28" t="inlineStr">
+        <is>
+          <t>极高</t>
+        </is>
+      </c>
+      <c r="H128" s="8" t="n">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="129" ht="28" customHeight="1">
+      <c r="A129" s="5" t="inlineStr">
+        <is>
+          <t>策略投资/量化</t>
+        </is>
+      </c>
+      <c r="B129" s="3" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="C129" s="3" t="inlineStr">
         <is>
           <t>F08-05</t>
         </is>
       </c>
-      <c r="D122" s="4" t="inlineStr">
+      <c r="D129" s="4" t="inlineStr">
         <is>
           <t>实时策略监控</t>
         </is>
       </c>
-      <c r="E122" s="5" t="inlineStr">
+      <c r="E129" s="5" t="inlineStr">
         <is>
           <t>持仓/PnL/回撤/Sharpe实时看板，风险触发自动平仓</t>
         </is>
       </c>
-      <c r="F122" s="5" t="inlineStr">
+      <c r="F129" s="5" t="inlineStr">
         <is>
           <t>功能测试通过/正确率100%</t>
         </is>
       </c>
-      <c r="G122" s="24" t="inlineStr">
+      <c r="G129" s="24" t="inlineStr">
         <is>
           <t>中</t>
         </is>
       </c>
-      <c r="H122" s="8" t="n">
+      <c r="H129" s="8" t="n">
         <v>20</v>
-      </c>
-    </row>
-    <row r="123" ht="20" customHeight="1">
-      <c r="A123" s="26" t="inlineStr">
-        <is>
-          <t>【P2】 定价平台  (Pricing Platform)</t>
-        </is>
-      </c>
-    </row>
-    <row r="124" ht="28" customHeight="1">
-      <c r="A124" s="11" t="inlineStr">
-        <is>
-          <t>定价平台</t>
-        </is>
-      </c>
-      <c r="B124" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
-        </is>
-      </c>
-      <c r="C124" s="10" t="inlineStr">
-        <is>
-          <t>F09-01</t>
-        </is>
-      </c>
-      <c r="D124" s="27" t="inlineStr">
-        <is>
-          <t>期限结构模型</t>
-        </is>
-      </c>
-      <c r="E124" s="11" t="inlineStr">
-        <is>
-          <t>Nelson-Siegel/Svensson/HJM等多模型参数拟合，实时曲线</t>
-        </is>
-      </c>
-      <c r="F124" s="11" t="inlineStr">
-        <is>
-          <t>p99延迟/误差率/精度验证/压测10k TPS</t>
-        </is>
-      </c>
-      <c r="G124" s="28" t="inlineStr">
-        <is>
-          <t>极高</t>
-        </is>
-      </c>
-      <c r="H124" s="13" t="n">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="125" ht="28" customHeight="1">
-      <c r="A125" s="11" t="inlineStr">
-        <is>
-          <t>定价平台</t>
-        </is>
-      </c>
-      <c r="B125" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
-        </is>
-      </c>
-      <c r="C125" s="10" t="inlineStr">
-        <is>
-          <t>F09-02</t>
-        </is>
-      </c>
-      <c r="D125" s="27" t="inlineStr">
-        <is>
-          <t>蒙特卡洛求解器</t>
-        </is>
-      </c>
-      <c r="E125" s="11" t="inlineStr">
-        <is>
-          <t>GPU加速MC，QMC低差异序列，支持路径相关期权定价</t>
-        </is>
-      </c>
-      <c r="F125" s="11" t="inlineStr">
-        <is>
-          <t>p99延迟/误差率/精度验证/压测10k TPS</t>
-        </is>
-      </c>
-      <c r="G125" s="28" t="inlineStr">
-        <is>
-          <t>极高</t>
-        </is>
-      </c>
-      <c r="H125" s="13" t="n">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="126" ht="28" customHeight="1">
-      <c r="A126" s="11" t="inlineStr">
-        <is>
-          <t>定价平台</t>
-        </is>
-      </c>
-      <c r="B126" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
-        </is>
-      </c>
-      <c r="C126" s="10" t="inlineStr">
-        <is>
-          <t>F09-03</t>
-        </is>
-      </c>
-      <c r="D126" s="27" t="inlineStr">
-        <is>
-          <t>有限差分（PDE）</t>
-        </is>
-      </c>
-      <c r="E126" s="11" t="inlineStr">
-        <is>
-          <t>Crank-Nicolson/ADI方法，含权债/可转债精确定价</t>
-        </is>
-      </c>
-      <c r="F126" s="11" t="inlineStr">
-        <is>
-          <t>p99延迟/误差率/精度验证/压测10k TPS</t>
-        </is>
-      </c>
-      <c r="G126" s="28" t="inlineStr">
-        <is>
-          <t>极高</t>
-        </is>
-      </c>
-      <c r="H126" s="13" t="n">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="127" ht="28" customHeight="1">
-      <c r="A127" s="11" t="inlineStr">
-        <is>
-          <t>定价平台</t>
-        </is>
-      </c>
-      <c r="B127" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
-        </is>
-      </c>
-      <c r="C127" s="10" t="inlineStr">
-        <is>
-          <t>F09-04</t>
-        </is>
-      </c>
-      <c r="D127" s="27" t="inlineStr">
-        <is>
-          <t>实时Greeks</t>
-        </is>
-      </c>
-      <c r="E127" s="11" t="inlineStr">
-        <is>
-          <t>Delta/Gamma/Vega/Theta/Rho分布式实时计算</t>
-        </is>
-      </c>
-      <c r="F127" s="11" t="inlineStr">
-        <is>
-          <t>功能完整/边界测试/集成冒烟/性能基线</t>
-        </is>
-      </c>
-      <c r="G127" s="23" t="inlineStr">
-        <is>
-          <t>高</t>
-        </is>
-      </c>
-      <c r="H127" s="13" t="n">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="128" ht="28" customHeight="1">
-      <c r="A128" s="11" t="inlineStr">
-        <is>
-          <t>定价平台</t>
-        </is>
-      </c>
-      <c r="B128" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
-        </is>
-      </c>
-      <c r="C128" s="10" t="inlineStr">
-        <is>
-          <t>F09-05</t>
-        </is>
-      </c>
-      <c r="D128" s="27" t="inlineStr">
-        <is>
-          <t>定价服务微服务架构</t>
-        </is>
-      </c>
-      <c r="E128" s="11" t="inlineStr">
-        <is>
-          <t>REST/gRPC定价API，支持横向扩展，p99&lt;100ms</t>
-        </is>
-      </c>
-      <c r="F128" s="11" t="inlineStr">
-        <is>
-          <t>功能完整/边界测试/集成冒烟/性能基线</t>
-        </is>
-      </c>
-      <c r="G128" s="23" t="inlineStr">
-        <is>
-          <t>高</t>
-        </is>
-      </c>
-      <c r="H128" s="13" t="n">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="129" ht="28" customHeight="1">
-      <c r="A129" s="11" t="inlineStr">
-        <is>
-          <t>定价平台</t>
-        </is>
-      </c>
-      <c r="B129" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
-        </is>
-      </c>
-      <c r="C129" s="10" t="inlineStr">
-        <is>
-          <t>F09-06</t>
-        </is>
-      </c>
-      <c r="D129" s="27" t="inlineStr">
-        <is>
-          <t>历史估值回测</t>
-        </is>
-      </c>
-      <c r="E129" s="11" t="inlineStr">
-        <is>
-          <t>基于历史行情重放定价误差分析，模型验证框架</t>
-        </is>
-      </c>
-      <c r="F129" s="11" t="inlineStr">
-        <is>
-          <t>功能完整/边界测试/集成冒烟/性能基线</t>
-        </is>
-      </c>
-      <c r="G129" s="23" t="inlineStr">
-        <is>
-          <t>高</t>
-        </is>
-      </c>
-      <c r="H129" s="13" t="n">
-        <v>30</v>
       </c>
     </row>
     <row r="130" ht="20" customHeight="1">
       <c r="A130" s="26" t="inlineStr">
         <is>
-          <t>【P2】 销售交易  (Sales Trading)</t>
+          <t>【P2】 定价平台  (Pricing Platform)</t>
         </is>
       </c>
     </row>
     <row r="131" ht="28" customHeight="1">
       <c r="A131" s="11" t="inlineStr">
         <is>
-          <t>销售交易</t>
+          <t>定价平台</t>
         </is>
       </c>
       <c r="B131" s="10" t="inlineStr">
@@ -6786,37 +6820,37 @@
       </c>
       <c r="C131" s="10" t="inlineStr">
         <is>
-          <t>F10-01</t>
+          <t>F09-01</t>
         </is>
       </c>
       <c r="D131" s="27" t="inlineStr">
         <is>
-          <t>销交工作台</t>
+          <t>期限结构模型</t>
         </is>
       </c>
       <c r="E131" s="11" t="inlineStr">
         <is>
-          <t>报价管理主界面，历史报价管理，当日报价快捷操作，导入/导出报价，一键unrefer操作</t>
+          <t>Nelson-Siegel/Svensson/HJM等多模型参数拟合，实时曲线</t>
         </is>
       </c>
       <c r="F131" s="11" t="inlineStr">
         <is>
-          <t>功能测试通过/正确率100%</t>
-        </is>
-      </c>
-      <c r="G131" s="24" t="inlineStr">
-        <is>
-          <t>中</t>
+          <t>p99延迟/误差率/精度验证/压测10k TPS</t>
+        </is>
+      </c>
+      <c r="G131" s="28" t="inlineStr">
+        <is>
+          <t>极高</t>
         </is>
       </c>
       <c r="H131" s="13" t="n">
-        <v>20</v>
+        <v>60</v>
       </c>
     </row>
     <row r="132" ht="28" customHeight="1">
       <c r="A132" s="11" t="inlineStr">
         <is>
-          <t>销售交易</t>
+          <t>定价平台</t>
         </is>
       </c>
       <c r="B132" s="10" t="inlineStr">
@@ -6826,37 +6860,37 @@
       </c>
       <c r="C132" s="10" t="inlineStr">
         <is>
-          <t>F10-02</t>
+          <t>F09-02</t>
         </is>
       </c>
       <c r="D132" s="27" t="inlineStr">
         <is>
-          <t>债券过滤与筛选</t>
+          <t>蒙特卡洛求解器</t>
         </is>
       </c>
       <c r="E132" s="11" t="inlineStr">
         <is>
-          <t>信用债/利率债过滤，信用债全品种过滤，利率债国债/证金债/地方债分类过滤，精确与模糊识别</t>
+          <t>GPU加速MC，QMC低差异序列，支持路径相关期权定价</t>
         </is>
       </c>
       <c r="F132" s="11" t="inlineStr">
         <is>
-          <t>功能测试通过</t>
-        </is>
-      </c>
-      <c r="G132" s="25" t="inlineStr">
-        <is>
-          <t>低</t>
+          <t>p99延迟/误差率/精度验证/压测10k TPS</t>
+        </is>
+      </c>
+      <c r="G132" s="28" t="inlineStr">
+        <is>
+          <t>极高</t>
         </is>
       </c>
       <c r="H132" s="13" t="n">
-        <v>10</v>
+        <v>70</v>
       </c>
     </row>
     <row r="133" ht="28" customHeight="1">
       <c r="A133" s="11" t="inlineStr">
         <is>
-          <t>销售交易</t>
+          <t>定价平台</t>
         </is>
       </c>
       <c r="B133" s="10" t="inlineStr">
@@ -6866,37 +6900,37 @@
       </c>
       <c r="C133" s="10" t="inlineStr">
         <is>
-          <t>F10-03</t>
+          <t>F09-03</t>
         </is>
       </c>
       <c r="D133" s="27" t="inlineStr">
         <is>
-          <t>报价撮合与对价</t>
+          <t>有限差分（PDE）</t>
         </is>
       </c>
       <c r="E133" s="11" t="inlineStr">
         <is>
-          <t>报价展示（对价/最优报价），撮合对价，报价提醒，交易包管理，报价成交确认</t>
+          <t>Crank-Nicolson/ADI方法，含权债/可转债精确定价</t>
         </is>
       </c>
       <c r="F133" s="11" t="inlineStr">
         <is>
-          <t>功能测试通过/正确率100%</t>
-        </is>
-      </c>
-      <c r="G133" s="24" t="inlineStr">
-        <is>
-          <t>中</t>
+          <t>p99延迟/误差率/精度验证/压测10k TPS</t>
+        </is>
+      </c>
+      <c r="G133" s="28" t="inlineStr">
+        <is>
+          <t>极高</t>
         </is>
       </c>
       <c r="H133" s="13" t="n">
-        <v>20</v>
+        <v>60</v>
       </c>
     </row>
     <row r="134" ht="28" customHeight="1">
       <c r="A134" s="11" t="inlineStr">
         <is>
-          <t>销售交易</t>
+          <t>定价平台</t>
         </is>
       </c>
       <c r="B134" s="10" t="inlineStr">
@@ -6906,37 +6940,37 @@
       </c>
       <c r="C134" s="10" t="inlineStr">
         <is>
-          <t>F10-04</t>
+          <t>F09-04</t>
         </is>
       </c>
       <c r="D134" s="27" t="inlineStr">
         <is>
-          <t>交易执行与审批</t>
+          <t>实时Greeks</t>
         </is>
       </c>
       <c r="E134" s="11" t="inlineStr">
         <is>
-          <t>意向达成，交易要素校验，手工价录入，业务审批流程，交易执行</t>
+          <t>Delta/Gamma/Vega/Theta/Rho分布式实时计算</t>
         </is>
       </c>
       <c r="F134" s="11" t="inlineStr">
         <is>
-          <t>功能测试通过/正确率100%</t>
-        </is>
-      </c>
-      <c r="G134" s="24" t="inlineStr">
-        <is>
-          <t>中</t>
+          <t>功能完整/边界测试/集成冒烟/性能基线</t>
+        </is>
+      </c>
+      <c r="G134" s="23" t="inlineStr">
+        <is>
+          <t>高</t>
         </is>
       </c>
       <c r="H134" s="13" t="n">
-        <v>15</v>
+        <v>40</v>
       </c>
     </row>
     <row r="135" ht="28" customHeight="1">
       <c r="A135" s="11" t="inlineStr">
         <is>
-          <t>销售交易</t>
+          <t>定价平台</t>
         </is>
       </c>
       <c r="B135" s="10" t="inlineStr">
@@ -6946,37 +6980,37 @@
       </c>
       <c r="C135" s="10" t="inlineStr">
         <is>
-          <t>F10-05</t>
+          <t>F09-05</t>
         </is>
       </c>
       <c r="D135" s="27" t="inlineStr">
         <is>
-          <t>风控检查</t>
+          <t>定价服务微服务架构</t>
         </is>
       </c>
       <c r="E135" s="11" t="inlineStr">
         <is>
-          <t>交易前风控规则校验，限额检查，合规拦截，风控记录留痕</t>
+          <t>REST/gRPC定价API，支持横向扩展，p99&lt;100ms</t>
         </is>
       </c>
       <c r="F135" s="11" t="inlineStr">
         <is>
-          <t>功能测试通过/正确率100%</t>
-        </is>
-      </c>
-      <c r="G135" s="24" t="inlineStr">
-        <is>
-          <t>中</t>
+          <t>功能完整/边界测试/集成冒烟/性能基线</t>
+        </is>
+      </c>
+      <c r="G135" s="23" t="inlineStr">
+        <is>
+          <t>高</t>
         </is>
       </c>
       <c r="H135" s="13" t="n">
-        <v>15</v>
+        <v>40</v>
       </c>
     </row>
     <row r="136" ht="28" customHeight="1">
       <c r="A136" s="11" t="inlineStr">
         <is>
-          <t>销售交易</t>
+          <t>定价平台</t>
         </is>
       </c>
       <c r="B136" s="10" t="inlineStr">
@@ -6986,17 +7020,17 @@
       </c>
       <c r="C136" s="10" t="inlineStr">
         <is>
-          <t>F10-06</t>
+          <t>F09-06</t>
         </is>
       </c>
       <c r="D136" s="27" t="inlineStr">
         <is>
-          <t>智能推荐系统</t>
+          <t>历史估值回测</t>
         </is>
       </c>
       <c r="E136" s="11" t="inlineStr">
         <is>
-          <t>从被动客户服务转向主动服务，基于客户画像与持仓分析智能推荐券种，提升客户响应效率</t>
+          <t>基于历史行情重放定价误差分析，模型验证框架</t>
         </is>
       </c>
       <c r="F136" s="11" t="inlineStr">
@@ -7010,20 +7044,20 @@
         </is>
       </c>
       <c r="H136" s="13" t="n">
-        <v>25</v>
+        <v>30</v>
       </c>
     </row>
     <row r="137" ht="20" customHeight="1">
       <c r="A137" s="26" t="inlineStr">
         <is>
-          <t>【P2】 信用债/信用衍生品  (Credit &amp; CDS)</t>
+          <t>【P2】 销售交易  (Sales Trading)</t>
         </is>
       </c>
     </row>
     <row r="138" ht="28" customHeight="1">
       <c r="A138" s="11" t="inlineStr">
         <is>
-          <t>信用债/信用衍生品</t>
+          <t>销售交易</t>
         </is>
       </c>
       <c r="B138" s="10" t="inlineStr">
@@ -7033,37 +7067,37 @@
       </c>
       <c r="C138" s="10" t="inlineStr">
         <is>
-          <t>F11-01</t>
+          <t>F10-01</t>
         </is>
       </c>
       <c r="D138" s="27" t="inlineStr">
         <is>
-          <t>信用利差分析</t>
+          <t>销交工作台</t>
         </is>
       </c>
       <c r="E138" s="11" t="inlineStr">
         <is>
-          <t>行业/评级/期限信用利差曲线实时计算，历史分位数分析</t>
+          <t>报价管理主界面，历史报价管理，当日报价快捷操作，导入/导出报价，一键unrefer操作</t>
         </is>
       </c>
       <c r="F138" s="11" t="inlineStr">
         <is>
-          <t>功能完整/边界测试/集成冒烟/性能基线</t>
-        </is>
-      </c>
-      <c r="G138" s="23" t="inlineStr">
-        <is>
-          <t>高</t>
+          <t>功能测试通过/正确率100%</t>
+        </is>
+      </c>
+      <c r="G138" s="24" t="inlineStr">
+        <is>
+          <t>中</t>
         </is>
       </c>
       <c r="H138" s="13" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
     </row>
     <row r="139" ht="28" customHeight="1">
       <c r="A139" s="11" t="inlineStr">
         <is>
-          <t>信用债/信用衍生品</t>
+          <t>销售交易</t>
         </is>
       </c>
       <c r="B139" s="10" t="inlineStr">
@@ -7073,37 +7107,37 @@
       </c>
       <c r="C139" s="10" t="inlineStr">
         <is>
-          <t>F11-02</t>
+          <t>F10-02</t>
         </is>
       </c>
       <c r="D139" s="27" t="inlineStr">
         <is>
-          <t>CDS/CLN定价</t>
+          <t>债券过滤与筛选</t>
         </is>
       </c>
       <c r="E139" s="11" t="inlineStr">
         <is>
-          <t>信用违约互换定价，ISDA标准，生存概率曲线校准</t>
+          <t>信用债/利率债过滤，信用债全品种过滤，利率债国债/证金债/地方债分类过滤，精确与模糊识别</t>
         </is>
       </c>
       <c r="F139" s="11" t="inlineStr">
         <is>
-          <t>p99延迟/误差率/精度验证/压测10k TPS</t>
-        </is>
-      </c>
-      <c r="G139" s="28" t="inlineStr">
-        <is>
-          <t>极高</t>
+          <t>功能测试通过</t>
+        </is>
+      </c>
+      <c r="G139" s="25" t="inlineStr">
+        <is>
+          <t>低</t>
         </is>
       </c>
       <c r="H139" s="13" t="n">
-        <v>50</v>
+        <v>10</v>
       </c>
     </row>
     <row r="140" ht="28" customHeight="1">
       <c r="A140" s="11" t="inlineStr">
         <is>
-          <t>信用债/信用衍生品</t>
+          <t>销售交易</t>
         </is>
       </c>
       <c r="B140" s="10" t="inlineStr">
@@ -7113,17 +7147,17 @@
       </c>
       <c r="C140" s="10" t="inlineStr">
         <is>
-          <t>F11-03</t>
+          <t>F10-03</t>
         </is>
       </c>
       <c r="D140" s="27" t="inlineStr">
         <is>
-          <t>信用评级动态监控</t>
+          <t>报价撮合与对价</t>
         </is>
       </c>
       <c r="E140" s="11" t="inlineStr">
         <is>
-          <t>对接外部评级机构（中诚信/联合/大公），评级下调预警</t>
+          <t>报价展示（对价/最优报价），撮合对价，报价提醒，交易包管理，报价成交确认</t>
         </is>
       </c>
       <c r="F140" s="11" t="inlineStr">
@@ -7143,7 +7177,7 @@
     <row r="141" ht="28" customHeight="1">
       <c r="A141" s="11" t="inlineStr">
         <is>
-          <t>信用债/信用衍生品</t>
+          <t>销售交易</t>
         </is>
       </c>
       <c r="B141" s="10" t="inlineStr">
@@ -7153,37 +7187,37 @@
       </c>
       <c r="C141" s="10" t="inlineStr">
         <is>
-          <t>F11-04</t>
+          <t>F10-04</t>
         </is>
       </c>
       <c r="D141" s="27" t="inlineStr">
         <is>
-          <t>违约概率（PD）建模</t>
+          <t>交易执行与审批</t>
         </is>
       </c>
       <c r="E141" s="11" t="inlineStr">
         <is>
-          <t>结构化Merton模型+市场隐含PD，信用风险计量</t>
+          <t>意向达成，交易要素校验，手工价录入，业务审批流程，交易执行</t>
         </is>
       </c>
       <c r="F141" s="11" t="inlineStr">
         <is>
-          <t>功能完整/边界测试/集成冒烟/性能基线</t>
-        </is>
-      </c>
-      <c r="G141" s="23" t="inlineStr">
-        <is>
-          <t>高</t>
+          <t>功能测试通过/正确率100%</t>
+        </is>
+      </c>
+      <c r="G141" s="24" t="inlineStr">
+        <is>
+          <t>中</t>
         </is>
       </c>
       <c r="H141" s="13" t="n">
-        <v>40</v>
+        <v>15</v>
       </c>
     </row>
     <row r="142" ht="28" customHeight="1">
       <c r="A142" s="11" t="inlineStr">
         <is>
-          <t>信用债/信用衍生品</t>
+          <t>销售交易</t>
         </is>
       </c>
       <c r="B142" s="10" t="inlineStr">
@@ -7193,17 +7227,17 @@
       </c>
       <c r="C142" s="10" t="inlineStr">
         <is>
-          <t>F11-05</t>
+          <t>F10-05</t>
         </is>
       </c>
       <c r="D142" s="27" t="inlineStr">
         <is>
-          <t>集中度限额管理</t>
+          <t>风控检查</t>
         </is>
       </c>
       <c r="E142" s="11" t="inlineStr">
         <is>
-          <t>行业/发行人/评级集中度多维限额，超限预警</t>
+          <t>交易前风控规则校验，限额检查，合规拦截，风控记录留痕</t>
         </is>
       </c>
       <c r="F142" s="11" t="inlineStr">
@@ -7217,60 +7251,60 @@
         </is>
       </c>
       <c r="H142" s="13" t="n">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="143" ht="20" customHeight="1">
-      <c r="A143" s="26" t="inlineStr">
-        <is>
-          <t>【P2】 投顾服务  (Investment Advisory)</t>
-        </is>
-      </c>
-    </row>
-    <row r="144" ht="28" customHeight="1">
-      <c r="A144" s="11" t="inlineStr">
-        <is>
-          <t>投顾服务</t>
-        </is>
-      </c>
-      <c r="B144" s="10" t="inlineStr">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="143" ht="28" customHeight="1">
+      <c r="A143" s="11" t="inlineStr">
+        <is>
+          <t>销售交易</t>
+        </is>
+      </c>
+      <c r="B143" s="10" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
       </c>
-      <c r="C144" s="10" t="inlineStr">
-        <is>
-          <t>F12-01</t>
-        </is>
-      </c>
-      <c r="D144" s="27" t="inlineStr">
-        <is>
-          <t>投顾工作台</t>
-        </is>
-      </c>
-      <c r="E144" s="11" t="inlineStr">
-        <is>
-          <t>投顾人员操作界面，管理客户委托，上传研究报告，发送投资建议，查看客户反馈</t>
-        </is>
-      </c>
-      <c r="F144" s="11" t="inlineStr">
-        <is>
-          <t>功能测试通过/正确率100%</t>
-        </is>
-      </c>
-      <c r="G144" s="24" t="inlineStr">
-        <is>
-          <t>中</t>
-        </is>
-      </c>
-      <c r="H144" s="13" t="n">
-        <v>20</v>
+      <c r="C143" s="10" t="inlineStr">
+        <is>
+          <t>F10-06</t>
+        </is>
+      </c>
+      <c r="D143" s="27" t="inlineStr">
+        <is>
+          <t>智能推荐系统</t>
+        </is>
+      </c>
+      <c r="E143" s="11" t="inlineStr">
+        <is>
+          <t>从被动客户服务转向主动服务，基于客户画像与持仓分析智能推荐券种，提升客户响应效率</t>
+        </is>
+      </c>
+      <c r="F143" s="11" t="inlineStr">
+        <is>
+          <t>功能完整/边界测试/集成冒烟/性能基线</t>
+        </is>
+      </c>
+      <c r="G143" s="23" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="H143" s="13" t="n">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="144" ht="20" customHeight="1">
+      <c r="A144" s="26" t="inlineStr">
+        <is>
+          <t>【P2】 信用债/信用衍生品  (Credit &amp; CDS)</t>
+        </is>
       </c>
     </row>
     <row r="145" ht="28" customHeight="1">
       <c r="A145" s="11" t="inlineStr">
         <is>
-          <t>投顾服务</t>
+          <t>信用债/信用衍生品</t>
         </is>
       </c>
       <c r="B145" s="10" t="inlineStr">
@@ -7280,37 +7314,37 @@
       </c>
       <c r="C145" s="10" t="inlineStr">
         <is>
-          <t>F12-02</t>
+          <t>F11-01</t>
         </is>
       </c>
       <c r="D145" s="27" t="inlineStr">
         <is>
-          <t>客户终端</t>
+          <t>信用利差分析</t>
         </is>
       </c>
       <c r="E145" s="11" t="inlineStr">
         <is>
-          <t>客户查看投资建议与分析报告，确认交易服务，查看账户净值走势、持仓明细、交易明细</t>
+          <t>行业/评级/期限信用利差曲线实时计算，历史分位数分析</t>
         </is>
       </c>
       <c r="F145" s="11" t="inlineStr">
         <is>
-          <t>功能测试通过/正确率100%</t>
-        </is>
-      </c>
-      <c r="G145" s="24" t="inlineStr">
-        <is>
-          <t>中</t>
+          <t>功能完整/边界测试/集成冒烟/性能基线</t>
+        </is>
+      </c>
+      <c r="G145" s="23" t="inlineStr">
+        <is>
+          <t>高</t>
         </is>
       </c>
       <c r="H145" s="13" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
     </row>
     <row r="146" ht="28" customHeight="1">
       <c r="A146" s="11" t="inlineStr">
         <is>
-          <t>投顾服务</t>
+          <t>信用债/信用衍生品</t>
         </is>
       </c>
       <c r="B146" s="10" t="inlineStr">
@@ -7320,37 +7354,37 @@
       </c>
       <c r="C146" s="10" t="inlineStr">
         <is>
-          <t>F12-03</t>
+          <t>F11-02</t>
         </is>
       </c>
       <c r="D146" s="27" t="inlineStr">
         <is>
-          <t>投资建议书管理</t>
+          <t>CDS/CLN定价</t>
         </is>
       </c>
       <c r="E146" s="11" t="inlineStr">
         <is>
-          <t>投资建议书线上生成、审批、确认全流程，留痕追溯，客户电子签收</t>
+          <t>信用违约互换定价，ISDA标准，生存概率曲线校准</t>
         </is>
       </c>
       <c r="F146" s="11" t="inlineStr">
         <is>
-          <t>功能测试通过/正确率100%</t>
-        </is>
-      </c>
-      <c r="G146" s="24" t="inlineStr">
-        <is>
-          <t>中</t>
+          <t>p99延迟/误差率/精度验证/压测10k TPS</t>
+        </is>
+      </c>
+      <c r="G146" s="28" t="inlineStr">
+        <is>
+          <t>极高</t>
         </is>
       </c>
       <c r="H146" s="13" t="n">
-        <v>15</v>
+        <v>50</v>
       </c>
     </row>
     <row r="147" ht="28" customHeight="1">
       <c r="A147" s="11" t="inlineStr">
         <is>
-          <t>投顾服务</t>
+          <t>信用债/信用衍生品</t>
         </is>
       </c>
       <c r="B147" s="10" t="inlineStr">
@@ -7360,37 +7394,37 @@
       </c>
       <c r="C147" s="10" t="inlineStr">
         <is>
-          <t>F12-04</t>
+          <t>F11-03</t>
         </is>
       </c>
       <c r="D147" s="27" t="inlineStr">
         <is>
-          <t>账户分析报告</t>
+          <t>信用评级动态监控</t>
         </is>
       </c>
       <c r="E147" s="11" t="inlineStr">
         <is>
-          <t>账户净值走势、久期走势、归因分析、估值台账等核心数据展示及定期报告生成</t>
+          <t>对接外部评级机构（中诚信/联合/大公），评级下调预警</t>
         </is>
       </c>
       <c r="F147" s="11" t="inlineStr">
         <is>
-          <t>功能完整/边界测试/集成冒烟/性能基线</t>
-        </is>
-      </c>
-      <c r="G147" s="23" t="inlineStr">
-        <is>
-          <t>高</t>
+          <t>功能测试通过/正确率100%</t>
+        </is>
+      </c>
+      <c r="G147" s="24" t="inlineStr">
+        <is>
+          <t>中</t>
         </is>
       </c>
       <c r="H147" s="13" t="n">
-        <v>25</v>
+        <v>20</v>
       </c>
     </row>
     <row r="148" ht="28" customHeight="1">
       <c r="A148" s="11" t="inlineStr">
         <is>
-          <t>投顾服务</t>
+          <t>信用债/信用衍生品</t>
         </is>
       </c>
       <c r="B148" s="10" t="inlineStr">
@@ -7400,37 +7434,37 @@
       </c>
       <c r="C148" s="10" t="inlineStr">
         <is>
-          <t>F12-05</t>
+          <t>F11-04</t>
         </is>
       </c>
       <c r="D148" s="27" t="inlineStr">
         <is>
-          <t>投研报告服务</t>
+          <t>违约概率（PD）建模</t>
         </is>
       </c>
       <c r="E148" s="11" t="inlineStr">
         <is>
-          <t>日/周/月研究报告上传与推送，RPA自动获取基础数据，报告分类管理</t>
+          <t>结构化Merton模型+市场隐含PD，信用风险计量</t>
         </is>
       </c>
       <c r="F148" s="11" t="inlineStr">
         <is>
-          <t>功能测试通过/正确率100%</t>
-        </is>
-      </c>
-      <c r="G148" s="24" t="inlineStr">
-        <is>
-          <t>中</t>
+          <t>功能完整/边界测试/集成冒烟/性能基线</t>
+        </is>
+      </c>
+      <c r="G148" s="23" t="inlineStr">
+        <is>
+          <t>高</t>
         </is>
       </c>
       <c r="H148" s="13" t="n">
-        <v>15</v>
+        <v>40</v>
       </c>
     </row>
     <row r="149" ht="28" customHeight="1">
       <c r="A149" s="11" t="inlineStr">
         <is>
-          <t>投顾服务</t>
+          <t>信用债/信用衍生品</t>
         </is>
       </c>
       <c r="B149" s="10" t="inlineStr">
@@ -7440,44 +7474,44 @@
       </c>
       <c r="C149" s="10" t="inlineStr">
         <is>
-          <t>F12-06</t>
+          <t>F11-05</t>
         </is>
       </c>
       <c r="D149" s="27" t="inlineStr">
         <is>
-          <t>客户服务与基础服务</t>
+          <t>集中度限额管理</t>
         </is>
       </c>
       <c r="E149" s="11" t="inlineStr">
         <is>
-          <t>服务中心、消息中心、问卷系统；用户/账户/数据管理，消息群发，登录注册</t>
+          <t>行业/发行人/评级集中度多维限额，超限预警</t>
         </is>
       </c>
       <c r="F149" s="11" t="inlineStr">
         <is>
-          <t>功能测试通过</t>
-        </is>
-      </c>
-      <c r="G149" s="25" t="inlineStr">
-        <is>
-          <t>低</t>
+          <t>功能测试通过/正确率100%</t>
+        </is>
+      </c>
+      <c r="G149" s="24" t="inlineStr">
+        <is>
+          <t>中</t>
         </is>
       </c>
       <c r="H149" s="13" t="n">
-        <v>10</v>
+        <v>20</v>
       </c>
     </row>
     <row r="150" ht="20" customHeight="1">
       <c r="A150" s="26" t="inlineStr">
         <is>
-          <t>【P2】 TRS收益互换  (Total Return Swap)</t>
+          <t>【P2】 投顾服务  (Investment Advisory)</t>
         </is>
       </c>
     </row>
     <row r="151" ht="28" customHeight="1">
       <c r="A151" s="11" t="inlineStr">
         <is>
-          <t>TRS收益互换</t>
+          <t>投顾服务</t>
         </is>
       </c>
       <c r="B151" s="10" t="inlineStr">
@@ -7487,37 +7521,37 @@
       </c>
       <c r="C151" s="10" t="inlineStr">
         <is>
-          <t>F13-01</t>
+          <t>F12-01</t>
         </is>
       </c>
       <c r="D151" s="27" t="inlineStr">
         <is>
-          <t>TRS交易端</t>
+          <t>投顾工作台</t>
         </is>
       </c>
       <c r="E151" s="11" t="inlineStr">
         <is>
-          <t>报价提供，成交回报，对冲委托与自动对冲，请求报价，行情与资讯，历史确认</t>
+          <t>投顾人员操作界面，管理客户委托，上传研究报告，发送投资建议，查看客户反馈</t>
         </is>
       </c>
       <c r="F151" s="11" t="inlineStr">
         <is>
-          <t>功能完整/边界测试/集成冒烟/性能基线</t>
-        </is>
-      </c>
-      <c r="G151" s="23" t="inlineStr">
-        <is>
-          <t>高</t>
+          <t>功能测试通过/正确率100%</t>
+        </is>
+      </c>
+      <c r="G151" s="24" t="inlineStr">
+        <is>
+          <t>中</t>
         </is>
       </c>
       <c r="H151" s="13" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
     </row>
     <row r="152" ht="28" customHeight="1">
       <c r="A152" s="11" t="inlineStr">
         <is>
-          <t>TRS收益互换</t>
+          <t>投顾服务</t>
         </is>
       </c>
       <c r="B152" s="10" t="inlineStr">
@@ -7527,37 +7561,37 @@
       </c>
       <c r="C152" s="10" t="inlineStr">
         <is>
-          <t>F13-02</t>
+          <t>F12-02</t>
         </is>
       </c>
       <c r="D152" s="27" t="inlineStr">
         <is>
-          <t>TRS客户端</t>
+          <t>客户终端</t>
         </is>
       </c>
       <c r="E152" s="11" t="inlineStr">
         <is>
-          <t>开户申请，客户委托，出入金申请，合约持仓，标的持仓，资金管理，行情矩阵，自主下单</t>
+          <t>客户查看投资建议与分析报告，确认交易服务，查看账户净值走势、持仓明细、交易明细</t>
         </is>
       </c>
       <c r="F152" s="11" t="inlineStr">
         <is>
-          <t>功能完整/边界测试/集成冒烟/性能基线</t>
-        </is>
-      </c>
-      <c r="G152" s="23" t="inlineStr">
-        <is>
-          <t>高</t>
+          <t>功能测试通过/正确率100%</t>
+        </is>
+      </c>
+      <c r="G152" s="24" t="inlineStr">
+        <is>
+          <t>中</t>
         </is>
       </c>
       <c r="H152" s="13" t="n">
-        <v>25</v>
+        <v>20</v>
       </c>
     </row>
     <row r="153" ht="28" customHeight="1">
       <c r="A153" s="11" t="inlineStr">
         <is>
-          <t>TRS收益互换</t>
+          <t>投顾服务</t>
         </is>
       </c>
       <c r="B153" s="10" t="inlineStr">
@@ -7567,17 +7601,17 @@
       </c>
       <c r="C153" s="10" t="inlineStr">
         <is>
-          <t>F13-03</t>
+          <t>F12-03</t>
         </is>
       </c>
       <c r="D153" s="27" t="inlineStr">
         <is>
-          <t>TRS管理端</t>
+          <t>投资建议书管理</t>
         </is>
       </c>
       <c r="E153" s="11" t="inlineStr">
         <is>
-          <t>开户申请审批，合约成交管理，出入金审批，运营管理，对账，库存，对冲录入</t>
+          <t>投资建议书线上生成、审批、确认全流程，留痕追溯，客户电子签收</t>
         </is>
       </c>
       <c r="F153" s="11" t="inlineStr">
@@ -7591,13 +7625,13 @@
         </is>
       </c>
       <c r="H153" s="13" t="n">
-        <v>20</v>
+        <v>15</v>
       </c>
     </row>
     <row r="154" ht="28" customHeight="1">
       <c r="A154" s="11" t="inlineStr">
         <is>
-          <t>TRS收益互换</t>
+          <t>投顾服务</t>
         </is>
       </c>
       <c r="B154" s="10" t="inlineStr">
@@ -7607,17 +7641,17 @@
       </c>
       <c r="C154" s="10" t="inlineStr">
         <is>
-          <t>F13-04</t>
+          <t>F12-04</t>
         </is>
       </c>
       <c r="D154" s="27" t="inlineStr">
         <is>
-          <t>自动对冲</t>
+          <t>账户分析报告</t>
         </is>
       </c>
       <c r="E154" s="11" t="inlineStr">
         <is>
-          <t>对冲委托自动触发，对冲回报处理，风险校验，组合重叠分析，开平仓设置</t>
+          <t>账户净值走势、久期走势、归因分析、估值台账等核心数据展示及定期报告生成</t>
         </is>
       </c>
       <c r="F154" s="11" t="inlineStr">
@@ -7637,7 +7671,7 @@
     <row r="155" ht="28" customHeight="1">
       <c r="A155" s="11" t="inlineStr">
         <is>
-          <t>TRS收益互换</t>
+          <t>投顾服务</t>
         </is>
       </c>
       <c r="B155" s="10" t="inlineStr">
@@ -7647,17 +7681,17 @@
       </c>
       <c r="C155" s="10" t="inlineStr">
         <is>
-          <t>F13-05</t>
+          <t>F12-05</t>
         </is>
       </c>
       <c r="D155" s="27" t="inlineStr">
         <is>
-          <t>通知与确认文件</t>
+          <t>投研报告服务</t>
         </is>
       </c>
       <c r="E155" s="11" t="inlineStr">
         <is>
-          <t>企微通知提醒，确认书/结算单/估值报告/出入金通知自动生成并通过邮箱发送</t>
+          <t>日/周/月研究报告上传与推送，RPA自动获取基础数据，报告分类管理</t>
         </is>
       </c>
       <c r="F155" s="11" t="inlineStr">
@@ -7677,278 +7711,525 @@
     <row r="156" ht="28" customHeight="1">
       <c r="A156" s="11" t="inlineStr">
         <is>
+          <t>投顾服务</t>
+        </is>
+      </c>
+      <c r="B156" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="C156" s="10" t="inlineStr">
+        <is>
+          <t>F12-06</t>
+        </is>
+      </c>
+      <c r="D156" s="27" t="inlineStr">
+        <is>
+          <t>客户服务与基础服务</t>
+        </is>
+      </c>
+      <c r="E156" s="11" t="inlineStr">
+        <is>
+          <t>服务中心、消息中心、问卷系统；用户/账户/数据管理，消息群发，登录注册</t>
+        </is>
+      </c>
+      <c r="F156" s="11" t="inlineStr">
+        <is>
+          <t>功能测试通过</t>
+        </is>
+      </c>
+      <c r="G156" s="25" t="inlineStr">
+        <is>
+          <t>低</t>
+        </is>
+      </c>
+      <c r="H156" s="13" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="157" ht="20" customHeight="1">
+      <c r="A157" s="26" t="inlineStr">
+        <is>
+          <t>【P2】 TRS收益互换  (Total Return Swap)</t>
+        </is>
+      </c>
+    </row>
+    <row r="158" ht="28" customHeight="1">
+      <c r="A158" s="11" t="inlineStr">
+        <is>
           <t>TRS收益互换</t>
         </is>
       </c>
-      <c r="B156" s="10" t="inlineStr">
+      <c r="B158" s="10" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
       </c>
-      <c r="C156" s="10" t="inlineStr">
+      <c r="C158" s="10" t="inlineStr">
+        <is>
+          <t>F13-01</t>
+        </is>
+      </c>
+      <c r="D158" s="27" t="inlineStr">
+        <is>
+          <t>TRS交易端</t>
+        </is>
+      </c>
+      <c r="E158" s="11" t="inlineStr">
+        <is>
+          <t>报价提供，成交回报，对冲委托与自动对冲，请求报价，行情与资讯，历史确认</t>
+        </is>
+      </c>
+      <c r="F158" s="11" t="inlineStr">
+        <is>
+          <t>功能完整/边界测试/集成冒烟/性能基线</t>
+        </is>
+      </c>
+      <c r="G158" s="23" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="H158" s="13" t="n">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="159" ht="28" customHeight="1">
+      <c r="A159" s="11" t="inlineStr">
+        <is>
+          <t>TRS收益互换</t>
+        </is>
+      </c>
+      <c r="B159" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="C159" s="10" t="inlineStr">
+        <is>
+          <t>F13-02</t>
+        </is>
+      </c>
+      <c r="D159" s="27" t="inlineStr">
+        <is>
+          <t>TRS客户端</t>
+        </is>
+      </c>
+      <c r="E159" s="11" t="inlineStr">
+        <is>
+          <t>开户申请，客户委托，出入金申请，合约持仓，标的持仓，资金管理，行情矩阵，自主下单</t>
+        </is>
+      </c>
+      <c r="F159" s="11" t="inlineStr">
+        <is>
+          <t>功能完整/边界测试/集成冒烟/性能基线</t>
+        </is>
+      </c>
+      <c r="G159" s="23" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="H159" s="13" t="n">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="160" ht="28" customHeight="1">
+      <c r="A160" s="11" t="inlineStr">
+        <is>
+          <t>TRS收益互换</t>
+        </is>
+      </c>
+      <c r="B160" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="C160" s="10" t="inlineStr">
+        <is>
+          <t>F13-03</t>
+        </is>
+      </c>
+      <c r="D160" s="27" t="inlineStr">
+        <is>
+          <t>TRS管理端</t>
+        </is>
+      </c>
+      <c r="E160" s="11" t="inlineStr">
+        <is>
+          <t>开户申请审批，合约成交管理，出入金审批，运营管理，对账，库存，对冲录入</t>
+        </is>
+      </c>
+      <c r="F160" s="11" t="inlineStr">
+        <is>
+          <t>功能测试通过/正确率100%</t>
+        </is>
+      </c>
+      <c r="G160" s="24" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="H160" s="13" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="161" ht="28" customHeight="1">
+      <c r="A161" s="11" t="inlineStr">
+        <is>
+          <t>TRS收益互换</t>
+        </is>
+      </c>
+      <c r="B161" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="C161" s="10" t="inlineStr">
+        <is>
+          <t>F13-04</t>
+        </is>
+      </c>
+      <c r="D161" s="27" t="inlineStr">
+        <is>
+          <t>自动对冲</t>
+        </is>
+      </c>
+      <c r="E161" s="11" t="inlineStr">
+        <is>
+          <t>对冲委托自动触发，对冲回报处理，风险校验，组合重叠分析，开平仓设置</t>
+        </is>
+      </c>
+      <c r="F161" s="11" t="inlineStr">
+        <is>
+          <t>功能完整/边界测试/集成冒烟/性能基线</t>
+        </is>
+      </c>
+      <c r="G161" s="23" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="H161" s="13" t="n">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="162" ht="28" customHeight="1">
+      <c r="A162" s="11" t="inlineStr">
+        <is>
+          <t>TRS收益互换</t>
+        </is>
+      </c>
+      <c r="B162" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="C162" s="10" t="inlineStr">
+        <is>
+          <t>F13-05</t>
+        </is>
+      </c>
+      <c r="D162" s="27" t="inlineStr">
+        <is>
+          <t>通知与确认文件</t>
+        </is>
+      </c>
+      <c r="E162" s="11" t="inlineStr">
+        <is>
+          <t>企微通知提醒，确认书/结算单/估值报告/出入金通知自动生成并通过邮箱发送</t>
+        </is>
+      </c>
+      <c r="F162" s="11" t="inlineStr">
+        <is>
+          <t>功能测试通过/正确率100%</t>
+        </is>
+      </c>
+      <c r="G162" s="24" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="H162" s="13" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="163" ht="28" customHeight="1">
+      <c r="A163" s="11" t="inlineStr">
+        <is>
+          <t>TRS收益互换</t>
+        </is>
+      </c>
+      <c r="B163" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="C163" s="10" t="inlineStr">
         <is>
           <t>F13-06</t>
         </is>
       </c>
-      <c r="D156" s="27" t="inlineStr">
+      <c r="D163" s="27" t="inlineStr">
         <is>
           <t>系统集成</t>
         </is>
       </c>
-      <c r="E156" s="11" t="inlineStr">
+      <c r="E163" s="11" t="inlineStr">
         <is>
           <t>与衡泰系统客户信息同步，QTrade聊天记录同步，交易管理系统对接，银行流水对接</t>
         </is>
       </c>
-      <c r="F156" s="11" t="inlineStr">
+      <c r="F163" s="11" t="inlineStr">
         <is>
           <t>功能完整/边界测试/集成冒烟/性能基线</t>
         </is>
       </c>
-      <c r="G156" s="23" t="inlineStr">
+      <c r="G163" s="23" t="inlineStr">
         <is>
           <t>高</t>
         </is>
       </c>
-      <c r="H156" s="13" t="n">
+      <c r="H163" s="13" t="n">
         <v>25</v>
       </c>
     </row>
-    <row r="157" ht="20" customHeight="1">
-      <c r="A157" s="29" t="inlineStr">
+    <row r="164" ht="20" customHeight="1">
+      <c r="A164" s="29" t="inlineStr">
         <is>
           <t>【P3】 做市商系统  (Market Making)</t>
         </is>
       </c>
     </row>
-    <row r="158" ht="28" customHeight="1">
-      <c r="A158" s="16" t="inlineStr">
+    <row r="165" ht="28" customHeight="1">
+      <c r="A165" s="16" t="inlineStr">
         <is>
           <t>做市商系统</t>
         </is>
       </c>
-      <c r="B158" s="15" t="inlineStr">
+      <c r="B165" s="15" t="inlineStr">
         <is>
           <t>P3</t>
         </is>
       </c>
-      <c r="C158" s="15" t="inlineStr">
+      <c r="C165" s="15" t="inlineStr">
         <is>
           <t>F15-01</t>
         </is>
       </c>
-      <c r="D158" s="30" t="inlineStr">
+      <c r="D165" s="30" t="inlineStr">
         <is>
           <t>双边报价引擎</t>
         </is>
       </c>
-      <c r="E158" s="16" t="inlineStr">
+      <c r="E165" s="16" t="inlineStr">
         <is>
           <t>多品种同时双边报价，延迟&lt;5ms，报价宽度动态优化</t>
         </is>
       </c>
-      <c r="F158" s="16" t="inlineStr">
+      <c r="F165" s="16" t="inlineStr">
         <is>
           <t>p99延迟/误差率/精度验证/压测10k TPS</t>
         </is>
       </c>
-      <c r="G158" s="28" t="inlineStr">
+      <c r="G165" s="28" t="inlineStr">
         <is>
           <t>极高</t>
         </is>
       </c>
-      <c r="H158" s="18" t="n">
+      <c r="H165" s="18" t="n">
         <v>70</v>
       </c>
     </row>
-    <row r="159" ht="28" customHeight="1">
-      <c r="A159" s="16" t="inlineStr">
+    <row r="166" ht="28" customHeight="1">
+      <c r="A166" s="16" t="inlineStr">
         <is>
           <t>做市商系统</t>
         </is>
       </c>
-      <c r="B159" s="15" t="inlineStr">
+      <c r="B166" s="15" t="inlineStr">
         <is>
           <t>P3</t>
         </is>
       </c>
-      <c r="C159" s="15" t="inlineStr">
+      <c r="C166" s="15" t="inlineStr">
         <is>
           <t>F15-02</t>
         </is>
       </c>
-      <c r="D159" s="30" t="inlineStr">
+      <c r="D166" s="30" t="inlineStr">
         <is>
           <t>库存风险实时管理</t>
         </is>
       </c>
-      <c r="E159" s="16" t="inlineStr">
+      <c r="E166" s="16" t="inlineStr">
         <is>
           <t>做市库存PnL实时监控，Delta对冲自动触发</t>
         </is>
       </c>
-      <c r="F159" s="16" t="inlineStr">
+      <c r="F166" s="16" t="inlineStr">
         <is>
           <t>p99延迟/误差率/精度验证/压测10k TPS</t>
         </is>
       </c>
-      <c r="G159" s="28" t="inlineStr">
+      <c r="G166" s="28" t="inlineStr">
         <is>
           <t>极高</t>
         </is>
       </c>
-      <c r="H159" s="18" t="n">
+      <c r="H166" s="18" t="n">
         <v>60</v>
       </c>
     </row>
-    <row r="160" ht="28" customHeight="1">
-      <c r="A160" s="16" t="inlineStr">
+    <row r="167" ht="28" customHeight="1">
+      <c r="A167" s="16" t="inlineStr">
         <is>
           <t>做市商系统</t>
         </is>
       </c>
-      <c r="B160" s="15" t="inlineStr">
+      <c r="B167" s="15" t="inlineStr">
         <is>
           <t>P3</t>
         </is>
       </c>
-      <c r="C160" s="15" t="inlineStr">
+      <c r="C167" s="15" t="inlineStr">
         <is>
           <t>F15-03</t>
         </is>
       </c>
-      <c r="D160" s="30" t="inlineStr">
+      <c r="D167" s="30" t="inlineStr">
         <is>
           <t>报价优化算法</t>
         </is>
       </c>
-      <c r="E160" s="16" t="inlineStr">
+      <c r="E167" s="16" t="inlineStr">
         <is>
           <t>基于市场微结构理论动态调整bid-ask spread</t>
         </is>
       </c>
-      <c r="F160" s="16" t="inlineStr">
+      <c r="F167" s="16" t="inlineStr">
         <is>
           <t>p99延迟/误差率/精度验证/压测10k TPS</t>
         </is>
       </c>
-      <c r="G160" s="28" t="inlineStr">
+      <c r="G167" s="28" t="inlineStr">
         <is>
           <t>极高</t>
         </is>
       </c>
-      <c r="H160" s="18" t="n">
+      <c r="H167" s="18" t="n">
         <v>50</v>
       </c>
     </row>
-    <row r="161" ht="28" customHeight="1">
-      <c r="A161" s="16" t="inlineStr">
+    <row r="168" ht="28" customHeight="1">
+      <c r="A168" s="16" t="inlineStr">
         <is>
           <t>做市商系统</t>
         </is>
       </c>
-      <c r="B161" s="15" t="inlineStr">
+      <c r="B168" s="15" t="inlineStr">
         <is>
           <t>P3</t>
         </is>
       </c>
-      <c r="C161" s="15" t="inlineStr">
+      <c r="C168" s="15" t="inlineStr">
         <is>
           <t>F15-04</t>
         </is>
       </c>
-      <c r="D161" s="30" t="inlineStr">
+      <c r="D168" s="30" t="inlineStr">
         <is>
           <t>竞争力分析</t>
         </is>
       </c>
-      <c r="E161" s="16" t="inlineStr">
+      <c r="E168" s="16" t="inlineStr">
         <is>
           <t>与市场最优报价对比，中签率分析，策略调优</t>
         </is>
       </c>
-      <c r="F161" s="16" t="inlineStr">
+      <c r="F168" s="16" t="inlineStr">
         <is>
           <t>功能完整/边界测试/集成冒烟/性能基线</t>
         </is>
       </c>
-      <c r="G161" s="23" t="inlineStr">
+      <c r="G168" s="23" t="inlineStr">
         <is>
           <t>高</t>
         </is>
       </c>
-      <c r="H161" s="18" t="n">
+      <c r="H168" s="18" t="n">
         <v>25</v>
       </c>
     </row>
-    <row r="162" ht="28" customHeight="1">
-      <c r="A162" s="16" t="inlineStr">
+    <row r="169" ht="28" customHeight="1">
+      <c r="A169" s="16" t="inlineStr">
         <is>
           <t>做市商系统</t>
         </is>
       </c>
-      <c r="B162" s="15" t="inlineStr">
+      <c r="B169" s="15" t="inlineStr">
         <is>
           <t>P3</t>
         </is>
       </c>
-      <c r="C162" s="15" t="inlineStr">
+      <c r="C169" s="15" t="inlineStr">
         <is>
           <t>F15-05</t>
         </is>
       </c>
-      <c r="D162" s="30" t="inlineStr">
+      <c r="D169" s="30" t="inlineStr">
         <is>
           <t>交易对手管理集成</t>
         </is>
       </c>
-      <c r="E162" s="16" t="inlineStr">
+      <c r="E169" s="16" t="inlineStr">
         <is>
           <t>做市交易对手信用实时检查，额度占用同步更新</t>
         </is>
       </c>
-      <c r="F162" s="16" t="inlineStr">
+      <c r="F169" s="16" t="inlineStr">
         <is>
           <t>功能测试通过/正确率100%</t>
         </is>
       </c>
-      <c r="G162" s="24" t="inlineStr">
+      <c r="G169" s="24" t="inlineStr">
         <is>
           <t>中</t>
         </is>
       </c>
-      <c r="H162" s="18" t="n">
+      <c r="H169" s="18" t="n">
         <v>20</v>
       </c>
     </row>
-    <row r="163">
-      <c r="A163" s="19" t="inlineStr">
+    <row r="170">
+      <c r="A170" s="19" t="inlineStr">
         <is>
           <t>总计功能数 / Total Function Points</t>
         </is>
       </c>
-      <c r="H163" s="20">
-        <f>SUM(H3:H162)</f>
+      <c r="H170" s="20">
+        <f>SUM(H3:H169)</f>
         <v/>
       </c>
     </row>
   </sheetData>
   <mergeCells count="16">
+    <mergeCell ref="A170:G170"/>
     <mergeCell ref="A67:H67"/>
-    <mergeCell ref="A143:H143"/>
+    <mergeCell ref="A100:H100"/>
     <mergeCell ref="A3:H3"/>
+    <mergeCell ref="A106:H106"/>
+    <mergeCell ref="A124:H124"/>
     <mergeCell ref="A130:H130"/>
     <mergeCell ref="A87:H87"/>
+    <mergeCell ref="A144:H144"/>
     <mergeCell ref="A157:H157"/>
-    <mergeCell ref="A99:H99"/>
-    <mergeCell ref="A117:H117"/>
+    <mergeCell ref="A164:H164"/>
+    <mergeCell ref="A137:H137"/>
     <mergeCell ref="A60:H60"/>
-    <mergeCell ref="A137:H137"/>
-    <mergeCell ref="A163:G163"/>
     <mergeCell ref="A1:H1"/>
     <mergeCell ref="A150:H150"/>
-    <mergeCell ref="A93:H93"/>
-    <mergeCell ref="A123:H123"/>
     <mergeCell ref="A31:H31"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -8660,7 +8941,7 @@
         </is>
       </c>
       <c r="H3" s="8" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="I3" s="8" t="n">
         <v>8</v>
@@ -12758,6 +13039,605 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:J20"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="48" customWidth="1" min="4" max="4"/>
+    <col width="26" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="6" max="6"/>
+    <col width="8" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="8" max="8"/>
+    <col width="7" customWidth="1" min="9" max="9"/>
+    <col width="18" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="24" customHeight="1">
+      <c r="A1" s="38" t="inlineStr">
+        <is>
+          <t>系统详情：异常交易风控  |  Abnormal Trade Monitor</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="36" customHeight="1">
+      <c r="A2" s="39" t="inlineStr">
+        <is>
+          <t>战略定位：监管驱动，AI差异化（LLM+RAG+Agent+MCP），快速商业化；对应PPT Slide 50   |   来源：Slide 50</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="28" customHeight="1">
+      <c r="A3" s="40" t="inlineStr">
+        <is>
+          <t>模块：异常交易风控  (Abnormal Trade Monitor)  |  优先级：P1  |  竞品：无主导者  |  华锐基础：ARC+AI规则引擎  |  工期：8月  团队：8人</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="28" customHeight="1">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>功能域</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>编号</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>功能名称</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>功能描述</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>验收标准</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>集成依赖</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>复杂度</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>预估(人天)</t>
+        </is>
+      </c>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t>优先级</t>
+        </is>
+      </c>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>备注</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="18" customHeight="1">
+      <c r="A5" s="22" t="inlineStr">
+        <is>
+          <t>D1. AI智能引擎</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="48" customHeight="1">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>D1. AI智能引擎</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>F05-01</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>LLM大语言模型应用</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>客户意图识别，自然语言处理交易描述，智能报告自动生成，新规合规解读</t>
+        </is>
+      </c>
+      <c r="E6" s="5" t="inlineStr"/>
+      <c r="F6" s="5" t="inlineStr"/>
+      <c r="G6" s="28" t="inlineStr">
+        <is>
+          <t>极高</t>
+        </is>
+      </c>
+      <c r="H6" s="8" t="n">
+        <v>40</v>
+      </c>
+      <c r="I6" s="6" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="J6" s="5" t="inlineStr"/>
+    </row>
+    <row r="7" ht="48" customHeight="1">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>D1. AI智能引擎</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>F05-02</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>RAG检索增强生成</t>
+        </is>
+      </c>
+      <c r="D7" s="5" t="inlineStr">
+        <is>
+          <t>监管规则知识库构建，新规则智能固化，合规智能问答，上下文理解与规则推理</t>
+        </is>
+      </c>
+      <c r="E7" s="5" t="inlineStr"/>
+      <c r="F7" s="5" t="inlineStr"/>
+      <c r="G7" s="41" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="H7" s="8" t="n">
+        <v>30</v>
+      </c>
+      <c r="I7" s="6" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="J7" s="5" t="inlineStr"/>
+    </row>
+    <row r="8" ht="48" customHeight="1">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>D1. AI智能引擎</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>F05-03</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="inlineStr">
+        <is>
+          <t>Agent智能体</t>
+        </is>
+      </c>
+      <c r="D8" s="5" t="inlineStr">
+        <is>
+          <t>异常处置任务自动化，决策支持工作流，多步骤异常核查流程优化，自动推送处置建议</t>
+        </is>
+      </c>
+      <c r="E8" s="5" t="inlineStr"/>
+      <c r="F8" s="5" t="inlineStr"/>
+      <c r="G8" s="41" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="H8" s="8" t="n">
+        <v>30</v>
+      </c>
+      <c r="I8" s="6" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="J8" s="5" t="inlineStr"/>
+    </row>
+    <row r="9" ht="48" customHeight="1">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>D1. AI智能引擎</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>F05-04</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>MCP外部服务集成</t>
+        </is>
+      </c>
+      <c r="D9" s="5" t="inlineStr">
+        <is>
+          <t>外部数据源调用接口，固化规则调用标准协议，与行情/持仓/交易系统数据对接</t>
+        </is>
+      </c>
+      <c r="E9" s="5" t="inlineStr"/>
+      <c r="F9" s="5" t="inlineStr"/>
+      <c r="G9" s="42" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="H9" s="8" t="n">
+        <v>20</v>
+      </c>
+      <c r="I9" s="6" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="J9" s="5" t="inlineStr"/>
+    </row>
+    <row r="10" ht="18" customHeight="1">
+      <c r="A10" s="40" t="inlineStr">
+        <is>
+          <t>D2. 异常识别引擎</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="48" customHeight="1">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>D2. 异常识别引擎</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>F05-05</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="inlineStr">
+        <is>
+          <t>代持与反向交易识别</t>
+        </is>
+      </c>
+      <c r="D11" s="5" t="inlineStr">
+        <is>
+          <t>代持相关交易检测，同券同额反向识别，多日反向低频交易模式识别</t>
+        </is>
+      </c>
+      <c r="E11" s="5" t="inlineStr"/>
+      <c r="F11" s="5" t="inlineStr"/>
+      <c r="G11" s="41" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="H11" s="8" t="n">
+        <v>25</v>
+      </c>
+      <c r="I11" s="6" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="J11" s="5" t="inlineStr"/>
+    </row>
+    <row r="12" ht="48" customHeight="1">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>D2. 异常识别引擎</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>F05-06</t>
+        </is>
+      </c>
+      <c r="C12" s="4" t="inlineStr">
+        <is>
+          <t>价格行为异常检测</t>
+        </is>
+      </c>
+      <c r="D12" s="5" t="inlineStr">
+        <is>
+          <t>高买低卖行为识别，信用债价格异常检测，基于历史分位数与实时行情动态偏离度计算</t>
+        </is>
+      </c>
+      <c r="E12" s="5" t="inlineStr"/>
+      <c r="F12" s="5" t="inlineStr"/>
+      <c r="G12" s="41" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="H12" s="8" t="n">
+        <v>25</v>
+      </c>
+      <c r="I12" s="6" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="J12" s="5" t="inlineStr"/>
+    </row>
+    <row r="13" ht="48" customHeight="1">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>D2. 异常识别引擎</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>F05-07</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="inlineStr">
+        <is>
+          <t>交易对手异常监控</t>
+        </is>
+      </c>
+      <c r="D13" s="5" t="inlineStr">
+        <is>
+          <t>同一交易对手频繁交易预警，多次修改交易对手行为识别，持仓结构异常检测</t>
+        </is>
+      </c>
+      <c r="E13" s="5" t="inlineStr"/>
+      <c r="F13" s="5" t="inlineStr"/>
+      <c r="G13" s="41" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="H13" s="8" t="n">
+        <v>20</v>
+      </c>
+      <c r="I13" s="6" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="J13" s="5" t="inlineStr"/>
+    </row>
+    <row r="14" ht="48" customHeight="1">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>D2. 异常识别引擎</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>F05-08</t>
+        </is>
+      </c>
+      <c r="C14" s="4" t="inlineStr">
+        <is>
+          <t>交易量异常检测</t>
+        </is>
+      </c>
+      <c r="D14" s="5" t="inlineStr">
+        <is>
+          <t>交易量统计异常识别，集中度异常告警，与历史基准对比的量级偏离检测</t>
+        </is>
+      </c>
+      <c r="E14" s="5" t="inlineStr"/>
+      <c r="F14" s="5" t="inlineStr"/>
+      <c r="G14" s="42" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="H14" s="8" t="n">
+        <v>15</v>
+      </c>
+      <c r="I14" s="6" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="J14" s="5" t="inlineStr"/>
+    </row>
+    <row r="15" ht="48" customHeight="1">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>D2. 异常识别引擎</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>F05-09</t>
+        </is>
+      </c>
+      <c r="C15" s="4" t="inlineStr">
+        <is>
+          <t>动态规则管理</t>
+        </is>
+      </c>
+      <c r="D15" s="5" t="inlineStr">
+        <is>
+          <t>异常模式智能探索与规则固化，No-Code规则配置界面，合规人员自助维护，规则版本管理</t>
+        </is>
+      </c>
+      <c r="E15" s="5" t="inlineStr"/>
+      <c r="F15" s="5" t="inlineStr"/>
+      <c r="G15" s="42" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="H15" s="8" t="n">
+        <v>20</v>
+      </c>
+      <c r="I15" s="6" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="J15" s="5" t="inlineStr"/>
+    </row>
+    <row r="16" ht="18" customHeight="1">
+      <c r="A16" s="43" t="inlineStr">
+        <is>
+          <t>D3. 运营与报告</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="48" customHeight="1">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>D3. 运营与报告</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>F05-10</t>
+        </is>
+      </c>
+      <c r="C17" s="4" t="inlineStr">
+        <is>
+          <t>异常交易定位</t>
+        </is>
+      </c>
+      <c r="D17" s="5" t="inlineStr">
+        <is>
+          <t>按时间范围快速查找历史异常交易，标记异常类型，可视化展示异常分布与趋势</t>
+        </is>
+      </c>
+      <c r="E17" s="5" t="inlineStr"/>
+      <c r="F17" s="5" t="inlineStr"/>
+      <c r="G17" s="42" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="H17" s="8" t="n">
+        <v>15</v>
+      </c>
+      <c r="I17" s="6" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="J17" s="5" t="inlineStr"/>
+    </row>
+    <row r="18" ht="48" customHeight="1">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>D3. 运营与报告</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>F05-11</t>
+        </is>
+      </c>
+      <c r="C18" s="4" t="inlineStr">
+        <is>
+          <t>数据上传校验</t>
+        </is>
+      </c>
+      <c r="D18" s="5" t="inlineStr">
+        <is>
+          <t>支持用户上传交易数据文件，瞬时完成异常交易校验并输出校验结果报告</t>
+        </is>
+      </c>
+      <c r="E18" s="5" t="inlineStr"/>
+      <c r="F18" s="5" t="inlineStr"/>
+      <c r="G18" s="42" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="H18" s="8" t="n">
+        <v>15</v>
+      </c>
+      <c r="I18" s="6" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="J18" s="5" t="inlineStr"/>
+    </row>
+    <row r="19" ht="48" customHeight="1">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t>D3. 运营与报告</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>F05-12</t>
+        </is>
+      </c>
+      <c r="C19" s="4" t="inlineStr">
+        <is>
+          <t>智能报告生成</t>
+        </is>
+      </c>
+      <c r="D19" s="5" t="inlineStr">
+        <is>
+          <t>模板自定义与场景数据一键应用，监管报送格式（证监会/人行），新业务过会合规分析报告</t>
+        </is>
+      </c>
+      <c r="E19" s="5" t="inlineStr"/>
+      <c r="F19" s="5" t="inlineStr"/>
+      <c r="G19" s="42" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="H19" s="8" t="n">
+        <v>20</v>
+      </c>
+      <c r="I19" s="6" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="J19" s="5" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="40" t="inlineStr">
+        <is>
+          <t>合计 12项功能  |  P1: 12项  |  P2: 0项</t>
+        </is>
+      </c>
+      <c r="H20" s="20">
+        <f>SUM(H5:H19)</f>
+        <v/>
+      </c>
+      <c r="I20" s="34" t="inlineStr"/>
+      <c r="J20" s="34" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <mergeCells count="7">
+    <mergeCell ref="A1:J1"/>
+    <mergeCell ref="A5:J5"/>
+    <mergeCell ref="A16:J16"/>
+    <mergeCell ref="A3:J3"/>
+    <mergeCell ref="A20:G20"/>
+    <mergeCell ref="A2:J2"/>
+    <mergeCell ref="A10:J10"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" fitToWidth="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:J28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>

</xml_diff>

<commit_message>
Expand module 08 策略投资/量化 from Slide 41
12 functions across 5 domains: 策略研发, 回测与模拟验证, 策略上线管理,
行情分析, 量化底座. Adds 模拟盘验证, 上线审批, AI辅助开发, AlphaLens,
6种策略类型, CEP流引擎, 宏观因子库. Duration 10→12m, 96→120pm.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Feasibility_analysis/FICC_Gap_Analysis.xlsx
+++ b/Feasibility_analysis/FICC_Gap_Analysis.xlsx
@@ -17,6 +17,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="详情_异常交易风控" sheetId="8" state="visible" r:id="rId8"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="详情_事前风控_合规" sheetId="9" state="visible" r:id="rId9"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="详情_组合管理+绩效归因" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="详情_策略投资_量化" sheetId="11" state="visible" r:id="rId11"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Area" localSheetId="0">'差距分析总表'!$A$1:$P$17</definedName>
@@ -1421,21 +1422,21 @@
       </c>
       <c r="L10" s="5" t="inlineStr">
         <is>
-          <t>低延迟ATP执行层</t>
+          <t>低延迟ATP执行层/定价平台</t>
         </is>
       </c>
       <c r="M10" s="3" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="N10" s="3" t="n">
         <v>12</v>
       </c>
       <c r="O10" s="8" t="n">
-        <v>96</v>
+        <v>120</v>
       </c>
       <c r="P10" s="5" t="inlineStr">
         <is>
-          <t>因子框架+回测引擎，低延迟执行</t>
+          <t>因子框架+回测引擎+模拟盘+AI辅助开发，覆盖利差/基差/跨市场套利等固收量化策略全流程；对应PPT Slide 41</t>
         </is>
       </c>
     </row>
@@ -2866,13 +2867,628 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J22"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="48" customWidth="1" min="4" max="4"/>
+    <col width="26" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="6" max="6"/>
+    <col width="8" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="8" max="8"/>
+    <col width="7" customWidth="1" min="9" max="9"/>
+    <col width="18" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="24" customHeight="1">
+      <c r="A1" s="38" t="inlineStr">
+        <is>
+          <t>系统详情：策略投资/量化  |  Quant Strategy</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="36" customHeight="1">
+      <c r="A2" s="39" t="inlineStr">
+        <is>
+          <t>战略定位：因子框架+回测引擎+模拟盘+AI辅助开发，覆盖利差/基差/跨市场套利等固收量化策略全流程；对应PPT Slide 41   |   来源：Slide 41</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="28" customHeight="1">
+      <c r="A3" s="40" t="inlineStr">
+        <is>
+          <t>模块：策略投资/量化  (Quant Strategy)  |  优先级：P1  |  竞品：无主导者  |  华锐基础：低延迟ATP执行层/定价平台  |  工期：12月  团队：12人</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="28" customHeight="1">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>功能域</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>编号</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>功能名称</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>功能描述</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>验收标准</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>集成依赖</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>复杂度</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>预估(人天)</t>
+        </is>
+      </c>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t>优先级</t>
+        </is>
+      </c>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>备注</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="18" customHeight="1">
+      <c r="A5" s="22" t="inlineStr">
+        <is>
+          <t>D1. 策略研发</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="48" customHeight="1">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>D1. 策略研发</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>F08-01</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>策略编写与版本管理</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>Python/C++策略脚本编写，沙箱隔离运行，策略版本管理，策略库分类管理（利差/基差/跨市场套利/网格/固收/量价）</t>
+        </is>
+      </c>
+      <c r="E6" s="5" t="inlineStr"/>
+      <c r="F6" s="5" t="inlineStr"/>
+      <c r="G6" s="41" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="H6" s="8" t="n">
+        <v>40</v>
+      </c>
+      <c r="I6" s="6" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="J6" s="5" t="inlineStr"/>
+    </row>
+    <row r="7" ht="48" customHeight="1">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>D1. 策略研发</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>F08-02</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>AI辅助策略开发</t>
+        </is>
+      </c>
+      <c r="D7" s="5" t="inlineStr">
+        <is>
+          <t>AI代码生成辅助，AI因子生成，AI参数优化建议，自然语言描述策略逻辑转代码</t>
+        </is>
+      </c>
+      <c r="E7" s="5" t="inlineStr"/>
+      <c r="F7" s="5" t="inlineStr"/>
+      <c r="G7" s="41" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="H7" s="8" t="n">
+        <v>35</v>
+      </c>
+      <c r="I7" s="6" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="J7" s="5" t="inlineStr"/>
+    </row>
+    <row r="8" ht="48" customHeight="1">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>D1. 策略研发</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>F08-03</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="inlineStr">
+        <is>
+          <t>因子挖掘与管理</t>
+        </is>
+      </c>
+      <c r="D8" s="5" t="inlineStr">
+        <is>
+          <t>因子编写，信号生成，因子库管理，AlphaLens因子有效性分析，量化模型库，宏观/技术/基本面因子</t>
+        </is>
+      </c>
+      <c r="E8" s="5" t="inlineStr"/>
+      <c r="F8" s="5" t="inlineStr"/>
+      <c r="G8" s="41" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="H8" s="8" t="n">
+        <v>40</v>
+      </c>
+      <c r="I8" s="6" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="J8" s="5" t="inlineStr"/>
+    </row>
+    <row r="9" ht="18" customHeight="1">
+      <c r="A9" s="40" t="inlineStr">
+        <is>
+          <t>D2. 回测与模拟验证</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="48" customHeight="1">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>D2. 回测与模拟验证</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>F08-04</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="inlineStr">
+        <is>
+          <t>Tick级回测引擎</t>
+        </is>
+      </c>
+      <c r="D10" s="5" t="inlineStr">
+        <is>
+          <t>Tick数据驱动回测，真实滑点/冲击模型，批量参数优化，风险计量，绩效归因，AlphaLens分析集成</t>
+        </is>
+      </c>
+      <c r="E10" s="5" t="inlineStr"/>
+      <c r="F10" s="5" t="inlineStr"/>
+      <c r="G10" s="28" t="inlineStr">
+        <is>
+          <t>极高</t>
+        </is>
+      </c>
+      <c r="H10" s="8" t="n">
+        <v>60</v>
+      </c>
+      <c r="I10" s="6" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="J10" s="5" t="inlineStr"/>
+    </row>
+    <row r="11" ht="48" customHeight="1">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>D2. 回测与模拟验证</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>F08-05</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="inlineStr">
+        <is>
+          <t>模拟盘验证</t>
+        </is>
+      </c>
+      <c r="D11" s="5" t="inlineStr">
+        <is>
+          <t>情景模拟，敏感度模拟，极端场景模拟，性能测试，模拟盘与实盘结果对比分析</t>
+        </is>
+      </c>
+      <c r="E11" s="5" t="inlineStr"/>
+      <c r="F11" s="5" t="inlineStr"/>
+      <c r="G11" s="41" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="H11" s="8" t="n">
+        <v>30</v>
+      </c>
+      <c r="I11" s="6" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="J11" s="5" t="inlineStr"/>
+    </row>
+    <row r="12" ht="18" customHeight="1">
+      <c r="A12" s="43" t="inlineStr">
+        <is>
+          <t>D3. 策略上线管理</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="48" customHeight="1">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>D3. 策略上线管理</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>F08-06</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="inlineStr">
+        <is>
+          <t>策略上线审批</t>
+        </is>
+      </c>
+      <c r="D13" s="5" t="inlineStr">
+        <is>
+          <t>模拟盘通过后触发上线审批流程，多级合规审核，审批留痕，参数锁定后方可实盘运行</t>
+        </is>
+      </c>
+      <c r="E13" s="5" t="inlineStr"/>
+      <c r="F13" s="5" t="inlineStr"/>
+      <c r="G13" s="42" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="H13" s="8" t="n">
+        <v>20</v>
+      </c>
+      <c r="I13" s="6" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="J13" s="5" t="inlineStr"/>
+    </row>
+    <row r="14" ht="48" customHeight="1">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>D3. 策略上线管理</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>F08-07</t>
+        </is>
+      </c>
+      <c r="C14" s="4" t="inlineStr">
+        <is>
+          <t>策略运行管理</t>
+        </is>
+      </c>
+      <c r="D14" s="5" t="inlineStr">
+        <is>
+          <t>实盘策略启停管理，策略状态实时监控，支持手动干预和自动触发停止，多策略并发调度</t>
+        </is>
+      </c>
+      <c r="E14" s="5" t="inlineStr"/>
+      <c r="F14" s="5" t="inlineStr"/>
+      <c r="G14" s="41" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="H14" s="8" t="n">
+        <v>30</v>
+      </c>
+      <c r="I14" s="6" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="J14" s="5" t="inlineStr"/>
+    </row>
+    <row r="15" ht="48" customHeight="1">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>D3. 策略上线管理</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>F08-08</t>
+        </is>
+      </c>
+      <c r="C15" s="4" t="inlineStr">
+        <is>
+          <t>策略绩效分析</t>
+        </is>
+      </c>
+      <c r="D15" s="5" t="inlineStr">
+        <is>
+          <t>实时PnL/持仓/回撤/Sharpe看板，策略归因分析，与基准对比，风险触发自动平仓</t>
+        </is>
+      </c>
+      <c r="E15" s="5" t="inlineStr"/>
+      <c r="F15" s="5" t="inlineStr"/>
+      <c r="G15" s="42" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="H15" s="8" t="n">
+        <v>25</v>
+      </c>
+      <c r="I15" s="6" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="J15" s="5" t="inlineStr"/>
+    </row>
+    <row r="16" ht="18" customHeight="1">
+      <c r="A16" s="43" t="inlineStr">
+        <is>
+          <t>D4. 行情分析</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="48" customHeight="1">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>D4. 行情分析</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>F08-09</t>
+        </is>
+      </c>
+      <c r="C17" s="4" t="inlineStr">
+        <is>
+          <t>实时多市场行情</t>
+        </is>
+      </c>
+      <c r="D17" s="5" t="inlineStr">
+        <is>
+          <t>现券/国债期货/股票/商品实时行情聚合展示，实时利差分析，跨市场价差监控，行情小窗</t>
+        </is>
+      </c>
+      <c r="E17" s="5" t="inlineStr"/>
+      <c r="F17" s="5" t="inlineStr"/>
+      <c r="G17" s="42" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="H17" s="8" t="n">
+        <v>20</v>
+      </c>
+      <c r="I17" s="6" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="J17" s="5" t="inlineStr"/>
+    </row>
+    <row r="18" ht="48" customHeight="1">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>D4. 行情分析</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>F08-10</t>
+        </is>
+      </c>
+      <c r="C18" s="4" t="inlineStr">
+        <is>
+          <t>历史行情回放</t>
+        </is>
+      </c>
+      <c r="D18" s="5" t="inlineStr">
+        <is>
+          <t>现券/国债期货/股票/商品历史行情回放，支持任意时间点快照，用于回测验证和策略复盘</t>
+        </is>
+      </c>
+      <c r="E18" s="5" t="inlineStr"/>
+      <c r="F18" s="5" t="inlineStr"/>
+      <c r="G18" s="42" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="H18" s="8" t="n">
+        <v>20</v>
+      </c>
+      <c r="I18" s="6" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="J18" s="5" t="inlineStr"/>
+    </row>
+    <row r="19" ht="18" customHeight="1">
+      <c r="A19" s="29" t="inlineStr">
+        <is>
+          <t>D5. 量化底座</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="48" customHeight="1">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>D5. 量化底座</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>F08-11</t>
+        </is>
+      </c>
+      <c r="C20" s="4" t="inlineStr">
+        <is>
+          <t>CEP流引擎与信号调度</t>
+        </is>
+      </c>
+      <c r="D20" s="5" t="inlineStr">
+        <is>
+          <t>复杂事件处理引擎，策略信号实时计算与调度，低延迟执行接口对接ATP超低延迟执行层</t>
+        </is>
+      </c>
+      <c r="E20" s="5" t="inlineStr"/>
+      <c r="F20" s="5" t="inlineStr"/>
+      <c r="G20" s="28" t="inlineStr">
+        <is>
+          <t>极高</t>
+        </is>
+      </c>
+      <c r="H20" s="8" t="n">
+        <v>45</v>
+      </c>
+      <c r="I20" s="6" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="J20" s="5" t="inlineStr"/>
+    </row>
+    <row r="21" ht="48" customHeight="1">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t>D5. 量化底座</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>F08-12</t>
+        </is>
+      </c>
+      <c r="C21" s="4" t="inlineStr">
+        <is>
+          <t>基础数据与模型底座</t>
+        </is>
+      </c>
+      <c r="D21" s="5" t="inlineStr">
+        <is>
+          <t>宏观因子库，债券曲线模型，估值数据接入，账户权限管理，AI引擎集成接口</t>
+        </is>
+      </c>
+      <c r="E21" s="5" t="inlineStr"/>
+      <c r="F21" s="5" t="inlineStr"/>
+      <c r="G21" s="41" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="H21" s="8" t="n">
+        <v>30</v>
+      </c>
+      <c r="I21" s="6" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="J21" s="5" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="40" t="inlineStr">
+        <is>
+          <t>合计 12项功能  |  P1: 12项  |  P2: 0项</t>
+        </is>
+      </c>
+      <c r="H22" s="20">
+        <f>SUM(H5:H21)</f>
+        <v/>
+      </c>
+      <c r="I22" s="34" t="inlineStr"/>
+      <c r="J22" s="34" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <mergeCells count="9">
+    <mergeCell ref="A1:J1"/>
+    <mergeCell ref="A5:J5"/>
+    <mergeCell ref="A16:J16"/>
+    <mergeCell ref="A9:J9"/>
+    <mergeCell ref="A22:G22"/>
+    <mergeCell ref="A3:J3"/>
+    <mergeCell ref="A12:J12"/>
+    <mergeCell ref="A2:J2"/>
+    <mergeCell ref="A19:J19"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" fitToWidth="1"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H175"/>
+  <dimension ref="A1:H182"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -7768,12 +8384,12 @@
       </c>
       <c r="D130" s="4" t="inlineStr">
         <is>
-          <t>因子模型框架</t>
+          <t>策略编写与版本管理</t>
         </is>
       </c>
       <c r="E130" s="5" t="inlineStr">
         <is>
-          <t>多因子Alpha模型+风险因子，支持自定义因子上传与测试</t>
+          <t>Python/C++策略脚本编写，沙箱隔离运行，策略版本管理，策略库分类管理（利差/基差/跨市场套利/网格/固收/量价）</t>
         </is>
       </c>
       <c r="F130" s="5" t="inlineStr">
@@ -7808,26 +8424,26 @@
       </c>
       <c r="D131" s="4" t="inlineStr">
         <is>
-          <t>Tick级回测引擎</t>
+          <t>AI辅助策略开发</t>
         </is>
       </c>
       <c r="E131" s="5" t="inlineStr">
         <is>
-          <t>Tick数据驱动回测，真实滑点/冲击模型，批量参数优化</t>
+          <t>AI代码生成辅助，AI因子生成，AI参数优化建议，自然语言描述策略逻辑转代码</t>
         </is>
       </c>
       <c r="F131" s="5" t="inlineStr">
         <is>
-          <t>p99延迟/误差率/精度验证/压测10k TPS</t>
-        </is>
-      </c>
-      <c r="G131" s="28" t="inlineStr">
-        <is>
-          <t>极高</t>
+          <t>功能完整/边界测试/集成冒烟/性能基线</t>
+        </is>
+      </c>
+      <c r="G131" s="23" t="inlineStr">
+        <is>
+          <t>高</t>
         </is>
       </c>
       <c r="H131" s="8" t="n">
-        <v>60</v>
+        <v>35</v>
       </c>
     </row>
     <row r="132" ht="28" customHeight="1">
@@ -7848,12 +8464,12 @@
       </c>
       <c r="D132" s="4" t="inlineStr">
         <is>
-          <t>信号生成与调度</t>
+          <t>因子挖掘与管理</t>
         </is>
       </c>
       <c r="E132" s="5" t="inlineStr">
         <is>
-          <t>策略信号实时计算，支持Python/C++策略脚本沙箱运行</t>
+          <t>因子编写，信号生成，因子库管理，AlphaLens因子有效性分析，量化模型库，宏观/技术/基本面因子</t>
         </is>
       </c>
       <c r="F132" s="5" t="inlineStr">
@@ -7888,12 +8504,12 @@
       </c>
       <c r="D133" s="4" t="inlineStr">
         <is>
-          <t>低延迟执行接口</t>
+          <t>Tick级回测引擎</t>
         </is>
       </c>
       <c r="E133" s="5" t="inlineStr">
         <is>
-          <t>与ATP超低延迟执行层对接，算法拆单（TWAP/VWAP/IS）</t>
+          <t>Tick数据驱动回测，真实滑点/冲击模型，批量参数优化，风险计量，绩效归因，AlphaLens分析集成</t>
         </is>
       </c>
       <c r="F133" s="5" t="inlineStr">
@@ -7907,7 +8523,7 @@
         </is>
       </c>
       <c r="H133" s="8" t="n">
-        <v>45</v>
+        <v>60</v>
       </c>
     </row>
     <row r="134" ht="28" customHeight="1">
@@ -7928,286 +8544,319 @@
       </c>
       <c r="D134" s="4" t="inlineStr">
         <is>
-          <t>实时策略监控</t>
+          <t>模拟盘验证</t>
         </is>
       </c>
       <c r="E134" s="5" t="inlineStr">
         <is>
-          <t>持仓/PnL/回撤/Sharpe实时看板，风险触发自动平仓</t>
+          <t>情景模拟，敏感度模拟，极端场景模拟，性能测试，模拟盘与实盘结果对比分析</t>
         </is>
       </c>
       <c r="F134" s="5" t="inlineStr">
         <is>
+          <t>功能完整/边界测试/集成冒烟/性能基线</t>
+        </is>
+      </c>
+      <c r="G134" s="23" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="H134" s="8" t="n">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="135" ht="28" customHeight="1">
+      <c r="A135" s="5" t="inlineStr">
+        <is>
+          <t>策略投资/量化</t>
+        </is>
+      </c>
+      <c r="B135" s="3" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="C135" s="3" t="inlineStr">
+        <is>
+          <t>F08-06</t>
+        </is>
+      </c>
+      <c r="D135" s="4" t="inlineStr">
+        <is>
+          <t>策略上线审批</t>
+        </is>
+      </c>
+      <c r="E135" s="5" t="inlineStr">
+        <is>
+          <t>模拟盘通过后触发上线审批流程，多级合规审核，审批留痕，参数锁定后方可实盘运行</t>
+        </is>
+      </c>
+      <c r="F135" s="5" t="inlineStr">
+        <is>
           <t>功能测试通过/正确率100%</t>
         </is>
       </c>
-      <c r="G134" s="24" t="inlineStr">
+      <c r="G135" s="24" t="inlineStr">
         <is>
           <t>中</t>
         </is>
       </c>
-      <c r="H134" s="8" t="n">
+      <c r="H135" s="8" t="n">
         <v>20</v>
       </c>
     </row>
-    <row r="135" ht="20" customHeight="1">
-      <c r="A135" s="26" t="inlineStr">
-        <is>
-          <t>【P2】 定价平台  (Pricing Platform)</t>
-        </is>
-      </c>
-    </row>
     <row r="136" ht="28" customHeight="1">
-      <c r="A136" s="11" t="inlineStr">
-        <is>
-          <t>定价平台</t>
-        </is>
-      </c>
-      <c r="B136" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
-        </is>
-      </c>
-      <c r="C136" s="10" t="inlineStr">
-        <is>
-          <t>F09-01</t>
-        </is>
-      </c>
-      <c r="D136" s="27" t="inlineStr">
-        <is>
-          <t>期限结构模型</t>
-        </is>
-      </c>
-      <c r="E136" s="11" t="inlineStr">
-        <is>
-          <t>Nelson-Siegel/Svensson/HJM等多模型参数拟合，实时曲线</t>
-        </is>
-      </c>
-      <c r="F136" s="11" t="inlineStr">
+      <c r="A136" s="5" t="inlineStr">
+        <is>
+          <t>策略投资/量化</t>
+        </is>
+      </c>
+      <c r="B136" s="3" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="C136" s="3" t="inlineStr">
+        <is>
+          <t>F08-07</t>
+        </is>
+      </c>
+      <c r="D136" s="4" t="inlineStr">
+        <is>
+          <t>策略运行管理</t>
+        </is>
+      </c>
+      <c r="E136" s="5" t="inlineStr">
+        <is>
+          <t>实盘策略启停管理，策略状态实时监控，支持手动干预和自动触发停止，多策略并发调度</t>
+        </is>
+      </c>
+      <c r="F136" s="5" t="inlineStr">
+        <is>
+          <t>功能完整/边界测试/集成冒烟/性能基线</t>
+        </is>
+      </c>
+      <c r="G136" s="23" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="H136" s="8" t="n">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="137" ht="28" customHeight="1">
+      <c r="A137" s="5" t="inlineStr">
+        <is>
+          <t>策略投资/量化</t>
+        </is>
+      </c>
+      <c r="B137" s="3" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="C137" s="3" t="inlineStr">
+        <is>
+          <t>F08-08</t>
+        </is>
+      </c>
+      <c r="D137" s="4" t="inlineStr">
+        <is>
+          <t>策略绩效分析</t>
+        </is>
+      </c>
+      <c r="E137" s="5" t="inlineStr">
+        <is>
+          <t>实时PnL/持仓/回撤/Sharpe看板，策略归因分析，与基准对比，风险触发自动平仓</t>
+        </is>
+      </c>
+      <c r="F137" s="5" t="inlineStr">
+        <is>
+          <t>功能测试通过/正确率100%</t>
+        </is>
+      </c>
+      <c r="G137" s="24" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="H137" s="8" t="n">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="138" ht="28" customHeight="1">
+      <c r="A138" s="5" t="inlineStr">
+        <is>
+          <t>策略投资/量化</t>
+        </is>
+      </c>
+      <c r="B138" s="3" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="C138" s="3" t="inlineStr">
+        <is>
+          <t>F08-09</t>
+        </is>
+      </c>
+      <c r="D138" s="4" t="inlineStr">
+        <is>
+          <t>实时多市场行情</t>
+        </is>
+      </c>
+      <c r="E138" s="5" t="inlineStr">
+        <is>
+          <t>现券/国债期货/股票/商品实时行情聚合展示，实时利差分析，跨市场价差监控，行情小窗</t>
+        </is>
+      </c>
+      <c r="F138" s="5" t="inlineStr">
+        <is>
+          <t>功能测试通过/正确率100%</t>
+        </is>
+      </c>
+      <c r="G138" s="24" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="H138" s="8" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="139" ht="28" customHeight="1">
+      <c r="A139" s="5" t="inlineStr">
+        <is>
+          <t>策略投资/量化</t>
+        </is>
+      </c>
+      <c r="B139" s="3" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="C139" s="3" t="inlineStr">
+        <is>
+          <t>F08-10</t>
+        </is>
+      </c>
+      <c r="D139" s="4" t="inlineStr">
+        <is>
+          <t>历史行情回放</t>
+        </is>
+      </c>
+      <c r="E139" s="5" t="inlineStr">
+        <is>
+          <t>现券/国债期货/股票/商品历史行情回放，支持任意时间点快照，用于回测验证和策略复盘</t>
+        </is>
+      </c>
+      <c r="F139" s="5" t="inlineStr">
+        <is>
+          <t>功能测试通过/正确率100%</t>
+        </is>
+      </c>
+      <c r="G139" s="24" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="H139" s="8" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="140" ht="28" customHeight="1">
+      <c r="A140" s="5" t="inlineStr">
+        <is>
+          <t>策略投资/量化</t>
+        </is>
+      </c>
+      <c r="B140" s="3" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="C140" s="3" t="inlineStr">
+        <is>
+          <t>F08-11</t>
+        </is>
+      </c>
+      <c r="D140" s="4" t="inlineStr">
+        <is>
+          <t>CEP流引擎与信号调度</t>
+        </is>
+      </c>
+      <c r="E140" s="5" t="inlineStr">
+        <is>
+          <t>复杂事件处理引擎，策略信号实时计算与调度，低延迟执行接口对接ATP超低延迟执行层</t>
+        </is>
+      </c>
+      <c r="F140" s="5" t="inlineStr">
         <is>
           <t>p99延迟/误差率/精度验证/压测10k TPS</t>
         </is>
       </c>
-      <c r="G136" s="28" t="inlineStr">
+      <c r="G140" s="28" t="inlineStr">
         <is>
           <t>极高</t>
         </is>
       </c>
-      <c r="H136" s="13" t="n">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="137" ht="28" customHeight="1">
-      <c r="A137" s="11" t="inlineStr">
-        <is>
-          <t>定价平台</t>
-        </is>
-      </c>
-      <c r="B137" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
-        </is>
-      </c>
-      <c r="C137" s="10" t="inlineStr">
-        <is>
-          <t>F09-02</t>
-        </is>
-      </c>
-      <c r="D137" s="27" t="inlineStr">
-        <is>
-          <t>蒙特卡洛求解器</t>
-        </is>
-      </c>
-      <c r="E137" s="11" t="inlineStr">
-        <is>
-          <t>GPU加速MC，QMC低差异序列，支持路径相关期权定价</t>
-        </is>
-      </c>
-      <c r="F137" s="11" t="inlineStr">
-        <is>
-          <t>p99延迟/误差率/精度验证/压测10k TPS</t>
-        </is>
-      </c>
-      <c r="G137" s="28" t="inlineStr">
-        <is>
-          <t>极高</t>
-        </is>
-      </c>
-      <c r="H137" s="13" t="n">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="138" ht="28" customHeight="1">
-      <c r="A138" s="11" t="inlineStr">
-        <is>
-          <t>定价平台</t>
-        </is>
-      </c>
-      <c r="B138" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
-        </is>
-      </c>
-      <c r="C138" s="10" t="inlineStr">
-        <is>
-          <t>F09-03</t>
-        </is>
-      </c>
-      <c r="D138" s="27" t="inlineStr">
-        <is>
-          <t>有限差分（PDE）</t>
-        </is>
-      </c>
-      <c r="E138" s="11" t="inlineStr">
-        <is>
-          <t>Crank-Nicolson/ADI方法，含权债/可转债精确定价</t>
-        </is>
-      </c>
-      <c r="F138" s="11" t="inlineStr">
-        <is>
-          <t>p99延迟/误差率/精度验证/压测10k TPS</t>
-        </is>
-      </c>
-      <c r="G138" s="28" t="inlineStr">
-        <is>
-          <t>极高</t>
-        </is>
-      </c>
-      <c r="H138" s="13" t="n">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="139" ht="28" customHeight="1">
-      <c r="A139" s="11" t="inlineStr">
-        <is>
-          <t>定价平台</t>
-        </is>
-      </c>
-      <c r="B139" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
-        </is>
-      </c>
-      <c r="C139" s="10" t="inlineStr">
-        <is>
-          <t>F09-04</t>
-        </is>
-      </c>
-      <c r="D139" s="27" t="inlineStr">
-        <is>
-          <t>实时Greeks</t>
-        </is>
-      </c>
-      <c r="E139" s="11" t="inlineStr">
-        <is>
-          <t>Delta/Gamma/Vega/Theta/Rho分布式实时计算</t>
-        </is>
-      </c>
-      <c r="F139" s="11" t="inlineStr">
+      <c r="H140" s="8" t="n">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="141" ht="28" customHeight="1">
+      <c r="A141" s="5" t="inlineStr">
+        <is>
+          <t>策略投资/量化</t>
+        </is>
+      </c>
+      <c r="B141" s="3" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="C141" s="3" t="inlineStr">
+        <is>
+          <t>F08-12</t>
+        </is>
+      </c>
+      <c r="D141" s="4" t="inlineStr">
+        <is>
+          <t>基础数据与模型底座</t>
+        </is>
+      </c>
+      <c r="E141" s="5" t="inlineStr">
+        <is>
+          <t>宏观因子库，债券曲线模型，估值数据接入，账户权限管理，AI引擎集成接口</t>
+        </is>
+      </c>
+      <c r="F141" s="5" t="inlineStr">
         <is>
           <t>功能完整/边界测试/集成冒烟/性能基线</t>
         </is>
       </c>
-      <c r="G139" s="23" t="inlineStr">
+      <c r="G141" s="23" t="inlineStr">
         <is>
           <t>高</t>
         </is>
       </c>
-      <c r="H139" s="13" t="n">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="140" ht="28" customHeight="1">
-      <c r="A140" s="11" t="inlineStr">
-        <is>
-          <t>定价平台</t>
-        </is>
-      </c>
-      <c r="B140" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
-        </is>
-      </c>
-      <c r="C140" s="10" t="inlineStr">
-        <is>
-          <t>F09-05</t>
-        </is>
-      </c>
-      <c r="D140" s="27" t="inlineStr">
-        <is>
-          <t>定价服务微服务架构</t>
-        </is>
-      </c>
-      <c r="E140" s="11" t="inlineStr">
-        <is>
-          <t>REST/gRPC定价API，支持横向扩展，p99&lt;100ms</t>
-        </is>
-      </c>
-      <c r="F140" s="11" t="inlineStr">
-        <is>
-          <t>功能完整/边界测试/集成冒烟/性能基线</t>
-        </is>
-      </c>
-      <c r="G140" s="23" t="inlineStr">
-        <is>
-          <t>高</t>
-        </is>
-      </c>
-      <c r="H140" s="13" t="n">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="141" ht="28" customHeight="1">
-      <c r="A141" s="11" t="inlineStr">
-        <is>
-          <t>定价平台</t>
-        </is>
-      </c>
-      <c r="B141" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
-        </is>
-      </c>
-      <c r="C141" s="10" t="inlineStr">
-        <is>
-          <t>F09-06</t>
-        </is>
-      </c>
-      <c r="D141" s="27" t="inlineStr">
-        <is>
-          <t>历史估值回测</t>
-        </is>
-      </c>
-      <c r="E141" s="11" t="inlineStr">
-        <is>
-          <t>基于历史行情重放定价误差分析，模型验证框架</t>
-        </is>
-      </c>
-      <c r="F141" s="11" t="inlineStr">
-        <is>
-          <t>功能完整/边界测试/集成冒烟/性能基线</t>
-        </is>
-      </c>
-      <c r="G141" s="23" t="inlineStr">
-        <is>
-          <t>高</t>
-        </is>
-      </c>
-      <c r="H141" s="13" t="n">
+      <c r="H141" s="8" t="n">
         <v>30</v>
       </c>
     </row>
     <row r="142" ht="20" customHeight="1">
       <c r="A142" s="26" t="inlineStr">
         <is>
-          <t>【P2】 销售交易  (Sales Trading)</t>
+          <t>【P2】 定价平台  (Pricing Platform)</t>
         </is>
       </c>
     </row>
     <row r="143" ht="28" customHeight="1">
       <c r="A143" s="11" t="inlineStr">
         <is>
-          <t>销售交易</t>
+          <t>定价平台</t>
         </is>
       </c>
       <c r="B143" s="10" t="inlineStr">
@@ -8217,37 +8866,37 @@
       </c>
       <c r="C143" s="10" t="inlineStr">
         <is>
-          <t>F10-01</t>
+          <t>F09-01</t>
         </is>
       </c>
       <c r="D143" s="27" t="inlineStr">
         <is>
-          <t>销交工作台</t>
+          <t>期限结构模型</t>
         </is>
       </c>
       <c r="E143" s="11" t="inlineStr">
         <is>
-          <t>报价管理主界面，历史报价管理，当日报价快捷操作，导入/导出报价，一键unrefer操作</t>
+          <t>Nelson-Siegel/Svensson/HJM等多模型参数拟合，实时曲线</t>
         </is>
       </c>
       <c r="F143" s="11" t="inlineStr">
         <is>
-          <t>功能测试通过/正确率100%</t>
-        </is>
-      </c>
-      <c r="G143" s="24" t="inlineStr">
-        <is>
-          <t>中</t>
+          <t>p99延迟/误差率/精度验证/压测10k TPS</t>
+        </is>
+      </c>
+      <c r="G143" s="28" t="inlineStr">
+        <is>
+          <t>极高</t>
         </is>
       </c>
       <c r="H143" s="13" t="n">
-        <v>20</v>
+        <v>60</v>
       </c>
     </row>
     <row r="144" ht="28" customHeight="1">
       <c r="A144" s="11" t="inlineStr">
         <is>
-          <t>销售交易</t>
+          <t>定价平台</t>
         </is>
       </c>
       <c r="B144" s="10" t="inlineStr">
@@ -8257,37 +8906,37 @@
       </c>
       <c r="C144" s="10" t="inlineStr">
         <is>
-          <t>F10-02</t>
+          <t>F09-02</t>
         </is>
       </c>
       <c r="D144" s="27" t="inlineStr">
         <is>
-          <t>债券过滤与筛选</t>
+          <t>蒙特卡洛求解器</t>
         </is>
       </c>
       <c r="E144" s="11" t="inlineStr">
         <is>
-          <t>信用债/利率债过滤，信用债全品种过滤，利率债国债/证金债/地方债分类过滤，精确与模糊识别</t>
+          <t>GPU加速MC，QMC低差异序列，支持路径相关期权定价</t>
         </is>
       </c>
       <c r="F144" s="11" t="inlineStr">
         <is>
-          <t>功能测试通过</t>
-        </is>
-      </c>
-      <c r="G144" s="25" t="inlineStr">
-        <is>
-          <t>低</t>
+          <t>p99延迟/误差率/精度验证/压测10k TPS</t>
+        </is>
+      </c>
+      <c r="G144" s="28" t="inlineStr">
+        <is>
+          <t>极高</t>
         </is>
       </c>
       <c r="H144" s="13" t="n">
-        <v>10</v>
+        <v>70</v>
       </c>
     </row>
     <row r="145" ht="28" customHeight="1">
       <c r="A145" s="11" t="inlineStr">
         <is>
-          <t>销售交易</t>
+          <t>定价平台</t>
         </is>
       </c>
       <c r="B145" s="10" t="inlineStr">
@@ -8297,37 +8946,37 @@
       </c>
       <c r="C145" s="10" t="inlineStr">
         <is>
-          <t>F10-03</t>
+          <t>F09-03</t>
         </is>
       </c>
       <c r="D145" s="27" t="inlineStr">
         <is>
-          <t>报价撮合与对价</t>
+          <t>有限差分（PDE）</t>
         </is>
       </c>
       <c r="E145" s="11" t="inlineStr">
         <is>
-          <t>报价展示（对价/最优报价），撮合对价，报价提醒，交易包管理，报价成交确认</t>
+          <t>Crank-Nicolson/ADI方法，含权债/可转债精确定价</t>
         </is>
       </c>
       <c r="F145" s="11" t="inlineStr">
         <is>
-          <t>功能测试通过/正确率100%</t>
-        </is>
-      </c>
-      <c r="G145" s="24" t="inlineStr">
-        <is>
-          <t>中</t>
+          <t>p99延迟/误差率/精度验证/压测10k TPS</t>
+        </is>
+      </c>
+      <c r="G145" s="28" t="inlineStr">
+        <is>
+          <t>极高</t>
         </is>
       </c>
       <c r="H145" s="13" t="n">
-        <v>20</v>
+        <v>60</v>
       </c>
     </row>
     <row r="146" ht="28" customHeight="1">
       <c r="A146" s="11" t="inlineStr">
         <is>
-          <t>销售交易</t>
+          <t>定价平台</t>
         </is>
       </c>
       <c r="B146" s="10" t="inlineStr">
@@ -8337,37 +8986,37 @@
       </c>
       <c r="C146" s="10" t="inlineStr">
         <is>
-          <t>F10-04</t>
+          <t>F09-04</t>
         </is>
       </c>
       <c r="D146" s="27" t="inlineStr">
         <is>
-          <t>交易执行与审批</t>
+          <t>实时Greeks</t>
         </is>
       </c>
       <c r="E146" s="11" t="inlineStr">
         <is>
-          <t>意向达成，交易要素校验，手工价录入，业务审批流程，交易执行</t>
+          <t>Delta/Gamma/Vega/Theta/Rho分布式实时计算</t>
         </is>
       </c>
       <c r="F146" s="11" t="inlineStr">
         <is>
-          <t>功能测试通过/正确率100%</t>
-        </is>
-      </c>
-      <c r="G146" s="24" t="inlineStr">
-        <is>
-          <t>中</t>
+          <t>功能完整/边界测试/集成冒烟/性能基线</t>
+        </is>
+      </c>
+      <c r="G146" s="23" t="inlineStr">
+        <is>
+          <t>高</t>
         </is>
       </c>
       <c r="H146" s="13" t="n">
-        <v>15</v>
+        <v>40</v>
       </c>
     </row>
     <row r="147" ht="28" customHeight="1">
       <c r="A147" s="11" t="inlineStr">
         <is>
-          <t>销售交易</t>
+          <t>定价平台</t>
         </is>
       </c>
       <c r="B147" s="10" t="inlineStr">
@@ -8377,37 +9026,37 @@
       </c>
       <c r="C147" s="10" t="inlineStr">
         <is>
-          <t>F10-05</t>
+          <t>F09-05</t>
         </is>
       </c>
       <c r="D147" s="27" t="inlineStr">
         <is>
-          <t>风控检查</t>
+          <t>定价服务微服务架构</t>
         </is>
       </c>
       <c r="E147" s="11" t="inlineStr">
         <is>
-          <t>交易前风控规则校验，限额检查，合规拦截，风控记录留痕</t>
+          <t>REST/gRPC定价API，支持横向扩展，p99&lt;100ms</t>
         </is>
       </c>
       <c r="F147" s="11" t="inlineStr">
         <is>
-          <t>功能测试通过/正确率100%</t>
-        </is>
-      </c>
-      <c r="G147" s="24" t="inlineStr">
-        <is>
-          <t>中</t>
+          <t>功能完整/边界测试/集成冒烟/性能基线</t>
+        </is>
+      </c>
+      <c r="G147" s="23" t="inlineStr">
+        <is>
+          <t>高</t>
         </is>
       </c>
       <c r="H147" s="13" t="n">
-        <v>15</v>
+        <v>40</v>
       </c>
     </row>
     <row r="148" ht="28" customHeight="1">
       <c r="A148" s="11" t="inlineStr">
         <is>
-          <t>销售交易</t>
+          <t>定价平台</t>
         </is>
       </c>
       <c r="B148" s="10" t="inlineStr">
@@ -8417,17 +9066,17 @@
       </c>
       <c r="C148" s="10" t="inlineStr">
         <is>
-          <t>F10-06</t>
+          <t>F09-06</t>
         </is>
       </c>
       <c r="D148" s="27" t="inlineStr">
         <is>
-          <t>智能推荐系统</t>
+          <t>历史估值回测</t>
         </is>
       </c>
       <c r="E148" s="11" t="inlineStr">
         <is>
-          <t>从被动客户服务转向主动服务，基于客户画像与持仓分析智能推荐券种，提升客户响应效率</t>
+          <t>基于历史行情重放定价误差分析，模型验证框架</t>
         </is>
       </c>
       <c r="F148" s="11" t="inlineStr">
@@ -8441,20 +9090,20 @@
         </is>
       </c>
       <c r="H148" s="13" t="n">
-        <v>25</v>
+        <v>30</v>
       </c>
     </row>
     <row r="149" ht="20" customHeight="1">
       <c r="A149" s="26" t="inlineStr">
         <is>
-          <t>【P2】 信用债/信用衍生品  (Credit &amp; CDS)</t>
+          <t>【P2】 销售交易  (Sales Trading)</t>
         </is>
       </c>
     </row>
     <row r="150" ht="28" customHeight="1">
       <c r="A150" s="11" t="inlineStr">
         <is>
-          <t>信用债/信用衍生品</t>
+          <t>销售交易</t>
         </is>
       </c>
       <c r="B150" s="10" t="inlineStr">
@@ -8464,37 +9113,37 @@
       </c>
       <c r="C150" s="10" t="inlineStr">
         <is>
-          <t>F11-01</t>
+          <t>F10-01</t>
         </is>
       </c>
       <c r="D150" s="27" t="inlineStr">
         <is>
-          <t>信用利差分析</t>
+          <t>销交工作台</t>
         </is>
       </c>
       <c r="E150" s="11" t="inlineStr">
         <is>
-          <t>行业/评级/期限信用利差曲线实时计算，历史分位数分析</t>
+          <t>报价管理主界面，历史报价管理，当日报价快捷操作，导入/导出报价，一键unrefer操作</t>
         </is>
       </c>
       <c r="F150" s="11" t="inlineStr">
         <is>
-          <t>功能完整/边界测试/集成冒烟/性能基线</t>
-        </is>
-      </c>
-      <c r="G150" s="23" t="inlineStr">
-        <is>
-          <t>高</t>
+          <t>功能测试通过/正确率100%</t>
+        </is>
+      </c>
+      <c r="G150" s="24" t="inlineStr">
+        <is>
+          <t>中</t>
         </is>
       </c>
       <c r="H150" s="13" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
     </row>
     <row r="151" ht="28" customHeight="1">
       <c r="A151" s="11" t="inlineStr">
         <is>
-          <t>信用债/信用衍生品</t>
+          <t>销售交易</t>
         </is>
       </c>
       <c r="B151" s="10" t="inlineStr">
@@ -8504,37 +9153,37 @@
       </c>
       <c r="C151" s="10" t="inlineStr">
         <is>
-          <t>F11-02</t>
+          <t>F10-02</t>
         </is>
       </c>
       <c r="D151" s="27" t="inlineStr">
         <is>
-          <t>CDS/CLN定价</t>
+          <t>债券过滤与筛选</t>
         </is>
       </c>
       <c r="E151" s="11" t="inlineStr">
         <is>
-          <t>信用违约互换定价，ISDA标准，生存概率曲线校准</t>
+          <t>信用债/利率债过滤，信用债全品种过滤，利率债国债/证金债/地方债分类过滤，精确与模糊识别</t>
         </is>
       </c>
       <c r="F151" s="11" t="inlineStr">
         <is>
-          <t>p99延迟/误差率/精度验证/压测10k TPS</t>
-        </is>
-      </c>
-      <c r="G151" s="28" t="inlineStr">
-        <is>
-          <t>极高</t>
+          <t>功能测试通过</t>
+        </is>
+      </c>
+      <c r="G151" s="25" t="inlineStr">
+        <is>
+          <t>低</t>
         </is>
       </c>
       <c r="H151" s="13" t="n">
-        <v>50</v>
+        <v>10</v>
       </c>
     </row>
     <row r="152" ht="28" customHeight="1">
       <c r="A152" s="11" t="inlineStr">
         <is>
-          <t>信用债/信用衍生品</t>
+          <t>销售交易</t>
         </is>
       </c>
       <c r="B152" s="10" t="inlineStr">
@@ -8544,17 +9193,17 @@
       </c>
       <c r="C152" s="10" t="inlineStr">
         <is>
-          <t>F11-03</t>
+          <t>F10-03</t>
         </is>
       </c>
       <c r="D152" s="27" t="inlineStr">
         <is>
-          <t>信用评级动态监控</t>
+          <t>报价撮合与对价</t>
         </is>
       </c>
       <c r="E152" s="11" t="inlineStr">
         <is>
-          <t>对接外部评级机构（中诚信/联合/大公），评级下调预警</t>
+          <t>报价展示（对价/最优报价），撮合对价，报价提醒，交易包管理，报价成交确认</t>
         </is>
       </c>
       <c r="F152" s="11" t="inlineStr">
@@ -8574,7 +9223,7 @@
     <row r="153" ht="28" customHeight="1">
       <c r="A153" s="11" t="inlineStr">
         <is>
-          <t>信用债/信用衍生品</t>
+          <t>销售交易</t>
         </is>
       </c>
       <c r="B153" s="10" t="inlineStr">
@@ -8584,37 +9233,37 @@
       </c>
       <c r="C153" s="10" t="inlineStr">
         <is>
-          <t>F11-04</t>
+          <t>F10-04</t>
         </is>
       </c>
       <c r="D153" s="27" t="inlineStr">
         <is>
-          <t>违约概率（PD）建模</t>
+          <t>交易执行与审批</t>
         </is>
       </c>
       <c r="E153" s="11" t="inlineStr">
         <is>
-          <t>结构化Merton模型+市场隐含PD，信用风险计量</t>
+          <t>意向达成，交易要素校验，手工价录入，业务审批流程，交易执行</t>
         </is>
       </c>
       <c r="F153" s="11" t="inlineStr">
         <is>
-          <t>功能完整/边界测试/集成冒烟/性能基线</t>
-        </is>
-      </c>
-      <c r="G153" s="23" t="inlineStr">
-        <is>
-          <t>高</t>
+          <t>功能测试通过/正确率100%</t>
+        </is>
+      </c>
+      <c r="G153" s="24" t="inlineStr">
+        <is>
+          <t>中</t>
         </is>
       </c>
       <c r="H153" s="13" t="n">
-        <v>40</v>
+        <v>15</v>
       </c>
     </row>
     <row r="154" ht="28" customHeight="1">
       <c r="A154" s="11" t="inlineStr">
         <is>
-          <t>信用债/信用衍生品</t>
+          <t>销售交易</t>
         </is>
       </c>
       <c r="B154" s="10" t="inlineStr">
@@ -8624,17 +9273,17 @@
       </c>
       <c r="C154" s="10" t="inlineStr">
         <is>
-          <t>F11-05</t>
+          <t>F10-05</t>
         </is>
       </c>
       <c r="D154" s="27" t="inlineStr">
         <is>
-          <t>集中度限额管理</t>
+          <t>风控检查</t>
         </is>
       </c>
       <c r="E154" s="11" t="inlineStr">
         <is>
-          <t>行业/发行人/评级集中度多维限额，超限预警</t>
+          <t>交易前风控规则校验，限额检查，合规拦截，风控记录留痕</t>
         </is>
       </c>
       <c r="F154" s="11" t="inlineStr">
@@ -8648,60 +9297,60 @@
         </is>
       </c>
       <c r="H154" s="13" t="n">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="155" ht="20" customHeight="1">
-      <c r="A155" s="26" t="inlineStr">
-        <is>
-          <t>【P2】 投顾服务  (Investment Advisory)</t>
-        </is>
-      </c>
-    </row>
-    <row r="156" ht="28" customHeight="1">
-      <c r="A156" s="11" t="inlineStr">
-        <is>
-          <t>投顾服务</t>
-        </is>
-      </c>
-      <c r="B156" s="10" t="inlineStr">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="155" ht="28" customHeight="1">
+      <c r="A155" s="11" t="inlineStr">
+        <is>
+          <t>销售交易</t>
+        </is>
+      </c>
+      <c r="B155" s="10" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
       </c>
-      <c r="C156" s="10" t="inlineStr">
-        <is>
-          <t>F12-01</t>
-        </is>
-      </c>
-      <c r="D156" s="27" t="inlineStr">
-        <is>
-          <t>投顾工作台</t>
-        </is>
-      </c>
-      <c r="E156" s="11" t="inlineStr">
-        <is>
-          <t>投顾人员操作界面，管理客户委托，上传研究报告，发送投资建议，查看客户反馈</t>
-        </is>
-      </c>
-      <c r="F156" s="11" t="inlineStr">
-        <is>
-          <t>功能测试通过/正确率100%</t>
-        </is>
-      </c>
-      <c r="G156" s="24" t="inlineStr">
-        <is>
-          <t>中</t>
-        </is>
-      </c>
-      <c r="H156" s="13" t="n">
-        <v>20</v>
+      <c r="C155" s="10" t="inlineStr">
+        <is>
+          <t>F10-06</t>
+        </is>
+      </c>
+      <c r="D155" s="27" t="inlineStr">
+        <is>
+          <t>智能推荐系统</t>
+        </is>
+      </c>
+      <c r="E155" s="11" t="inlineStr">
+        <is>
+          <t>从被动客户服务转向主动服务，基于客户画像与持仓分析智能推荐券种，提升客户响应效率</t>
+        </is>
+      </c>
+      <c r="F155" s="11" t="inlineStr">
+        <is>
+          <t>功能完整/边界测试/集成冒烟/性能基线</t>
+        </is>
+      </c>
+      <c r="G155" s="23" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="H155" s="13" t="n">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="156" ht="20" customHeight="1">
+      <c r="A156" s="26" t="inlineStr">
+        <is>
+          <t>【P2】 信用债/信用衍生品  (Credit &amp; CDS)</t>
+        </is>
       </c>
     </row>
     <row r="157" ht="28" customHeight="1">
       <c r="A157" s="11" t="inlineStr">
         <is>
-          <t>投顾服务</t>
+          <t>信用债/信用衍生品</t>
         </is>
       </c>
       <c r="B157" s="10" t="inlineStr">
@@ -8711,37 +9360,37 @@
       </c>
       <c r="C157" s="10" t="inlineStr">
         <is>
-          <t>F12-02</t>
+          <t>F11-01</t>
         </is>
       </c>
       <c r="D157" s="27" t="inlineStr">
         <is>
-          <t>客户终端</t>
+          <t>信用利差分析</t>
         </is>
       </c>
       <c r="E157" s="11" t="inlineStr">
         <is>
-          <t>客户查看投资建议与分析报告，确认交易服务，查看账户净值走势、持仓明细、交易明细</t>
+          <t>行业/评级/期限信用利差曲线实时计算，历史分位数分析</t>
         </is>
       </c>
       <c r="F157" s="11" t="inlineStr">
         <is>
-          <t>功能测试通过/正确率100%</t>
-        </is>
-      </c>
-      <c r="G157" s="24" t="inlineStr">
-        <is>
-          <t>中</t>
+          <t>功能完整/边界测试/集成冒烟/性能基线</t>
+        </is>
+      </c>
+      <c r="G157" s="23" t="inlineStr">
+        <is>
+          <t>高</t>
         </is>
       </c>
       <c r="H157" s="13" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
     </row>
     <row r="158" ht="28" customHeight="1">
       <c r="A158" s="11" t="inlineStr">
         <is>
-          <t>投顾服务</t>
+          <t>信用债/信用衍生品</t>
         </is>
       </c>
       <c r="B158" s="10" t="inlineStr">
@@ -8751,37 +9400,37 @@
       </c>
       <c r="C158" s="10" t="inlineStr">
         <is>
-          <t>F12-03</t>
+          <t>F11-02</t>
         </is>
       </c>
       <c r="D158" s="27" t="inlineStr">
         <is>
-          <t>投资建议书管理</t>
+          <t>CDS/CLN定价</t>
         </is>
       </c>
       <c r="E158" s="11" t="inlineStr">
         <is>
-          <t>投资建议书线上生成、审批、确认全流程，留痕追溯，客户电子签收</t>
+          <t>信用违约互换定价，ISDA标准，生存概率曲线校准</t>
         </is>
       </c>
       <c r="F158" s="11" t="inlineStr">
         <is>
-          <t>功能测试通过/正确率100%</t>
-        </is>
-      </c>
-      <c r="G158" s="24" t="inlineStr">
-        <is>
-          <t>中</t>
+          <t>p99延迟/误差率/精度验证/压测10k TPS</t>
+        </is>
+      </c>
+      <c r="G158" s="28" t="inlineStr">
+        <is>
+          <t>极高</t>
         </is>
       </c>
       <c r="H158" s="13" t="n">
-        <v>15</v>
+        <v>50</v>
       </c>
     </row>
     <row r="159" ht="28" customHeight="1">
       <c r="A159" s="11" t="inlineStr">
         <is>
-          <t>投顾服务</t>
+          <t>信用债/信用衍生品</t>
         </is>
       </c>
       <c r="B159" s="10" t="inlineStr">
@@ -8791,37 +9440,37 @@
       </c>
       <c r="C159" s="10" t="inlineStr">
         <is>
-          <t>F12-04</t>
+          <t>F11-03</t>
         </is>
       </c>
       <c r="D159" s="27" t="inlineStr">
         <is>
-          <t>账户分析报告</t>
+          <t>信用评级动态监控</t>
         </is>
       </c>
       <c r="E159" s="11" t="inlineStr">
         <is>
-          <t>账户净值走势、久期走势、归因分析、估值台账等核心数据展示及定期报告生成</t>
+          <t>对接外部评级机构（中诚信/联合/大公），评级下调预警</t>
         </is>
       </c>
       <c r="F159" s="11" t="inlineStr">
         <is>
-          <t>功能完整/边界测试/集成冒烟/性能基线</t>
-        </is>
-      </c>
-      <c r="G159" s="23" t="inlineStr">
-        <is>
-          <t>高</t>
+          <t>功能测试通过/正确率100%</t>
+        </is>
+      </c>
+      <c r="G159" s="24" t="inlineStr">
+        <is>
+          <t>中</t>
         </is>
       </c>
       <c r="H159" s="13" t="n">
-        <v>25</v>
+        <v>20</v>
       </c>
     </row>
     <row r="160" ht="28" customHeight="1">
       <c r="A160" s="11" t="inlineStr">
         <is>
-          <t>投顾服务</t>
+          <t>信用债/信用衍生品</t>
         </is>
       </c>
       <c r="B160" s="10" t="inlineStr">
@@ -8831,37 +9480,37 @@
       </c>
       <c r="C160" s="10" t="inlineStr">
         <is>
-          <t>F12-05</t>
+          <t>F11-04</t>
         </is>
       </c>
       <c r="D160" s="27" t="inlineStr">
         <is>
-          <t>投研报告服务</t>
+          <t>违约概率（PD）建模</t>
         </is>
       </c>
       <c r="E160" s="11" t="inlineStr">
         <is>
-          <t>日/周/月研究报告上传与推送，RPA自动获取基础数据，报告分类管理</t>
+          <t>结构化Merton模型+市场隐含PD，信用风险计量</t>
         </is>
       </c>
       <c r="F160" s="11" t="inlineStr">
         <is>
-          <t>功能测试通过/正确率100%</t>
-        </is>
-      </c>
-      <c r="G160" s="24" t="inlineStr">
-        <is>
-          <t>中</t>
+          <t>功能完整/边界测试/集成冒烟/性能基线</t>
+        </is>
+      </c>
+      <c r="G160" s="23" t="inlineStr">
+        <is>
+          <t>高</t>
         </is>
       </c>
       <c r="H160" s="13" t="n">
-        <v>15</v>
+        <v>40</v>
       </c>
     </row>
     <row r="161" ht="28" customHeight="1">
       <c r="A161" s="11" t="inlineStr">
         <is>
-          <t>投顾服务</t>
+          <t>信用债/信用衍生品</t>
         </is>
       </c>
       <c r="B161" s="10" t="inlineStr">
@@ -8871,44 +9520,44 @@
       </c>
       <c r="C161" s="10" t="inlineStr">
         <is>
-          <t>F12-06</t>
+          <t>F11-05</t>
         </is>
       </c>
       <c r="D161" s="27" t="inlineStr">
         <is>
-          <t>客户服务与基础服务</t>
+          <t>集中度限额管理</t>
         </is>
       </c>
       <c r="E161" s="11" t="inlineStr">
         <is>
-          <t>服务中心、消息中心、问卷系统；用户/账户/数据管理，消息群发，登录注册</t>
+          <t>行业/发行人/评级集中度多维限额，超限预警</t>
         </is>
       </c>
       <c r="F161" s="11" t="inlineStr">
         <is>
-          <t>功能测试通过</t>
-        </is>
-      </c>
-      <c r="G161" s="25" t="inlineStr">
-        <is>
-          <t>低</t>
+          <t>功能测试通过/正确率100%</t>
+        </is>
+      </c>
+      <c r="G161" s="24" t="inlineStr">
+        <is>
+          <t>中</t>
         </is>
       </c>
       <c r="H161" s="13" t="n">
-        <v>10</v>
+        <v>20</v>
       </c>
     </row>
     <row r="162" ht="20" customHeight="1">
       <c r="A162" s="26" t="inlineStr">
         <is>
-          <t>【P2】 TRS收益互换  (Total Return Swap)</t>
+          <t>【P2】 投顾服务  (Investment Advisory)</t>
         </is>
       </c>
     </row>
     <row r="163" ht="28" customHeight="1">
       <c r="A163" s="11" t="inlineStr">
         <is>
-          <t>TRS收益互换</t>
+          <t>投顾服务</t>
         </is>
       </c>
       <c r="B163" s="10" t="inlineStr">
@@ -8918,37 +9567,37 @@
       </c>
       <c r="C163" s="10" t="inlineStr">
         <is>
-          <t>F13-01</t>
+          <t>F12-01</t>
         </is>
       </c>
       <c r="D163" s="27" t="inlineStr">
         <is>
-          <t>TRS交易端</t>
+          <t>投顾工作台</t>
         </is>
       </c>
       <c r="E163" s="11" t="inlineStr">
         <is>
-          <t>报价提供，成交回报，对冲委托与自动对冲，请求报价，行情与资讯，历史确认</t>
+          <t>投顾人员操作界面，管理客户委托，上传研究报告，发送投资建议，查看客户反馈</t>
         </is>
       </c>
       <c r="F163" s="11" t="inlineStr">
         <is>
-          <t>功能完整/边界测试/集成冒烟/性能基线</t>
-        </is>
-      </c>
-      <c r="G163" s="23" t="inlineStr">
-        <is>
-          <t>高</t>
+          <t>功能测试通过/正确率100%</t>
+        </is>
+      </c>
+      <c r="G163" s="24" t="inlineStr">
+        <is>
+          <t>中</t>
         </is>
       </c>
       <c r="H163" s="13" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
     </row>
     <row r="164" ht="28" customHeight="1">
       <c r="A164" s="11" t="inlineStr">
         <is>
-          <t>TRS收益互换</t>
+          <t>投顾服务</t>
         </is>
       </c>
       <c r="B164" s="10" t="inlineStr">
@@ -8958,37 +9607,37 @@
       </c>
       <c r="C164" s="10" t="inlineStr">
         <is>
-          <t>F13-02</t>
+          <t>F12-02</t>
         </is>
       </c>
       <c r="D164" s="27" t="inlineStr">
         <is>
-          <t>TRS客户端</t>
+          <t>客户终端</t>
         </is>
       </c>
       <c r="E164" s="11" t="inlineStr">
         <is>
-          <t>开户申请，客户委托，出入金申请，合约持仓，标的持仓，资金管理，行情矩阵，自主下单</t>
+          <t>客户查看投资建议与分析报告，确认交易服务，查看账户净值走势、持仓明细、交易明细</t>
         </is>
       </c>
       <c r="F164" s="11" t="inlineStr">
         <is>
-          <t>功能完整/边界测试/集成冒烟/性能基线</t>
-        </is>
-      </c>
-      <c r="G164" s="23" t="inlineStr">
-        <is>
-          <t>高</t>
+          <t>功能测试通过/正确率100%</t>
+        </is>
+      </c>
+      <c r="G164" s="24" t="inlineStr">
+        <is>
+          <t>中</t>
         </is>
       </c>
       <c r="H164" s="13" t="n">
-        <v>25</v>
+        <v>20</v>
       </c>
     </row>
     <row r="165" ht="28" customHeight="1">
       <c r="A165" s="11" t="inlineStr">
         <is>
-          <t>TRS收益互换</t>
+          <t>投顾服务</t>
         </is>
       </c>
       <c r="B165" s="10" t="inlineStr">
@@ -8998,17 +9647,17 @@
       </c>
       <c r="C165" s="10" t="inlineStr">
         <is>
-          <t>F13-03</t>
+          <t>F12-03</t>
         </is>
       </c>
       <c r="D165" s="27" t="inlineStr">
         <is>
-          <t>TRS管理端</t>
+          <t>投资建议书管理</t>
         </is>
       </c>
       <c r="E165" s="11" t="inlineStr">
         <is>
-          <t>开户申请审批，合约成交管理，出入金审批，运营管理，对账，库存，对冲录入</t>
+          <t>投资建议书线上生成、审批、确认全流程，留痕追溯，客户电子签收</t>
         </is>
       </c>
       <c r="F165" s="11" t="inlineStr">
@@ -9022,13 +9671,13 @@
         </is>
       </c>
       <c r="H165" s="13" t="n">
-        <v>20</v>
+        <v>15</v>
       </c>
     </row>
     <row r="166" ht="28" customHeight="1">
       <c r="A166" s="11" t="inlineStr">
         <is>
-          <t>TRS收益互换</t>
+          <t>投顾服务</t>
         </is>
       </c>
       <c r="B166" s="10" t="inlineStr">
@@ -9038,17 +9687,17 @@
       </c>
       <c r="C166" s="10" t="inlineStr">
         <is>
-          <t>F13-04</t>
+          <t>F12-04</t>
         </is>
       </c>
       <c r="D166" s="27" t="inlineStr">
         <is>
-          <t>自动对冲</t>
+          <t>账户分析报告</t>
         </is>
       </c>
       <c r="E166" s="11" t="inlineStr">
         <is>
-          <t>对冲委托自动触发，对冲回报处理，风险校验，组合重叠分析，开平仓设置</t>
+          <t>账户净值走势、久期走势、归因分析、估值台账等核心数据展示及定期报告生成</t>
         </is>
       </c>
       <c r="F166" s="11" t="inlineStr">
@@ -9068,7 +9717,7 @@
     <row r="167" ht="28" customHeight="1">
       <c r="A167" s="11" t="inlineStr">
         <is>
-          <t>TRS收益互换</t>
+          <t>投顾服务</t>
         </is>
       </c>
       <c r="B167" s="10" t="inlineStr">
@@ -9078,17 +9727,17 @@
       </c>
       <c r="C167" s="10" t="inlineStr">
         <is>
-          <t>F13-05</t>
+          <t>F12-05</t>
         </is>
       </c>
       <c r="D167" s="27" t="inlineStr">
         <is>
-          <t>通知与确认文件</t>
+          <t>投研报告服务</t>
         </is>
       </c>
       <c r="E167" s="11" t="inlineStr">
         <is>
-          <t>企微通知提醒，确认书/结算单/估值报告/出入金通知自动生成并通过邮箱发送</t>
+          <t>日/周/月研究报告上传与推送，RPA自动获取基础数据，报告分类管理</t>
         </is>
       </c>
       <c r="F167" s="11" t="inlineStr">
@@ -9108,258 +9757,505 @@
     <row r="168" ht="28" customHeight="1">
       <c r="A168" s="11" t="inlineStr">
         <is>
+          <t>投顾服务</t>
+        </is>
+      </c>
+      <c r="B168" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="C168" s="10" t="inlineStr">
+        <is>
+          <t>F12-06</t>
+        </is>
+      </c>
+      <c r="D168" s="27" t="inlineStr">
+        <is>
+          <t>客户服务与基础服务</t>
+        </is>
+      </c>
+      <c r="E168" s="11" t="inlineStr">
+        <is>
+          <t>服务中心、消息中心、问卷系统；用户/账户/数据管理，消息群发，登录注册</t>
+        </is>
+      </c>
+      <c r="F168" s="11" t="inlineStr">
+        <is>
+          <t>功能测试通过</t>
+        </is>
+      </c>
+      <c r="G168" s="25" t="inlineStr">
+        <is>
+          <t>低</t>
+        </is>
+      </c>
+      <c r="H168" s="13" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="169" ht="20" customHeight="1">
+      <c r="A169" s="26" t="inlineStr">
+        <is>
+          <t>【P2】 TRS收益互换  (Total Return Swap)</t>
+        </is>
+      </c>
+    </row>
+    <row r="170" ht="28" customHeight="1">
+      <c r="A170" s="11" t="inlineStr">
+        <is>
           <t>TRS收益互换</t>
         </is>
       </c>
-      <c r="B168" s="10" t="inlineStr">
+      <c r="B170" s="10" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
       </c>
-      <c r="C168" s="10" t="inlineStr">
+      <c r="C170" s="10" t="inlineStr">
+        <is>
+          <t>F13-01</t>
+        </is>
+      </c>
+      <c r="D170" s="27" t="inlineStr">
+        <is>
+          <t>TRS交易端</t>
+        </is>
+      </c>
+      <c r="E170" s="11" t="inlineStr">
+        <is>
+          <t>报价提供，成交回报，对冲委托与自动对冲，请求报价，行情与资讯，历史确认</t>
+        </is>
+      </c>
+      <c r="F170" s="11" t="inlineStr">
+        <is>
+          <t>功能完整/边界测试/集成冒烟/性能基线</t>
+        </is>
+      </c>
+      <c r="G170" s="23" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="H170" s="13" t="n">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="171" ht="28" customHeight="1">
+      <c r="A171" s="11" t="inlineStr">
+        <is>
+          <t>TRS收益互换</t>
+        </is>
+      </c>
+      <c r="B171" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="C171" s="10" t="inlineStr">
+        <is>
+          <t>F13-02</t>
+        </is>
+      </c>
+      <c r="D171" s="27" t="inlineStr">
+        <is>
+          <t>TRS客户端</t>
+        </is>
+      </c>
+      <c r="E171" s="11" t="inlineStr">
+        <is>
+          <t>开户申请，客户委托，出入金申请，合约持仓，标的持仓，资金管理，行情矩阵，自主下单</t>
+        </is>
+      </c>
+      <c r="F171" s="11" t="inlineStr">
+        <is>
+          <t>功能完整/边界测试/集成冒烟/性能基线</t>
+        </is>
+      </c>
+      <c r="G171" s="23" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="H171" s="13" t="n">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="172" ht="28" customHeight="1">
+      <c r="A172" s="11" t="inlineStr">
+        <is>
+          <t>TRS收益互换</t>
+        </is>
+      </c>
+      <c r="B172" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="C172" s="10" t="inlineStr">
+        <is>
+          <t>F13-03</t>
+        </is>
+      </c>
+      <c r="D172" s="27" t="inlineStr">
+        <is>
+          <t>TRS管理端</t>
+        </is>
+      </c>
+      <c r="E172" s="11" t="inlineStr">
+        <is>
+          <t>开户申请审批，合约成交管理，出入金审批，运营管理，对账，库存，对冲录入</t>
+        </is>
+      </c>
+      <c r="F172" s="11" t="inlineStr">
+        <is>
+          <t>功能测试通过/正确率100%</t>
+        </is>
+      </c>
+      <c r="G172" s="24" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="H172" s="13" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="173" ht="28" customHeight="1">
+      <c r="A173" s="11" t="inlineStr">
+        <is>
+          <t>TRS收益互换</t>
+        </is>
+      </c>
+      <c r="B173" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="C173" s="10" t="inlineStr">
+        <is>
+          <t>F13-04</t>
+        </is>
+      </c>
+      <c r="D173" s="27" t="inlineStr">
+        <is>
+          <t>自动对冲</t>
+        </is>
+      </c>
+      <c r="E173" s="11" t="inlineStr">
+        <is>
+          <t>对冲委托自动触发，对冲回报处理，风险校验，组合重叠分析，开平仓设置</t>
+        </is>
+      </c>
+      <c r="F173" s="11" t="inlineStr">
+        <is>
+          <t>功能完整/边界测试/集成冒烟/性能基线</t>
+        </is>
+      </c>
+      <c r="G173" s="23" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="H173" s="13" t="n">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="174" ht="28" customHeight="1">
+      <c r="A174" s="11" t="inlineStr">
+        <is>
+          <t>TRS收益互换</t>
+        </is>
+      </c>
+      <c r="B174" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="C174" s="10" t="inlineStr">
+        <is>
+          <t>F13-05</t>
+        </is>
+      </c>
+      <c r="D174" s="27" t="inlineStr">
+        <is>
+          <t>通知与确认文件</t>
+        </is>
+      </c>
+      <c r="E174" s="11" t="inlineStr">
+        <is>
+          <t>企微通知提醒，确认书/结算单/估值报告/出入金通知自动生成并通过邮箱发送</t>
+        </is>
+      </c>
+      <c r="F174" s="11" t="inlineStr">
+        <is>
+          <t>功能测试通过/正确率100%</t>
+        </is>
+      </c>
+      <c r="G174" s="24" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="H174" s="13" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="175" ht="28" customHeight="1">
+      <c r="A175" s="11" t="inlineStr">
+        <is>
+          <t>TRS收益互换</t>
+        </is>
+      </c>
+      <c r="B175" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="C175" s="10" t="inlineStr">
         <is>
           <t>F13-06</t>
         </is>
       </c>
-      <c r="D168" s="27" t="inlineStr">
+      <c r="D175" s="27" t="inlineStr">
         <is>
           <t>系统集成</t>
         </is>
       </c>
-      <c r="E168" s="11" t="inlineStr">
+      <c r="E175" s="11" t="inlineStr">
         <is>
           <t>与衡泰系统客户信息同步，QTrade聊天记录同步，交易管理系统对接，银行流水对接</t>
         </is>
       </c>
-      <c r="F168" s="11" t="inlineStr">
+      <c r="F175" s="11" t="inlineStr">
         <is>
           <t>功能完整/边界测试/集成冒烟/性能基线</t>
         </is>
       </c>
-      <c r="G168" s="23" t="inlineStr">
+      <c r="G175" s="23" t="inlineStr">
         <is>
           <t>高</t>
         </is>
       </c>
-      <c r="H168" s="13" t="n">
+      <c r="H175" s="13" t="n">
         <v>25</v>
       </c>
     </row>
-    <row r="169" ht="20" customHeight="1">
-      <c r="A169" s="29" t="inlineStr">
+    <row r="176" ht="20" customHeight="1">
+      <c r="A176" s="29" t="inlineStr">
         <is>
           <t>【P3】 做市商系统  (Market Making)</t>
         </is>
       </c>
     </row>
-    <row r="170" ht="28" customHeight="1">
-      <c r="A170" s="16" t="inlineStr">
+    <row r="177" ht="28" customHeight="1">
+      <c r="A177" s="16" t="inlineStr">
         <is>
           <t>做市商系统</t>
         </is>
       </c>
-      <c r="B170" s="15" t="inlineStr">
+      <c r="B177" s="15" t="inlineStr">
         <is>
           <t>P3</t>
         </is>
       </c>
-      <c r="C170" s="15" t="inlineStr">
+      <c r="C177" s="15" t="inlineStr">
         <is>
           <t>F15-01</t>
         </is>
       </c>
-      <c r="D170" s="30" t="inlineStr">
+      <c r="D177" s="30" t="inlineStr">
         <is>
           <t>双边报价引擎</t>
         </is>
       </c>
-      <c r="E170" s="16" t="inlineStr">
+      <c r="E177" s="16" t="inlineStr">
         <is>
           <t>多品种同时双边报价，延迟&lt;5ms，报价宽度动态优化</t>
         </is>
       </c>
-      <c r="F170" s="16" t="inlineStr">
+      <c r="F177" s="16" t="inlineStr">
         <is>
           <t>p99延迟/误差率/精度验证/压测10k TPS</t>
         </is>
       </c>
-      <c r="G170" s="28" t="inlineStr">
+      <c r="G177" s="28" t="inlineStr">
         <is>
           <t>极高</t>
         </is>
       </c>
-      <c r="H170" s="18" t="n">
+      <c r="H177" s="18" t="n">
         <v>70</v>
       </c>
     </row>
-    <row r="171" ht="28" customHeight="1">
-      <c r="A171" s="16" t="inlineStr">
+    <row r="178" ht="28" customHeight="1">
+      <c r="A178" s="16" t="inlineStr">
         <is>
           <t>做市商系统</t>
         </is>
       </c>
-      <c r="B171" s="15" t="inlineStr">
+      <c r="B178" s="15" t="inlineStr">
         <is>
           <t>P3</t>
         </is>
       </c>
-      <c r="C171" s="15" t="inlineStr">
+      <c r="C178" s="15" t="inlineStr">
         <is>
           <t>F15-02</t>
         </is>
       </c>
-      <c r="D171" s="30" t="inlineStr">
+      <c r="D178" s="30" t="inlineStr">
         <is>
           <t>库存风险实时管理</t>
         </is>
       </c>
-      <c r="E171" s="16" t="inlineStr">
+      <c r="E178" s="16" t="inlineStr">
         <is>
           <t>做市库存PnL实时监控，Delta对冲自动触发</t>
         </is>
       </c>
-      <c r="F171" s="16" t="inlineStr">
+      <c r="F178" s="16" t="inlineStr">
         <is>
           <t>p99延迟/误差率/精度验证/压测10k TPS</t>
         </is>
       </c>
-      <c r="G171" s="28" t="inlineStr">
+      <c r="G178" s="28" t="inlineStr">
         <is>
           <t>极高</t>
         </is>
       </c>
-      <c r="H171" s="18" t="n">
+      <c r="H178" s="18" t="n">
         <v>60</v>
       </c>
     </row>
-    <row r="172" ht="28" customHeight="1">
-      <c r="A172" s="16" t="inlineStr">
+    <row r="179" ht="28" customHeight="1">
+      <c r="A179" s="16" t="inlineStr">
         <is>
           <t>做市商系统</t>
         </is>
       </c>
-      <c r="B172" s="15" t="inlineStr">
+      <c r="B179" s="15" t="inlineStr">
         <is>
           <t>P3</t>
         </is>
       </c>
-      <c r="C172" s="15" t="inlineStr">
+      <c r="C179" s="15" t="inlineStr">
         <is>
           <t>F15-03</t>
         </is>
       </c>
-      <c r="D172" s="30" t="inlineStr">
+      <c r="D179" s="30" t="inlineStr">
         <is>
           <t>报价优化算法</t>
         </is>
       </c>
-      <c r="E172" s="16" t="inlineStr">
+      <c r="E179" s="16" t="inlineStr">
         <is>
           <t>基于市场微结构理论动态调整bid-ask spread</t>
         </is>
       </c>
-      <c r="F172" s="16" t="inlineStr">
+      <c r="F179" s="16" t="inlineStr">
         <is>
           <t>p99延迟/误差率/精度验证/压测10k TPS</t>
         </is>
       </c>
-      <c r="G172" s="28" t="inlineStr">
+      <c r="G179" s="28" t="inlineStr">
         <is>
           <t>极高</t>
         </is>
       </c>
-      <c r="H172" s="18" t="n">
+      <c r="H179" s="18" t="n">
         <v>50</v>
       </c>
     </row>
-    <row r="173" ht="28" customHeight="1">
-      <c r="A173" s="16" t="inlineStr">
+    <row r="180" ht="28" customHeight="1">
+      <c r="A180" s="16" t="inlineStr">
         <is>
           <t>做市商系统</t>
         </is>
       </c>
-      <c r="B173" s="15" t="inlineStr">
+      <c r="B180" s="15" t="inlineStr">
         <is>
           <t>P3</t>
         </is>
       </c>
-      <c r="C173" s="15" t="inlineStr">
+      <c r="C180" s="15" t="inlineStr">
         <is>
           <t>F15-04</t>
         </is>
       </c>
-      <c r="D173" s="30" t="inlineStr">
+      <c r="D180" s="30" t="inlineStr">
         <is>
           <t>竞争力分析</t>
         </is>
       </c>
-      <c r="E173" s="16" t="inlineStr">
+      <c r="E180" s="16" t="inlineStr">
         <is>
           <t>与市场最优报价对比，中签率分析，策略调优</t>
         </is>
       </c>
-      <c r="F173" s="16" t="inlineStr">
+      <c r="F180" s="16" t="inlineStr">
         <is>
           <t>功能完整/边界测试/集成冒烟/性能基线</t>
         </is>
       </c>
-      <c r="G173" s="23" t="inlineStr">
+      <c r="G180" s="23" t="inlineStr">
         <is>
           <t>高</t>
         </is>
       </c>
-      <c r="H173" s="18" t="n">
+      <c r="H180" s="18" t="n">
         <v>25</v>
       </c>
     </row>
-    <row r="174" ht="28" customHeight="1">
-      <c r="A174" s="16" t="inlineStr">
+    <row r="181" ht="28" customHeight="1">
+      <c r="A181" s="16" t="inlineStr">
         <is>
           <t>做市商系统</t>
         </is>
       </c>
-      <c r="B174" s="15" t="inlineStr">
+      <c r="B181" s="15" t="inlineStr">
         <is>
           <t>P3</t>
         </is>
       </c>
-      <c r="C174" s="15" t="inlineStr">
+      <c r="C181" s="15" t="inlineStr">
         <is>
           <t>F15-05</t>
         </is>
       </c>
-      <c r="D174" s="30" t="inlineStr">
+      <c r="D181" s="30" t="inlineStr">
         <is>
           <t>交易对手管理集成</t>
         </is>
       </c>
-      <c r="E174" s="16" t="inlineStr">
+      <c r="E181" s="16" t="inlineStr">
         <is>
           <t>做市交易对手信用实时检查，额度占用同步更新</t>
         </is>
       </c>
-      <c r="F174" s="16" t="inlineStr">
+      <c r="F181" s="16" t="inlineStr">
         <is>
           <t>功能测试通过/正确率100%</t>
         </is>
       </c>
-      <c r="G174" s="24" t="inlineStr">
+      <c r="G181" s="24" t="inlineStr">
         <is>
           <t>中</t>
         </is>
       </c>
-      <c r="H174" s="18" t="n">
+      <c r="H181" s="18" t="n">
         <v>20</v>
       </c>
     </row>
-    <row r="175">
-      <c r="A175" s="19" t="inlineStr">
+    <row r="182">
+      <c r="A182" s="19" t="inlineStr">
         <is>
           <t>总计功能数 / Total Function Points</t>
         </is>
       </c>
-      <c r="H175" s="20">
-        <f>SUM(H3:H174)</f>
+      <c r="H182" s="20">
+        <f>SUM(H3:H181)</f>
         <v/>
       </c>
     </row>
@@ -9368,19 +10264,19 @@
     <mergeCell ref="A67:H67"/>
     <mergeCell ref="A100:H100"/>
     <mergeCell ref="A3:H3"/>
-    <mergeCell ref="A155:H155"/>
     <mergeCell ref="A162:H162"/>
+    <mergeCell ref="A176:H176"/>
     <mergeCell ref="A87:H87"/>
-    <mergeCell ref="A175:G175"/>
+    <mergeCell ref="A156:H156"/>
     <mergeCell ref="A129:H129"/>
     <mergeCell ref="A60:H60"/>
     <mergeCell ref="A142:H142"/>
     <mergeCell ref="A169:H169"/>
     <mergeCell ref="A1:H1"/>
+    <mergeCell ref="A182:G182"/>
     <mergeCell ref="A111:H111"/>
     <mergeCell ref="A31:H31"/>
     <mergeCell ref="A149:H149"/>
-    <mergeCell ref="A135:H135"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -10379,7 +11275,7 @@
         </is>
       </c>
       <c r="H9" s="8" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="I9" s="8" t="n">
         <v>12</v>

</xml_diff>

<commit_message>
Expand module 09 定价平台: 15 functions/5 domains + tech_design
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Feasibility_analysis/FICC_Gap_Analysis.xlsx
+++ b/Feasibility_analysis/FICC_Gap_Analysis.xlsx
@@ -19,6 +19,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="详情_事前风控_合规" sheetId="10" state="visible" r:id="rId10"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="详情_组合管理+绩效归因" sheetId="11" state="visible" r:id="rId11"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="详情_策略投资_量化" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="详情_定价平台" sheetId="13" state="visible" r:id="rId13"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Area" localSheetId="0">'差距分析总表'!$A$1:$P$17</definedName>
@@ -1511,7 +1512,7 @@
       </c>
       <c r="P11" s="11" t="inlineStr">
         <is>
-          <t>蒙特卡洛/有限差分，替代衡泰核心</t>
+          <t>蒙特卡洛/有限差分，替代衡泰核心，覆盖权益/利率/大宗商品/外汇/衍生品全品种；对应PPT Slide 56</t>
         </is>
       </c>
     </row>
@@ -4006,13 +4007,742 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J25"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="48" customWidth="1" min="4" max="4"/>
+    <col width="26" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="6" max="6"/>
+    <col width="8" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="8" max="8"/>
+    <col width="7" customWidth="1" min="9" max="9"/>
+    <col width="18" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="24" customHeight="1">
+      <c r="A1" s="38" t="inlineStr">
+        <is>
+          <t>系统详情：定价平台  |  Pricing Platform</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="36" customHeight="1">
+      <c r="A2" s="39" t="inlineStr">
+        <is>
+          <t>战略定位：蒙特卡洛/有限差分，替代衡泰核心，覆盖权益/利率/大宗商品/外汇/衍生品全品种；对应PPT Slide 56   |   来源：Slide 56</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="28" customHeight="1">
+      <c r="A3" s="40" t="inlineStr">
+        <is>
+          <t>模块：定价平台  (Pricing Platform)  |  优先级：P2  |  竞品：衡泰(垄断)  |  华锐基础：ARC基础数值库  |  工期：18月  团队：15人</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="28" customHeight="1">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>功能域</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>编号</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>功能名称</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>功能描述</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>验收标准</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>集成依赖</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>复杂度</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>预估(人天)</t>
+        </is>
+      </c>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t>优先级</t>
+        </is>
+      </c>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>备注</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="18" customHeight="1">
+      <c r="A5" s="22" t="inlineStr">
+        <is>
+          <t>D1. 金融产品覆盖</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="48" customHeight="1">
+      <c r="A6" s="11" t="inlineStr">
+        <is>
+          <t>D1. 金融产品覆盖</t>
+        </is>
+      </c>
+      <c r="B6" s="10" t="inlineStr">
+        <is>
+          <t>F09-01</t>
+        </is>
+      </c>
+      <c r="C6" s="27" t="inlineStr">
+        <is>
+          <t>期权收益结构定价</t>
+        </is>
+      </c>
+      <c r="D6" s="11" t="inlineStr">
+        <is>
+          <t>香草期权/价差期权/欧式/美式/雪球/自定义期权定价，挂钩标的覆盖国债/期货/股票/指数/商品</t>
+        </is>
+      </c>
+      <c r="E6" s="11" t="inlineStr"/>
+      <c r="F6" s="11" t="inlineStr"/>
+      <c r="G6" s="28" t="inlineStr">
+        <is>
+          <t>极高</t>
+        </is>
+      </c>
+      <c r="H6" s="13" t="n">
+        <v>60</v>
+      </c>
+      <c r="I6" s="12" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="J6" s="11" t="inlineStr"/>
+    </row>
+    <row r="7" ht="48" customHeight="1">
+      <c r="A7" s="11" t="inlineStr">
+        <is>
+          <t>D1. 金融产品覆盖</t>
+        </is>
+      </c>
+      <c r="B7" s="10" t="inlineStr">
+        <is>
+          <t>F09-02</t>
+        </is>
+      </c>
+      <c r="C7" s="27" t="inlineStr">
+        <is>
+          <t>结构化产品定价</t>
+        </is>
+      </c>
+      <c r="D7" s="11" t="inlineStr">
+        <is>
+          <t>场外期权/远期/收益凭证/收益互换/融资融券/合约型互换定价，支持自定义结构化产品</t>
+        </is>
+      </c>
+      <c r="E7" s="11" t="inlineStr"/>
+      <c r="F7" s="11" t="inlineStr"/>
+      <c r="G7" s="28" t="inlineStr">
+        <is>
+          <t>极高</t>
+        </is>
+      </c>
+      <c r="H7" s="13" t="n">
+        <v>50</v>
+      </c>
+      <c r="I7" s="12" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="J7" s="11" t="inlineStr"/>
+    </row>
+    <row r="8" ht="48" customHeight="1">
+      <c r="A8" s="11" t="inlineStr">
+        <is>
+          <t>D1. 金融产品覆盖</t>
+        </is>
+      </c>
+      <c r="B8" s="10" t="inlineStr">
+        <is>
+          <t>F09-03</t>
+        </is>
+      </c>
+      <c r="C8" s="27" t="inlineStr">
+        <is>
+          <t>固收品种定价</t>
+        </is>
+      </c>
+      <c r="D8" s="11" t="inlineStr">
+        <is>
+          <t>固息/浮息国债，含权债，可转债精确定价，信用债估值，ABS定价</t>
+        </is>
+      </c>
+      <c r="E8" s="11" t="inlineStr"/>
+      <c r="F8" s="11" t="inlineStr"/>
+      <c r="G8" s="41" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="H8" s="13" t="n">
+        <v>40</v>
+      </c>
+      <c r="I8" s="12" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="J8" s="11" t="inlineStr"/>
+    </row>
+    <row r="9" ht="18" customHeight="1">
+      <c r="A9" s="40" t="inlineStr">
+        <is>
+          <t>D2. 市场数据底座</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="48" customHeight="1">
+      <c r="A10" s="11" t="inlineStr">
+        <is>
+          <t>D2. 市场数据底座</t>
+        </is>
+      </c>
+      <c r="B10" s="10" t="inlineStr">
+        <is>
+          <t>F09-04</t>
+        </is>
+      </c>
+      <c r="C10" s="27" t="inlineStr">
+        <is>
+          <t>利率与信用曲线构建</t>
+        </is>
+      </c>
+      <c r="D10" s="11" t="inlineStr">
+        <is>
+          <t>利率曲线（多插值方法），信用利差曲线，利差曲线，违约曲线，全品种统一曲线服务</t>
+        </is>
+      </c>
+      <c r="E10" s="11" t="inlineStr"/>
+      <c r="F10" s="11" t="inlineStr"/>
+      <c r="G10" s="28" t="inlineStr">
+        <is>
+          <t>极高</t>
+        </is>
+      </c>
+      <c r="H10" s="13" t="n">
+        <v>60</v>
+      </c>
+      <c r="I10" s="12" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="J10" s="11" t="inlineStr"/>
+    </row>
+    <row r="11" ht="48" customHeight="1">
+      <c r="A11" s="11" t="inlineStr">
+        <is>
+          <t>D2. 市场数据底座</t>
+        </is>
+      </c>
+      <c r="B11" s="10" t="inlineStr">
+        <is>
+          <t>F09-05</t>
+        </is>
+      </c>
+      <c r="C11" s="27" t="inlineStr">
+        <is>
+          <t>波动率曲面构建</t>
+        </is>
+      </c>
+      <c r="D11" s="11" t="inlineStr">
+        <is>
+          <t>隐含波动率曲面，红利曲线，汇率曲线，Local Volatility曲面，波动率微笑校准</t>
+        </is>
+      </c>
+      <c r="E11" s="11" t="inlineStr"/>
+      <c r="F11" s="11" t="inlineStr"/>
+      <c r="G11" s="28" t="inlineStr">
+        <is>
+          <t>极高</t>
+        </is>
+      </c>
+      <c r="H11" s="13" t="n">
+        <v>50</v>
+      </c>
+      <c r="I11" s="12" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="J11" s="11" t="inlineStr"/>
+    </row>
+    <row r="12" ht="48" customHeight="1">
+      <c r="A12" s="11" t="inlineStr">
+        <is>
+          <t>D2. 市场数据底座</t>
+        </is>
+      </c>
+      <c r="B12" s="10" t="inlineStr">
+        <is>
+          <t>F09-06</t>
+        </is>
+      </c>
+      <c r="C12" s="27" t="inlineStr">
+        <is>
+          <t>市场数据管理</t>
+        </is>
+      </c>
+      <c r="D12" s="11" t="inlineStr">
+        <is>
+          <t>境内外权益/债券/外汇/商品资讯统一接入，数据清洗，异常值处理，数据质量监控</t>
+        </is>
+      </c>
+      <c r="E12" s="11" t="inlineStr"/>
+      <c r="F12" s="11" t="inlineStr"/>
+      <c r="G12" s="41" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="H12" s="13" t="n">
+        <v>30</v>
+      </c>
+      <c r="I12" s="12" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="J12" s="11" t="inlineStr"/>
+    </row>
+    <row r="13" ht="18" customHeight="1">
+      <c r="A13" s="43" t="inlineStr">
+        <is>
+          <t>D3. 定价模型引擎</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="48" customHeight="1">
+      <c r="A14" s="11" t="inlineStr">
+        <is>
+          <t>D3. 定价模型引擎</t>
+        </is>
+      </c>
+      <c r="B14" s="10" t="inlineStr">
+        <is>
+          <t>F09-07</t>
+        </is>
+      </c>
+      <c r="C14" s="27" t="inlineStr">
+        <is>
+          <t>蒙特卡洛求解器</t>
+        </is>
+      </c>
+      <c r="D14" s="11" t="inlineStr">
+        <is>
+          <t>GPU加速MC，QMC低差异序列，支持路径相关期权定价，并行情景模拟</t>
+        </is>
+      </c>
+      <c r="E14" s="11" t="inlineStr"/>
+      <c r="F14" s="11" t="inlineStr"/>
+      <c r="G14" s="28" t="inlineStr">
+        <is>
+          <t>极高</t>
+        </is>
+      </c>
+      <c r="H14" s="13" t="n">
+        <v>70</v>
+      </c>
+      <c r="I14" s="12" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="J14" s="11" t="inlineStr"/>
+    </row>
+    <row r="15" ht="48" customHeight="1">
+      <c r="A15" s="11" t="inlineStr">
+        <is>
+          <t>D3. 定价模型引擎</t>
+        </is>
+      </c>
+      <c r="B15" s="10" t="inlineStr">
+        <is>
+          <t>F09-08</t>
+        </is>
+      </c>
+      <c r="C15" s="27" t="inlineStr">
+        <is>
+          <t>解析解与数值解</t>
+        </is>
+      </c>
+      <c r="D15" s="11" t="inlineStr">
+        <is>
+          <t>Black-Scholes解析解，Hull-White利率模型，SABR波动率模型，二叉树/三叉树数值解</t>
+        </is>
+      </c>
+      <c r="E15" s="11" t="inlineStr"/>
+      <c r="F15" s="11" t="inlineStr"/>
+      <c r="G15" s="28" t="inlineStr">
+        <is>
+          <t>极高</t>
+        </is>
+      </c>
+      <c r="H15" s="13" t="n">
+        <v>60</v>
+      </c>
+      <c r="I15" s="12" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="J15" s="11" t="inlineStr"/>
+    </row>
+    <row r="16" ht="48" customHeight="1">
+      <c r="A16" s="11" t="inlineStr">
+        <is>
+          <t>D3. 定价模型引擎</t>
+        </is>
+      </c>
+      <c r="B16" s="10" t="inlineStr">
+        <is>
+          <t>F09-09</t>
+        </is>
+      </c>
+      <c r="C16" s="27" t="inlineStr">
+        <is>
+          <t>有限差分（PDE）</t>
+        </is>
+      </c>
+      <c r="D16" s="11" t="inlineStr">
+        <is>
+          <t>Crank-Nicolson/ADI方法，含权债/可转债精确定价，局部波动率模型数值解</t>
+        </is>
+      </c>
+      <c r="E16" s="11" t="inlineStr"/>
+      <c r="F16" s="11" t="inlineStr"/>
+      <c r="G16" s="28" t="inlineStr">
+        <is>
+          <t>极高</t>
+        </is>
+      </c>
+      <c r="H16" s="13" t="n">
+        <v>60</v>
+      </c>
+      <c r="I16" s="12" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="J16" s="11" t="inlineStr"/>
+    </row>
+    <row r="17" ht="48" customHeight="1">
+      <c r="A17" s="11" t="inlineStr">
+        <is>
+          <t>D3. 定价模型引擎</t>
+        </is>
+      </c>
+      <c r="B17" s="10" t="inlineStr">
+        <is>
+          <t>F09-10</t>
+        </is>
+      </c>
+      <c r="C17" s="27" t="inlineStr">
+        <is>
+          <t>实时Greeks计算</t>
+        </is>
+      </c>
+      <c r="D17" s="11" t="inlineStr">
+        <is>
+          <t>Delta/Gamma/Vega/Theta/Rho分布式实时计算，DV01/CS01，分桶敏感度</t>
+        </is>
+      </c>
+      <c r="E17" s="11" t="inlineStr"/>
+      <c r="F17" s="11" t="inlineStr"/>
+      <c r="G17" s="41" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="H17" s="13" t="n">
+        <v>40</v>
+      </c>
+      <c r="I17" s="12" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="J17" s="11" t="inlineStr"/>
+    </row>
+    <row r="18" ht="18" customHeight="1">
+      <c r="A18" s="43" t="inlineStr">
+        <is>
+          <t>D4. 定价应用场景</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="48" customHeight="1">
+      <c r="A19" s="11" t="inlineStr">
+        <is>
+          <t>D4. 定价应用场景</t>
+        </is>
+      </c>
+      <c r="B19" s="10" t="inlineStr">
+        <is>
+          <t>F09-11</t>
+        </is>
+      </c>
+      <c r="C19" s="27" t="inlineStr">
+        <is>
+          <t>估值与结算计算</t>
+        </is>
+      </c>
+      <c r="D19" s="11" t="inlineStr">
+        <is>
+          <t>日终估值，盯市计算，保证金计算，结算价格，历史估值回测与误差分析</t>
+        </is>
+      </c>
+      <c r="E19" s="11" t="inlineStr"/>
+      <c r="F19" s="11" t="inlineStr"/>
+      <c r="G19" s="41" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="H19" s="13" t="n">
+        <v>40</v>
+      </c>
+      <c r="I19" s="12" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="J19" s="11" t="inlineStr"/>
+    </row>
+    <row r="20" ht="48" customHeight="1">
+      <c r="A20" s="11" t="inlineStr">
+        <is>
+          <t>D4. 定价应用场景</t>
+        </is>
+      </c>
+      <c r="B20" s="10" t="inlineStr">
+        <is>
+          <t>F09-12</t>
+        </is>
+      </c>
+      <c r="C20" s="27" t="inlineStr">
+        <is>
+          <t>风控与情景计算</t>
+        </is>
+      </c>
+      <c r="D20" s="11" t="inlineStr">
+        <is>
+          <t>风险计量（VaR/压力测试）调用，情景分析，保证金计算，为风控平台提供统一定价接口</t>
+        </is>
+      </c>
+      <c r="E20" s="11" t="inlineStr"/>
+      <c r="F20" s="11" t="inlineStr"/>
+      <c r="G20" s="41" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="H20" s="13" t="n">
+        <v>35</v>
+      </c>
+      <c r="I20" s="12" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="J20" s="11" t="inlineStr"/>
+    </row>
+    <row r="21" ht="48" customHeight="1">
+      <c r="A21" s="11" t="inlineStr">
+        <is>
+          <t>D4. 定价应用场景</t>
+        </is>
+      </c>
+      <c r="B21" s="10" t="inlineStr">
+        <is>
+          <t>F09-13</t>
+        </is>
+      </c>
+      <c r="C21" s="27" t="inlineStr">
+        <is>
+          <t>客需报价服务</t>
+        </is>
+      </c>
+      <c r="D21" s="11" t="inlineStr">
+        <is>
+          <t>为销售交易/TRS系统提供实时报价，一站式报价接口，支持结构化产品定制化快速报价</t>
+        </is>
+      </c>
+      <c r="E21" s="11" t="inlineStr"/>
+      <c r="F21" s="11" t="inlineStr"/>
+      <c r="G21" s="41" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="H21" s="13" t="n">
+        <v>35</v>
+      </c>
+      <c r="I21" s="12" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="J21" s="11" t="inlineStr"/>
+    </row>
+    <row r="22" ht="18" customHeight="1">
+      <c r="A22" s="29" t="inlineStr">
+        <is>
+          <t>D5. 平台基础设施</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="48" customHeight="1">
+      <c r="A23" s="11" t="inlineStr">
+        <is>
+          <t>D5. 平台基础设施</t>
+        </is>
+      </c>
+      <c r="B23" s="10" t="inlineStr">
+        <is>
+          <t>F09-14</t>
+        </is>
+      </c>
+      <c r="C23" s="27" t="inlineStr">
+        <is>
+          <t>定价微服务架构</t>
+        </is>
+      </c>
+      <c r="D23" s="11" t="inlineStr">
+        <is>
+          <t>REST/gRPC定价API，横向弹性扩容，p99&lt;100ms，模型插件化注册，版本管理</t>
+        </is>
+      </c>
+      <c r="E23" s="11" t="inlineStr"/>
+      <c r="F23" s="11" t="inlineStr"/>
+      <c r="G23" s="41" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="H23" s="13" t="n">
+        <v>40</v>
+      </c>
+      <c r="I23" s="12" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="J23" s="11" t="inlineStr"/>
+    </row>
+    <row r="24" ht="48" customHeight="1">
+      <c r="A24" s="11" t="inlineStr">
+        <is>
+          <t>D5. 平台基础设施</t>
+        </is>
+      </c>
+      <c r="B24" s="10" t="inlineStr">
+        <is>
+          <t>F09-15</t>
+        </is>
+      </c>
+      <c r="C24" s="27" t="inlineStr">
+        <is>
+          <t>灵活二次开发能力</t>
+        </is>
+      </c>
+      <c r="D24" s="11" t="inlineStr">
+        <is>
+          <t>全平台级/单功能模块级/系统框架级可扩展，支持自定义模型接入，策略团队自助扩展</t>
+        </is>
+      </c>
+      <c r="E24" s="11" t="inlineStr"/>
+      <c r="F24" s="11" t="inlineStr"/>
+      <c r="G24" s="41" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="H24" s="13" t="n">
+        <v>30</v>
+      </c>
+      <c r="I24" s="12" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="J24" s="11" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="40" t="inlineStr">
+        <is>
+          <t>合计 15项功能  |  P1: 0项  |  P2: 15项</t>
+        </is>
+      </c>
+      <c r="H25" s="20">
+        <f>SUM(H5:H24)</f>
+        <v/>
+      </c>
+      <c r="I25" s="34" t="inlineStr"/>
+      <c r="J25" s="34" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <mergeCells count="9">
+    <mergeCell ref="A1:J1"/>
+    <mergeCell ref="A5:J5"/>
+    <mergeCell ref="A22:J22"/>
+    <mergeCell ref="A9:J9"/>
+    <mergeCell ref="A18:J18"/>
+    <mergeCell ref="A3:J3"/>
+    <mergeCell ref="A25:G25"/>
+    <mergeCell ref="A2:J2"/>
+    <mergeCell ref="A13:J13"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" fitToWidth="1"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H183"/>
+  <dimension ref="A1:H192"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -9435,12 +10165,12 @@
       </c>
       <c r="D144" s="27" t="inlineStr">
         <is>
-          <t>期限结构模型</t>
+          <t>期权收益结构定价</t>
         </is>
       </c>
       <c r="E144" s="11" t="inlineStr">
         <is>
-          <t>Nelson-Siegel/Svensson/HJM等多模型参数拟合，实时曲线</t>
+          <t>香草期权/价差期权/欧式/美式/雪球/自定义期权定价，挂钩标的覆盖国债/期货/股票/指数/商品</t>
         </is>
       </c>
       <c r="F144" s="11" t="inlineStr">
@@ -9475,12 +10205,12 @@
       </c>
       <c r="D145" s="27" t="inlineStr">
         <is>
-          <t>蒙特卡洛求解器</t>
+          <t>结构化产品定价</t>
         </is>
       </c>
       <c r="E145" s="11" t="inlineStr">
         <is>
-          <t>GPU加速MC，QMC低差异序列，支持路径相关期权定价</t>
+          <t>场外期权/远期/收益凭证/收益互换/融资融券/合约型互换定价，支持自定义结构化产品</t>
         </is>
       </c>
       <c r="F145" s="11" t="inlineStr">
@@ -9494,7 +10224,7 @@
         </is>
       </c>
       <c r="H145" s="13" t="n">
-        <v>70</v>
+        <v>50</v>
       </c>
     </row>
     <row r="146" ht="28" customHeight="1">
@@ -9515,26 +10245,26 @@
       </c>
       <c r="D146" s="27" t="inlineStr">
         <is>
-          <t>有限差分（PDE）</t>
+          <t>固收品种定价</t>
         </is>
       </c>
       <c r="E146" s="11" t="inlineStr">
         <is>
-          <t>Crank-Nicolson/ADI方法，含权债/可转债精确定价</t>
+          <t>固息/浮息国债，含权债，可转债精确定价，信用债估值，ABS定价</t>
         </is>
       </c>
       <c r="F146" s="11" t="inlineStr">
         <is>
-          <t>p99延迟/误差率/精度验证/压测10k TPS</t>
-        </is>
-      </c>
-      <c r="G146" s="28" t="inlineStr">
-        <is>
-          <t>极高</t>
+          <t>功能完整/边界测试/集成冒烟/性能基线</t>
+        </is>
+      </c>
+      <c r="G146" s="23" t="inlineStr">
+        <is>
+          <t>高</t>
         </is>
       </c>
       <c r="H146" s="13" t="n">
-        <v>60</v>
+        <v>40</v>
       </c>
     </row>
     <row r="147" ht="28" customHeight="1">
@@ -9555,26 +10285,26 @@
       </c>
       <c r="D147" s="27" t="inlineStr">
         <is>
-          <t>实时Greeks</t>
+          <t>利率与信用曲线构建</t>
         </is>
       </c>
       <c r="E147" s="11" t="inlineStr">
         <is>
-          <t>Delta/Gamma/Vega/Theta/Rho分布式实时计算</t>
+          <t>利率曲线（多插值方法），信用利差曲线，利差曲线，违约曲线，全品种统一曲线服务</t>
         </is>
       </c>
       <c r="F147" s="11" t="inlineStr">
         <is>
-          <t>功能完整/边界测试/集成冒烟/性能基线</t>
-        </is>
-      </c>
-      <c r="G147" s="23" t="inlineStr">
-        <is>
-          <t>高</t>
+          <t>p99延迟/误差率/精度验证/压测10k TPS</t>
+        </is>
+      </c>
+      <c r="G147" s="28" t="inlineStr">
+        <is>
+          <t>极高</t>
         </is>
       </c>
       <c r="H147" s="13" t="n">
-        <v>40</v>
+        <v>60</v>
       </c>
     </row>
     <row r="148" ht="28" customHeight="1">
@@ -9595,26 +10325,26 @@
       </c>
       <c r="D148" s="27" t="inlineStr">
         <is>
-          <t>定价服务微服务架构</t>
+          <t>波动率曲面构建</t>
         </is>
       </c>
       <c r="E148" s="11" t="inlineStr">
         <is>
-          <t>REST/gRPC定价API，支持横向扩展，p99&lt;100ms</t>
+          <t>隐含波动率曲面，红利曲线，汇率曲线，Local Volatility曲面，波动率微笑校准</t>
         </is>
       </c>
       <c r="F148" s="11" t="inlineStr">
         <is>
-          <t>功能完整/边界测试/集成冒烟/性能基线</t>
-        </is>
-      </c>
-      <c r="G148" s="23" t="inlineStr">
-        <is>
-          <t>高</t>
+          <t>p99延迟/误差率/精度验证/压测10k TPS</t>
+        </is>
+      </c>
+      <c r="G148" s="28" t="inlineStr">
+        <is>
+          <t>极高</t>
         </is>
       </c>
       <c r="H148" s="13" t="n">
-        <v>40</v>
+        <v>50</v>
       </c>
     </row>
     <row r="149" ht="28" customHeight="1">
@@ -9635,12 +10365,12 @@
       </c>
       <c r="D149" s="27" t="inlineStr">
         <is>
-          <t>历史估值回测</t>
+          <t>市场数据管理</t>
         </is>
       </c>
       <c r="E149" s="11" t="inlineStr">
         <is>
-          <t>基于历史行情重放定价误差分析，模型验证框架</t>
+          <t>境内外权益/债券/外汇/商品资讯统一接入，数据清洗，异常值处理，数据质量监控</t>
         </is>
       </c>
       <c r="F149" s="11" t="inlineStr">
@@ -9657,17 +10387,50 @@
         <v>30</v>
       </c>
     </row>
-    <row r="150" ht="20" customHeight="1">
-      <c r="A150" s="26" t="inlineStr">
-        <is>
-          <t>【P2】 销售交易  (Sales Trading)</t>
-        </is>
+    <row r="150" ht="28" customHeight="1">
+      <c r="A150" s="11" t="inlineStr">
+        <is>
+          <t>定价平台</t>
+        </is>
+      </c>
+      <c r="B150" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="C150" s="10" t="inlineStr">
+        <is>
+          <t>F09-07</t>
+        </is>
+      </c>
+      <c r="D150" s="27" t="inlineStr">
+        <is>
+          <t>蒙特卡洛求解器</t>
+        </is>
+      </c>
+      <c r="E150" s="11" t="inlineStr">
+        <is>
+          <t>GPU加速MC，QMC低差异序列，支持路径相关期权定价，并行情景模拟</t>
+        </is>
+      </c>
+      <c r="F150" s="11" t="inlineStr">
+        <is>
+          <t>p99延迟/误差率/精度验证/压测10k TPS</t>
+        </is>
+      </c>
+      <c r="G150" s="28" t="inlineStr">
+        <is>
+          <t>极高</t>
+        </is>
+      </c>
+      <c r="H150" s="13" t="n">
+        <v>70</v>
       </c>
     </row>
     <row r="151" ht="28" customHeight="1">
       <c r="A151" s="11" t="inlineStr">
         <is>
-          <t>销售交易</t>
+          <t>定价平台</t>
         </is>
       </c>
       <c r="B151" s="10" t="inlineStr">
@@ -9677,37 +10440,37 @@
       </c>
       <c r="C151" s="10" t="inlineStr">
         <is>
-          <t>F10-01</t>
+          <t>F09-08</t>
         </is>
       </c>
       <c r="D151" s="27" t="inlineStr">
         <is>
-          <t>销交工作台</t>
+          <t>解析解与数值解</t>
         </is>
       </c>
       <c r="E151" s="11" t="inlineStr">
         <is>
-          <t>报价管理主界面，历史报价管理，当日报价快捷操作，导入/导出报价，一键unrefer操作</t>
+          <t>Black-Scholes解析解，Hull-White利率模型，SABR波动率模型，二叉树/三叉树数值解</t>
         </is>
       </c>
       <c r="F151" s="11" t="inlineStr">
         <is>
-          <t>功能测试通过/正确率100%</t>
-        </is>
-      </c>
-      <c r="G151" s="24" t="inlineStr">
-        <is>
-          <t>中</t>
+          <t>p99延迟/误差率/精度验证/压测10k TPS</t>
+        </is>
+      </c>
+      <c r="G151" s="28" t="inlineStr">
+        <is>
+          <t>极高</t>
         </is>
       </c>
       <c r="H151" s="13" t="n">
-        <v>20</v>
+        <v>60</v>
       </c>
     </row>
     <row r="152" ht="28" customHeight="1">
       <c r="A152" s="11" t="inlineStr">
         <is>
-          <t>销售交易</t>
+          <t>定价平台</t>
         </is>
       </c>
       <c r="B152" s="10" t="inlineStr">
@@ -9717,37 +10480,37 @@
       </c>
       <c r="C152" s="10" t="inlineStr">
         <is>
-          <t>F10-02</t>
+          <t>F09-09</t>
         </is>
       </c>
       <c r="D152" s="27" t="inlineStr">
         <is>
-          <t>债券过滤与筛选</t>
+          <t>有限差分（PDE）</t>
         </is>
       </c>
       <c r="E152" s="11" t="inlineStr">
         <is>
-          <t>信用债/利率债过滤，信用债全品种过滤，利率债国债/证金债/地方债分类过滤，精确与模糊识别</t>
+          <t>Crank-Nicolson/ADI方法，含权债/可转债精确定价，局部波动率模型数值解</t>
         </is>
       </c>
       <c r="F152" s="11" t="inlineStr">
         <is>
-          <t>功能测试通过</t>
-        </is>
-      </c>
-      <c r="G152" s="25" t="inlineStr">
-        <is>
-          <t>低</t>
+          <t>p99延迟/误差率/精度验证/压测10k TPS</t>
+        </is>
+      </c>
+      <c r="G152" s="28" t="inlineStr">
+        <is>
+          <t>极高</t>
         </is>
       </c>
       <c r="H152" s="13" t="n">
-        <v>10</v>
+        <v>60</v>
       </c>
     </row>
     <row r="153" ht="28" customHeight="1">
       <c r="A153" s="11" t="inlineStr">
         <is>
-          <t>销售交易</t>
+          <t>定价平台</t>
         </is>
       </c>
       <c r="B153" s="10" t="inlineStr">
@@ -9757,37 +10520,37 @@
       </c>
       <c r="C153" s="10" t="inlineStr">
         <is>
-          <t>F10-03</t>
+          <t>F09-10</t>
         </is>
       </c>
       <c r="D153" s="27" t="inlineStr">
         <is>
-          <t>报价撮合与对价</t>
+          <t>实时Greeks计算</t>
         </is>
       </c>
       <c r="E153" s="11" t="inlineStr">
         <is>
-          <t>报价展示（对价/最优报价），撮合对价，报价提醒，交易包管理，报价成交确认</t>
+          <t>Delta/Gamma/Vega/Theta/Rho分布式实时计算，DV01/CS01，分桶敏感度</t>
         </is>
       </c>
       <c r="F153" s="11" t="inlineStr">
         <is>
-          <t>功能测试通过/正确率100%</t>
-        </is>
-      </c>
-      <c r="G153" s="24" t="inlineStr">
-        <is>
-          <t>中</t>
+          <t>功能完整/边界测试/集成冒烟/性能基线</t>
+        </is>
+      </c>
+      <c r="G153" s="23" t="inlineStr">
+        <is>
+          <t>高</t>
         </is>
       </c>
       <c r="H153" s="13" t="n">
-        <v>20</v>
+        <v>40</v>
       </c>
     </row>
     <row r="154" ht="28" customHeight="1">
       <c r="A154" s="11" t="inlineStr">
         <is>
-          <t>销售交易</t>
+          <t>定价平台</t>
         </is>
       </c>
       <c r="B154" s="10" t="inlineStr">
@@ -9797,37 +10560,37 @@
       </c>
       <c r="C154" s="10" t="inlineStr">
         <is>
-          <t>F10-04</t>
+          <t>F09-11</t>
         </is>
       </c>
       <c r="D154" s="27" t="inlineStr">
         <is>
-          <t>交易执行与审批</t>
+          <t>估值与结算计算</t>
         </is>
       </c>
       <c r="E154" s="11" t="inlineStr">
         <is>
-          <t>意向达成，交易要素校验，手工价录入，业务审批流程，交易执行</t>
+          <t>日终估值，盯市计算，保证金计算，结算价格，历史估值回测与误差分析</t>
         </is>
       </c>
       <c r="F154" s="11" t="inlineStr">
         <is>
-          <t>功能测试通过/正确率100%</t>
-        </is>
-      </c>
-      <c r="G154" s="24" t="inlineStr">
-        <is>
-          <t>中</t>
+          <t>功能完整/边界测试/集成冒烟/性能基线</t>
+        </is>
+      </c>
+      <c r="G154" s="23" t="inlineStr">
+        <is>
+          <t>高</t>
         </is>
       </c>
       <c r="H154" s="13" t="n">
-        <v>15</v>
+        <v>40</v>
       </c>
     </row>
     <row r="155" ht="28" customHeight="1">
       <c r="A155" s="11" t="inlineStr">
         <is>
-          <t>销售交易</t>
+          <t>定价平台</t>
         </is>
       </c>
       <c r="B155" s="10" t="inlineStr">
@@ -9837,37 +10600,37 @@
       </c>
       <c r="C155" s="10" t="inlineStr">
         <is>
-          <t>F10-05</t>
+          <t>F09-12</t>
         </is>
       </c>
       <c r="D155" s="27" t="inlineStr">
         <is>
-          <t>风控检查</t>
+          <t>风控与情景计算</t>
         </is>
       </c>
       <c r="E155" s="11" t="inlineStr">
         <is>
-          <t>交易前风控规则校验，限额检查，合规拦截，风控记录留痕</t>
+          <t>风险计量（VaR/压力测试）调用，情景分析，保证金计算，为风控平台提供统一定价接口</t>
         </is>
       </c>
       <c r="F155" s="11" t="inlineStr">
         <is>
-          <t>功能测试通过/正确率100%</t>
-        </is>
-      </c>
-      <c r="G155" s="24" t="inlineStr">
-        <is>
-          <t>中</t>
+          <t>功能完整/边界测试/集成冒烟/性能基线</t>
+        </is>
+      </c>
+      <c r="G155" s="23" t="inlineStr">
+        <is>
+          <t>高</t>
         </is>
       </c>
       <c r="H155" s="13" t="n">
-        <v>15</v>
+        <v>35</v>
       </c>
     </row>
     <row r="156" ht="28" customHeight="1">
       <c r="A156" s="11" t="inlineStr">
         <is>
-          <t>销售交易</t>
+          <t>定价平台</t>
         </is>
       </c>
       <c r="B156" s="10" t="inlineStr">
@@ -9877,17 +10640,17 @@
       </c>
       <c r="C156" s="10" t="inlineStr">
         <is>
-          <t>F10-06</t>
+          <t>F09-13</t>
         </is>
       </c>
       <c r="D156" s="27" t="inlineStr">
         <is>
-          <t>智能推荐系统</t>
+          <t>客需报价服务</t>
         </is>
       </c>
       <c r="E156" s="11" t="inlineStr">
         <is>
-          <t>从被动客户服务转向主动服务，基于客户画像与持仓分析智能推荐券种，提升客户响应效率</t>
+          <t>为销售交易/TRS系统提供实时报价，一站式报价接口，支持结构化产品定制化快速报价</t>
         </is>
       </c>
       <c r="F156" s="11" t="inlineStr">
@@ -9901,20 +10664,53 @@
         </is>
       </c>
       <c r="H156" s="13" t="n">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="157" ht="20" customHeight="1">
-      <c r="A157" s="26" t="inlineStr">
-        <is>
-          <t>【P2】 信用债/信用衍生品  (Credit &amp; CDS)</t>
-        </is>
+        <v>35</v>
+      </c>
+    </row>
+    <row r="157" ht="28" customHeight="1">
+      <c r="A157" s="11" t="inlineStr">
+        <is>
+          <t>定价平台</t>
+        </is>
+      </c>
+      <c r="B157" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="C157" s="10" t="inlineStr">
+        <is>
+          <t>F09-14</t>
+        </is>
+      </c>
+      <c r="D157" s="27" t="inlineStr">
+        <is>
+          <t>定价微服务架构</t>
+        </is>
+      </c>
+      <c r="E157" s="11" t="inlineStr">
+        <is>
+          <t>REST/gRPC定价API，横向弹性扩容，p99&lt;100ms，模型插件化注册，版本管理</t>
+        </is>
+      </c>
+      <c r="F157" s="11" t="inlineStr">
+        <is>
+          <t>功能完整/边界测试/集成冒烟/性能基线</t>
+        </is>
+      </c>
+      <c r="G157" s="23" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="H157" s="13" t="n">
+        <v>40</v>
       </c>
     </row>
     <row r="158" ht="28" customHeight="1">
       <c r="A158" s="11" t="inlineStr">
         <is>
-          <t>信用债/信用衍生品</t>
+          <t>定价平台</t>
         </is>
       </c>
       <c r="B158" s="10" t="inlineStr">
@@ -9924,17 +10720,17 @@
       </c>
       <c r="C158" s="10" t="inlineStr">
         <is>
-          <t>F11-01</t>
+          <t>F09-15</t>
         </is>
       </c>
       <c r="D158" s="27" t="inlineStr">
         <is>
-          <t>信用利差分析</t>
+          <t>灵活二次开发能力</t>
         </is>
       </c>
       <c r="E158" s="11" t="inlineStr">
         <is>
-          <t>行业/评级/期限信用利差曲线实时计算，历史分位数分析</t>
+          <t>全平台级/单功能模块级/系统框架级可扩展，支持自定义模型接入，策略团队自助扩展</t>
         </is>
       </c>
       <c r="F158" s="11" t="inlineStr">
@@ -9951,50 +10747,17 @@
         <v>30</v>
       </c>
     </row>
-    <row r="159" ht="28" customHeight="1">
-      <c r="A159" s="11" t="inlineStr">
-        <is>
-          <t>信用债/信用衍生品</t>
-        </is>
-      </c>
-      <c r="B159" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
-        </is>
-      </c>
-      <c r="C159" s="10" t="inlineStr">
-        <is>
-          <t>F11-02</t>
-        </is>
-      </c>
-      <c r="D159" s="27" t="inlineStr">
-        <is>
-          <t>CDS/CLN定价</t>
-        </is>
-      </c>
-      <c r="E159" s="11" t="inlineStr">
-        <is>
-          <t>信用违约互换定价，ISDA标准，生存概率曲线校准</t>
-        </is>
-      </c>
-      <c r="F159" s="11" t="inlineStr">
-        <is>
-          <t>p99延迟/误差率/精度验证/压测10k TPS</t>
-        </is>
-      </c>
-      <c r="G159" s="28" t="inlineStr">
-        <is>
-          <t>极高</t>
-        </is>
-      </c>
-      <c r="H159" s="13" t="n">
-        <v>50</v>
+    <row r="159" ht="20" customHeight="1">
+      <c r="A159" s="26" t="inlineStr">
+        <is>
+          <t>【P2】 销售交易  (Sales Trading)</t>
+        </is>
       </c>
     </row>
     <row r="160" ht="28" customHeight="1">
       <c r="A160" s="11" t="inlineStr">
         <is>
-          <t>信用债/信用衍生品</t>
+          <t>销售交易</t>
         </is>
       </c>
       <c r="B160" s="10" t="inlineStr">
@@ -10004,17 +10767,17 @@
       </c>
       <c r="C160" s="10" t="inlineStr">
         <is>
-          <t>F11-03</t>
+          <t>F10-01</t>
         </is>
       </c>
       <c r="D160" s="27" t="inlineStr">
         <is>
-          <t>信用评级动态监控</t>
+          <t>销交工作台</t>
         </is>
       </c>
       <c r="E160" s="11" t="inlineStr">
         <is>
-          <t>对接外部评级机构（中诚信/联合/大公），评级下调预警</t>
+          <t>报价管理主界面，历史报价管理，当日报价快捷操作，导入/导出报价，一键unrefer操作</t>
         </is>
       </c>
       <c r="F160" s="11" t="inlineStr">
@@ -10034,7 +10797,7 @@
     <row r="161" ht="28" customHeight="1">
       <c r="A161" s="11" t="inlineStr">
         <is>
-          <t>信用债/信用衍生品</t>
+          <t>销售交易</t>
         </is>
       </c>
       <c r="B161" s="10" t="inlineStr">
@@ -10044,37 +10807,37 @@
       </c>
       <c r="C161" s="10" t="inlineStr">
         <is>
-          <t>F11-04</t>
+          <t>F10-02</t>
         </is>
       </c>
       <c r="D161" s="27" t="inlineStr">
         <is>
-          <t>违约概率（PD）建模</t>
+          <t>债券过滤与筛选</t>
         </is>
       </c>
       <c r="E161" s="11" t="inlineStr">
         <is>
-          <t>结构化Merton模型+市场隐含PD，信用风险计量</t>
+          <t>信用债/利率债过滤，信用债全品种过滤，利率债国债/证金债/地方债分类过滤，精确与模糊识别</t>
         </is>
       </c>
       <c r="F161" s="11" t="inlineStr">
         <is>
-          <t>功能完整/边界测试/集成冒烟/性能基线</t>
-        </is>
-      </c>
-      <c r="G161" s="23" t="inlineStr">
-        <is>
-          <t>高</t>
+          <t>功能测试通过</t>
+        </is>
+      </c>
+      <c r="G161" s="25" t="inlineStr">
+        <is>
+          <t>低</t>
         </is>
       </c>
       <c r="H161" s="13" t="n">
-        <v>40</v>
+        <v>10</v>
       </c>
     </row>
     <row r="162" ht="28" customHeight="1">
       <c r="A162" s="11" t="inlineStr">
         <is>
-          <t>信用债/信用衍生品</t>
+          <t>销售交易</t>
         </is>
       </c>
       <c r="B162" s="10" t="inlineStr">
@@ -10084,17 +10847,17 @@
       </c>
       <c r="C162" s="10" t="inlineStr">
         <is>
-          <t>F11-05</t>
+          <t>F10-03</t>
         </is>
       </c>
       <c r="D162" s="27" t="inlineStr">
         <is>
-          <t>集中度限额管理</t>
+          <t>报价撮合与对价</t>
         </is>
       </c>
       <c r="E162" s="11" t="inlineStr">
         <is>
-          <t>行业/发行人/评级集中度多维限额，超限预警</t>
+          <t>报价展示（对价/最优报价），撮合对价，报价提醒，交易包管理，报价成交确认</t>
         </is>
       </c>
       <c r="F162" s="11" t="inlineStr">
@@ -10111,17 +10874,50 @@
         <v>20</v>
       </c>
     </row>
-    <row r="163" ht="20" customHeight="1">
-      <c r="A163" s="26" t="inlineStr">
-        <is>
-          <t>【P2】 投顾服务  (Investment Advisory)</t>
-        </is>
+    <row r="163" ht="28" customHeight="1">
+      <c r="A163" s="11" t="inlineStr">
+        <is>
+          <t>销售交易</t>
+        </is>
+      </c>
+      <c r="B163" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="C163" s="10" t="inlineStr">
+        <is>
+          <t>F10-04</t>
+        </is>
+      </c>
+      <c r="D163" s="27" t="inlineStr">
+        <is>
+          <t>交易执行与审批</t>
+        </is>
+      </c>
+      <c r="E163" s="11" t="inlineStr">
+        <is>
+          <t>意向达成，交易要素校验，手工价录入，业务审批流程，交易执行</t>
+        </is>
+      </c>
+      <c r="F163" s="11" t="inlineStr">
+        <is>
+          <t>功能测试通过/正确率100%</t>
+        </is>
+      </c>
+      <c r="G163" s="24" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="H163" s="13" t="n">
+        <v>15</v>
       </c>
     </row>
     <row r="164" ht="28" customHeight="1">
       <c r="A164" s="11" t="inlineStr">
         <is>
-          <t>投顾服务</t>
+          <t>销售交易</t>
         </is>
       </c>
       <c r="B164" s="10" t="inlineStr">
@@ -10131,17 +10927,17 @@
       </c>
       <c r="C164" s="10" t="inlineStr">
         <is>
-          <t>F12-01</t>
+          <t>F10-05</t>
         </is>
       </c>
       <c r="D164" s="27" t="inlineStr">
         <is>
-          <t>投顾工作台</t>
+          <t>风控检查</t>
         </is>
       </c>
       <c r="E164" s="11" t="inlineStr">
         <is>
-          <t>投顾人员操作界面，管理客户委托，上传研究报告，发送投资建议，查看客户反馈</t>
+          <t>交易前风控规则校验，限额检查，合规拦截，风控记录留痕</t>
         </is>
       </c>
       <c r="F164" s="11" t="inlineStr">
@@ -10155,13 +10951,13 @@
         </is>
       </c>
       <c r="H164" s="13" t="n">
-        <v>20</v>
+        <v>15</v>
       </c>
     </row>
     <row r="165" ht="28" customHeight="1">
       <c r="A165" s="11" t="inlineStr">
         <is>
-          <t>投顾服务</t>
+          <t>销售交易</t>
         </is>
       </c>
       <c r="B165" s="10" t="inlineStr">
@@ -10171,77 +10967,44 @@
       </c>
       <c r="C165" s="10" t="inlineStr">
         <is>
-          <t>F12-02</t>
+          <t>F10-06</t>
         </is>
       </c>
       <c r="D165" s="27" t="inlineStr">
         <is>
-          <t>客户终端</t>
+          <t>智能推荐系统</t>
         </is>
       </c>
       <c r="E165" s="11" t="inlineStr">
         <is>
-          <t>客户查看投资建议与分析报告，确认交易服务，查看账户净值走势、持仓明细、交易明细</t>
+          <t>从被动客户服务转向主动服务，基于客户画像与持仓分析智能推荐券种，提升客户响应效率</t>
         </is>
       </c>
       <c r="F165" s="11" t="inlineStr">
         <is>
-          <t>功能测试通过/正确率100%</t>
-        </is>
-      </c>
-      <c r="G165" s="24" t="inlineStr">
-        <is>
-          <t>中</t>
+          <t>功能完整/边界测试/集成冒烟/性能基线</t>
+        </is>
+      </c>
+      <c r="G165" s="23" t="inlineStr">
+        <is>
+          <t>高</t>
         </is>
       </c>
       <c r="H165" s="13" t="n">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="166" ht="28" customHeight="1">
-      <c r="A166" s="11" t="inlineStr">
-        <is>
-          <t>投顾服务</t>
-        </is>
-      </c>
-      <c r="B166" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
-        </is>
-      </c>
-      <c r="C166" s="10" t="inlineStr">
-        <is>
-          <t>F12-03</t>
-        </is>
-      </c>
-      <c r="D166" s="27" t="inlineStr">
-        <is>
-          <t>投资建议书管理</t>
-        </is>
-      </c>
-      <c r="E166" s="11" t="inlineStr">
-        <is>
-          <t>投资建议书线上生成、审批、确认全流程，留痕追溯，客户电子签收</t>
-        </is>
-      </c>
-      <c r="F166" s="11" t="inlineStr">
-        <is>
-          <t>功能测试通过/正确率100%</t>
-        </is>
-      </c>
-      <c r="G166" s="24" t="inlineStr">
-        <is>
-          <t>中</t>
-        </is>
-      </c>
-      <c r="H166" s="13" t="n">
-        <v>15</v>
+        <v>25</v>
+      </c>
+    </row>
+    <row r="166" ht="20" customHeight="1">
+      <c r="A166" s="26" t="inlineStr">
+        <is>
+          <t>【P2】 信用债/信用衍生品  (Credit &amp; CDS)</t>
+        </is>
       </c>
     </row>
     <row r="167" ht="28" customHeight="1">
       <c r="A167" s="11" t="inlineStr">
         <is>
-          <t>投顾服务</t>
+          <t>信用债/信用衍生品</t>
         </is>
       </c>
       <c r="B167" s="10" t="inlineStr">
@@ -10251,17 +11014,17 @@
       </c>
       <c r="C167" s="10" t="inlineStr">
         <is>
-          <t>F12-04</t>
+          <t>F11-01</t>
         </is>
       </c>
       <c r="D167" s="27" t="inlineStr">
         <is>
-          <t>账户分析报告</t>
+          <t>信用利差分析</t>
         </is>
       </c>
       <c r="E167" s="11" t="inlineStr">
         <is>
-          <t>账户净值走势、久期走势、归因分析、估值台账等核心数据展示及定期报告生成</t>
+          <t>行业/评级/期限信用利差曲线实时计算，历史分位数分析</t>
         </is>
       </c>
       <c r="F167" s="11" t="inlineStr">
@@ -10275,13 +11038,13 @@
         </is>
       </c>
       <c r="H167" s="13" t="n">
-        <v>25</v>
+        <v>30</v>
       </c>
     </row>
     <row r="168" ht="28" customHeight="1">
       <c r="A168" s="11" t="inlineStr">
         <is>
-          <t>投顾服务</t>
+          <t>信用债/信用衍生品</t>
         </is>
       </c>
       <c r="B168" s="10" t="inlineStr">
@@ -10291,37 +11054,37 @@
       </c>
       <c r="C168" s="10" t="inlineStr">
         <is>
-          <t>F12-05</t>
+          <t>F11-02</t>
         </is>
       </c>
       <c r="D168" s="27" t="inlineStr">
         <is>
-          <t>投研报告服务</t>
+          <t>CDS/CLN定价</t>
         </is>
       </c>
       <c r="E168" s="11" t="inlineStr">
         <is>
-          <t>日/周/月研究报告上传与推送，RPA自动获取基础数据，报告分类管理</t>
+          <t>信用违约互换定价，ISDA标准，生存概率曲线校准</t>
         </is>
       </c>
       <c r="F168" s="11" t="inlineStr">
         <is>
-          <t>功能测试通过/正确率100%</t>
-        </is>
-      </c>
-      <c r="G168" s="24" t="inlineStr">
-        <is>
-          <t>中</t>
+          <t>p99延迟/误差率/精度验证/压测10k TPS</t>
+        </is>
+      </c>
+      <c r="G168" s="28" t="inlineStr">
+        <is>
+          <t>极高</t>
         </is>
       </c>
       <c r="H168" s="13" t="n">
-        <v>15</v>
+        <v>50</v>
       </c>
     </row>
     <row r="169" ht="28" customHeight="1">
       <c r="A169" s="11" t="inlineStr">
         <is>
-          <t>投顾服务</t>
+          <t>信用债/信用衍生品</t>
         </is>
       </c>
       <c r="B169" s="10" t="inlineStr">
@@ -10331,44 +11094,77 @@
       </c>
       <c r="C169" s="10" t="inlineStr">
         <is>
-          <t>F12-06</t>
+          <t>F11-03</t>
         </is>
       </c>
       <c r="D169" s="27" t="inlineStr">
         <is>
-          <t>客户服务与基础服务</t>
+          <t>信用评级动态监控</t>
         </is>
       </c>
       <c r="E169" s="11" t="inlineStr">
         <is>
-          <t>服务中心、消息中心、问卷系统；用户/账户/数据管理，消息群发，登录注册</t>
+          <t>对接外部评级机构（中诚信/联合/大公），评级下调预警</t>
         </is>
       </c>
       <c r="F169" s="11" t="inlineStr">
         <is>
-          <t>功能测试通过</t>
-        </is>
-      </c>
-      <c r="G169" s="25" t="inlineStr">
-        <is>
-          <t>低</t>
+          <t>功能测试通过/正确率100%</t>
+        </is>
+      </c>
+      <c r="G169" s="24" t="inlineStr">
+        <is>
+          <t>中</t>
         </is>
       </c>
       <c r="H169" s="13" t="n">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="170" ht="20" customHeight="1">
-      <c r="A170" s="26" t="inlineStr">
-        <is>
-          <t>【P2】 TRS收益互换  (Total Return Swap)</t>
-        </is>
+        <v>20</v>
+      </c>
+    </row>
+    <row r="170" ht="28" customHeight="1">
+      <c r="A170" s="11" t="inlineStr">
+        <is>
+          <t>信用债/信用衍生品</t>
+        </is>
+      </c>
+      <c r="B170" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="C170" s="10" t="inlineStr">
+        <is>
+          <t>F11-04</t>
+        </is>
+      </c>
+      <c r="D170" s="27" t="inlineStr">
+        <is>
+          <t>违约概率（PD）建模</t>
+        </is>
+      </c>
+      <c r="E170" s="11" t="inlineStr">
+        <is>
+          <t>结构化Merton模型+市场隐含PD，信用风险计量</t>
+        </is>
+      </c>
+      <c r="F170" s="11" t="inlineStr">
+        <is>
+          <t>功能完整/边界测试/集成冒烟/性能基线</t>
+        </is>
+      </c>
+      <c r="G170" s="23" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="H170" s="13" t="n">
+        <v>40</v>
       </c>
     </row>
     <row r="171" ht="28" customHeight="1">
       <c r="A171" s="11" t="inlineStr">
         <is>
-          <t>TRS收益互换</t>
+          <t>信用债/信用衍生品</t>
         </is>
       </c>
       <c r="B171" s="10" t="inlineStr">
@@ -10378,77 +11174,44 @@
       </c>
       <c r="C171" s="10" t="inlineStr">
         <is>
-          <t>F13-01</t>
+          <t>F11-05</t>
         </is>
       </c>
       <c r="D171" s="27" t="inlineStr">
         <is>
-          <t>TRS交易端</t>
+          <t>集中度限额管理</t>
         </is>
       </c>
       <c r="E171" s="11" t="inlineStr">
         <is>
-          <t>报价提供，成交回报，对冲委托与自动对冲，请求报价，行情与资讯，历史确认</t>
+          <t>行业/发行人/评级集中度多维限额，超限预警</t>
         </is>
       </c>
       <c r="F171" s="11" t="inlineStr">
         <is>
-          <t>功能完整/边界测试/集成冒烟/性能基线</t>
-        </is>
-      </c>
-      <c r="G171" s="23" t="inlineStr">
-        <is>
-          <t>高</t>
+          <t>功能测试通过/正确率100%</t>
+        </is>
+      </c>
+      <c r="G171" s="24" t="inlineStr">
+        <is>
+          <t>中</t>
         </is>
       </c>
       <c r="H171" s="13" t="n">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="172" ht="28" customHeight="1">
-      <c r="A172" s="11" t="inlineStr">
-        <is>
-          <t>TRS收益互换</t>
-        </is>
-      </c>
-      <c r="B172" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
-        </is>
-      </c>
-      <c r="C172" s="10" t="inlineStr">
-        <is>
-          <t>F13-02</t>
-        </is>
-      </c>
-      <c r="D172" s="27" t="inlineStr">
-        <is>
-          <t>TRS客户端</t>
-        </is>
-      </c>
-      <c r="E172" s="11" t="inlineStr">
-        <is>
-          <t>开户申请，客户委托，出入金申请，合约持仓，标的持仓，资金管理，行情矩阵，自主下单</t>
-        </is>
-      </c>
-      <c r="F172" s="11" t="inlineStr">
-        <is>
-          <t>功能完整/边界测试/集成冒烟/性能基线</t>
-        </is>
-      </c>
-      <c r="G172" s="23" t="inlineStr">
-        <is>
-          <t>高</t>
-        </is>
-      </c>
-      <c r="H172" s="13" t="n">
-        <v>25</v>
+        <v>20</v>
+      </c>
+    </row>
+    <row r="172" ht="20" customHeight="1">
+      <c r="A172" s="26" t="inlineStr">
+        <is>
+          <t>【P2】 投顾服务  (Investment Advisory)</t>
+        </is>
       </c>
     </row>
     <row r="173" ht="28" customHeight="1">
       <c r="A173" s="11" t="inlineStr">
         <is>
-          <t>TRS收益互换</t>
+          <t>投顾服务</t>
         </is>
       </c>
       <c r="B173" s="10" t="inlineStr">
@@ -10458,17 +11221,17 @@
       </c>
       <c r="C173" s="10" t="inlineStr">
         <is>
-          <t>F13-03</t>
+          <t>F12-01</t>
         </is>
       </c>
       <c r="D173" s="27" t="inlineStr">
         <is>
-          <t>TRS管理端</t>
+          <t>投顾工作台</t>
         </is>
       </c>
       <c r="E173" s="11" t="inlineStr">
         <is>
-          <t>开户申请审批，合约成交管理，出入金审批，运营管理，对账，库存，对冲录入</t>
+          <t>投顾人员操作界面，管理客户委托，上传研究报告，发送投资建议，查看客户反馈</t>
         </is>
       </c>
       <c r="F173" s="11" t="inlineStr">
@@ -10488,7 +11251,7 @@
     <row r="174" ht="28" customHeight="1">
       <c r="A174" s="11" t="inlineStr">
         <is>
-          <t>TRS收益互换</t>
+          <t>投顾服务</t>
         </is>
       </c>
       <c r="B174" s="10" t="inlineStr">
@@ -10498,37 +11261,37 @@
       </c>
       <c r="C174" s="10" t="inlineStr">
         <is>
-          <t>F13-04</t>
+          <t>F12-02</t>
         </is>
       </c>
       <c r="D174" s="27" t="inlineStr">
         <is>
-          <t>自动对冲</t>
+          <t>客户终端</t>
         </is>
       </c>
       <c r="E174" s="11" t="inlineStr">
         <is>
-          <t>对冲委托自动触发，对冲回报处理，风险校验，组合重叠分析，开平仓设置</t>
+          <t>客户查看投资建议与分析报告，确认交易服务，查看账户净值走势、持仓明细、交易明细</t>
         </is>
       </c>
       <c r="F174" s="11" t="inlineStr">
         <is>
-          <t>功能完整/边界测试/集成冒烟/性能基线</t>
-        </is>
-      </c>
-      <c r="G174" s="23" t="inlineStr">
-        <is>
-          <t>高</t>
+          <t>功能测试通过/正确率100%</t>
+        </is>
+      </c>
+      <c r="G174" s="24" t="inlineStr">
+        <is>
+          <t>中</t>
         </is>
       </c>
       <c r="H174" s="13" t="n">
-        <v>25</v>
+        <v>20</v>
       </c>
     </row>
     <row r="175" ht="28" customHeight="1">
       <c r="A175" s="11" t="inlineStr">
         <is>
-          <t>TRS收益互换</t>
+          <t>投顾服务</t>
         </is>
       </c>
       <c r="B175" s="10" t="inlineStr">
@@ -10538,17 +11301,17 @@
       </c>
       <c r="C175" s="10" t="inlineStr">
         <is>
-          <t>F13-05</t>
+          <t>F12-03</t>
         </is>
       </c>
       <c r="D175" s="27" t="inlineStr">
         <is>
-          <t>通知与确认文件</t>
+          <t>投资建议书管理</t>
         </is>
       </c>
       <c r="E175" s="11" t="inlineStr">
         <is>
-          <t>企微通知提醒，确认书/结算单/估值报告/出入金通知自动生成并通过邮箱发送</t>
+          <t>投资建议书线上生成、审批、确认全流程，留痕追溯，客户电子签收</t>
         </is>
       </c>
       <c r="F175" s="11" t="inlineStr">
@@ -10568,7 +11331,7 @@
     <row r="176" ht="28" customHeight="1">
       <c r="A176" s="11" t="inlineStr">
         <is>
-          <t>TRS收益互换</t>
+          <t>投顾服务</t>
         </is>
       </c>
       <c r="B176" s="10" t="inlineStr">
@@ -10578,17 +11341,17 @@
       </c>
       <c r="C176" s="10" t="inlineStr">
         <is>
-          <t>F13-06</t>
+          <t>F12-04</t>
         </is>
       </c>
       <c r="D176" s="27" t="inlineStr">
         <is>
-          <t>系统集成</t>
+          <t>账户分析报告</t>
         </is>
       </c>
       <c r="E176" s="11" t="inlineStr">
         <is>
-          <t>与衡泰系统客户信息同步，QTrade聊天记录同步，交易管理系统对接，银行流水对接</t>
+          <t>账户净值走势、久期走势、归因分析、估值台账等核心数据展示及定期报告生成</t>
         </is>
       </c>
       <c r="F176" s="11" t="inlineStr">
@@ -10605,241 +11368,568 @@
         <v>25</v>
       </c>
     </row>
-    <row r="177" ht="20" customHeight="1">
-      <c r="A177" s="29" t="inlineStr">
+    <row r="177" ht="28" customHeight="1">
+      <c r="A177" s="11" t="inlineStr">
+        <is>
+          <t>投顾服务</t>
+        </is>
+      </c>
+      <c r="B177" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="C177" s="10" t="inlineStr">
+        <is>
+          <t>F12-05</t>
+        </is>
+      </c>
+      <c r="D177" s="27" t="inlineStr">
+        <is>
+          <t>投研报告服务</t>
+        </is>
+      </c>
+      <c r="E177" s="11" t="inlineStr">
+        <is>
+          <t>日/周/月研究报告上传与推送，RPA自动获取基础数据，报告分类管理</t>
+        </is>
+      </c>
+      <c r="F177" s="11" t="inlineStr">
+        <is>
+          <t>功能测试通过/正确率100%</t>
+        </is>
+      </c>
+      <c r="G177" s="24" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="H177" s="13" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="178" ht="28" customHeight="1">
+      <c r="A178" s="11" t="inlineStr">
+        <is>
+          <t>投顾服务</t>
+        </is>
+      </c>
+      <c r="B178" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="C178" s="10" t="inlineStr">
+        <is>
+          <t>F12-06</t>
+        </is>
+      </c>
+      <c r="D178" s="27" t="inlineStr">
+        <is>
+          <t>客户服务与基础服务</t>
+        </is>
+      </c>
+      <c r="E178" s="11" t="inlineStr">
+        <is>
+          <t>服务中心、消息中心、问卷系统；用户/账户/数据管理，消息群发，登录注册</t>
+        </is>
+      </c>
+      <c r="F178" s="11" t="inlineStr">
+        <is>
+          <t>功能测试通过</t>
+        </is>
+      </c>
+      <c r="G178" s="25" t="inlineStr">
+        <is>
+          <t>低</t>
+        </is>
+      </c>
+      <c r="H178" s="13" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="179" ht="20" customHeight="1">
+      <c r="A179" s="26" t="inlineStr">
+        <is>
+          <t>【P2】 TRS收益互换  (Total Return Swap)</t>
+        </is>
+      </c>
+    </row>
+    <row r="180" ht="28" customHeight="1">
+      <c r="A180" s="11" t="inlineStr">
+        <is>
+          <t>TRS收益互换</t>
+        </is>
+      </c>
+      <c r="B180" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="C180" s="10" t="inlineStr">
+        <is>
+          <t>F13-01</t>
+        </is>
+      </c>
+      <c r="D180" s="27" t="inlineStr">
+        <is>
+          <t>TRS交易端</t>
+        </is>
+      </c>
+      <c r="E180" s="11" t="inlineStr">
+        <is>
+          <t>报价提供，成交回报，对冲委托与自动对冲，请求报价，行情与资讯，历史确认</t>
+        </is>
+      </c>
+      <c r="F180" s="11" t="inlineStr">
+        <is>
+          <t>功能完整/边界测试/集成冒烟/性能基线</t>
+        </is>
+      </c>
+      <c r="G180" s="23" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="H180" s="13" t="n">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="181" ht="28" customHeight="1">
+      <c r="A181" s="11" t="inlineStr">
+        <is>
+          <t>TRS收益互换</t>
+        </is>
+      </c>
+      <c r="B181" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="C181" s="10" t="inlineStr">
+        <is>
+          <t>F13-02</t>
+        </is>
+      </c>
+      <c r="D181" s="27" t="inlineStr">
+        <is>
+          <t>TRS客户端</t>
+        </is>
+      </c>
+      <c r="E181" s="11" t="inlineStr">
+        <is>
+          <t>开户申请，客户委托，出入金申请，合约持仓，标的持仓，资金管理，行情矩阵，自主下单</t>
+        </is>
+      </c>
+      <c r="F181" s="11" t="inlineStr">
+        <is>
+          <t>功能完整/边界测试/集成冒烟/性能基线</t>
+        </is>
+      </c>
+      <c r="G181" s="23" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="H181" s="13" t="n">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="182" ht="28" customHeight="1">
+      <c r="A182" s="11" t="inlineStr">
+        <is>
+          <t>TRS收益互换</t>
+        </is>
+      </c>
+      <c r="B182" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="C182" s="10" t="inlineStr">
+        <is>
+          <t>F13-03</t>
+        </is>
+      </c>
+      <c r="D182" s="27" t="inlineStr">
+        <is>
+          <t>TRS管理端</t>
+        </is>
+      </c>
+      <c r="E182" s="11" t="inlineStr">
+        <is>
+          <t>开户申请审批，合约成交管理，出入金审批，运营管理，对账，库存，对冲录入</t>
+        </is>
+      </c>
+      <c r="F182" s="11" t="inlineStr">
+        <is>
+          <t>功能测试通过/正确率100%</t>
+        </is>
+      </c>
+      <c r="G182" s="24" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="H182" s="13" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="183" ht="28" customHeight="1">
+      <c r="A183" s="11" t="inlineStr">
+        <is>
+          <t>TRS收益互换</t>
+        </is>
+      </c>
+      <c r="B183" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="C183" s="10" t="inlineStr">
+        <is>
+          <t>F13-04</t>
+        </is>
+      </c>
+      <c r="D183" s="27" t="inlineStr">
+        <is>
+          <t>自动对冲</t>
+        </is>
+      </c>
+      <c r="E183" s="11" t="inlineStr">
+        <is>
+          <t>对冲委托自动触发，对冲回报处理，风险校验，组合重叠分析，开平仓设置</t>
+        </is>
+      </c>
+      <c r="F183" s="11" t="inlineStr">
+        <is>
+          <t>功能完整/边界测试/集成冒烟/性能基线</t>
+        </is>
+      </c>
+      <c r="G183" s="23" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="H183" s="13" t="n">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="184" ht="28" customHeight="1">
+      <c r="A184" s="11" t="inlineStr">
+        <is>
+          <t>TRS收益互换</t>
+        </is>
+      </c>
+      <c r="B184" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="C184" s="10" t="inlineStr">
+        <is>
+          <t>F13-05</t>
+        </is>
+      </c>
+      <c r="D184" s="27" t="inlineStr">
+        <is>
+          <t>通知与确认文件</t>
+        </is>
+      </c>
+      <c r="E184" s="11" t="inlineStr">
+        <is>
+          <t>企微通知提醒，确认书/结算单/估值报告/出入金通知自动生成并通过邮箱发送</t>
+        </is>
+      </c>
+      <c r="F184" s="11" t="inlineStr">
+        <is>
+          <t>功能测试通过/正确率100%</t>
+        </is>
+      </c>
+      <c r="G184" s="24" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="H184" s="13" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="185" ht="28" customHeight="1">
+      <c r="A185" s="11" t="inlineStr">
+        <is>
+          <t>TRS收益互换</t>
+        </is>
+      </c>
+      <c r="B185" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="C185" s="10" t="inlineStr">
+        <is>
+          <t>F13-06</t>
+        </is>
+      </c>
+      <c r="D185" s="27" t="inlineStr">
+        <is>
+          <t>系统集成</t>
+        </is>
+      </c>
+      <c r="E185" s="11" t="inlineStr">
+        <is>
+          <t>与衡泰系统客户信息同步，QTrade聊天记录同步，交易管理系统对接，银行流水对接</t>
+        </is>
+      </c>
+      <c r="F185" s="11" t="inlineStr">
+        <is>
+          <t>功能完整/边界测试/集成冒烟/性能基线</t>
+        </is>
+      </c>
+      <c r="G185" s="23" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="H185" s="13" t="n">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="186" ht="20" customHeight="1">
+      <c r="A186" s="29" t="inlineStr">
         <is>
           <t>【P3】 做市商系统  (Market Making)</t>
         </is>
       </c>
     </row>
-    <row r="178" ht="28" customHeight="1">
-      <c r="A178" s="16" t="inlineStr">
+    <row r="187" ht="28" customHeight="1">
+      <c r="A187" s="16" t="inlineStr">
         <is>
           <t>做市商系统</t>
         </is>
       </c>
-      <c r="B178" s="15" t="inlineStr">
+      <c r="B187" s="15" t="inlineStr">
         <is>
           <t>P3</t>
         </is>
       </c>
-      <c r="C178" s="15" t="inlineStr">
+      <c r="C187" s="15" t="inlineStr">
         <is>
           <t>F15-01</t>
         </is>
       </c>
-      <c r="D178" s="30" t="inlineStr">
+      <c r="D187" s="30" t="inlineStr">
         <is>
           <t>双边报价引擎</t>
         </is>
       </c>
-      <c r="E178" s="16" t="inlineStr">
+      <c r="E187" s="16" t="inlineStr">
         <is>
           <t>多品种同时双边报价，延迟&lt;5ms，报价宽度动态优化</t>
         </is>
       </c>
-      <c r="F178" s="16" t="inlineStr">
+      <c r="F187" s="16" t="inlineStr">
         <is>
           <t>p99延迟/误差率/精度验证/压测10k TPS</t>
         </is>
       </c>
-      <c r="G178" s="28" t="inlineStr">
+      <c r="G187" s="28" t="inlineStr">
         <is>
           <t>极高</t>
         </is>
       </c>
-      <c r="H178" s="18" t="n">
+      <c r="H187" s="18" t="n">
         <v>70</v>
       </c>
     </row>
-    <row r="179" ht="28" customHeight="1">
-      <c r="A179" s="16" t="inlineStr">
+    <row r="188" ht="28" customHeight="1">
+      <c r="A188" s="16" t="inlineStr">
         <is>
           <t>做市商系统</t>
         </is>
       </c>
-      <c r="B179" s="15" t="inlineStr">
+      <c r="B188" s="15" t="inlineStr">
         <is>
           <t>P3</t>
         </is>
       </c>
-      <c r="C179" s="15" t="inlineStr">
+      <c r="C188" s="15" t="inlineStr">
         <is>
           <t>F15-02</t>
         </is>
       </c>
-      <c r="D179" s="30" t="inlineStr">
+      <c r="D188" s="30" t="inlineStr">
         <is>
           <t>库存风险实时管理</t>
         </is>
       </c>
-      <c r="E179" s="16" t="inlineStr">
+      <c r="E188" s="16" t="inlineStr">
         <is>
           <t>做市库存PnL实时监控，Delta对冲自动触发</t>
         </is>
       </c>
-      <c r="F179" s="16" t="inlineStr">
+      <c r="F188" s="16" t="inlineStr">
         <is>
           <t>p99延迟/误差率/精度验证/压测10k TPS</t>
         </is>
       </c>
-      <c r="G179" s="28" t="inlineStr">
+      <c r="G188" s="28" t="inlineStr">
         <is>
           <t>极高</t>
         </is>
       </c>
-      <c r="H179" s="18" t="n">
+      <c r="H188" s="18" t="n">
         <v>60</v>
       </c>
     </row>
-    <row r="180" ht="28" customHeight="1">
-      <c r="A180" s="16" t="inlineStr">
+    <row r="189" ht="28" customHeight="1">
+      <c r="A189" s="16" t="inlineStr">
         <is>
           <t>做市商系统</t>
         </is>
       </c>
-      <c r="B180" s="15" t="inlineStr">
+      <c r="B189" s="15" t="inlineStr">
         <is>
           <t>P3</t>
         </is>
       </c>
-      <c r="C180" s="15" t="inlineStr">
+      <c r="C189" s="15" t="inlineStr">
         <is>
           <t>F15-03</t>
         </is>
       </c>
-      <c r="D180" s="30" t="inlineStr">
+      <c r="D189" s="30" t="inlineStr">
         <is>
           <t>报价优化算法</t>
         </is>
       </c>
-      <c r="E180" s="16" t="inlineStr">
+      <c r="E189" s="16" t="inlineStr">
         <is>
           <t>基于市场微结构理论动态调整bid-ask spread</t>
         </is>
       </c>
-      <c r="F180" s="16" t="inlineStr">
+      <c r="F189" s="16" t="inlineStr">
         <is>
           <t>p99延迟/误差率/精度验证/压测10k TPS</t>
         </is>
       </c>
-      <c r="G180" s="28" t="inlineStr">
+      <c r="G189" s="28" t="inlineStr">
         <is>
           <t>极高</t>
         </is>
       </c>
-      <c r="H180" s="18" t="n">
+      <c r="H189" s="18" t="n">
         <v>50</v>
       </c>
     </row>
-    <row r="181" ht="28" customHeight="1">
-      <c r="A181" s="16" t="inlineStr">
+    <row r="190" ht="28" customHeight="1">
+      <c r="A190" s="16" t="inlineStr">
         <is>
           <t>做市商系统</t>
         </is>
       </c>
-      <c r="B181" s="15" t="inlineStr">
+      <c r="B190" s="15" t="inlineStr">
         <is>
           <t>P3</t>
         </is>
       </c>
-      <c r="C181" s="15" t="inlineStr">
+      <c r="C190" s="15" t="inlineStr">
         <is>
           <t>F15-04</t>
         </is>
       </c>
-      <c r="D181" s="30" t="inlineStr">
+      <c r="D190" s="30" t="inlineStr">
         <is>
           <t>竞争力分析</t>
         </is>
       </c>
-      <c r="E181" s="16" t="inlineStr">
+      <c r="E190" s="16" t="inlineStr">
         <is>
           <t>与市场最优报价对比，中签率分析，策略调优</t>
         </is>
       </c>
-      <c r="F181" s="16" t="inlineStr">
+      <c r="F190" s="16" t="inlineStr">
         <is>
           <t>功能完整/边界测试/集成冒烟/性能基线</t>
         </is>
       </c>
-      <c r="G181" s="23" t="inlineStr">
+      <c r="G190" s="23" t="inlineStr">
         <is>
           <t>高</t>
         </is>
       </c>
-      <c r="H181" s="18" t="n">
+      <c r="H190" s="18" t="n">
         <v>25</v>
       </c>
     </row>
-    <row r="182" ht="28" customHeight="1">
-      <c r="A182" s="16" t="inlineStr">
+    <row r="191" ht="28" customHeight="1">
+      <c r="A191" s="16" t="inlineStr">
         <is>
           <t>做市商系统</t>
         </is>
       </c>
-      <c r="B182" s="15" t="inlineStr">
+      <c r="B191" s="15" t="inlineStr">
         <is>
           <t>P3</t>
         </is>
       </c>
-      <c r="C182" s="15" t="inlineStr">
+      <c r="C191" s="15" t="inlineStr">
         <is>
           <t>F15-05</t>
         </is>
       </c>
-      <c r="D182" s="30" t="inlineStr">
+      <c r="D191" s="30" t="inlineStr">
         <is>
           <t>交易对手管理集成</t>
         </is>
       </c>
-      <c r="E182" s="16" t="inlineStr">
+      <c r="E191" s="16" t="inlineStr">
         <is>
           <t>做市交易对手信用实时检查，额度占用同步更新</t>
         </is>
       </c>
-      <c r="F182" s="16" t="inlineStr">
+      <c r="F191" s="16" t="inlineStr">
         <is>
           <t>功能测试通过/正确率100%</t>
         </is>
       </c>
-      <c r="G182" s="24" t="inlineStr">
+      <c r="G191" s="24" t="inlineStr">
         <is>
           <t>中</t>
         </is>
       </c>
-      <c r="H182" s="18" t="n">
+      <c r="H191" s="18" t="n">
         <v>20</v>
       </c>
     </row>
-    <row r="183">
-      <c r="A183" s="19" t="inlineStr">
+    <row r="192">
+      <c r="A192" s="19" t="inlineStr">
         <is>
           <t>总计功能数 / Total Function Points</t>
         </is>
       </c>
-      <c r="H183" s="20">
-        <f>SUM(H3:H182)</f>
+      <c r="H192" s="20">
+        <f>SUM(H3:H191)</f>
         <v/>
       </c>
     </row>
   </sheetData>
   <mergeCells count="16">
     <mergeCell ref="A143:H143"/>
-    <mergeCell ref="A163:H163"/>
     <mergeCell ref="A3:H3"/>
     <mergeCell ref="A101:H101"/>
     <mergeCell ref="A130:H130"/>
-    <mergeCell ref="A157:H157"/>
+    <mergeCell ref="A179:H179"/>
+    <mergeCell ref="A166:H166"/>
+    <mergeCell ref="A186:H186"/>
+    <mergeCell ref="A172:H172"/>
+    <mergeCell ref="A192:G192"/>
     <mergeCell ref="A60:H60"/>
     <mergeCell ref="A112:H112"/>
     <mergeCell ref="A68:H68"/>
-    <mergeCell ref="A170:H170"/>
-    <mergeCell ref="A177:H177"/>
-    <mergeCell ref="A183:G183"/>
     <mergeCell ref="A1:H1"/>
-    <mergeCell ref="A150:H150"/>
     <mergeCell ref="A31:H31"/>
+    <mergeCell ref="A159:H159"/>
     <mergeCell ref="A88:H88"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Expand module 10 销售交易: 7 functions/3 domains + tech_design
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Feasibility_analysis/FICC_Gap_Analysis.xlsx
+++ b/Feasibility_analysis/FICC_Gap_Analysis.xlsx
@@ -20,6 +20,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="详情_组合管理+绩效归因" sheetId="11" state="visible" r:id="rId11"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="详情_策略投资_量化" sheetId="12" state="visible" r:id="rId12"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="详情_定价平台" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="详情_销售交易" sheetId="14" state="visible" r:id="rId14"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Area" localSheetId="0">'差距分析总表'!$A$1:$P$17</definedName>
@@ -1576,13 +1577,13 @@
         </is>
       </c>
       <c r="M12" s="10" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="N12" s="10" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="O12" s="13" t="n">
-        <v>14</v>
+        <v>20</v>
       </c>
       <c r="P12" s="11" t="inlineStr">
         <is>
@@ -4736,13 +4737,422 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="48" customWidth="1" min="4" max="4"/>
+    <col width="26" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="6" max="6"/>
+    <col width="8" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="8" max="8"/>
+    <col width="7" customWidth="1" min="9" max="9"/>
+    <col width="18" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="24" customHeight="1">
+      <c r="A1" s="38" t="inlineStr">
+        <is>
+          <t>系统详情：销售交易  |  Sales Trading</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="36" customHeight="1">
+      <c r="A2" s="39" t="inlineStr">
+        <is>
+          <t>战略定位：面向对客服务的销售交易工作台，报价聚合、智能推荐、交易执行一体化；对应PPT Slide 47   |   来源：Slide 47</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="28" customHeight="1">
+      <c r="A3" s="40" t="inlineStr">
+        <is>
+          <t>模块：销售交易  (Sales Trading)  |  优先级：P2  |  竞品：金证/顶点  |  华锐基础：现券交易系统/IBOR  |  工期：5月  团队：5人</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="28" customHeight="1">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>功能域</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>编号</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>功能名称</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>功能描述</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>验收标准</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>集成依赖</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>复杂度</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>预估(人天)</t>
+        </is>
+      </c>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t>优先级</t>
+        </is>
+      </c>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>备注</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="18" customHeight="1">
+      <c r="A5" s="22" t="inlineStr">
+        <is>
+          <t>D1. 报价管理</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="48" customHeight="1">
+      <c r="A6" s="11" t="inlineStr">
+        <is>
+          <t>D1. 报价管理</t>
+        </is>
+      </c>
+      <c r="B6" s="10" t="inlineStr">
+        <is>
+          <t>F10-01</t>
+        </is>
+      </c>
+      <c r="C6" s="27" t="inlineStr">
+        <is>
+          <t>报价工作台</t>
+        </is>
+      </c>
+      <c r="D6" s="11" t="inlineStr">
+        <is>
+          <t>历史报价管理，当日报价快捷操作，导入/导出报价，一键unrefer，报价提醒功能</t>
+        </is>
+      </c>
+      <c r="E6" s="11" t="inlineStr"/>
+      <c r="F6" s="11" t="inlineStr"/>
+      <c r="G6" s="42" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="H6" s="13" t="n">
+        <v>20</v>
+      </c>
+      <c r="I6" s="12" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="J6" s="11" t="inlineStr"/>
+    </row>
+    <row r="7" ht="48" customHeight="1">
+      <c r="A7" s="11" t="inlineStr">
+        <is>
+          <t>D1. 报价管理</t>
+        </is>
+      </c>
+      <c r="B7" s="10" t="inlineStr">
+        <is>
+          <t>F10-02</t>
+        </is>
+      </c>
+      <c r="C7" s="27" t="inlineStr">
+        <is>
+          <t>债券过滤与筛选</t>
+        </is>
+      </c>
+      <c r="D7" s="11" t="inlineStr">
+        <is>
+          <t>信用债全品种过滤，利率债（国债/证金债/地方债）过滤，精确识别与模糊识别双模式</t>
+        </is>
+      </c>
+      <c r="E7" s="11" t="inlineStr"/>
+      <c r="F7" s="11" t="inlineStr"/>
+      <c r="G7" s="42" t="inlineStr">
+        <is>
+          <t>低</t>
+        </is>
+      </c>
+      <c r="H7" s="13" t="n">
+        <v>10</v>
+      </c>
+      <c r="I7" s="12" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="J7" s="11" t="inlineStr"/>
+    </row>
+    <row r="8" ht="48" customHeight="1">
+      <c r="A8" s="11" t="inlineStr">
+        <is>
+          <t>D1. 报价管理</t>
+        </is>
+      </c>
+      <c r="B8" s="10" t="inlineStr">
+        <is>
+          <t>F10-03</t>
+        </is>
+      </c>
+      <c r="C8" s="27" t="inlineStr">
+        <is>
+          <t>报价撮合与对价</t>
+        </is>
+      </c>
+      <c r="D8" s="11" t="inlineStr">
+        <is>
+          <t>对价/最优报价聚合展示，撮合对价，交易包管理，报价成交确认，一键成交</t>
+        </is>
+      </c>
+      <c r="E8" s="11" t="inlineStr"/>
+      <c r="F8" s="11" t="inlineStr"/>
+      <c r="G8" s="42" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="H8" s="13" t="n">
+        <v>20</v>
+      </c>
+      <c r="I8" s="12" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="J8" s="11" t="inlineStr"/>
+    </row>
+    <row r="9" ht="18" customHeight="1">
+      <c r="A9" s="40" t="inlineStr">
+        <is>
+          <t>D2. 交易执行</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="48" customHeight="1">
+      <c r="A10" s="11" t="inlineStr">
+        <is>
+          <t>D2. 交易执行</t>
+        </is>
+      </c>
+      <c r="B10" s="10" t="inlineStr">
+        <is>
+          <t>F10-04</t>
+        </is>
+      </c>
+      <c r="C10" s="27" t="inlineStr">
+        <is>
+          <t>交易执行与要素校验</t>
+        </is>
+      </c>
+      <c r="D10" s="11" t="inlineStr">
+        <is>
+          <t>意向达成，交易要素自动校验，手工价录入，业务审批流程，交易记录管理</t>
+        </is>
+      </c>
+      <c r="E10" s="11" t="inlineStr"/>
+      <c r="F10" s="11" t="inlineStr"/>
+      <c r="G10" s="42" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="H10" s="13" t="n">
+        <v>15</v>
+      </c>
+      <c r="I10" s="12" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="J10" s="11" t="inlineStr"/>
+    </row>
+    <row r="11" ht="48" customHeight="1">
+      <c r="A11" s="11" t="inlineStr">
+        <is>
+          <t>D2. 交易执行</t>
+        </is>
+      </c>
+      <c r="B11" s="10" t="inlineStr">
+        <is>
+          <t>F10-05</t>
+        </is>
+      </c>
+      <c r="C11" s="27" t="inlineStr">
+        <is>
+          <t>风控检查</t>
+        </is>
+      </c>
+      <c r="D11" s="11" t="inlineStr">
+        <is>
+          <t>交易前风控规则同步校验，限额检查，合规拦截，风控记录留痕，不通过自动拦截</t>
+        </is>
+      </c>
+      <c r="E11" s="11" t="inlineStr"/>
+      <c r="F11" s="11" t="inlineStr"/>
+      <c r="G11" s="42" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="H11" s="13" t="n">
+        <v>15</v>
+      </c>
+      <c r="I11" s="12" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="J11" s="11" t="inlineStr"/>
+    </row>
+    <row r="12" ht="18" customHeight="1">
+      <c r="A12" s="43" t="inlineStr">
+        <is>
+          <t>D3. 智能服务</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="48" customHeight="1">
+      <c r="A13" s="11" t="inlineStr">
+        <is>
+          <t>D3. 智能服务</t>
+        </is>
+      </c>
+      <c r="B13" s="10" t="inlineStr">
+        <is>
+          <t>F10-06</t>
+        </is>
+      </c>
+      <c r="C13" s="27" t="inlineStr">
+        <is>
+          <t>智能推荐系统</t>
+        </is>
+      </c>
+      <c r="D13" s="11" t="inlineStr">
+        <is>
+          <t>基于客户画像与历史交易数据主动推荐券种，从被动服务转向主动服务，提升客户响应效率</t>
+        </is>
+      </c>
+      <c r="E13" s="11" t="inlineStr"/>
+      <c r="F13" s="11" t="inlineStr"/>
+      <c r="G13" s="41" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="H13" s="13" t="n">
+        <v>25</v>
+      </c>
+      <c r="I13" s="12" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="J13" s="11" t="inlineStr"/>
+    </row>
+    <row r="14" ht="48" customHeight="1">
+      <c r="A14" s="11" t="inlineStr">
+        <is>
+          <t>D3. 智能服务</t>
+        </is>
+      </c>
+      <c r="B14" s="10" t="inlineStr">
+        <is>
+          <t>F10-07</t>
+        </is>
+      </c>
+      <c r="C14" s="27" t="inlineStr">
+        <is>
+          <t>综合业务平台</t>
+        </is>
+      </c>
+      <c r="D14" s="11" t="inlineStr">
+        <is>
+          <t>解决交易员分散办公与客户交易信息共享问题，报价聚合展示，客户快速服务，多地协同</t>
+        </is>
+      </c>
+      <c r="E14" s="11" t="inlineStr"/>
+      <c r="F14" s="11" t="inlineStr"/>
+      <c r="G14" s="42" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="H14" s="13" t="n">
+        <v>15</v>
+      </c>
+      <c r="I14" s="12" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="J14" s="11" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="40" t="inlineStr">
+        <is>
+          <t>合计 7项功能  |  P1: 0项  |  P2: 7项</t>
+        </is>
+      </c>
+      <c r="H15" s="20">
+        <f>SUM(H5:H14)</f>
+        <v/>
+      </c>
+      <c r="I15" s="34" t="inlineStr"/>
+      <c r="J15" s="34" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <mergeCells count="7">
+    <mergeCell ref="A1:J1"/>
+    <mergeCell ref="A5:J5"/>
+    <mergeCell ref="A9:J9"/>
+    <mergeCell ref="A3:J3"/>
+    <mergeCell ref="A12:J12"/>
+    <mergeCell ref="A15:G15"/>
+    <mergeCell ref="A2:J2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" fitToWidth="1"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H192"/>
+  <dimension ref="A1:H193"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -10772,12 +11182,12 @@
       </c>
       <c r="D160" s="27" t="inlineStr">
         <is>
-          <t>销交工作台</t>
+          <t>报价工作台</t>
         </is>
       </c>
       <c r="E160" s="11" t="inlineStr">
         <is>
-          <t>报价管理主界面，历史报价管理，当日报价快捷操作，导入/导出报价，一键unrefer操作</t>
+          <t>历史报价管理，当日报价快捷操作，导入/导出报价，一键unrefer，报价提醒功能</t>
         </is>
       </c>
       <c r="F160" s="11" t="inlineStr">
@@ -10817,7 +11227,7 @@
       </c>
       <c r="E161" s="11" t="inlineStr">
         <is>
-          <t>信用债/利率债过滤，信用债全品种过滤，利率债国债/证金债/地方债分类过滤，精确与模糊识别</t>
+          <t>信用债全品种过滤，利率债（国债/证金债/地方债）过滤，精确识别与模糊识别双模式</t>
         </is>
       </c>
       <c r="F161" s="11" t="inlineStr">
@@ -10857,7 +11267,7 @@
       </c>
       <c r="E162" s="11" t="inlineStr">
         <is>
-          <t>报价展示（对价/最优报价），撮合对价，报价提醒，交易包管理，报价成交确认</t>
+          <t>对价/最优报价聚合展示，撮合对价，交易包管理，报价成交确认，一键成交</t>
         </is>
       </c>
       <c r="F162" s="11" t="inlineStr">
@@ -10892,12 +11302,12 @@
       </c>
       <c r="D163" s="27" t="inlineStr">
         <is>
-          <t>交易执行与审批</t>
+          <t>交易执行与要素校验</t>
         </is>
       </c>
       <c r="E163" s="11" t="inlineStr">
         <is>
-          <t>意向达成，交易要素校验，手工价录入，业务审批流程，交易执行</t>
+          <t>意向达成，交易要素自动校验，手工价录入，业务审批流程，交易记录管理</t>
         </is>
       </c>
       <c r="F163" s="11" t="inlineStr">
@@ -10937,7 +11347,7 @@
       </c>
       <c r="E164" s="11" t="inlineStr">
         <is>
-          <t>交易前风控规则校验，限额检查，合规拦截，风控记录留痕</t>
+          <t>交易前风控规则同步校验，限额检查，合规拦截，风控记录留痕，不通过自动拦截</t>
         </is>
       </c>
       <c r="F164" s="11" t="inlineStr">
@@ -10977,7 +11387,7 @@
       </c>
       <c r="E165" s="11" t="inlineStr">
         <is>
-          <t>从被动客户服务转向主动服务，基于客户画像与持仓分析智能推荐券种，提升客户响应效率</t>
+          <t>基于客户画像与历史交易数据主动推荐券种，从被动服务转向主动服务，提升客户响应效率</t>
         </is>
       </c>
       <c r="F165" s="11" t="inlineStr">
@@ -10994,51 +11404,51 @@
         <v>25</v>
       </c>
     </row>
-    <row r="166" ht="20" customHeight="1">
-      <c r="A166" s="26" t="inlineStr">
+    <row r="166" ht="28" customHeight="1">
+      <c r="A166" s="11" t="inlineStr">
+        <is>
+          <t>销售交易</t>
+        </is>
+      </c>
+      <c r="B166" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="C166" s="10" t="inlineStr">
+        <is>
+          <t>F10-07</t>
+        </is>
+      </c>
+      <c r="D166" s="27" t="inlineStr">
+        <is>
+          <t>综合业务平台</t>
+        </is>
+      </c>
+      <c r="E166" s="11" t="inlineStr">
+        <is>
+          <t>解决交易员分散办公与客户交易信息共享问题，报价聚合展示，客户快速服务，多地协同</t>
+        </is>
+      </c>
+      <c r="F166" s="11" t="inlineStr">
+        <is>
+          <t>功能测试通过/正确率100%</t>
+        </is>
+      </c>
+      <c r="G166" s="24" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="H166" s="13" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="167" ht="20" customHeight="1">
+      <c r="A167" s="26" t="inlineStr">
         <is>
           <t>【P2】 信用债/信用衍生品  (Credit &amp; CDS)</t>
         </is>
-      </c>
-    </row>
-    <row r="167" ht="28" customHeight="1">
-      <c r="A167" s="11" t="inlineStr">
-        <is>
-          <t>信用债/信用衍生品</t>
-        </is>
-      </c>
-      <c r="B167" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
-        </is>
-      </c>
-      <c r="C167" s="10" t="inlineStr">
-        <is>
-          <t>F11-01</t>
-        </is>
-      </c>
-      <c r="D167" s="27" t="inlineStr">
-        <is>
-          <t>信用利差分析</t>
-        </is>
-      </c>
-      <c r="E167" s="11" t="inlineStr">
-        <is>
-          <t>行业/评级/期限信用利差曲线实时计算，历史分位数分析</t>
-        </is>
-      </c>
-      <c r="F167" s="11" t="inlineStr">
-        <is>
-          <t>功能完整/边界测试/集成冒烟/性能基线</t>
-        </is>
-      </c>
-      <c r="G167" s="23" t="inlineStr">
-        <is>
-          <t>高</t>
-        </is>
-      </c>
-      <c r="H167" s="13" t="n">
-        <v>30</v>
       </c>
     </row>
     <row r="168" ht="28" customHeight="1">
@@ -11054,31 +11464,31 @@
       </c>
       <c r="C168" s="10" t="inlineStr">
         <is>
-          <t>F11-02</t>
+          <t>F11-01</t>
         </is>
       </c>
       <c r="D168" s="27" t="inlineStr">
         <is>
-          <t>CDS/CLN定价</t>
+          <t>信用利差分析</t>
         </is>
       </c>
       <c r="E168" s="11" t="inlineStr">
         <is>
-          <t>信用违约互换定价，ISDA标准，生存概率曲线校准</t>
+          <t>行业/评级/期限信用利差曲线实时计算，历史分位数分析</t>
         </is>
       </c>
       <c r="F168" s="11" t="inlineStr">
         <is>
-          <t>p99延迟/误差率/精度验证/压测10k TPS</t>
-        </is>
-      </c>
-      <c r="G168" s="28" t="inlineStr">
-        <is>
-          <t>极高</t>
+          <t>功能完整/边界测试/集成冒烟/性能基线</t>
+        </is>
+      </c>
+      <c r="G168" s="23" t="inlineStr">
+        <is>
+          <t>高</t>
         </is>
       </c>
       <c r="H168" s="13" t="n">
-        <v>50</v>
+        <v>30</v>
       </c>
     </row>
     <row r="169" ht="28" customHeight="1">
@@ -11094,31 +11504,31 @@
       </c>
       <c r="C169" s="10" t="inlineStr">
         <is>
-          <t>F11-03</t>
+          <t>F11-02</t>
         </is>
       </c>
       <c r="D169" s="27" t="inlineStr">
         <is>
-          <t>信用评级动态监控</t>
+          <t>CDS/CLN定价</t>
         </is>
       </c>
       <c r="E169" s="11" t="inlineStr">
         <is>
-          <t>对接外部评级机构（中诚信/联合/大公），评级下调预警</t>
+          <t>信用违约互换定价，ISDA标准，生存概率曲线校准</t>
         </is>
       </c>
       <c r="F169" s="11" t="inlineStr">
         <is>
-          <t>功能测试通过/正确率100%</t>
-        </is>
-      </c>
-      <c r="G169" s="24" t="inlineStr">
-        <is>
-          <t>中</t>
+          <t>p99延迟/误差率/精度验证/压测10k TPS</t>
+        </is>
+      </c>
+      <c r="G169" s="28" t="inlineStr">
+        <is>
+          <t>极高</t>
         </is>
       </c>
       <c r="H169" s="13" t="n">
-        <v>20</v>
+        <v>50</v>
       </c>
     </row>
     <row r="170" ht="28" customHeight="1">
@@ -11134,31 +11544,31 @@
       </c>
       <c r="C170" s="10" t="inlineStr">
         <is>
-          <t>F11-04</t>
+          <t>F11-03</t>
         </is>
       </c>
       <c r="D170" s="27" t="inlineStr">
         <is>
-          <t>违约概率（PD）建模</t>
+          <t>信用评级动态监控</t>
         </is>
       </c>
       <c r="E170" s="11" t="inlineStr">
         <is>
-          <t>结构化Merton模型+市场隐含PD，信用风险计量</t>
+          <t>对接外部评级机构（中诚信/联合/大公），评级下调预警</t>
         </is>
       </c>
       <c r="F170" s="11" t="inlineStr">
         <is>
-          <t>功能完整/边界测试/集成冒烟/性能基线</t>
-        </is>
-      </c>
-      <c r="G170" s="23" t="inlineStr">
-        <is>
-          <t>高</t>
+          <t>功能测试通过/正确率100%</t>
+        </is>
+      </c>
+      <c r="G170" s="24" t="inlineStr">
+        <is>
+          <t>中</t>
         </is>
       </c>
       <c r="H170" s="13" t="n">
-        <v>40</v>
+        <v>20</v>
       </c>
     </row>
     <row r="171" ht="28" customHeight="1">
@@ -11174,78 +11584,78 @@
       </c>
       <c r="C171" s="10" t="inlineStr">
         <is>
+          <t>F11-04</t>
+        </is>
+      </c>
+      <c r="D171" s="27" t="inlineStr">
+        <is>
+          <t>违约概率（PD）建模</t>
+        </is>
+      </c>
+      <c r="E171" s="11" t="inlineStr">
+        <is>
+          <t>结构化Merton模型+市场隐含PD，信用风险计量</t>
+        </is>
+      </c>
+      <c r="F171" s="11" t="inlineStr">
+        <is>
+          <t>功能完整/边界测试/集成冒烟/性能基线</t>
+        </is>
+      </c>
+      <c r="G171" s="23" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="H171" s="13" t="n">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="172" ht="28" customHeight="1">
+      <c r="A172" s="11" t="inlineStr">
+        <is>
+          <t>信用债/信用衍生品</t>
+        </is>
+      </c>
+      <c r="B172" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="C172" s="10" t="inlineStr">
+        <is>
           <t>F11-05</t>
         </is>
       </c>
-      <c r="D171" s="27" t="inlineStr">
+      <c r="D172" s="27" t="inlineStr">
         <is>
           <t>集中度限额管理</t>
         </is>
       </c>
-      <c r="E171" s="11" t="inlineStr">
+      <c r="E172" s="11" t="inlineStr">
         <is>
           <t>行业/发行人/评级集中度多维限额，超限预警</t>
         </is>
       </c>
-      <c r="F171" s="11" t="inlineStr">
+      <c r="F172" s="11" t="inlineStr">
         <is>
           <t>功能测试通过/正确率100%</t>
         </is>
       </c>
-      <c r="G171" s="24" t="inlineStr">
+      <c r="G172" s="24" t="inlineStr">
         <is>
           <t>中</t>
         </is>
       </c>
-      <c r="H171" s="13" t="n">
+      <c r="H172" s="13" t="n">
         <v>20</v>
       </c>
     </row>
-    <row r="172" ht="20" customHeight="1">
-      <c r="A172" s="26" t="inlineStr">
+    <row r="173" ht="20" customHeight="1">
+      <c r="A173" s="26" t="inlineStr">
         <is>
           <t>【P2】 投顾服务  (Investment Advisory)</t>
         </is>
-      </c>
-    </row>
-    <row r="173" ht="28" customHeight="1">
-      <c r="A173" s="11" t="inlineStr">
-        <is>
-          <t>投顾服务</t>
-        </is>
-      </c>
-      <c r="B173" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
-        </is>
-      </c>
-      <c r="C173" s="10" t="inlineStr">
-        <is>
-          <t>F12-01</t>
-        </is>
-      </c>
-      <c r="D173" s="27" t="inlineStr">
-        <is>
-          <t>投顾工作台</t>
-        </is>
-      </c>
-      <c r="E173" s="11" t="inlineStr">
-        <is>
-          <t>投顾人员操作界面，管理客户委托，上传研究报告，发送投资建议，查看客户反馈</t>
-        </is>
-      </c>
-      <c r="F173" s="11" t="inlineStr">
-        <is>
-          <t>功能测试通过/正确率100%</t>
-        </is>
-      </c>
-      <c r="G173" s="24" t="inlineStr">
-        <is>
-          <t>中</t>
-        </is>
-      </c>
-      <c r="H173" s="13" t="n">
-        <v>20</v>
       </c>
     </row>
     <row r="174" ht="28" customHeight="1">
@@ -11261,17 +11671,17 @@
       </c>
       <c r="C174" s="10" t="inlineStr">
         <is>
-          <t>F12-02</t>
+          <t>F12-01</t>
         </is>
       </c>
       <c r="D174" s="27" t="inlineStr">
         <is>
-          <t>客户终端</t>
+          <t>投顾工作台</t>
         </is>
       </c>
       <c r="E174" s="11" t="inlineStr">
         <is>
-          <t>客户查看投资建议与分析报告，确认交易服务，查看账户净值走势、持仓明细、交易明细</t>
+          <t>投顾人员操作界面，管理客户委托，上传研究报告，发送投资建议，查看客户反馈</t>
         </is>
       </c>
       <c r="F174" s="11" t="inlineStr">
@@ -11301,17 +11711,17 @@
       </c>
       <c r="C175" s="10" t="inlineStr">
         <is>
-          <t>F12-03</t>
+          <t>F12-02</t>
         </is>
       </c>
       <c r="D175" s="27" t="inlineStr">
         <is>
-          <t>投资建议书管理</t>
+          <t>客户终端</t>
         </is>
       </c>
       <c r="E175" s="11" t="inlineStr">
         <is>
-          <t>投资建议书线上生成、审批、确认全流程，留痕追溯，客户电子签收</t>
+          <t>客户查看投资建议与分析报告，确认交易服务，查看账户净值走势、持仓明细、交易明细</t>
         </is>
       </c>
       <c r="F175" s="11" t="inlineStr">
@@ -11325,7 +11735,7 @@
         </is>
       </c>
       <c r="H175" s="13" t="n">
-        <v>15</v>
+        <v>20</v>
       </c>
     </row>
     <row r="176" ht="28" customHeight="1">
@@ -11341,31 +11751,31 @@
       </c>
       <c r="C176" s="10" t="inlineStr">
         <is>
-          <t>F12-04</t>
+          <t>F12-03</t>
         </is>
       </c>
       <c r="D176" s="27" t="inlineStr">
         <is>
-          <t>账户分析报告</t>
+          <t>投资建议书管理</t>
         </is>
       </c>
       <c r="E176" s="11" t="inlineStr">
         <is>
-          <t>账户净值走势、久期走势、归因分析、估值台账等核心数据展示及定期报告生成</t>
+          <t>投资建议书线上生成、审批、确认全流程，留痕追溯，客户电子签收</t>
         </is>
       </c>
       <c r="F176" s="11" t="inlineStr">
         <is>
-          <t>功能完整/边界测试/集成冒烟/性能基线</t>
-        </is>
-      </c>
-      <c r="G176" s="23" t="inlineStr">
-        <is>
-          <t>高</t>
+          <t>功能测试通过/正确率100%</t>
+        </is>
+      </c>
+      <c r="G176" s="24" t="inlineStr">
+        <is>
+          <t>中</t>
         </is>
       </c>
       <c r="H176" s="13" t="n">
-        <v>25</v>
+        <v>15</v>
       </c>
     </row>
     <row r="177" ht="28" customHeight="1">
@@ -11381,31 +11791,31 @@
       </c>
       <c r="C177" s="10" t="inlineStr">
         <is>
-          <t>F12-05</t>
+          <t>F12-04</t>
         </is>
       </c>
       <c r="D177" s="27" t="inlineStr">
         <is>
-          <t>投研报告服务</t>
+          <t>账户分析报告</t>
         </is>
       </c>
       <c r="E177" s="11" t="inlineStr">
         <is>
-          <t>日/周/月研究报告上传与推送，RPA自动获取基础数据，报告分类管理</t>
+          <t>账户净值走势、久期走势、归因分析、估值台账等核心数据展示及定期报告生成</t>
         </is>
       </c>
       <c r="F177" s="11" t="inlineStr">
         <is>
-          <t>功能测试通过/正确率100%</t>
-        </is>
-      </c>
-      <c r="G177" s="24" t="inlineStr">
-        <is>
-          <t>中</t>
+          <t>功能完整/边界测试/集成冒烟/性能基线</t>
+        </is>
+      </c>
+      <c r="G177" s="23" t="inlineStr">
+        <is>
+          <t>高</t>
         </is>
       </c>
       <c r="H177" s="13" t="n">
-        <v>15</v>
+        <v>25</v>
       </c>
     </row>
     <row r="178" ht="28" customHeight="1">
@@ -11421,78 +11831,78 @@
       </c>
       <c r="C178" s="10" t="inlineStr">
         <is>
+          <t>F12-05</t>
+        </is>
+      </c>
+      <c r="D178" s="27" t="inlineStr">
+        <is>
+          <t>投研报告服务</t>
+        </is>
+      </c>
+      <c r="E178" s="11" t="inlineStr">
+        <is>
+          <t>日/周/月研究报告上传与推送，RPA自动获取基础数据，报告分类管理</t>
+        </is>
+      </c>
+      <c r="F178" s="11" t="inlineStr">
+        <is>
+          <t>功能测试通过/正确率100%</t>
+        </is>
+      </c>
+      <c r="G178" s="24" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="H178" s="13" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="179" ht="28" customHeight="1">
+      <c r="A179" s="11" t="inlineStr">
+        <is>
+          <t>投顾服务</t>
+        </is>
+      </c>
+      <c r="B179" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="C179" s="10" t="inlineStr">
+        <is>
           <t>F12-06</t>
         </is>
       </c>
-      <c r="D178" s="27" t="inlineStr">
+      <c r="D179" s="27" t="inlineStr">
         <is>
           <t>客户服务与基础服务</t>
         </is>
       </c>
-      <c r="E178" s="11" t="inlineStr">
+      <c r="E179" s="11" t="inlineStr">
         <is>
           <t>服务中心、消息中心、问卷系统；用户/账户/数据管理，消息群发，登录注册</t>
         </is>
       </c>
-      <c r="F178" s="11" t="inlineStr">
+      <c r="F179" s="11" t="inlineStr">
         <is>
           <t>功能测试通过</t>
         </is>
       </c>
-      <c r="G178" s="25" t="inlineStr">
+      <c r="G179" s="25" t="inlineStr">
         <is>
           <t>低</t>
         </is>
       </c>
-      <c r="H178" s="13" t="n">
+      <c r="H179" s="13" t="n">
         <v>10</v>
       </c>
     </row>
-    <row r="179" ht="20" customHeight="1">
-      <c r="A179" s="26" t="inlineStr">
+    <row r="180" ht="20" customHeight="1">
+      <c r="A180" s="26" t="inlineStr">
         <is>
           <t>【P2】 TRS收益互换  (Total Return Swap)</t>
         </is>
-      </c>
-    </row>
-    <row r="180" ht="28" customHeight="1">
-      <c r="A180" s="11" t="inlineStr">
-        <is>
-          <t>TRS收益互换</t>
-        </is>
-      </c>
-      <c r="B180" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
-        </is>
-      </c>
-      <c r="C180" s="10" t="inlineStr">
-        <is>
-          <t>F13-01</t>
-        </is>
-      </c>
-      <c r="D180" s="27" t="inlineStr">
-        <is>
-          <t>TRS交易端</t>
-        </is>
-      </c>
-      <c r="E180" s="11" t="inlineStr">
-        <is>
-          <t>报价提供，成交回报，对冲委托与自动对冲，请求报价，行情与资讯，历史确认</t>
-        </is>
-      </c>
-      <c r="F180" s="11" t="inlineStr">
-        <is>
-          <t>功能完整/边界测试/集成冒烟/性能基线</t>
-        </is>
-      </c>
-      <c r="G180" s="23" t="inlineStr">
-        <is>
-          <t>高</t>
-        </is>
-      </c>
-      <c r="H180" s="13" t="n">
-        <v>30</v>
       </c>
     </row>
     <row r="181" ht="28" customHeight="1">
@@ -11508,17 +11918,17 @@
       </c>
       <c r="C181" s="10" t="inlineStr">
         <is>
-          <t>F13-02</t>
+          <t>F13-01</t>
         </is>
       </c>
       <c r="D181" s="27" t="inlineStr">
         <is>
-          <t>TRS客户端</t>
+          <t>TRS交易端</t>
         </is>
       </c>
       <c r="E181" s="11" t="inlineStr">
         <is>
-          <t>开户申请，客户委托，出入金申请，合约持仓，标的持仓，资金管理，行情矩阵，自主下单</t>
+          <t>报价提供，成交回报，对冲委托与自动对冲，请求报价，行情与资讯，历史确认</t>
         </is>
       </c>
       <c r="F181" s="11" t="inlineStr">
@@ -11532,7 +11942,7 @@
         </is>
       </c>
       <c r="H181" s="13" t="n">
-        <v>25</v>
+        <v>30</v>
       </c>
     </row>
     <row r="182" ht="28" customHeight="1">
@@ -11548,31 +11958,31 @@
       </c>
       <c r="C182" s="10" t="inlineStr">
         <is>
-          <t>F13-03</t>
+          <t>F13-02</t>
         </is>
       </c>
       <c r="D182" s="27" t="inlineStr">
         <is>
-          <t>TRS管理端</t>
+          <t>TRS客户端</t>
         </is>
       </c>
       <c r="E182" s="11" t="inlineStr">
         <is>
-          <t>开户申请审批，合约成交管理，出入金审批，运营管理，对账，库存，对冲录入</t>
+          <t>开户申请，客户委托，出入金申请，合约持仓，标的持仓，资金管理，行情矩阵，自主下单</t>
         </is>
       </c>
       <c r="F182" s="11" t="inlineStr">
         <is>
-          <t>功能测试通过/正确率100%</t>
-        </is>
-      </c>
-      <c r="G182" s="24" t="inlineStr">
-        <is>
-          <t>中</t>
+          <t>功能完整/边界测试/集成冒烟/性能基线</t>
+        </is>
+      </c>
+      <c r="G182" s="23" t="inlineStr">
+        <is>
+          <t>高</t>
         </is>
       </c>
       <c r="H182" s="13" t="n">
-        <v>20</v>
+        <v>25</v>
       </c>
     </row>
     <row r="183" ht="28" customHeight="1">
@@ -11588,31 +11998,31 @@
       </c>
       <c r="C183" s="10" t="inlineStr">
         <is>
-          <t>F13-04</t>
+          <t>F13-03</t>
         </is>
       </c>
       <c r="D183" s="27" t="inlineStr">
         <is>
-          <t>自动对冲</t>
+          <t>TRS管理端</t>
         </is>
       </c>
       <c r="E183" s="11" t="inlineStr">
         <is>
-          <t>对冲委托自动触发，对冲回报处理，风险校验，组合重叠分析，开平仓设置</t>
+          <t>开户申请审批，合约成交管理，出入金审批，运营管理，对账，库存，对冲录入</t>
         </is>
       </c>
       <c r="F183" s="11" t="inlineStr">
         <is>
-          <t>功能完整/边界测试/集成冒烟/性能基线</t>
-        </is>
-      </c>
-      <c r="G183" s="23" t="inlineStr">
-        <is>
-          <t>高</t>
+          <t>功能测试通过/正确率100%</t>
+        </is>
+      </c>
+      <c r="G183" s="24" t="inlineStr">
+        <is>
+          <t>中</t>
         </is>
       </c>
       <c r="H183" s="13" t="n">
-        <v>25</v>
+        <v>20</v>
       </c>
     </row>
     <row r="184" ht="28" customHeight="1">
@@ -11628,31 +12038,31 @@
       </c>
       <c r="C184" s="10" t="inlineStr">
         <is>
-          <t>F13-05</t>
+          <t>F13-04</t>
         </is>
       </c>
       <c r="D184" s="27" t="inlineStr">
         <is>
-          <t>通知与确认文件</t>
+          <t>自动对冲</t>
         </is>
       </c>
       <c r="E184" s="11" t="inlineStr">
         <is>
-          <t>企微通知提醒，确认书/结算单/估值报告/出入金通知自动生成并通过邮箱发送</t>
+          <t>对冲委托自动触发，对冲回报处理，风险校验，组合重叠分析，开平仓设置</t>
         </is>
       </c>
       <c r="F184" s="11" t="inlineStr">
         <is>
-          <t>功能测试通过/正确率100%</t>
-        </is>
-      </c>
-      <c r="G184" s="24" t="inlineStr">
-        <is>
-          <t>中</t>
+          <t>功能完整/边界测试/集成冒烟/性能基线</t>
+        </is>
+      </c>
+      <c r="G184" s="23" t="inlineStr">
+        <is>
+          <t>高</t>
         </is>
       </c>
       <c r="H184" s="13" t="n">
-        <v>15</v>
+        <v>25</v>
       </c>
     </row>
     <row r="185" ht="28" customHeight="1">
@@ -11668,78 +12078,78 @@
       </c>
       <c r="C185" s="10" t="inlineStr">
         <is>
+          <t>F13-05</t>
+        </is>
+      </c>
+      <c r="D185" s="27" t="inlineStr">
+        <is>
+          <t>通知与确认文件</t>
+        </is>
+      </c>
+      <c r="E185" s="11" t="inlineStr">
+        <is>
+          <t>企微通知提醒，确认书/结算单/估值报告/出入金通知自动生成并通过邮箱发送</t>
+        </is>
+      </c>
+      <c r="F185" s="11" t="inlineStr">
+        <is>
+          <t>功能测试通过/正确率100%</t>
+        </is>
+      </c>
+      <c r="G185" s="24" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="H185" s="13" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="186" ht="28" customHeight="1">
+      <c r="A186" s="11" t="inlineStr">
+        <is>
+          <t>TRS收益互换</t>
+        </is>
+      </c>
+      <c r="B186" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="C186" s="10" t="inlineStr">
+        <is>
           <t>F13-06</t>
         </is>
       </c>
-      <c r="D185" s="27" t="inlineStr">
+      <c r="D186" s="27" t="inlineStr">
         <is>
           <t>系统集成</t>
         </is>
       </c>
-      <c r="E185" s="11" t="inlineStr">
+      <c r="E186" s="11" t="inlineStr">
         <is>
           <t>与衡泰系统客户信息同步，QTrade聊天记录同步，交易管理系统对接，银行流水对接</t>
         </is>
       </c>
-      <c r="F185" s="11" t="inlineStr">
+      <c r="F186" s="11" t="inlineStr">
         <is>
           <t>功能完整/边界测试/集成冒烟/性能基线</t>
         </is>
       </c>
-      <c r="G185" s="23" t="inlineStr">
+      <c r="G186" s="23" t="inlineStr">
         <is>
           <t>高</t>
         </is>
       </c>
-      <c r="H185" s="13" t="n">
+      <c r="H186" s="13" t="n">
         <v>25</v>
       </c>
     </row>
-    <row r="186" ht="20" customHeight="1">
-      <c r="A186" s="29" t="inlineStr">
+    <row r="187" ht="20" customHeight="1">
+      <c r="A187" s="29" t="inlineStr">
         <is>
           <t>【P3】 做市商系统  (Market Making)</t>
         </is>
-      </c>
-    </row>
-    <row r="187" ht="28" customHeight="1">
-      <c r="A187" s="16" t="inlineStr">
-        <is>
-          <t>做市商系统</t>
-        </is>
-      </c>
-      <c r="B187" s="15" t="inlineStr">
-        <is>
-          <t>P3</t>
-        </is>
-      </c>
-      <c r="C187" s="15" t="inlineStr">
-        <is>
-          <t>F15-01</t>
-        </is>
-      </c>
-      <c r="D187" s="30" t="inlineStr">
-        <is>
-          <t>双边报价引擎</t>
-        </is>
-      </c>
-      <c r="E187" s="16" t="inlineStr">
-        <is>
-          <t>多品种同时双边报价，延迟&lt;5ms，报价宽度动态优化</t>
-        </is>
-      </c>
-      <c r="F187" s="16" t="inlineStr">
-        <is>
-          <t>p99延迟/误差率/精度验证/压测10k TPS</t>
-        </is>
-      </c>
-      <c r="G187" s="28" t="inlineStr">
-        <is>
-          <t>极高</t>
-        </is>
-      </c>
-      <c r="H187" s="18" t="n">
-        <v>70</v>
       </c>
     </row>
     <row r="188" ht="28" customHeight="1">
@@ -11755,17 +12165,17 @@
       </c>
       <c r="C188" s="15" t="inlineStr">
         <is>
-          <t>F15-02</t>
+          <t>F15-01</t>
         </is>
       </c>
       <c r="D188" s="30" t="inlineStr">
         <is>
-          <t>库存风险实时管理</t>
+          <t>双边报价引擎</t>
         </is>
       </c>
       <c r="E188" s="16" t="inlineStr">
         <is>
-          <t>做市库存PnL实时监控，Delta对冲自动触发</t>
+          <t>多品种同时双边报价，延迟&lt;5ms，报价宽度动态优化</t>
         </is>
       </c>
       <c r="F188" s="16" t="inlineStr">
@@ -11779,7 +12189,7 @@
         </is>
       </c>
       <c r="H188" s="18" t="n">
-        <v>60</v>
+        <v>70</v>
       </c>
     </row>
     <row r="189" ht="28" customHeight="1">
@@ -11795,17 +12205,17 @@
       </c>
       <c r="C189" s="15" t="inlineStr">
         <is>
-          <t>F15-03</t>
+          <t>F15-02</t>
         </is>
       </c>
       <c r="D189" s="30" t="inlineStr">
         <is>
-          <t>报价优化算法</t>
+          <t>库存风险实时管理</t>
         </is>
       </c>
       <c r="E189" s="16" t="inlineStr">
         <is>
-          <t>基于市场微结构理论动态调整bid-ask spread</t>
+          <t>做市库存PnL实时监控，Delta对冲自动触发</t>
         </is>
       </c>
       <c r="F189" s="16" t="inlineStr">
@@ -11819,7 +12229,7 @@
         </is>
       </c>
       <c r="H189" s="18" t="n">
-        <v>50</v>
+        <v>60</v>
       </c>
     </row>
     <row r="190" ht="28" customHeight="1">
@@ -11835,31 +12245,31 @@
       </c>
       <c r="C190" s="15" t="inlineStr">
         <is>
-          <t>F15-04</t>
+          <t>F15-03</t>
         </is>
       </c>
       <c r="D190" s="30" t="inlineStr">
         <is>
-          <t>竞争力分析</t>
+          <t>报价优化算法</t>
         </is>
       </c>
       <c r="E190" s="16" t="inlineStr">
         <is>
-          <t>与市场最优报价对比，中签率分析，策略调优</t>
+          <t>基于市场微结构理论动态调整bid-ask spread</t>
         </is>
       </c>
       <c r="F190" s="16" t="inlineStr">
         <is>
-          <t>功能完整/边界测试/集成冒烟/性能基线</t>
-        </is>
-      </c>
-      <c r="G190" s="23" t="inlineStr">
-        <is>
-          <t>高</t>
+          <t>p99延迟/误差率/精度验证/压测10k TPS</t>
+        </is>
+      </c>
+      <c r="G190" s="28" t="inlineStr">
+        <is>
+          <t>极高</t>
         </is>
       </c>
       <c r="H190" s="18" t="n">
-        <v>25</v>
+        <v>50</v>
       </c>
     </row>
     <row r="191" ht="28" customHeight="1">
@@ -11875,62 +12285,102 @@
       </c>
       <c r="C191" s="15" t="inlineStr">
         <is>
+          <t>F15-04</t>
+        </is>
+      </c>
+      <c r="D191" s="30" t="inlineStr">
+        <is>
+          <t>竞争力分析</t>
+        </is>
+      </c>
+      <c r="E191" s="16" t="inlineStr">
+        <is>
+          <t>与市场最优报价对比，中签率分析，策略调优</t>
+        </is>
+      </c>
+      <c r="F191" s="16" t="inlineStr">
+        <is>
+          <t>功能完整/边界测试/集成冒烟/性能基线</t>
+        </is>
+      </c>
+      <c r="G191" s="23" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="H191" s="18" t="n">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="192" ht="28" customHeight="1">
+      <c r="A192" s="16" t="inlineStr">
+        <is>
+          <t>做市商系统</t>
+        </is>
+      </c>
+      <c r="B192" s="15" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="C192" s="15" t="inlineStr">
+        <is>
           <t>F15-05</t>
         </is>
       </c>
-      <c r="D191" s="30" t="inlineStr">
+      <c r="D192" s="30" t="inlineStr">
         <is>
           <t>交易对手管理集成</t>
         </is>
       </c>
-      <c r="E191" s="16" t="inlineStr">
+      <c r="E192" s="16" t="inlineStr">
         <is>
           <t>做市交易对手信用实时检查，额度占用同步更新</t>
         </is>
       </c>
-      <c r="F191" s="16" t="inlineStr">
+      <c r="F192" s="16" t="inlineStr">
         <is>
           <t>功能测试通过/正确率100%</t>
         </is>
       </c>
-      <c r="G191" s="24" t="inlineStr">
+      <c r="G192" s="24" t="inlineStr">
         <is>
           <t>中</t>
         </is>
       </c>
-      <c r="H191" s="18" t="n">
+      <c r="H192" s="18" t="n">
         <v>20</v>
       </c>
     </row>
-    <row r="192">
-      <c r="A192" s="19" t="inlineStr">
+    <row r="193">
+      <c r="A193" s="19" t="inlineStr">
         <is>
           <t>总计功能数 / Total Function Points</t>
         </is>
       </c>
-      <c r="H192" s="20">
-        <f>SUM(H3:H191)</f>
+      <c r="H193" s="20">
+        <f>SUM(H3:H192)</f>
         <v/>
       </c>
     </row>
   </sheetData>
   <mergeCells count="16">
     <mergeCell ref="A143:H143"/>
+    <mergeCell ref="A193:G193"/>
     <mergeCell ref="A3:H3"/>
     <mergeCell ref="A101:H101"/>
     <mergeCell ref="A130:H130"/>
-    <mergeCell ref="A179:H179"/>
-    <mergeCell ref="A166:H166"/>
-    <mergeCell ref="A186:H186"/>
-    <mergeCell ref="A172:H172"/>
-    <mergeCell ref="A192:G192"/>
+    <mergeCell ref="A180:H180"/>
+    <mergeCell ref="A187:H187"/>
     <mergeCell ref="A60:H60"/>
     <mergeCell ref="A112:H112"/>
     <mergeCell ref="A68:H68"/>
     <mergeCell ref="A1:H1"/>
+    <mergeCell ref="A173:H173"/>
     <mergeCell ref="A31:H31"/>
     <mergeCell ref="A159:H159"/>
     <mergeCell ref="A88:H88"/>
+    <mergeCell ref="A167:H167"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Expand module 11 信用债/信用衍生品: 12 functions/4 domains + tech_design
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Feasibility_analysis/FICC_Gap_Analysis.xlsx
+++ b/Feasibility_analysis/FICC_Gap_Analysis.xlsx
@@ -21,6 +21,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="详情_策略投资_量化" sheetId="12" state="visible" r:id="rId12"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="详情_定价平台" sheetId="13" state="visible" r:id="rId13"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="详情_销售交易" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="详情_信用债_信用衍生品" sheetId="15" state="visible" r:id="rId15"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Area" localSheetId="0">'差距分析总表'!$A$1:$P$17</definedName>
@@ -1602,7 +1603,7 @@
       </c>
       <c r="C13" s="11" t="inlineStr">
         <is>
-          <t>Credit &amp; CDS</t>
+          <t>Credit Bond &amp; CDS</t>
         </is>
       </c>
       <c r="D13" s="11" t="inlineStr">
@@ -1622,46 +1623,46 @@
       </c>
       <c r="G13" s="10" t="inlineStr">
         <is>
-          <t>★★★★☆</t>
+          <t>★★★☆☆</t>
         </is>
       </c>
       <c r="H13" s="10" t="inlineStr">
         <is>
-          <t>L1</t>
+          <t>L2</t>
         </is>
       </c>
       <c r="I13" s="10" t="inlineStr">
         <is>
-          <t>L3</t>
-        </is>
-      </c>
-      <c r="J13" s="14" t="inlineStr">
-        <is>
-          <t>大</t>
+          <t>L4</t>
+        </is>
+      </c>
+      <c r="J13" s="7" t="inlineStr">
+        <is>
+          <t>中</t>
         </is>
       </c>
       <c r="K13" s="11" t="inlineStr">
         <is>
-          <t>衡泰/Bloomberg</t>
+          <t>衡泰/恒生</t>
         </is>
       </c>
       <c r="L13" s="11" t="inlineStr">
         <is>
-          <t>ARC信用风险框架</t>
+          <t>IBOR持仓账薄/定价平台</t>
         </is>
       </c>
       <c r="M13" s="10" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="N13" s="10" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="O13" s="13" t="n">
-        <v>80</v>
+        <v>55</v>
       </c>
       <c r="P13" s="11" t="inlineStr">
         <is>
-          <t>CDS定价+信用利差分析</t>
+          <t>信用评级/投资池/全生命周期信用风险管理，打通从评级审批到交易下单全链路；对应PPT Slide 42</t>
         </is>
       </c>
     </row>
@@ -5146,13 +5147,620 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J21"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="48" customWidth="1" min="4" max="4"/>
+    <col width="26" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="6" max="6"/>
+    <col width="8" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="8" max="8"/>
+    <col width="7" customWidth="1" min="9" max="9"/>
+    <col width="18" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="24" customHeight="1">
+      <c r="A1" s="38" t="inlineStr">
+        <is>
+          <t>系统详情：信用债/信用衍生品  |  Credit Bond &amp; CDS</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="36" customHeight="1">
+      <c r="A2" s="39" t="inlineStr">
+        <is>
+          <t>战略定位：信用评级/投资池/全生命周期信用风险管理，打通从评级审批到交易下单全链路；对应PPT Slide 42   |   来源：Slide 42</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="28" customHeight="1">
+      <c r="A3" s="40" t="inlineStr">
+        <is>
+          <t>模块：信用债/信用衍生品  (Credit Bond &amp; CDS)  |  优先级：P2  |  竞品：衡泰/恒生  |  华锐基础：IBOR持仓账薄/定价平台  |  工期：8月  团队：8人</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="28" customHeight="1">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>功能域</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>编号</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>功能名称</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>功能描述</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>验收标准</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>集成依赖</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>复杂度</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>预估(人天)</t>
+        </is>
+      </c>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t>优先级</t>
+        </is>
+      </c>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>备注</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="18" customHeight="1">
+      <c r="A5" s="22" t="inlineStr">
+        <is>
+          <t>D1. 信用数据与评估</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="48" customHeight="1">
+      <c r="A6" s="11" t="inlineStr">
+        <is>
+          <t>D1. 信用数据与评估</t>
+        </is>
+      </c>
+      <c r="B6" s="10" t="inlineStr">
+        <is>
+          <t>F11-01</t>
+        </is>
+      </c>
+      <c r="C6" s="27" t="inlineStr">
+        <is>
+          <t>信用风险数据接入</t>
+        </is>
+      </c>
+      <c r="D6" s="11" t="inlineStr">
+        <is>
+          <t>外部信用数据服务接入（Wind/中诚信/联合评级等），内部数据整合，数据质量检查，信用风险数据集市</t>
+        </is>
+      </c>
+      <c r="E6" s="11" t="inlineStr"/>
+      <c r="F6" s="11" t="inlineStr"/>
+      <c r="G6" s="41" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="H6" s="13" t="n">
+        <v>30</v>
+      </c>
+      <c r="I6" s="12" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="J6" s="11" t="inlineStr"/>
+    </row>
+    <row r="7" ht="48" customHeight="1">
+      <c r="A7" s="11" t="inlineStr">
+        <is>
+          <t>D1. 信用数据与评估</t>
+        </is>
+      </c>
+      <c r="B7" s="10" t="inlineStr">
+        <is>
+          <t>F11-02</t>
+        </is>
+      </c>
+      <c r="C7" s="27" t="inlineStr">
+        <is>
+          <t>信用评估引擎</t>
+        </is>
+      </c>
+      <c r="D7" s="11" t="inlineStr">
+        <is>
+          <t>持续迭代信用评价引擎，资产证券化评价，交易对手评价，违约概率（PD）建模，信用评分</t>
+        </is>
+      </c>
+      <c r="E7" s="11" t="inlineStr"/>
+      <c r="F7" s="11" t="inlineStr"/>
+      <c r="G7" s="28" t="inlineStr">
+        <is>
+          <t>极高</t>
+        </is>
+      </c>
+      <c r="H7" s="13" t="n">
+        <v>40</v>
+      </c>
+      <c r="I7" s="12" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="J7" s="11" t="inlineStr"/>
+    </row>
+    <row r="8" ht="48" customHeight="1">
+      <c r="A8" s="11" t="inlineStr">
+        <is>
+          <t>D1. 信用数据与评估</t>
+        </is>
+      </c>
+      <c r="B8" s="10" t="inlineStr">
+        <is>
+          <t>F11-03</t>
+        </is>
+      </c>
+      <c r="C8" s="27" t="inlineStr">
+        <is>
+          <t>信用预警系统</t>
+        </is>
+      </c>
+      <c r="D8" s="11" t="inlineStr">
+        <is>
+          <t>市场数据自动触发预警，评级下调动态预警，投后预警跟踪与信号处理，预警规则配置</t>
+        </is>
+      </c>
+      <c r="E8" s="11" t="inlineStr"/>
+      <c r="F8" s="11" t="inlineStr"/>
+      <c r="G8" s="41" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="H8" s="13" t="n">
+        <v>30</v>
+      </c>
+      <c r="I8" s="12" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="J8" s="11" t="inlineStr"/>
+    </row>
+    <row r="9" ht="18" customHeight="1">
+      <c r="A9" s="40" t="inlineStr">
+        <is>
+          <t>D2. 投资池与准入管理</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="48" customHeight="1">
+      <c r="A10" s="11" t="inlineStr">
+        <is>
+          <t>D2. 投资池与准入管理</t>
+        </is>
+      </c>
+      <c r="B10" s="10" t="inlineStr">
+        <is>
+          <t>F11-04</t>
+        </is>
+      </c>
+      <c r="C10" s="27" t="inlineStr">
+        <is>
+          <t>投资池管理</t>
+        </is>
+      </c>
+      <c r="D10" s="11" t="inlineStr">
+        <is>
+          <t>债券池配置与维护，债券准入/退出规则，白名单/黑名单管理，池状态实时更新</t>
+        </is>
+      </c>
+      <c r="E10" s="11" t="inlineStr"/>
+      <c r="F10" s="11" t="inlineStr"/>
+      <c r="G10" s="42" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="H10" s="13" t="n">
+        <v>20</v>
+      </c>
+      <c r="I10" s="12" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="J10" s="11" t="inlineStr"/>
+    </row>
+    <row r="11" ht="48" customHeight="1">
+      <c r="A11" s="11" t="inlineStr">
+        <is>
+          <t>D2. 投资池与准入管理</t>
+        </is>
+      </c>
+      <c r="B11" s="10" t="inlineStr">
+        <is>
+          <t>F11-05</t>
+        </is>
+      </c>
+      <c r="C11" s="27" t="inlineStr">
+        <is>
+          <t>评级管理</t>
+        </is>
+      </c>
+      <c r="D11" s="11" t="inlineStr">
+        <is>
+          <t>内部评级录入与更新，外部评级同步（中诚信/联合/大公），评级变更历史追踪，评级模型管理</t>
+        </is>
+      </c>
+      <c r="E11" s="11" t="inlineStr"/>
+      <c r="F11" s="11" t="inlineStr"/>
+      <c r="G11" s="42" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="H11" s="13" t="n">
+        <v>20</v>
+      </c>
+      <c r="I11" s="12" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="J11" s="11" t="inlineStr"/>
+    </row>
+    <row r="12" ht="48" customHeight="1">
+      <c r="A12" s="11" t="inlineStr">
+        <is>
+          <t>D2. 投资池与准入管理</t>
+        </is>
+      </c>
+      <c r="B12" s="10" t="inlineStr">
+        <is>
+          <t>F11-06</t>
+        </is>
+      </c>
+      <c r="C12" s="27" t="inlineStr">
+        <is>
+          <t>投前审批管理</t>
+        </is>
+      </c>
+      <c r="D12" s="11" t="inlineStr">
+        <is>
+          <t>新券投资准入审批流程，信用额度申请，投资决策材料生成，审批记录留痕</t>
+        </is>
+      </c>
+      <c r="E12" s="11" t="inlineStr"/>
+      <c r="F12" s="11" t="inlineStr"/>
+      <c r="G12" s="42" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="H12" s="13" t="n">
+        <v>20</v>
+      </c>
+      <c r="I12" s="12" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="J12" s="11" t="inlineStr"/>
+    </row>
+    <row r="13" ht="18" customHeight="1">
+      <c r="A13" s="43" t="inlineStr">
+        <is>
+          <t>D3. 持仓与风险监控</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="48" customHeight="1">
+      <c r="A14" s="11" t="inlineStr">
+        <is>
+          <t>D3. 持仓与风险监控</t>
+        </is>
+      </c>
+      <c r="B14" s="10" t="inlineStr">
+        <is>
+          <t>F11-07</t>
+        </is>
+      </c>
+      <c r="C14" s="27" t="inlineStr">
+        <is>
+          <t>持仓与敞口管理</t>
+        </is>
+      </c>
+      <c r="D14" s="11" t="inlineStr">
+        <is>
+          <t>信用债持仓实时查询，敞口管理，集中度分析（行业/评级/发行人），到期提醒</t>
+        </is>
+      </c>
+      <c r="E14" s="11" t="inlineStr"/>
+      <c r="F14" s="11" t="inlineStr"/>
+      <c r="G14" s="42" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="H14" s="13" t="n">
+        <v>20</v>
+      </c>
+      <c r="I14" s="12" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="J14" s="11" t="inlineStr"/>
+    </row>
+    <row r="15" ht="48" customHeight="1">
+      <c r="A15" s="11" t="inlineStr">
+        <is>
+          <t>D3. 持仓与风险监控</t>
+        </is>
+      </c>
+      <c r="B15" s="10" t="inlineStr">
+        <is>
+          <t>F11-08</t>
+        </is>
+      </c>
+      <c r="C15" s="27" t="inlineStr">
+        <is>
+          <t>信用风险监控看板</t>
+        </is>
+      </c>
+      <c r="D15" s="11" t="inlineStr">
+        <is>
+          <t>多维度风险指标实时监控，信用利差走势，主体信用事件推送，指标监控与查询统计</t>
+        </is>
+      </c>
+      <c r="E15" s="11" t="inlineStr"/>
+      <c r="F15" s="11" t="inlineStr"/>
+      <c r="G15" s="41" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="H15" s="13" t="n">
+        <v>25</v>
+      </c>
+      <c r="I15" s="12" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="J15" s="11" t="inlineStr"/>
+    </row>
+    <row r="16" ht="48" customHeight="1">
+      <c r="A16" s="11" t="inlineStr">
+        <is>
+          <t>D3. 持仓与风险监控</t>
+        </is>
+      </c>
+      <c r="B16" s="10" t="inlineStr">
+        <is>
+          <t>F11-09</t>
+        </is>
+      </c>
+      <c r="C16" s="27" t="inlineStr">
+        <is>
+          <t>违约管理</t>
+        </is>
+      </c>
+      <c r="D16" s="11" t="inlineStr">
+        <is>
+          <t>违约事件记录，违约债券处置跟踪，损失估算，监管报送，违约主体黑名单自动更新</t>
+        </is>
+      </c>
+      <c r="E16" s="11" t="inlineStr"/>
+      <c r="F16" s="11" t="inlineStr"/>
+      <c r="G16" s="41" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="H16" s="13" t="n">
+        <v>25</v>
+      </c>
+      <c r="I16" s="12" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="J16" s="11" t="inlineStr"/>
+    </row>
+    <row r="17" ht="18" customHeight="1">
+      <c r="A17" s="43" t="inlineStr">
+        <is>
+          <t>D4. 信用利差与衍生品</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="48" customHeight="1">
+      <c r="A18" s="11" t="inlineStr">
+        <is>
+          <t>D4. 信用利差与衍生品</t>
+        </is>
+      </c>
+      <c r="B18" s="10" t="inlineStr">
+        <is>
+          <t>F11-10</t>
+        </is>
+      </c>
+      <c r="C18" s="27" t="inlineStr">
+        <is>
+          <t>信用利差分析</t>
+        </is>
+      </c>
+      <c r="D18" s="11" t="inlineStr">
+        <is>
+          <t>行业/评级/期限信用利差曲线实时计算，历史分位数分析，利差走势，相对价值分析</t>
+        </is>
+      </c>
+      <c r="E18" s="11" t="inlineStr"/>
+      <c r="F18" s="11" t="inlineStr"/>
+      <c r="G18" s="41" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="H18" s="13" t="n">
+        <v>30</v>
+      </c>
+      <c r="I18" s="12" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="J18" s="11" t="inlineStr"/>
+    </row>
+    <row r="19" ht="48" customHeight="1">
+      <c r="A19" s="11" t="inlineStr">
+        <is>
+          <t>D4. 信用利差与衍生品</t>
+        </is>
+      </c>
+      <c r="B19" s="10" t="inlineStr">
+        <is>
+          <t>F11-11</t>
+        </is>
+      </c>
+      <c r="C19" s="27" t="inlineStr">
+        <is>
+          <t>CDS定价与管理</t>
+        </is>
+      </c>
+      <c r="D19" s="11" t="inlineStr">
+        <is>
+          <t>信用违约互换定价（ISDA标准），生存概率曲线校准，CDS交易录入与持仓管理</t>
+        </is>
+      </c>
+      <c r="E19" s="11" t="inlineStr"/>
+      <c r="F19" s="11" t="inlineStr"/>
+      <c r="G19" s="28" t="inlineStr">
+        <is>
+          <t>极高</t>
+        </is>
+      </c>
+      <c r="H19" s="13" t="n">
+        <v>40</v>
+      </c>
+      <c r="I19" s="12" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="J19" s="11" t="inlineStr"/>
+    </row>
+    <row r="20" ht="48" customHeight="1">
+      <c r="A20" s="11" t="inlineStr">
+        <is>
+          <t>D4. 信用利差与衍生品</t>
+        </is>
+      </c>
+      <c r="B20" s="10" t="inlineStr">
+        <is>
+          <t>F11-12</t>
+        </is>
+      </c>
+      <c r="C20" s="27" t="inlineStr">
+        <is>
+          <t>配置与权限管理</t>
+        </is>
+      </c>
+      <c r="D20" s="11" t="inlineStr">
+        <is>
+          <t>预警规则配置，指标库管理，评级模型管理，用户权限管理，债券池配置管理</t>
+        </is>
+      </c>
+      <c r="E20" s="11" t="inlineStr"/>
+      <c r="F20" s="11" t="inlineStr"/>
+      <c r="G20" s="42" t="inlineStr">
+        <is>
+          <t>低</t>
+        </is>
+      </c>
+      <c r="H20" s="13" t="n">
+        <v>15</v>
+      </c>
+      <c r="I20" s="12" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="J20" s="11" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="40" t="inlineStr">
+        <is>
+          <t>合计 12项功能  |  P1: 0项  |  P2: 12项</t>
+        </is>
+      </c>
+      <c r="H21" s="20">
+        <f>SUM(H5:H20)</f>
+        <v/>
+      </c>
+      <c r="I21" s="34" t="inlineStr"/>
+      <c r="J21" s="34" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <mergeCells count="8">
+    <mergeCell ref="A1:J1"/>
+    <mergeCell ref="A5:J5"/>
+    <mergeCell ref="A17:J17"/>
+    <mergeCell ref="A9:J9"/>
+    <mergeCell ref="A21:G21"/>
+    <mergeCell ref="A3:J3"/>
+    <mergeCell ref="A2:J2"/>
+    <mergeCell ref="A13:J13"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" fitToWidth="1"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H193"/>
+  <dimension ref="A1:H200"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -11447,7 +12055,7 @@
     <row r="167" ht="20" customHeight="1">
       <c r="A167" s="26" t="inlineStr">
         <is>
-          <t>【P2】 信用债/信用衍生品  (Credit &amp; CDS)</t>
+          <t>【P2】 信用债/信用衍生品  (Credit Bond &amp; CDS)</t>
         </is>
       </c>
     </row>
@@ -11469,12 +12077,12 @@
       </c>
       <c r="D168" s="27" t="inlineStr">
         <is>
-          <t>信用利差分析</t>
+          <t>信用风险数据接入</t>
         </is>
       </c>
       <c r="E168" s="11" t="inlineStr">
         <is>
-          <t>行业/评级/期限信用利差曲线实时计算，历史分位数分析</t>
+          <t>外部信用数据服务接入（Wind/中诚信/联合评级等），内部数据整合，数据质量检查，信用风险数据集市</t>
         </is>
       </c>
       <c r="F168" s="11" t="inlineStr">
@@ -11509,12 +12117,12 @@
       </c>
       <c r="D169" s="27" t="inlineStr">
         <is>
-          <t>CDS/CLN定价</t>
+          <t>信用评估引擎</t>
         </is>
       </c>
       <c r="E169" s="11" t="inlineStr">
         <is>
-          <t>信用违约互换定价，ISDA标准，生存概率曲线校准</t>
+          <t>持续迭代信用评价引擎，资产证券化评价，交易对手评价，违约概率（PD）建模，信用评分</t>
         </is>
       </c>
       <c r="F169" s="11" t="inlineStr">
@@ -11528,7 +12136,7 @@
         </is>
       </c>
       <c r="H169" s="13" t="n">
-        <v>50</v>
+        <v>40</v>
       </c>
     </row>
     <row r="170" ht="28" customHeight="1">
@@ -11549,26 +12157,26 @@
       </c>
       <c r="D170" s="27" t="inlineStr">
         <is>
-          <t>信用评级动态监控</t>
+          <t>信用预警系统</t>
         </is>
       </c>
       <c r="E170" s="11" t="inlineStr">
         <is>
-          <t>对接外部评级机构（中诚信/联合/大公），评级下调预警</t>
+          <t>市场数据自动触发预警，评级下调动态预警，投后预警跟踪与信号处理，预警规则配置</t>
         </is>
       </c>
       <c r="F170" s="11" t="inlineStr">
         <is>
-          <t>功能测试通过/正确率100%</t>
-        </is>
-      </c>
-      <c r="G170" s="24" t="inlineStr">
-        <is>
-          <t>中</t>
+          <t>功能完整/边界测试/集成冒烟/性能基线</t>
+        </is>
+      </c>
+      <c r="G170" s="23" t="inlineStr">
+        <is>
+          <t>高</t>
         </is>
       </c>
       <c r="H170" s="13" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
     </row>
     <row r="171" ht="28" customHeight="1">
@@ -11589,26 +12197,26 @@
       </c>
       <c r="D171" s="27" t="inlineStr">
         <is>
-          <t>违约概率（PD）建模</t>
+          <t>投资池管理</t>
         </is>
       </c>
       <c r="E171" s="11" t="inlineStr">
         <is>
-          <t>结构化Merton模型+市场隐含PD，信用风险计量</t>
+          <t>债券池配置与维护，债券准入/退出规则，白名单/黑名单管理，池状态实时更新</t>
         </is>
       </c>
       <c r="F171" s="11" t="inlineStr">
         <is>
-          <t>功能完整/边界测试/集成冒烟/性能基线</t>
-        </is>
-      </c>
-      <c r="G171" s="23" t="inlineStr">
-        <is>
-          <t>高</t>
+          <t>功能测试通过/正确率100%</t>
+        </is>
+      </c>
+      <c r="G171" s="24" t="inlineStr">
+        <is>
+          <t>中</t>
         </is>
       </c>
       <c r="H171" s="13" t="n">
-        <v>40</v>
+        <v>20</v>
       </c>
     </row>
     <row r="172" ht="28" customHeight="1">
@@ -11629,12 +12237,12 @@
       </c>
       <c r="D172" s="27" t="inlineStr">
         <is>
-          <t>集中度限额管理</t>
+          <t>评级管理</t>
         </is>
       </c>
       <c r="E172" s="11" t="inlineStr">
         <is>
-          <t>行业/发行人/评级集中度多维限额，超限预警</t>
+          <t>内部评级录入与更新，外部评级同步（中诚信/联合/大公），评级变更历史追踪，评级模型管理</t>
         </is>
       </c>
       <c r="F172" s="11" t="inlineStr">
@@ -11651,17 +12259,50 @@
         <v>20</v>
       </c>
     </row>
-    <row r="173" ht="20" customHeight="1">
-      <c r="A173" s="26" t="inlineStr">
-        <is>
-          <t>【P2】 投顾服务  (Investment Advisory)</t>
-        </is>
+    <row r="173" ht="28" customHeight="1">
+      <c r="A173" s="11" t="inlineStr">
+        <is>
+          <t>信用债/信用衍生品</t>
+        </is>
+      </c>
+      <c r="B173" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="C173" s="10" t="inlineStr">
+        <is>
+          <t>F11-06</t>
+        </is>
+      </c>
+      <c r="D173" s="27" t="inlineStr">
+        <is>
+          <t>投前审批管理</t>
+        </is>
+      </c>
+      <c r="E173" s="11" t="inlineStr">
+        <is>
+          <t>新券投资准入审批流程，信用额度申请，投资决策材料生成，审批记录留痕</t>
+        </is>
+      </c>
+      <c r="F173" s="11" t="inlineStr">
+        <is>
+          <t>功能测试通过/正确率100%</t>
+        </is>
+      </c>
+      <c r="G173" s="24" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="H173" s="13" t="n">
+        <v>20</v>
       </c>
     </row>
     <row r="174" ht="28" customHeight="1">
       <c r="A174" s="11" t="inlineStr">
         <is>
-          <t>投顾服务</t>
+          <t>信用债/信用衍生品</t>
         </is>
       </c>
       <c r="B174" s="10" t="inlineStr">
@@ -11671,17 +12312,17 @@
       </c>
       <c r="C174" s="10" t="inlineStr">
         <is>
-          <t>F12-01</t>
+          <t>F11-07</t>
         </is>
       </c>
       <c r="D174" s="27" t="inlineStr">
         <is>
-          <t>投顾工作台</t>
+          <t>持仓与敞口管理</t>
         </is>
       </c>
       <c r="E174" s="11" t="inlineStr">
         <is>
-          <t>投顾人员操作界面，管理客户委托，上传研究报告，发送投资建议，查看客户反馈</t>
+          <t>信用债持仓实时查询，敞口管理，集中度分析（行业/评级/发行人），到期提醒</t>
         </is>
       </c>
       <c r="F174" s="11" t="inlineStr">
@@ -11701,7 +12342,7 @@
     <row r="175" ht="28" customHeight="1">
       <c r="A175" s="11" t="inlineStr">
         <is>
-          <t>投顾服务</t>
+          <t>信用债/信用衍生品</t>
         </is>
       </c>
       <c r="B175" s="10" t="inlineStr">
@@ -11711,37 +12352,37 @@
       </c>
       <c r="C175" s="10" t="inlineStr">
         <is>
-          <t>F12-02</t>
+          <t>F11-08</t>
         </is>
       </c>
       <c r="D175" s="27" t="inlineStr">
         <is>
-          <t>客户终端</t>
+          <t>信用风险监控看板</t>
         </is>
       </c>
       <c r="E175" s="11" t="inlineStr">
         <is>
-          <t>客户查看投资建议与分析报告，确认交易服务，查看账户净值走势、持仓明细、交易明细</t>
+          <t>多维度风险指标实时监控，信用利差走势，主体信用事件推送，指标监控与查询统计</t>
         </is>
       </c>
       <c r="F175" s="11" t="inlineStr">
         <is>
-          <t>功能测试通过/正确率100%</t>
-        </is>
-      </c>
-      <c r="G175" s="24" t="inlineStr">
-        <is>
-          <t>中</t>
+          <t>功能完整/边界测试/集成冒烟/性能基线</t>
+        </is>
+      </c>
+      <c r="G175" s="23" t="inlineStr">
+        <is>
+          <t>高</t>
         </is>
       </c>
       <c r="H175" s="13" t="n">
-        <v>20</v>
+        <v>25</v>
       </c>
     </row>
     <row r="176" ht="28" customHeight="1">
       <c r="A176" s="11" t="inlineStr">
         <is>
-          <t>投顾服务</t>
+          <t>信用债/信用衍生品</t>
         </is>
       </c>
       <c r="B176" s="10" t="inlineStr">
@@ -11751,37 +12392,37 @@
       </c>
       <c r="C176" s="10" t="inlineStr">
         <is>
-          <t>F12-03</t>
+          <t>F11-09</t>
         </is>
       </c>
       <c r="D176" s="27" t="inlineStr">
         <is>
-          <t>投资建议书管理</t>
+          <t>违约管理</t>
         </is>
       </c>
       <c r="E176" s="11" t="inlineStr">
         <is>
-          <t>投资建议书线上生成、审批、确认全流程，留痕追溯，客户电子签收</t>
+          <t>违约事件记录，违约债券处置跟踪，损失估算，监管报送，违约主体黑名单自动更新</t>
         </is>
       </c>
       <c r="F176" s="11" t="inlineStr">
         <is>
-          <t>功能测试通过/正确率100%</t>
-        </is>
-      </c>
-      <c r="G176" s="24" t="inlineStr">
-        <is>
-          <t>中</t>
+          <t>功能完整/边界测试/集成冒烟/性能基线</t>
+        </is>
+      </c>
+      <c r="G176" s="23" t="inlineStr">
+        <is>
+          <t>高</t>
         </is>
       </c>
       <c r="H176" s="13" t="n">
-        <v>15</v>
+        <v>25</v>
       </c>
     </row>
     <row r="177" ht="28" customHeight="1">
       <c r="A177" s="11" t="inlineStr">
         <is>
-          <t>投顾服务</t>
+          <t>信用债/信用衍生品</t>
         </is>
       </c>
       <c r="B177" s="10" t="inlineStr">
@@ -11791,17 +12432,17 @@
       </c>
       <c r="C177" s="10" t="inlineStr">
         <is>
-          <t>F12-04</t>
+          <t>F11-10</t>
         </is>
       </c>
       <c r="D177" s="27" t="inlineStr">
         <is>
-          <t>账户分析报告</t>
+          <t>信用利差分析</t>
         </is>
       </c>
       <c r="E177" s="11" t="inlineStr">
         <is>
-          <t>账户净值走势、久期走势、归因分析、估值台账等核心数据展示及定期报告生成</t>
+          <t>行业/评级/期限信用利差曲线实时计算，历史分位数分析，利差走势，相对价值分析</t>
         </is>
       </c>
       <c r="F177" s="11" t="inlineStr">
@@ -11815,13 +12456,13 @@
         </is>
       </c>
       <c r="H177" s="13" t="n">
-        <v>25</v>
+        <v>30</v>
       </c>
     </row>
     <row r="178" ht="28" customHeight="1">
       <c r="A178" s="11" t="inlineStr">
         <is>
-          <t>投顾服务</t>
+          <t>信用债/信用衍生品</t>
         </is>
       </c>
       <c r="B178" s="10" t="inlineStr">
@@ -11831,37 +12472,37 @@
       </c>
       <c r="C178" s="10" t="inlineStr">
         <is>
-          <t>F12-05</t>
+          <t>F11-11</t>
         </is>
       </c>
       <c r="D178" s="27" t="inlineStr">
         <is>
-          <t>投研报告服务</t>
+          <t>CDS定价与管理</t>
         </is>
       </c>
       <c r="E178" s="11" t="inlineStr">
         <is>
-          <t>日/周/月研究报告上传与推送，RPA自动获取基础数据，报告分类管理</t>
+          <t>信用违约互换定价（ISDA标准），生存概率曲线校准，CDS交易录入与持仓管理</t>
         </is>
       </c>
       <c r="F178" s="11" t="inlineStr">
         <is>
-          <t>功能测试通过/正确率100%</t>
-        </is>
-      </c>
-      <c r="G178" s="24" t="inlineStr">
-        <is>
-          <t>中</t>
+          <t>p99延迟/误差率/精度验证/压测10k TPS</t>
+        </is>
+      </c>
+      <c r="G178" s="28" t="inlineStr">
+        <is>
+          <t>极高</t>
         </is>
       </c>
       <c r="H178" s="13" t="n">
-        <v>15</v>
+        <v>40</v>
       </c>
     </row>
     <row r="179" ht="28" customHeight="1">
       <c r="A179" s="11" t="inlineStr">
         <is>
-          <t>投顾服务</t>
+          <t>信用债/信用衍生品</t>
         </is>
       </c>
       <c r="B179" s="10" t="inlineStr">
@@ -11871,17 +12512,17 @@
       </c>
       <c r="C179" s="10" t="inlineStr">
         <is>
-          <t>F12-06</t>
+          <t>F11-12</t>
         </is>
       </c>
       <c r="D179" s="27" t="inlineStr">
         <is>
-          <t>客户服务与基础服务</t>
+          <t>配置与权限管理</t>
         </is>
       </c>
       <c r="E179" s="11" t="inlineStr">
         <is>
-          <t>服务中心、消息中心、问卷系统；用户/账户/数据管理，消息群发，登录注册</t>
+          <t>预警规则配置，指标库管理，评级模型管理，用户权限管理，债券池配置管理</t>
         </is>
       </c>
       <c r="F179" s="11" t="inlineStr">
@@ -11895,20 +12536,20 @@
         </is>
       </c>
       <c r="H179" s="13" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="180" ht="20" customHeight="1">
       <c r="A180" s="26" t="inlineStr">
         <is>
-          <t>【P2】 TRS收益互换  (Total Return Swap)</t>
+          <t>【P2】 投顾服务  (Investment Advisory)</t>
         </is>
       </c>
     </row>
     <row r="181" ht="28" customHeight="1">
       <c r="A181" s="11" t="inlineStr">
         <is>
-          <t>TRS收益互换</t>
+          <t>投顾服务</t>
         </is>
       </c>
       <c r="B181" s="10" t="inlineStr">
@@ -11918,37 +12559,37 @@
       </c>
       <c r="C181" s="10" t="inlineStr">
         <is>
-          <t>F13-01</t>
+          <t>F12-01</t>
         </is>
       </c>
       <c r="D181" s="27" t="inlineStr">
         <is>
-          <t>TRS交易端</t>
+          <t>投顾工作台</t>
         </is>
       </c>
       <c r="E181" s="11" t="inlineStr">
         <is>
-          <t>报价提供，成交回报，对冲委托与自动对冲，请求报价，行情与资讯，历史确认</t>
+          <t>投顾人员操作界面，管理客户委托，上传研究报告，发送投资建议，查看客户反馈</t>
         </is>
       </c>
       <c r="F181" s="11" t="inlineStr">
         <is>
-          <t>功能完整/边界测试/集成冒烟/性能基线</t>
-        </is>
-      </c>
-      <c r="G181" s="23" t="inlineStr">
-        <is>
-          <t>高</t>
+          <t>功能测试通过/正确率100%</t>
+        </is>
+      </c>
+      <c r="G181" s="24" t="inlineStr">
+        <is>
+          <t>中</t>
         </is>
       </c>
       <c r="H181" s="13" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
     </row>
     <row r="182" ht="28" customHeight="1">
       <c r="A182" s="11" t="inlineStr">
         <is>
-          <t>TRS收益互换</t>
+          <t>投顾服务</t>
         </is>
       </c>
       <c r="B182" s="10" t="inlineStr">
@@ -11958,37 +12599,37 @@
       </c>
       <c r="C182" s="10" t="inlineStr">
         <is>
-          <t>F13-02</t>
+          <t>F12-02</t>
         </is>
       </c>
       <c r="D182" s="27" t="inlineStr">
         <is>
-          <t>TRS客户端</t>
+          <t>客户终端</t>
         </is>
       </c>
       <c r="E182" s="11" t="inlineStr">
         <is>
-          <t>开户申请，客户委托，出入金申请，合约持仓，标的持仓，资金管理，行情矩阵，自主下单</t>
+          <t>客户查看投资建议与分析报告，确认交易服务，查看账户净值走势、持仓明细、交易明细</t>
         </is>
       </c>
       <c r="F182" s="11" t="inlineStr">
         <is>
-          <t>功能完整/边界测试/集成冒烟/性能基线</t>
-        </is>
-      </c>
-      <c r="G182" s="23" t="inlineStr">
-        <is>
-          <t>高</t>
+          <t>功能测试通过/正确率100%</t>
+        </is>
+      </c>
+      <c r="G182" s="24" t="inlineStr">
+        <is>
+          <t>中</t>
         </is>
       </c>
       <c r="H182" s="13" t="n">
-        <v>25</v>
+        <v>20</v>
       </c>
     </row>
     <row r="183" ht="28" customHeight="1">
       <c r="A183" s="11" t="inlineStr">
         <is>
-          <t>TRS收益互换</t>
+          <t>投顾服务</t>
         </is>
       </c>
       <c r="B183" s="10" t="inlineStr">
@@ -11998,17 +12639,17 @@
       </c>
       <c r="C183" s="10" t="inlineStr">
         <is>
-          <t>F13-03</t>
+          <t>F12-03</t>
         </is>
       </c>
       <c r="D183" s="27" t="inlineStr">
         <is>
-          <t>TRS管理端</t>
+          <t>投资建议书管理</t>
         </is>
       </c>
       <c r="E183" s="11" t="inlineStr">
         <is>
-          <t>开户申请审批，合约成交管理，出入金审批，运营管理，对账，库存，对冲录入</t>
+          <t>投资建议书线上生成、审批、确认全流程，留痕追溯，客户电子签收</t>
         </is>
       </c>
       <c r="F183" s="11" t="inlineStr">
@@ -12022,13 +12663,13 @@
         </is>
       </c>
       <c r="H183" s="13" t="n">
-        <v>20</v>
+        <v>15</v>
       </c>
     </row>
     <row r="184" ht="28" customHeight="1">
       <c r="A184" s="11" t="inlineStr">
         <is>
-          <t>TRS收益互换</t>
+          <t>投顾服务</t>
         </is>
       </c>
       <c r="B184" s="10" t="inlineStr">
@@ -12038,17 +12679,17 @@
       </c>
       <c r="C184" s="10" t="inlineStr">
         <is>
-          <t>F13-04</t>
+          <t>F12-04</t>
         </is>
       </c>
       <c r="D184" s="27" t="inlineStr">
         <is>
-          <t>自动对冲</t>
+          <t>账户分析报告</t>
         </is>
       </c>
       <c r="E184" s="11" t="inlineStr">
         <is>
-          <t>对冲委托自动触发，对冲回报处理，风险校验，组合重叠分析，开平仓设置</t>
+          <t>账户净值走势、久期走势、归因分析、估值台账等核心数据展示及定期报告生成</t>
         </is>
       </c>
       <c r="F184" s="11" t="inlineStr">
@@ -12068,7 +12709,7 @@
     <row r="185" ht="28" customHeight="1">
       <c r="A185" s="11" t="inlineStr">
         <is>
-          <t>TRS收益互换</t>
+          <t>投顾服务</t>
         </is>
       </c>
       <c r="B185" s="10" t="inlineStr">
@@ -12078,17 +12719,17 @@
       </c>
       <c r="C185" s="10" t="inlineStr">
         <is>
-          <t>F13-05</t>
+          <t>F12-05</t>
         </is>
       </c>
       <c r="D185" s="27" t="inlineStr">
         <is>
-          <t>通知与确认文件</t>
+          <t>投研报告服务</t>
         </is>
       </c>
       <c r="E185" s="11" t="inlineStr">
         <is>
-          <t>企微通知提醒，确认书/结算单/估值报告/出入金通知自动生成并通过邮箱发送</t>
+          <t>日/周/月研究报告上传与推送，RPA自动获取基础数据，报告分类管理</t>
         </is>
       </c>
       <c r="F185" s="11" t="inlineStr">
@@ -12108,275 +12749,522 @@
     <row r="186" ht="28" customHeight="1">
       <c r="A186" s="11" t="inlineStr">
         <is>
+          <t>投顾服务</t>
+        </is>
+      </c>
+      <c r="B186" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="C186" s="10" t="inlineStr">
+        <is>
+          <t>F12-06</t>
+        </is>
+      </c>
+      <c r="D186" s="27" t="inlineStr">
+        <is>
+          <t>客户服务与基础服务</t>
+        </is>
+      </c>
+      <c r="E186" s="11" t="inlineStr">
+        <is>
+          <t>服务中心、消息中心、问卷系统；用户/账户/数据管理，消息群发，登录注册</t>
+        </is>
+      </c>
+      <c r="F186" s="11" t="inlineStr">
+        <is>
+          <t>功能测试通过</t>
+        </is>
+      </c>
+      <c r="G186" s="25" t="inlineStr">
+        <is>
+          <t>低</t>
+        </is>
+      </c>
+      <c r="H186" s="13" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="187" ht="20" customHeight="1">
+      <c r="A187" s="26" t="inlineStr">
+        <is>
+          <t>【P2】 TRS收益互换  (Total Return Swap)</t>
+        </is>
+      </c>
+    </row>
+    <row r="188" ht="28" customHeight="1">
+      <c r="A188" s="11" t="inlineStr">
+        <is>
           <t>TRS收益互换</t>
         </is>
       </c>
-      <c r="B186" s="10" t="inlineStr">
+      <c r="B188" s="10" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
       </c>
-      <c r="C186" s="10" t="inlineStr">
+      <c r="C188" s="10" t="inlineStr">
+        <is>
+          <t>F13-01</t>
+        </is>
+      </c>
+      <c r="D188" s="27" t="inlineStr">
+        <is>
+          <t>TRS交易端</t>
+        </is>
+      </c>
+      <c r="E188" s="11" t="inlineStr">
+        <is>
+          <t>报价提供，成交回报，对冲委托与自动对冲，请求报价，行情与资讯，历史确认</t>
+        </is>
+      </c>
+      <c r="F188" s="11" t="inlineStr">
+        <is>
+          <t>功能完整/边界测试/集成冒烟/性能基线</t>
+        </is>
+      </c>
+      <c r="G188" s="23" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="H188" s="13" t="n">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="189" ht="28" customHeight="1">
+      <c r="A189" s="11" t="inlineStr">
+        <is>
+          <t>TRS收益互换</t>
+        </is>
+      </c>
+      <c r="B189" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="C189" s="10" t="inlineStr">
+        <is>
+          <t>F13-02</t>
+        </is>
+      </c>
+      <c r="D189" s="27" t="inlineStr">
+        <is>
+          <t>TRS客户端</t>
+        </is>
+      </c>
+      <c r="E189" s="11" t="inlineStr">
+        <is>
+          <t>开户申请，客户委托，出入金申请，合约持仓，标的持仓，资金管理，行情矩阵，自主下单</t>
+        </is>
+      </c>
+      <c r="F189" s="11" t="inlineStr">
+        <is>
+          <t>功能完整/边界测试/集成冒烟/性能基线</t>
+        </is>
+      </c>
+      <c r="G189" s="23" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="H189" s="13" t="n">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="190" ht="28" customHeight="1">
+      <c r="A190" s="11" t="inlineStr">
+        <is>
+          <t>TRS收益互换</t>
+        </is>
+      </c>
+      <c r="B190" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="C190" s="10" t="inlineStr">
+        <is>
+          <t>F13-03</t>
+        </is>
+      </c>
+      <c r="D190" s="27" t="inlineStr">
+        <is>
+          <t>TRS管理端</t>
+        </is>
+      </c>
+      <c r="E190" s="11" t="inlineStr">
+        <is>
+          <t>开户申请审批，合约成交管理，出入金审批，运营管理，对账，库存，对冲录入</t>
+        </is>
+      </c>
+      <c r="F190" s="11" t="inlineStr">
+        <is>
+          <t>功能测试通过/正确率100%</t>
+        </is>
+      </c>
+      <c r="G190" s="24" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="H190" s="13" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="191" ht="28" customHeight="1">
+      <c r="A191" s="11" t="inlineStr">
+        <is>
+          <t>TRS收益互换</t>
+        </is>
+      </c>
+      <c r="B191" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="C191" s="10" t="inlineStr">
+        <is>
+          <t>F13-04</t>
+        </is>
+      </c>
+      <c r="D191" s="27" t="inlineStr">
+        <is>
+          <t>自动对冲</t>
+        </is>
+      </c>
+      <c r="E191" s="11" t="inlineStr">
+        <is>
+          <t>对冲委托自动触发，对冲回报处理，风险校验，组合重叠分析，开平仓设置</t>
+        </is>
+      </c>
+      <c r="F191" s="11" t="inlineStr">
+        <is>
+          <t>功能完整/边界测试/集成冒烟/性能基线</t>
+        </is>
+      </c>
+      <c r="G191" s="23" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="H191" s="13" t="n">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="192" ht="28" customHeight="1">
+      <c r="A192" s="11" t="inlineStr">
+        <is>
+          <t>TRS收益互换</t>
+        </is>
+      </c>
+      <c r="B192" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="C192" s="10" t="inlineStr">
+        <is>
+          <t>F13-05</t>
+        </is>
+      </c>
+      <c r="D192" s="27" t="inlineStr">
+        <is>
+          <t>通知与确认文件</t>
+        </is>
+      </c>
+      <c r="E192" s="11" t="inlineStr">
+        <is>
+          <t>企微通知提醒，确认书/结算单/估值报告/出入金通知自动生成并通过邮箱发送</t>
+        </is>
+      </c>
+      <c r="F192" s="11" t="inlineStr">
+        <is>
+          <t>功能测试通过/正确率100%</t>
+        </is>
+      </c>
+      <c r="G192" s="24" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="H192" s="13" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="193" ht="28" customHeight="1">
+      <c r="A193" s="11" t="inlineStr">
+        <is>
+          <t>TRS收益互换</t>
+        </is>
+      </c>
+      <c r="B193" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="C193" s="10" t="inlineStr">
         <is>
           <t>F13-06</t>
         </is>
       </c>
-      <c r="D186" s="27" t="inlineStr">
+      <c r="D193" s="27" t="inlineStr">
         <is>
           <t>系统集成</t>
         </is>
       </c>
-      <c r="E186" s="11" t="inlineStr">
+      <c r="E193" s="11" t="inlineStr">
         <is>
           <t>与衡泰系统客户信息同步，QTrade聊天记录同步，交易管理系统对接，银行流水对接</t>
         </is>
       </c>
-      <c r="F186" s="11" t="inlineStr">
+      <c r="F193" s="11" t="inlineStr">
         <is>
           <t>功能完整/边界测试/集成冒烟/性能基线</t>
         </is>
       </c>
-      <c r="G186" s="23" t="inlineStr">
+      <c r="G193" s="23" t="inlineStr">
         <is>
           <t>高</t>
         </is>
       </c>
-      <c r="H186" s="13" t="n">
+      <c r="H193" s="13" t="n">
         <v>25</v>
       </c>
     </row>
-    <row r="187" ht="20" customHeight="1">
-      <c r="A187" s="29" t="inlineStr">
+    <row r="194" ht="20" customHeight="1">
+      <c r="A194" s="29" t="inlineStr">
         <is>
           <t>【P3】 做市商系统  (Market Making)</t>
         </is>
       </c>
     </row>
-    <row r="188" ht="28" customHeight="1">
-      <c r="A188" s="16" t="inlineStr">
+    <row r="195" ht="28" customHeight="1">
+      <c r="A195" s="16" t="inlineStr">
         <is>
           <t>做市商系统</t>
         </is>
       </c>
-      <c r="B188" s="15" t="inlineStr">
+      <c r="B195" s="15" t="inlineStr">
         <is>
           <t>P3</t>
         </is>
       </c>
-      <c r="C188" s="15" t="inlineStr">
+      <c r="C195" s="15" t="inlineStr">
         <is>
           <t>F15-01</t>
         </is>
       </c>
-      <c r="D188" s="30" t="inlineStr">
+      <c r="D195" s="30" t="inlineStr">
         <is>
           <t>双边报价引擎</t>
         </is>
       </c>
-      <c r="E188" s="16" t="inlineStr">
+      <c r="E195" s="16" t="inlineStr">
         <is>
           <t>多品种同时双边报价，延迟&lt;5ms，报价宽度动态优化</t>
         </is>
       </c>
-      <c r="F188" s="16" t="inlineStr">
+      <c r="F195" s="16" t="inlineStr">
         <is>
           <t>p99延迟/误差率/精度验证/压测10k TPS</t>
         </is>
       </c>
-      <c r="G188" s="28" t="inlineStr">
+      <c r="G195" s="28" t="inlineStr">
         <is>
           <t>极高</t>
         </is>
       </c>
-      <c r="H188" s="18" t="n">
+      <c r="H195" s="18" t="n">
         <v>70</v>
       </c>
     </row>
-    <row r="189" ht="28" customHeight="1">
-      <c r="A189" s="16" t="inlineStr">
+    <row r="196" ht="28" customHeight="1">
+      <c r="A196" s="16" t="inlineStr">
         <is>
           <t>做市商系统</t>
         </is>
       </c>
-      <c r="B189" s="15" t="inlineStr">
+      <c r="B196" s="15" t="inlineStr">
         <is>
           <t>P3</t>
         </is>
       </c>
-      <c r="C189" s="15" t="inlineStr">
+      <c r="C196" s="15" t="inlineStr">
         <is>
           <t>F15-02</t>
         </is>
       </c>
-      <c r="D189" s="30" t="inlineStr">
+      <c r="D196" s="30" t="inlineStr">
         <is>
           <t>库存风险实时管理</t>
         </is>
       </c>
-      <c r="E189" s="16" t="inlineStr">
+      <c r="E196" s="16" t="inlineStr">
         <is>
           <t>做市库存PnL实时监控，Delta对冲自动触发</t>
         </is>
       </c>
-      <c r="F189" s="16" t="inlineStr">
+      <c r="F196" s="16" t="inlineStr">
         <is>
           <t>p99延迟/误差率/精度验证/压测10k TPS</t>
         </is>
       </c>
-      <c r="G189" s="28" t="inlineStr">
+      <c r="G196" s="28" t="inlineStr">
         <is>
           <t>极高</t>
         </is>
       </c>
-      <c r="H189" s="18" t="n">
+      <c r="H196" s="18" t="n">
         <v>60</v>
       </c>
     </row>
-    <row r="190" ht="28" customHeight="1">
-      <c r="A190" s="16" t="inlineStr">
+    <row r="197" ht="28" customHeight="1">
+      <c r="A197" s="16" t="inlineStr">
         <is>
           <t>做市商系统</t>
         </is>
       </c>
-      <c r="B190" s="15" t="inlineStr">
+      <c r="B197" s="15" t="inlineStr">
         <is>
           <t>P3</t>
         </is>
       </c>
-      <c r="C190" s="15" t="inlineStr">
+      <c r="C197" s="15" t="inlineStr">
         <is>
           <t>F15-03</t>
         </is>
       </c>
-      <c r="D190" s="30" t="inlineStr">
+      <c r="D197" s="30" t="inlineStr">
         <is>
           <t>报价优化算法</t>
         </is>
       </c>
-      <c r="E190" s="16" t="inlineStr">
+      <c r="E197" s="16" t="inlineStr">
         <is>
           <t>基于市场微结构理论动态调整bid-ask spread</t>
         </is>
       </c>
-      <c r="F190" s="16" t="inlineStr">
+      <c r="F197" s="16" t="inlineStr">
         <is>
           <t>p99延迟/误差率/精度验证/压测10k TPS</t>
         </is>
       </c>
-      <c r="G190" s="28" t="inlineStr">
+      <c r="G197" s="28" t="inlineStr">
         <is>
           <t>极高</t>
         </is>
       </c>
-      <c r="H190" s="18" t="n">
+      <c r="H197" s="18" t="n">
         <v>50</v>
       </c>
     </row>
-    <row r="191" ht="28" customHeight="1">
-      <c r="A191" s="16" t="inlineStr">
+    <row r="198" ht="28" customHeight="1">
+      <c r="A198" s="16" t="inlineStr">
         <is>
           <t>做市商系统</t>
         </is>
       </c>
-      <c r="B191" s="15" t="inlineStr">
+      <c r="B198" s="15" t="inlineStr">
         <is>
           <t>P3</t>
         </is>
       </c>
-      <c r="C191" s="15" t="inlineStr">
+      <c r="C198" s="15" t="inlineStr">
         <is>
           <t>F15-04</t>
         </is>
       </c>
-      <c r="D191" s="30" t="inlineStr">
+      <c r="D198" s="30" t="inlineStr">
         <is>
           <t>竞争力分析</t>
         </is>
       </c>
-      <c r="E191" s="16" t="inlineStr">
+      <c r="E198" s="16" t="inlineStr">
         <is>
           <t>与市场最优报价对比，中签率分析，策略调优</t>
         </is>
       </c>
-      <c r="F191" s="16" t="inlineStr">
+      <c r="F198" s="16" t="inlineStr">
         <is>
           <t>功能完整/边界测试/集成冒烟/性能基线</t>
         </is>
       </c>
-      <c r="G191" s="23" t="inlineStr">
+      <c r="G198" s="23" t="inlineStr">
         <is>
           <t>高</t>
         </is>
       </c>
-      <c r="H191" s="18" t="n">
+      <c r="H198" s="18" t="n">
         <v>25</v>
       </c>
     </row>
-    <row r="192" ht="28" customHeight="1">
-      <c r="A192" s="16" t="inlineStr">
+    <row r="199" ht="28" customHeight="1">
+      <c r="A199" s="16" t="inlineStr">
         <is>
           <t>做市商系统</t>
         </is>
       </c>
-      <c r="B192" s="15" t="inlineStr">
+      <c r="B199" s="15" t="inlineStr">
         <is>
           <t>P3</t>
         </is>
       </c>
-      <c r="C192" s="15" t="inlineStr">
+      <c r="C199" s="15" t="inlineStr">
         <is>
           <t>F15-05</t>
         </is>
       </c>
-      <c r="D192" s="30" t="inlineStr">
+      <c r="D199" s="30" t="inlineStr">
         <is>
           <t>交易对手管理集成</t>
         </is>
       </c>
-      <c r="E192" s="16" t="inlineStr">
+      <c r="E199" s="16" t="inlineStr">
         <is>
           <t>做市交易对手信用实时检查，额度占用同步更新</t>
         </is>
       </c>
-      <c r="F192" s="16" t="inlineStr">
+      <c r="F199" s="16" t="inlineStr">
         <is>
           <t>功能测试通过/正确率100%</t>
         </is>
       </c>
-      <c r="G192" s="24" t="inlineStr">
+      <c r="G199" s="24" t="inlineStr">
         <is>
           <t>中</t>
         </is>
       </c>
-      <c r="H192" s="18" t="n">
+      <c r="H199" s="18" t="n">
         <v>20</v>
       </c>
     </row>
-    <row r="193">
-      <c r="A193" s="19" t="inlineStr">
+    <row r="200">
+      <c r="A200" s="19" t="inlineStr">
         <is>
           <t>总计功能数 / Total Function Points</t>
         </is>
       </c>
-      <c r="H193" s="20">
-        <f>SUM(H3:H192)</f>
+      <c r="H200" s="20">
+        <f>SUM(H3:H199)</f>
         <v/>
       </c>
     </row>
   </sheetData>
   <mergeCells count="16">
     <mergeCell ref="A143:H143"/>
-    <mergeCell ref="A193:G193"/>
     <mergeCell ref="A3:H3"/>
     <mergeCell ref="A101:H101"/>
     <mergeCell ref="A130:H130"/>
     <mergeCell ref="A180:H180"/>
     <mergeCell ref="A187:H187"/>
+    <mergeCell ref="A200:G200"/>
     <mergeCell ref="A60:H60"/>
     <mergeCell ref="A112:H112"/>
     <mergeCell ref="A68:H68"/>
     <mergeCell ref="A1:H1"/>
-    <mergeCell ref="A173:H173"/>
+    <mergeCell ref="A194:H194"/>
     <mergeCell ref="A31:H31"/>
     <mergeCell ref="A159:H159"/>
     <mergeCell ref="A88:H88"/>

</xml_diff>

<commit_message>
Expand module 12 投顾服务: 8 functions/3 domains + tech_design
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Feasibility_analysis/FICC_Gap_Analysis.xlsx
+++ b/Feasibility_analysis/FICC_Gap_Analysis.xlsx
@@ -22,6 +22,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="详情_定价平台" sheetId="13" state="visible" r:id="rId13"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="详情_销售交易" sheetId="14" state="visible" r:id="rId14"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="详情_信用债_信用衍生品" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="详情_投顾服务" sheetId="16" state="visible" r:id="rId16"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Area" localSheetId="0">'差距分析总表'!$A$1:$P$17</definedName>
@@ -1726,13 +1727,13 @@
         </is>
       </c>
       <c r="M14" s="10" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="N14" s="10" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="O14" s="13" t="n">
-        <v>14</v>
+        <v>20</v>
       </c>
       <c r="P14" s="11" t="inlineStr">
         <is>
@@ -5754,13 +5755,460 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J16"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="48" customWidth="1" min="4" max="4"/>
+    <col width="26" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="6" max="6"/>
+    <col width="8" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="8" max="8"/>
+    <col width="7" customWidth="1" min="9" max="9"/>
+    <col width="18" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="24" customHeight="1">
+      <c r="A1" s="38" t="inlineStr">
+        <is>
+          <t>系统详情：投顾服务  |  Investment Advisory</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="36" customHeight="1">
+      <c r="A2" s="39" t="inlineStr">
+        <is>
+          <t>战略定位：全链条数字化债券投顾服务，覆盖投资建议、账户分析、投研报告；对应PPT Slide 48   |   来源：Slide 48</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="28" customHeight="1">
+      <c r="A3" s="40" t="inlineStr">
+        <is>
+          <t>模块：投顾服务  (Investment Advisory)  |  优先级：P2  |  竞品：衡泰/金证  |  华锐基础：IBOR持仓账薄  |  工期：5月  团队：5人</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="28" customHeight="1">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>功能域</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>编号</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>功能名称</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>功能描述</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>验收标准</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>集成依赖</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>复杂度</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>预估(人天)</t>
+        </is>
+      </c>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t>优先级</t>
+        </is>
+      </c>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>备注</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="18" customHeight="1">
+      <c r="A5" s="22" t="inlineStr">
+        <is>
+          <t>D1. 投顾工作台</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="48" customHeight="1">
+      <c r="A6" s="11" t="inlineStr">
+        <is>
+          <t>D1. 投顾工作台</t>
+        </is>
+      </c>
+      <c r="B6" s="10" t="inlineStr">
+        <is>
+          <t>F12-01</t>
+        </is>
+      </c>
+      <c r="C6" s="27" t="inlineStr">
+        <is>
+          <t>投顾操作工作台</t>
+        </is>
+      </c>
+      <c r="D6" s="11" t="inlineStr">
+        <is>
+          <t>投顾人员管理客户委托，上传研究报告，发送投资建议，查看客户反馈与确认状态</t>
+        </is>
+      </c>
+      <c r="E6" s="11" t="inlineStr"/>
+      <c r="F6" s="11" t="inlineStr"/>
+      <c r="G6" s="42" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="H6" s="13" t="n">
+        <v>20</v>
+      </c>
+      <c r="I6" s="12" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="J6" s="11" t="inlineStr"/>
+    </row>
+    <row r="7" ht="48" customHeight="1">
+      <c r="A7" s="11" t="inlineStr">
+        <is>
+          <t>D1. 投顾工作台</t>
+        </is>
+      </c>
+      <c r="B7" s="10" t="inlineStr">
+        <is>
+          <t>F12-02</t>
+        </is>
+      </c>
+      <c r="C7" s="27" t="inlineStr">
+        <is>
+          <t>投资建议书管理</t>
+        </is>
+      </c>
+      <c r="D7" s="11" t="inlineStr">
+        <is>
+          <t>投资建议书线上生成与审批，客户确认全流程，留痕追溯，电子签收，历史建议书归档</t>
+        </is>
+      </c>
+      <c r="E7" s="11" t="inlineStr"/>
+      <c r="F7" s="11" t="inlineStr"/>
+      <c r="G7" s="42" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="H7" s="13" t="n">
+        <v>20</v>
+      </c>
+      <c r="I7" s="12" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="J7" s="11" t="inlineStr"/>
+    </row>
+    <row r="8" ht="48" customHeight="1">
+      <c r="A8" s="11" t="inlineStr">
+        <is>
+          <t>D1. 投顾工作台</t>
+        </is>
+      </c>
+      <c r="B8" s="10" t="inlineStr">
+        <is>
+          <t>F12-03</t>
+        </is>
+      </c>
+      <c r="C8" s="27" t="inlineStr">
+        <is>
+          <t>投研报告服务</t>
+        </is>
+      </c>
+      <c r="D8" s="11" t="inlineStr">
+        <is>
+          <t>日/周/月研究报告上传与定向推送，RPA自动获取基础数据，报告分类管理与检索</t>
+        </is>
+      </c>
+      <c r="E8" s="11" t="inlineStr"/>
+      <c r="F8" s="11" t="inlineStr"/>
+      <c r="G8" s="42" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="H8" s="13" t="n">
+        <v>15</v>
+      </c>
+      <c r="I8" s="12" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="J8" s="11" t="inlineStr"/>
+    </row>
+    <row r="9" ht="18" customHeight="1">
+      <c r="A9" s="40" t="inlineStr">
+        <is>
+          <t>D2. 客户终端</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="48" customHeight="1">
+      <c r="A10" s="11" t="inlineStr">
+        <is>
+          <t>D2. 客户终端</t>
+        </is>
+      </c>
+      <c r="B10" s="10" t="inlineStr">
+        <is>
+          <t>F12-04</t>
+        </is>
+      </c>
+      <c r="C10" s="27" t="inlineStr">
+        <is>
+          <t>客户投资服务界面</t>
+        </is>
+      </c>
+      <c r="D10" s="11" t="inlineStr">
+        <is>
+          <t>客户查看投资建议与分析报告，发送确认，查看账户净值走势、持仓明细、交易明细</t>
+        </is>
+      </c>
+      <c r="E10" s="11" t="inlineStr"/>
+      <c r="F10" s="11" t="inlineStr"/>
+      <c r="G10" s="42" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="H10" s="13" t="n">
+        <v>20</v>
+      </c>
+      <c r="I10" s="12" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="J10" s="11" t="inlineStr"/>
+    </row>
+    <row r="11" ht="48" customHeight="1">
+      <c r="A11" s="11" t="inlineStr">
+        <is>
+          <t>D2. 客户终端</t>
+        </is>
+      </c>
+      <c r="B11" s="10" t="inlineStr">
+        <is>
+          <t>F12-05</t>
+        </is>
+      </c>
+      <c r="C11" s="27" t="inlineStr">
+        <is>
+          <t>账户深度分析</t>
+        </is>
+      </c>
+      <c r="D11" s="11" t="inlineStr">
+        <is>
+          <t>账户净值走势，久期走势，归因分析，估值台账，持仓明细，交易明细，定期分析报告生成</t>
+        </is>
+      </c>
+      <c r="E11" s="11" t="inlineStr"/>
+      <c r="F11" s="11" t="inlineStr"/>
+      <c r="G11" s="41" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="H11" s="13" t="n">
+        <v>25</v>
+      </c>
+      <c r="I11" s="12" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="J11" s="11" t="inlineStr"/>
+    </row>
+    <row r="12" ht="48" customHeight="1">
+      <c r="A12" s="11" t="inlineStr">
+        <is>
+          <t>D2. 客户终端</t>
+        </is>
+      </c>
+      <c r="B12" s="10" t="inlineStr">
+        <is>
+          <t>F12-06</t>
+        </is>
+      </c>
+      <c r="C12" s="27" t="inlineStr">
+        <is>
+          <t>交易服务对接</t>
+        </is>
+      </c>
+      <c r="D12" s="11" t="inlineStr">
+        <is>
+          <t>客户查看投资建议后直接触发交易委托，与销售交易系统对接，全程数字化交易确认</t>
+        </is>
+      </c>
+      <c r="E12" s="11" t="inlineStr"/>
+      <c r="F12" s="11" t="inlineStr"/>
+      <c r="G12" s="42" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="H12" s="13" t="n">
+        <v>15</v>
+      </c>
+      <c r="I12" s="12" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="J12" s="11" t="inlineStr"/>
+    </row>
+    <row r="13" ht="18" customHeight="1">
+      <c r="A13" s="43" t="inlineStr">
+        <is>
+          <t>D3. 基础服务</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="48" customHeight="1">
+      <c r="A14" s="11" t="inlineStr">
+        <is>
+          <t>D3. 基础服务</t>
+        </is>
+      </c>
+      <c r="B14" s="10" t="inlineStr">
+        <is>
+          <t>F12-07</t>
+        </is>
+      </c>
+      <c r="C14" s="27" t="inlineStr">
+        <is>
+          <t>客户服务中心</t>
+        </is>
+      </c>
+      <c r="D14" s="11" t="inlineStr">
+        <is>
+          <t>服务中心，消息中心，常见问题，问卷系统，客户满意度管理</t>
+        </is>
+      </c>
+      <c r="E14" s="11" t="inlineStr"/>
+      <c r="F14" s="11" t="inlineStr"/>
+      <c r="G14" s="42" t="inlineStr">
+        <is>
+          <t>低</t>
+        </is>
+      </c>
+      <c r="H14" s="13" t="n">
+        <v>10</v>
+      </c>
+      <c r="I14" s="12" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="J14" s="11" t="inlineStr"/>
+    </row>
+    <row r="15" ht="48" customHeight="1">
+      <c r="A15" s="11" t="inlineStr">
+        <is>
+          <t>D3. 基础服务</t>
+        </is>
+      </c>
+      <c r="B15" s="10" t="inlineStr">
+        <is>
+          <t>F12-08</t>
+        </is>
+      </c>
+      <c r="C15" s="27" t="inlineStr">
+        <is>
+          <t>平台基础管理</t>
+        </is>
+      </c>
+      <c r="D15" s="11" t="inlineStr">
+        <is>
+          <t>用户管理，账户管理，数据管理，消息群发，登录注册，权限控制</t>
+        </is>
+      </c>
+      <c r="E15" s="11" t="inlineStr"/>
+      <c r="F15" s="11" t="inlineStr"/>
+      <c r="G15" s="42" t="inlineStr">
+        <is>
+          <t>低</t>
+        </is>
+      </c>
+      <c r="H15" s="13" t="n">
+        <v>10</v>
+      </c>
+      <c r="I15" s="12" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="J15" s="11" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="40" t="inlineStr">
+        <is>
+          <t>合计 8项功能  |  P1: 0项  |  P2: 8项</t>
+        </is>
+      </c>
+      <c r="H16" s="20">
+        <f>SUM(H5:H15)</f>
+        <v/>
+      </c>
+      <c r="I16" s="34" t="inlineStr"/>
+      <c r="J16" s="34" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <mergeCells count="7">
+    <mergeCell ref="A1:J1"/>
+    <mergeCell ref="A5:J5"/>
+    <mergeCell ref="A9:J9"/>
+    <mergeCell ref="A3:J3"/>
+    <mergeCell ref="A16:G16"/>
+    <mergeCell ref="A2:J2"/>
+    <mergeCell ref="A13:J13"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" fitToWidth="1"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H200"/>
+  <dimension ref="A1:H202"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -12564,12 +13012,12 @@
       </c>
       <c r="D181" s="27" t="inlineStr">
         <is>
-          <t>投顾工作台</t>
+          <t>投顾操作工作台</t>
         </is>
       </c>
       <c r="E181" s="11" t="inlineStr">
         <is>
-          <t>投顾人员操作界面，管理客户委托，上传研究报告，发送投资建议，查看客户反馈</t>
+          <t>投顾人员管理客户委托，上传研究报告，发送投资建议，查看客户反馈与确认状态</t>
         </is>
       </c>
       <c r="F181" s="11" t="inlineStr">
@@ -12604,12 +13052,12 @@
       </c>
       <c r="D182" s="27" t="inlineStr">
         <is>
-          <t>客户终端</t>
+          <t>投资建议书管理</t>
         </is>
       </c>
       <c r="E182" s="11" t="inlineStr">
         <is>
-          <t>客户查看投资建议与分析报告，确认交易服务，查看账户净值走势、持仓明细、交易明细</t>
+          <t>投资建议书线上生成与审批，客户确认全流程，留痕追溯，电子签收，历史建议书归档</t>
         </is>
       </c>
       <c r="F182" s="11" t="inlineStr">
@@ -12644,12 +13092,12 @@
       </c>
       <c r="D183" s="27" t="inlineStr">
         <is>
-          <t>投资建议书管理</t>
+          <t>投研报告服务</t>
         </is>
       </c>
       <c r="E183" s="11" t="inlineStr">
         <is>
-          <t>投资建议书线上生成、审批、确认全流程，留痕追溯，客户电子签收</t>
+          <t>日/周/月研究报告上传与定向推送，RPA自动获取基础数据，报告分类管理与检索</t>
         </is>
       </c>
       <c r="F183" s="11" t="inlineStr">
@@ -12684,26 +13132,26 @@
       </c>
       <c r="D184" s="27" t="inlineStr">
         <is>
-          <t>账户分析报告</t>
+          <t>客户投资服务界面</t>
         </is>
       </c>
       <c r="E184" s="11" t="inlineStr">
         <is>
-          <t>账户净值走势、久期走势、归因分析、估值台账等核心数据展示及定期报告生成</t>
+          <t>客户查看投资建议与分析报告，发送确认，查看账户净值走势、持仓明细、交易明细</t>
         </is>
       </c>
       <c r="F184" s="11" t="inlineStr">
         <is>
-          <t>功能完整/边界测试/集成冒烟/性能基线</t>
-        </is>
-      </c>
-      <c r="G184" s="23" t="inlineStr">
-        <is>
-          <t>高</t>
+          <t>功能测试通过/正确率100%</t>
+        </is>
+      </c>
+      <c r="G184" s="24" t="inlineStr">
+        <is>
+          <t>中</t>
         </is>
       </c>
       <c r="H184" s="13" t="n">
-        <v>25</v>
+        <v>20</v>
       </c>
     </row>
     <row r="185" ht="28" customHeight="1">
@@ -12724,26 +13172,26 @@
       </c>
       <c r="D185" s="27" t="inlineStr">
         <is>
-          <t>投研报告服务</t>
+          <t>账户深度分析</t>
         </is>
       </c>
       <c r="E185" s="11" t="inlineStr">
         <is>
-          <t>日/周/月研究报告上传与推送，RPA自动获取基础数据，报告分类管理</t>
+          <t>账户净值走势，久期走势，归因分析，估值台账，持仓明细，交易明细，定期分析报告生成</t>
         </is>
       </c>
       <c r="F185" s="11" t="inlineStr">
         <is>
-          <t>功能测试通过/正确率100%</t>
-        </is>
-      </c>
-      <c r="G185" s="24" t="inlineStr">
-        <is>
-          <t>中</t>
+          <t>功能完整/边界测试/集成冒烟/性能基线</t>
+        </is>
+      </c>
+      <c r="G185" s="23" t="inlineStr">
+        <is>
+          <t>高</t>
         </is>
       </c>
       <c r="H185" s="13" t="n">
-        <v>15</v>
+        <v>25</v>
       </c>
     </row>
     <row r="186" ht="28" customHeight="1">
@@ -12764,39 +13212,72 @@
       </c>
       <c r="D186" s="27" t="inlineStr">
         <is>
-          <t>客户服务与基础服务</t>
+          <t>交易服务对接</t>
         </is>
       </c>
       <c r="E186" s="11" t="inlineStr">
         <is>
-          <t>服务中心、消息中心、问卷系统；用户/账户/数据管理，消息群发，登录注册</t>
+          <t>客户查看投资建议后直接触发交易委托，与销售交易系统对接，全程数字化交易确认</t>
         </is>
       </c>
       <c r="F186" s="11" t="inlineStr">
         <is>
+          <t>功能测试通过/正确率100%</t>
+        </is>
+      </c>
+      <c r="G186" s="24" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="H186" s="13" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="187" ht="28" customHeight="1">
+      <c r="A187" s="11" t="inlineStr">
+        <is>
+          <t>投顾服务</t>
+        </is>
+      </c>
+      <c r="B187" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="C187" s="10" t="inlineStr">
+        <is>
+          <t>F12-07</t>
+        </is>
+      </c>
+      <c r="D187" s="27" t="inlineStr">
+        <is>
+          <t>客户服务中心</t>
+        </is>
+      </c>
+      <c r="E187" s="11" t="inlineStr">
+        <is>
+          <t>服务中心，消息中心，常见问题，问卷系统，客户满意度管理</t>
+        </is>
+      </c>
+      <c r="F187" s="11" t="inlineStr">
+        <is>
           <t>功能测试通过</t>
         </is>
       </c>
-      <c r="G186" s="25" t="inlineStr">
+      <c r="G187" s="25" t="inlineStr">
         <is>
           <t>低</t>
         </is>
       </c>
-      <c r="H186" s="13" t="n">
+      <c r="H187" s="13" t="n">
         <v>10</v>
-      </c>
-    </row>
-    <row r="187" ht="20" customHeight="1">
-      <c r="A187" s="26" t="inlineStr">
-        <is>
-          <t>【P2】 TRS收益互换  (Total Return Swap)</t>
-        </is>
       </c>
     </row>
     <row r="188" ht="28" customHeight="1">
       <c r="A188" s="11" t="inlineStr">
         <is>
-          <t>TRS收益互换</t>
+          <t>投顾服务</t>
         </is>
       </c>
       <c r="B188" s="10" t="inlineStr">
@@ -12806,71 +13287,38 @@
       </c>
       <c r="C188" s="10" t="inlineStr">
         <is>
-          <t>F13-01</t>
+          <t>F12-08</t>
         </is>
       </c>
       <c r="D188" s="27" t="inlineStr">
         <is>
-          <t>TRS交易端</t>
+          <t>平台基础管理</t>
         </is>
       </c>
       <c r="E188" s="11" t="inlineStr">
         <is>
-          <t>报价提供，成交回报，对冲委托与自动对冲，请求报价，行情与资讯，历史确认</t>
+          <t>用户管理，账户管理，数据管理，消息群发，登录注册，权限控制</t>
         </is>
       </c>
       <c r="F188" s="11" t="inlineStr">
         <is>
-          <t>功能完整/边界测试/集成冒烟/性能基线</t>
-        </is>
-      </c>
-      <c r="G188" s="23" t="inlineStr">
-        <is>
-          <t>高</t>
+          <t>功能测试通过</t>
+        </is>
+      </c>
+      <c r="G188" s="25" t="inlineStr">
+        <is>
+          <t>低</t>
         </is>
       </c>
       <c r="H188" s="13" t="n">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="189" ht="28" customHeight="1">
-      <c r="A189" s="11" t="inlineStr">
-        <is>
-          <t>TRS收益互换</t>
-        </is>
-      </c>
-      <c r="B189" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
-        </is>
-      </c>
-      <c r="C189" s="10" t="inlineStr">
-        <is>
-          <t>F13-02</t>
-        </is>
-      </c>
-      <c r="D189" s="27" t="inlineStr">
-        <is>
-          <t>TRS客户端</t>
-        </is>
-      </c>
-      <c r="E189" s="11" t="inlineStr">
-        <is>
-          <t>开户申请，客户委托，出入金申请，合约持仓，标的持仓，资金管理，行情矩阵，自主下单</t>
-        </is>
-      </c>
-      <c r="F189" s="11" t="inlineStr">
-        <is>
-          <t>功能完整/边界测试/集成冒烟/性能基线</t>
-        </is>
-      </c>
-      <c r="G189" s="23" t="inlineStr">
-        <is>
-          <t>高</t>
-        </is>
-      </c>
-      <c r="H189" s="13" t="n">
-        <v>25</v>
+        <v>10</v>
+      </c>
+    </row>
+    <row r="189" ht="20" customHeight="1">
+      <c r="A189" s="26" t="inlineStr">
+        <is>
+          <t>【P2】 TRS收益互换  (Total Return Swap)</t>
+        </is>
       </c>
     </row>
     <row r="190" ht="28" customHeight="1">
@@ -12886,31 +13334,31 @@
       </c>
       <c r="C190" s="10" t="inlineStr">
         <is>
-          <t>F13-03</t>
+          <t>F13-01</t>
         </is>
       </c>
       <c r="D190" s="27" t="inlineStr">
         <is>
-          <t>TRS管理端</t>
+          <t>TRS交易端</t>
         </is>
       </c>
       <c r="E190" s="11" t="inlineStr">
         <is>
-          <t>开户申请审批，合约成交管理，出入金审批，运营管理，对账，库存，对冲录入</t>
+          <t>报价提供，成交回报，对冲委托与自动对冲，请求报价，行情与资讯，历史确认</t>
         </is>
       </c>
       <c r="F190" s="11" t="inlineStr">
         <is>
-          <t>功能测试通过/正确率100%</t>
-        </is>
-      </c>
-      <c r="G190" s="24" t="inlineStr">
-        <is>
-          <t>中</t>
+          <t>功能完整/边界测试/集成冒烟/性能基线</t>
+        </is>
+      </c>
+      <c r="G190" s="23" t="inlineStr">
+        <is>
+          <t>高</t>
         </is>
       </c>
       <c r="H190" s="13" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
     </row>
     <row r="191" ht="28" customHeight="1">
@@ -12926,17 +13374,17 @@
       </c>
       <c r="C191" s="10" t="inlineStr">
         <is>
-          <t>F13-04</t>
+          <t>F13-02</t>
         </is>
       </c>
       <c r="D191" s="27" t="inlineStr">
         <is>
-          <t>自动对冲</t>
+          <t>TRS客户端</t>
         </is>
       </c>
       <c r="E191" s="11" t="inlineStr">
         <is>
-          <t>对冲委托自动触发，对冲回报处理，风险校验，组合重叠分析，开平仓设置</t>
+          <t>开户申请，客户委托，出入金申请，合约持仓，标的持仓，资金管理，行情矩阵，自主下单</t>
         </is>
       </c>
       <c r="F191" s="11" t="inlineStr">
@@ -12966,17 +13414,17 @@
       </c>
       <c r="C192" s="10" t="inlineStr">
         <is>
-          <t>F13-05</t>
+          <t>F13-03</t>
         </is>
       </c>
       <c r="D192" s="27" t="inlineStr">
         <is>
-          <t>通知与确认文件</t>
+          <t>TRS管理端</t>
         </is>
       </c>
       <c r="E192" s="11" t="inlineStr">
         <is>
-          <t>企微通知提醒，确认书/结算单/估值报告/出入金通知自动生成并通过邮箱发送</t>
+          <t>开户申请审批，合约成交管理，出入金审批，运营管理，对账，库存，对冲录入</t>
         </is>
       </c>
       <c r="F192" s="11" t="inlineStr">
@@ -12990,7 +13438,7 @@
         </is>
       </c>
       <c r="H192" s="13" t="n">
-        <v>15</v>
+        <v>20</v>
       </c>
     </row>
     <row r="193" ht="28" customHeight="1">
@@ -13006,17 +13454,17 @@
       </c>
       <c r="C193" s="10" t="inlineStr">
         <is>
-          <t>F13-06</t>
+          <t>F13-04</t>
         </is>
       </c>
       <c r="D193" s="27" t="inlineStr">
         <is>
-          <t>系统集成</t>
+          <t>自动对冲</t>
         </is>
       </c>
       <c r="E193" s="11" t="inlineStr">
         <is>
-          <t>与衡泰系统客户信息同步，QTrade聊天记录同步，交易管理系统对接，银行流水对接</t>
+          <t>对冲委托自动触发，对冲回报处理，风险校验，组合重叠分析，开平仓设置</t>
         </is>
       </c>
       <c r="F193" s="11" t="inlineStr">
@@ -13033,91 +13481,91 @@
         <v>25</v>
       </c>
     </row>
-    <row r="194" ht="20" customHeight="1">
-      <c r="A194" s="29" t="inlineStr">
+    <row r="194" ht="28" customHeight="1">
+      <c r="A194" s="11" t="inlineStr">
+        <is>
+          <t>TRS收益互换</t>
+        </is>
+      </c>
+      <c r="B194" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="C194" s="10" t="inlineStr">
+        <is>
+          <t>F13-05</t>
+        </is>
+      </c>
+      <c r="D194" s="27" t="inlineStr">
+        <is>
+          <t>通知与确认文件</t>
+        </is>
+      </c>
+      <c r="E194" s="11" t="inlineStr">
+        <is>
+          <t>企微通知提醒，确认书/结算单/估值报告/出入金通知自动生成并通过邮箱发送</t>
+        </is>
+      </c>
+      <c r="F194" s="11" t="inlineStr">
+        <is>
+          <t>功能测试通过/正确率100%</t>
+        </is>
+      </c>
+      <c r="G194" s="24" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="H194" s="13" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="195" ht="28" customHeight="1">
+      <c r="A195" s="11" t="inlineStr">
+        <is>
+          <t>TRS收益互换</t>
+        </is>
+      </c>
+      <c r="B195" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="C195" s="10" t="inlineStr">
+        <is>
+          <t>F13-06</t>
+        </is>
+      </c>
+      <c r="D195" s="27" t="inlineStr">
+        <is>
+          <t>系统集成</t>
+        </is>
+      </c>
+      <c r="E195" s="11" t="inlineStr">
+        <is>
+          <t>与衡泰系统客户信息同步，QTrade聊天记录同步，交易管理系统对接，银行流水对接</t>
+        </is>
+      </c>
+      <c r="F195" s="11" t="inlineStr">
+        <is>
+          <t>功能完整/边界测试/集成冒烟/性能基线</t>
+        </is>
+      </c>
+      <c r="G195" s="23" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="H195" s="13" t="n">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="196" ht="20" customHeight="1">
+      <c r="A196" s="29" t="inlineStr">
         <is>
           <t>【P3】 做市商系统  (Market Making)</t>
         </is>
-      </c>
-    </row>
-    <row r="195" ht="28" customHeight="1">
-      <c r="A195" s="16" t="inlineStr">
-        <is>
-          <t>做市商系统</t>
-        </is>
-      </c>
-      <c r="B195" s="15" t="inlineStr">
-        <is>
-          <t>P3</t>
-        </is>
-      </c>
-      <c r="C195" s="15" t="inlineStr">
-        <is>
-          <t>F15-01</t>
-        </is>
-      </c>
-      <c r="D195" s="30" t="inlineStr">
-        <is>
-          <t>双边报价引擎</t>
-        </is>
-      </c>
-      <c r="E195" s="16" t="inlineStr">
-        <is>
-          <t>多品种同时双边报价，延迟&lt;5ms，报价宽度动态优化</t>
-        </is>
-      </c>
-      <c r="F195" s="16" t="inlineStr">
-        <is>
-          <t>p99延迟/误差率/精度验证/压测10k TPS</t>
-        </is>
-      </c>
-      <c r="G195" s="28" t="inlineStr">
-        <is>
-          <t>极高</t>
-        </is>
-      </c>
-      <c r="H195" s="18" t="n">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="196" ht="28" customHeight="1">
-      <c r="A196" s="16" t="inlineStr">
-        <is>
-          <t>做市商系统</t>
-        </is>
-      </c>
-      <c r="B196" s="15" t="inlineStr">
-        <is>
-          <t>P3</t>
-        </is>
-      </c>
-      <c r="C196" s="15" t="inlineStr">
-        <is>
-          <t>F15-02</t>
-        </is>
-      </c>
-      <c r="D196" s="30" t="inlineStr">
-        <is>
-          <t>库存风险实时管理</t>
-        </is>
-      </c>
-      <c r="E196" s="16" t="inlineStr">
-        <is>
-          <t>做市库存PnL实时监控，Delta对冲自动触发</t>
-        </is>
-      </c>
-      <c r="F196" s="16" t="inlineStr">
-        <is>
-          <t>p99延迟/误差率/精度验证/压测10k TPS</t>
-        </is>
-      </c>
-      <c r="G196" s="28" t="inlineStr">
-        <is>
-          <t>极高</t>
-        </is>
-      </c>
-      <c r="H196" s="18" t="n">
-        <v>60</v>
       </c>
     </row>
     <row r="197" ht="28" customHeight="1">
@@ -13133,17 +13581,17 @@
       </c>
       <c r="C197" s="15" t="inlineStr">
         <is>
-          <t>F15-03</t>
+          <t>F15-01</t>
         </is>
       </c>
       <c r="D197" s="30" t="inlineStr">
         <is>
-          <t>报价优化算法</t>
+          <t>双边报价引擎</t>
         </is>
       </c>
       <c r="E197" s="16" t="inlineStr">
         <is>
-          <t>基于市场微结构理论动态调整bid-ask spread</t>
+          <t>多品种同时双边报价，延迟&lt;5ms，报价宽度动态优化</t>
         </is>
       </c>
       <c r="F197" s="16" t="inlineStr">
@@ -13157,7 +13605,7 @@
         </is>
       </c>
       <c r="H197" s="18" t="n">
-        <v>50</v>
+        <v>70</v>
       </c>
     </row>
     <row r="198" ht="28" customHeight="1">
@@ -13173,31 +13621,31 @@
       </c>
       <c r="C198" s="15" t="inlineStr">
         <is>
-          <t>F15-04</t>
+          <t>F15-02</t>
         </is>
       </c>
       <c r="D198" s="30" t="inlineStr">
         <is>
-          <t>竞争力分析</t>
+          <t>库存风险实时管理</t>
         </is>
       </c>
       <c r="E198" s="16" t="inlineStr">
         <is>
-          <t>与市场最优报价对比，中签率分析，策略调优</t>
+          <t>做市库存PnL实时监控，Delta对冲自动触发</t>
         </is>
       </c>
       <c r="F198" s="16" t="inlineStr">
         <is>
-          <t>功能完整/边界测试/集成冒烟/性能基线</t>
-        </is>
-      </c>
-      <c r="G198" s="23" t="inlineStr">
-        <is>
-          <t>高</t>
+          <t>p99延迟/误差率/精度验证/压测10k TPS</t>
+        </is>
+      </c>
+      <c r="G198" s="28" t="inlineStr">
+        <is>
+          <t>极高</t>
         </is>
       </c>
       <c r="H198" s="18" t="n">
-        <v>25</v>
+        <v>60</v>
       </c>
     </row>
     <row r="199" ht="28" customHeight="1">
@@ -13213,58 +13661,138 @@
       </c>
       <c r="C199" s="15" t="inlineStr">
         <is>
+          <t>F15-03</t>
+        </is>
+      </c>
+      <c r="D199" s="30" t="inlineStr">
+        <is>
+          <t>报价优化算法</t>
+        </is>
+      </c>
+      <c r="E199" s="16" t="inlineStr">
+        <is>
+          <t>基于市场微结构理论动态调整bid-ask spread</t>
+        </is>
+      </c>
+      <c r="F199" s="16" t="inlineStr">
+        <is>
+          <t>p99延迟/误差率/精度验证/压测10k TPS</t>
+        </is>
+      </c>
+      <c r="G199" s="28" t="inlineStr">
+        <is>
+          <t>极高</t>
+        </is>
+      </c>
+      <c r="H199" s="18" t="n">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="200" ht="28" customHeight="1">
+      <c r="A200" s="16" t="inlineStr">
+        <is>
+          <t>做市商系统</t>
+        </is>
+      </c>
+      <c r="B200" s="15" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="C200" s="15" t="inlineStr">
+        <is>
+          <t>F15-04</t>
+        </is>
+      </c>
+      <c r="D200" s="30" t="inlineStr">
+        <is>
+          <t>竞争力分析</t>
+        </is>
+      </c>
+      <c r="E200" s="16" t="inlineStr">
+        <is>
+          <t>与市场最优报价对比，中签率分析，策略调优</t>
+        </is>
+      </c>
+      <c r="F200" s="16" t="inlineStr">
+        <is>
+          <t>功能完整/边界测试/集成冒烟/性能基线</t>
+        </is>
+      </c>
+      <c r="G200" s="23" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="H200" s="18" t="n">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="201" ht="28" customHeight="1">
+      <c r="A201" s="16" t="inlineStr">
+        <is>
+          <t>做市商系统</t>
+        </is>
+      </c>
+      <c r="B201" s="15" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="C201" s="15" t="inlineStr">
+        <is>
           <t>F15-05</t>
         </is>
       </c>
-      <c r="D199" s="30" t="inlineStr">
+      <c r="D201" s="30" t="inlineStr">
         <is>
           <t>交易对手管理集成</t>
         </is>
       </c>
-      <c r="E199" s="16" t="inlineStr">
+      <c r="E201" s="16" t="inlineStr">
         <is>
           <t>做市交易对手信用实时检查，额度占用同步更新</t>
         </is>
       </c>
-      <c r="F199" s="16" t="inlineStr">
+      <c r="F201" s="16" t="inlineStr">
         <is>
           <t>功能测试通过/正确率100%</t>
         </is>
       </c>
-      <c r="G199" s="24" t="inlineStr">
+      <c r="G201" s="24" t="inlineStr">
         <is>
           <t>中</t>
         </is>
       </c>
-      <c r="H199" s="18" t="n">
+      <c r="H201" s="18" t="n">
         <v>20</v>
       </c>
     </row>
-    <row r="200">
-      <c r="A200" s="19" t="inlineStr">
+    <row r="202">
+      <c r="A202" s="19" t="inlineStr">
         <is>
           <t>总计功能数 / Total Function Points</t>
         </is>
       </c>
-      <c r="H200" s="20">
-        <f>SUM(H3:H199)</f>
+      <c r="H202" s="20">
+        <f>SUM(H3:H201)</f>
         <v/>
       </c>
     </row>
   </sheetData>
   <mergeCells count="16">
     <mergeCell ref="A143:H143"/>
+    <mergeCell ref="A202:G202"/>
     <mergeCell ref="A3:H3"/>
     <mergeCell ref="A101:H101"/>
     <mergeCell ref="A130:H130"/>
     <mergeCell ref="A180:H180"/>
-    <mergeCell ref="A187:H187"/>
-    <mergeCell ref="A200:G200"/>
+    <mergeCell ref="A196:H196"/>
     <mergeCell ref="A60:H60"/>
     <mergeCell ref="A112:H112"/>
     <mergeCell ref="A68:H68"/>
     <mergeCell ref="A1:H1"/>
-    <mergeCell ref="A194:H194"/>
+    <mergeCell ref="A189:H189"/>
     <mergeCell ref="A31:H31"/>
     <mergeCell ref="A159:H159"/>
     <mergeCell ref="A88:H88"/>

</xml_diff>

<commit_message>
Expand module 13 TRS收益互换: 10 functions/4 domains + tech_design
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Feasibility_analysis/FICC_Gap_Analysis.xlsx
+++ b/Feasibility_analysis/FICC_Gap_Analysis.xlsx
@@ -23,6 +23,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="详情_销售交易" sheetId="14" state="visible" r:id="rId14"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="详情_信用债_信用衍生品" sheetId="15" state="visible" r:id="rId15"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="详情_投顾服务" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="详情_TRS收益互换" sheetId="17" state="visible" r:id="rId17"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Area" localSheetId="0">'差距分析总表'!$A$1:$P$17</definedName>
@@ -1797,21 +1798,21 @@
       </c>
       <c r="L15" s="11" t="inlineStr">
         <is>
-          <t>现券交易系统/IBOR</t>
+          <t>现券交易系统/IBOR/定价平台</t>
         </is>
       </c>
       <c r="M15" s="10" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="N15" s="10" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="O15" s="13" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="P15" s="11" t="inlineStr">
         <is>
-          <t>场外衍生品主经纪商客需服务，覆盖TRS交易端/客户端/管理端及自动对冲；对应PPT Slide 49</t>
+          <t>场外衍生品主经纪商客需服务，三端架构（交易端/客户端/管理端），自动对冲与运营一体化；对应PPT Slide 49</t>
         </is>
       </c>
     </row>
@@ -6202,13 +6203,544 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J19"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="48" customWidth="1" min="4" max="4"/>
+    <col width="26" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="6" max="6"/>
+    <col width="8" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="8" max="8"/>
+    <col width="7" customWidth="1" min="9" max="9"/>
+    <col width="18" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="24" customHeight="1">
+      <c r="A1" s="38" t="inlineStr">
+        <is>
+          <t>系统详情：TRS收益互换  |  Total Return Swap</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="36" customHeight="1">
+      <c r="A2" s="39" t="inlineStr">
+        <is>
+          <t>战略定位：场外衍生品主经纪商客需服务，三端架构（交易端/客户端/管理端），自动对冲与运营一体化；对应PPT Slide 49   |   来源：Slide 49</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="28" customHeight="1">
+      <c r="A3" s="40" t="inlineStr">
+        <is>
+          <t>模块：TRS收益互换  (Total Return Swap)  |  优先级：P2  |  竞品：衡泰/森浦(STC)  |  华锐基础：现券交易系统/IBOR/定价平台  |  工期：6月  团队：6人</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="28" customHeight="1">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>功能域</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>编号</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>功能名称</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>功能描述</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>验收标准</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>集成依赖</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>复杂度</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>预估(人天)</t>
+        </is>
+      </c>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t>优先级</t>
+        </is>
+      </c>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>备注</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="18" customHeight="1">
+      <c r="A5" s="22" t="inlineStr">
+        <is>
+          <t>D1. TRS交易端（内部）</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="48" customHeight="1">
+      <c r="A6" s="11" t="inlineStr">
+        <is>
+          <t>D1. TRS交易端（内部）</t>
+        </is>
+      </c>
+      <c r="B6" s="10" t="inlineStr">
+        <is>
+          <t>F13-01</t>
+        </is>
+      </c>
+      <c r="C6" s="27" t="inlineStr">
+        <is>
+          <t>报价与成交管理</t>
+        </is>
+      </c>
+      <c r="D6" s="11" t="inlineStr">
+        <is>
+          <t>一站式报价（市场各渠道 + 内部自营），成交回报处理，请求报价（RFQ），历史确认查询</t>
+        </is>
+      </c>
+      <c r="E6" s="11" t="inlineStr"/>
+      <c r="F6" s="11" t="inlineStr"/>
+      <c r="G6" s="41" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="H6" s="13" t="n">
+        <v>30</v>
+      </c>
+      <c r="I6" s="12" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="J6" s="11" t="inlineStr"/>
+    </row>
+    <row r="7" ht="48" customHeight="1">
+      <c r="A7" s="11" t="inlineStr">
+        <is>
+          <t>D1. TRS交易端（内部）</t>
+        </is>
+      </c>
+      <c r="B7" s="10" t="inlineStr">
+        <is>
+          <t>F13-02</t>
+        </is>
+      </c>
+      <c r="C7" s="27" t="inlineStr">
+        <is>
+          <t>自动对冲</t>
+        </is>
+      </c>
+      <c r="D7" s="11" t="inlineStr">
+        <is>
+          <t>对冲委托自动触发，对冲回报处理，风险校验，组合重叠分析，开平仓设置，对冲策略配置</t>
+        </is>
+      </c>
+      <c r="E7" s="11" t="inlineStr"/>
+      <c r="F7" s="11" t="inlineStr"/>
+      <c r="G7" s="41" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="H7" s="13" t="n">
+        <v>30</v>
+      </c>
+      <c r="I7" s="12" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="J7" s="11" t="inlineStr"/>
+    </row>
+    <row r="8" ht="48" customHeight="1">
+      <c r="A8" s="11" t="inlineStr">
+        <is>
+          <t>D1. TRS交易端（内部）</t>
+        </is>
+      </c>
+      <c r="B8" s="10" t="inlineStr">
+        <is>
+          <t>F13-03</t>
+        </is>
+      </c>
+      <c r="C8" s="27" t="inlineStr">
+        <is>
+          <t>行情与资讯</t>
+        </is>
+      </c>
+      <c r="D8" s="11" t="inlineStr">
+        <is>
+          <t>实时行情矩阵展示，债券行情，我的关注，历史行情，资讯推送</t>
+        </is>
+      </c>
+      <c r="E8" s="11" t="inlineStr"/>
+      <c r="F8" s="11" t="inlineStr"/>
+      <c r="G8" s="42" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="H8" s="13" t="n">
+        <v>15</v>
+      </c>
+      <c r="I8" s="12" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="J8" s="11" t="inlineStr"/>
+    </row>
+    <row r="9" ht="18" customHeight="1">
+      <c r="A9" s="40" t="inlineStr">
+        <is>
+          <t>D2. TRS客户端（外部）</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="48" customHeight="1">
+      <c r="A10" s="11" t="inlineStr">
+        <is>
+          <t>D2. TRS客户端（外部）</t>
+        </is>
+      </c>
+      <c r="B10" s="10" t="inlineStr">
+        <is>
+          <t>F13-04</t>
+        </is>
+      </c>
+      <c r="C10" s="27" t="inlineStr">
+        <is>
+          <t>开户与账户管理</t>
+        </is>
+      </c>
+      <c r="D10" s="11" t="inlineStr">
+        <is>
+          <t>客户开户申请，账户信息管理，出入金申请，银行账号绑定，资金管理</t>
+        </is>
+      </c>
+      <c r="E10" s="11" t="inlineStr"/>
+      <c r="F10" s="11" t="inlineStr"/>
+      <c r="G10" s="42" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="H10" s="13" t="n">
+        <v>20</v>
+      </c>
+      <c r="I10" s="12" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="J10" s="11" t="inlineStr"/>
+    </row>
+    <row r="11" ht="48" customHeight="1">
+      <c r="A11" s="11" t="inlineStr">
+        <is>
+          <t>D2. TRS客户端（外部）</t>
+        </is>
+      </c>
+      <c r="B11" s="10" t="inlineStr">
+        <is>
+          <t>F13-05</t>
+        </is>
+      </c>
+      <c r="C11" s="27" t="inlineStr">
+        <is>
+          <t>客户自主交易</t>
+        </is>
+      </c>
+      <c r="D11" s="11" t="inlineStr">
+        <is>
+          <t>客户委托下单，合约持仓查询，标的持仓查询，当日委托，行情矩阵，历史确认，开平仓设置</t>
+        </is>
+      </c>
+      <c r="E11" s="11" t="inlineStr"/>
+      <c r="F11" s="11" t="inlineStr"/>
+      <c r="G11" s="41" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="H11" s="13" t="n">
+        <v>25</v>
+      </c>
+      <c r="I11" s="12" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="J11" s="11" t="inlineStr"/>
+    </row>
+    <row r="12" ht="18" customHeight="1">
+      <c r="A12" s="43" t="inlineStr">
+        <is>
+          <t>D3. TRS管理端（运营）</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="48" customHeight="1">
+      <c r="A13" s="11" t="inlineStr">
+        <is>
+          <t>D3. TRS管理端（运营）</t>
+        </is>
+      </c>
+      <c r="B13" s="10" t="inlineStr">
+        <is>
+          <t>F13-06</t>
+        </is>
+      </c>
+      <c r="C13" s="27" t="inlineStr">
+        <is>
+          <t>审批管理</t>
+        </is>
+      </c>
+      <c r="D13" s="11" t="inlineStr">
+        <is>
+          <t>开户申请审批，出入金审批，合约成交审核，多级审批工作流，审批留痕</t>
+        </is>
+      </c>
+      <c r="E13" s="11" t="inlineStr"/>
+      <c r="F13" s="11" t="inlineStr"/>
+      <c r="G13" s="42" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="H13" s="13" t="n">
+        <v>20</v>
+      </c>
+      <c r="I13" s="12" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="J13" s="11" t="inlineStr"/>
+    </row>
+    <row r="14" ht="48" customHeight="1">
+      <c r="A14" s="11" t="inlineStr">
+        <is>
+          <t>D3. TRS管理端（运营）</t>
+        </is>
+      </c>
+      <c r="B14" s="10" t="inlineStr">
+        <is>
+          <t>F13-07</t>
+        </is>
+      </c>
+      <c r="C14" s="27" t="inlineStr">
+        <is>
+          <t>运营管理</t>
+        </is>
+      </c>
+      <c r="D14" s="11" t="inlineStr">
+        <is>
+          <t>对账，库存管理，对冲录入，合约生命周期管理，日终结算处理</t>
+        </is>
+      </c>
+      <c r="E14" s="11" t="inlineStr"/>
+      <c r="F14" s="11" t="inlineStr"/>
+      <c r="G14" s="41" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="H14" s="13" t="n">
+        <v>25</v>
+      </c>
+      <c r="I14" s="12" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="J14" s="11" t="inlineStr"/>
+    </row>
+    <row r="15" ht="48" customHeight="1">
+      <c r="A15" s="11" t="inlineStr">
+        <is>
+          <t>D3. TRS管理端（运营）</t>
+        </is>
+      </c>
+      <c r="B15" s="10" t="inlineStr">
+        <is>
+          <t>F13-08</t>
+        </is>
+      </c>
+      <c r="C15" s="27" t="inlineStr">
+        <is>
+          <t>通知与文件生成</t>
+        </is>
+      </c>
+      <c r="D15" s="11" t="inlineStr">
+        <is>
+          <t>企微通知提醒，确认书/结算单/估值报告/出入金通知自动生成并通过邮箱发送</t>
+        </is>
+      </c>
+      <c r="E15" s="11" t="inlineStr"/>
+      <c r="F15" s="11" t="inlineStr"/>
+      <c r="G15" s="42" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="H15" s="13" t="n">
+        <v>15</v>
+      </c>
+      <c r="I15" s="12" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="J15" s="11" t="inlineStr"/>
+    </row>
+    <row r="16" ht="18" customHeight="1">
+      <c r="A16" s="43" t="inlineStr">
+        <is>
+          <t>D4. 系统集成</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="48" customHeight="1">
+      <c r="A17" s="11" t="inlineStr">
+        <is>
+          <t>D4. 系统集成</t>
+        </is>
+      </c>
+      <c r="B17" s="10" t="inlineStr">
+        <is>
+          <t>F13-09</t>
+        </is>
+      </c>
+      <c r="C17" s="27" t="inlineStr">
+        <is>
+          <t>外部系统集成</t>
+        </is>
+      </c>
+      <c r="D17" s="11" t="inlineStr">
+        <is>
+          <t>衡泰系统客户信息同步，QTrade聊天记录同步，银行流水对接，公司邮箱系统集成</t>
+        </is>
+      </c>
+      <c r="E17" s="11" t="inlineStr"/>
+      <c r="F17" s="11" t="inlineStr"/>
+      <c r="G17" s="41" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="H17" s="13" t="n">
+        <v>25</v>
+      </c>
+      <c r="I17" s="12" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="J17" s="11" t="inlineStr"/>
+    </row>
+    <row r="18" ht="48" customHeight="1">
+      <c r="A18" s="11" t="inlineStr">
+        <is>
+          <t>D4. 系统集成</t>
+        </is>
+      </c>
+      <c r="B18" s="10" t="inlineStr">
+        <is>
+          <t>F13-10</t>
+        </is>
+      </c>
+      <c r="C18" s="27" t="inlineStr">
+        <is>
+          <t>内部系统集成</t>
+        </is>
+      </c>
+      <c r="D18" s="11" t="inlineStr">
+        <is>
+          <t>现券交易系统（对冲交易执行），IBOR（持仓记录），定价平台（估值报告），事前风控（合规校验）</t>
+        </is>
+      </c>
+      <c r="E18" s="11" t="inlineStr"/>
+      <c r="F18" s="11" t="inlineStr"/>
+      <c r="G18" s="41" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="H18" s="13" t="n">
+        <v>20</v>
+      </c>
+      <c r="I18" s="12" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="J18" s="11" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="40" t="inlineStr">
+        <is>
+          <t>合计 10项功能  |  P1: 0项  |  P2: 10项</t>
+        </is>
+      </c>
+      <c r="H19" s="20">
+        <f>SUM(H5:H18)</f>
+        <v/>
+      </c>
+      <c r="I19" s="34" t="inlineStr"/>
+      <c r="J19" s="34" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <mergeCells count="8">
+    <mergeCell ref="A1:J1"/>
+    <mergeCell ref="A5:J5"/>
+    <mergeCell ref="A16:J16"/>
+    <mergeCell ref="A9:J9"/>
+    <mergeCell ref="A3:J3"/>
+    <mergeCell ref="A12:J12"/>
+    <mergeCell ref="A2:J2"/>
+    <mergeCell ref="A19:G19"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" fitToWidth="1"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H202"/>
+  <dimension ref="A1:H206"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -13339,12 +13871,12 @@
       </c>
       <c r="D190" s="27" t="inlineStr">
         <is>
-          <t>TRS交易端</t>
+          <t>报价与成交管理</t>
         </is>
       </c>
       <c r="E190" s="11" t="inlineStr">
         <is>
-          <t>报价提供，成交回报，对冲委托与自动对冲，请求报价，行情与资讯，历史确认</t>
+          <t>一站式报价（市场各渠道 + 内部自营），成交回报处理，请求报价（RFQ），历史确认查询</t>
         </is>
       </c>
       <c r="F190" s="11" t="inlineStr">
@@ -13379,12 +13911,12 @@
       </c>
       <c r="D191" s="27" t="inlineStr">
         <is>
-          <t>TRS客户端</t>
+          <t>自动对冲</t>
         </is>
       </c>
       <c r="E191" s="11" t="inlineStr">
         <is>
-          <t>开户申请，客户委托，出入金申请，合约持仓，标的持仓，资金管理，行情矩阵，自主下单</t>
+          <t>对冲委托自动触发，对冲回报处理，风险校验，组合重叠分析，开平仓设置，对冲策略配置</t>
         </is>
       </c>
       <c r="F191" s="11" t="inlineStr">
@@ -13398,7 +13930,7 @@
         </is>
       </c>
       <c r="H191" s="13" t="n">
-        <v>25</v>
+        <v>30</v>
       </c>
     </row>
     <row r="192" ht="28" customHeight="1">
@@ -13419,12 +13951,12 @@
       </c>
       <c r="D192" s="27" t="inlineStr">
         <is>
-          <t>TRS管理端</t>
+          <t>行情与资讯</t>
         </is>
       </c>
       <c r="E192" s="11" t="inlineStr">
         <is>
-          <t>开户申请审批，合约成交管理，出入金审批，运营管理，对账，库存，对冲录入</t>
+          <t>实时行情矩阵展示，债券行情，我的关注，历史行情，资讯推送</t>
         </is>
       </c>
       <c r="F192" s="11" t="inlineStr">
@@ -13438,7 +13970,7 @@
         </is>
       </c>
       <c r="H192" s="13" t="n">
-        <v>20</v>
+        <v>15</v>
       </c>
     </row>
     <row r="193" ht="28" customHeight="1">
@@ -13459,26 +13991,26 @@
       </c>
       <c r="D193" s="27" t="inlineStr">
         <is>
-          <t>自动对冲</t>
+          <t>开户与账户管理</t>
         </is>
       </c>
       <c r="E193" s="11" t="inlineStr">
         <is>
-          <t>对冲委托自动触发，对冲回报处理，风险校验，组合重叠分析，开平仓设置</t>
+          <t>客户开户申请，账户信息管理，出入金申请，银行账号绑定，资金管理</t>
         </is>
       </c>
       <c r="F193" s="11" t="inlineStr">
         <is>
-          <t>功能完整/边界测试/集成冒烟/性能基线</t>
-        </is>
-      </c>
-      <c r="G193" s="23" t="inlineStr">
-        <is>
-          <t>高</t>
+          <t>功能测试通过/正确率100%</t>
+        </is>
+      </c>
+      <c r="G193" s="24" t="inlineStr">
+        <is>
+          <t>中</t>
         </is>
       </c>
       <c r="H193" s="13" t="n">
-        <v>25</v>
+        <v>20</v>
       </c>
     </row>
     <row r="194" ht="28" customHeight="1">
@@ -13499,26 +14031,26 @@
       </c>
       <c r="D194" s="27" t="inlineStr">
         <is>
-          <t>通知与确认文件</t>
+          <t>客户自主交易</t>
         </is>
       </c>
       <c r="E194" s="11" t="inlineStr">
         <is>
-          <t>企微通知提醒，确认书/结算单/估值报告/出入金通知自动生成并通过邮箱发送</t>
+          <t>客户委托下单，合约持仓查询，标的持仓查询，当日委托，行情矩阵，历史确认，开平仓设置</t>
         </is>
       </c>
       <c r="F194" s="11" t="inlineStr">
         <is>
-          <t>功能测试通过/正确率100%</t>
-        </is>
-      </c>
-      <c r="G194" s="24" t="inlineStr">
-        <is>
-          <t>中</t>
+          <t>功能完整/边界测试/集成冒烟/性能基线</t>
+        </is>
+      </c>
+      <c r="G194" s="23" t="inlineStr">
+        <is>
+          <t>高</t>
         </is>
       </c>
       <c r="H194" s="13" t="n">
-        <v>15</v>
+        <v>25</v>
       </c>
     </row>
     <row r="195" ht="28" customHeight="1">
@@ -13539,193 +14071,193 @@
       </c>
       <c r="D195" s="27" t="inlineStr">
         <is>
-          <t>系统集成</t>
+          <t>审批管理</t>
         </is>
       </c>
       <c r="E195" s="11" t="inlineStr">
         <is>
-          <t>与衡泰系统客户信息同步，QTrade聊天记录同步，交易管理系统对接，银行流水对接</t>
+          <t>开户申请审批，出入金审批，合约成交审核，多级审批工作流，审批留痕</t>
         </is>
       </c>
       <c r="F195" s="11" t="inlineStr">
         <is>
+          <t>功能测试通过/正确率100%</t>
+        </is>
+      </c>
+      <c r="G195" s="24" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="H195" s="13" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="196" ht="28" customHeight="1">
+      <c r="A196" s="11" t="inlineStr">
+        <is>
+          <t>TRS收益互换</t>
+        </is>
+      </c>
+      <c r="B196" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="C196" s="10" t="inlineStr">
+        <is>
+          <t>F13-07</t>
+        </is>
+      </c>
+      <c r="D196" s="27" t="inlineStr">
+        <is>
+          <t>运营管理</t>
+        </is>
+      </c>
+      <c r="E196" s="11" t="inlineStr">
+        <is>
+          <t>对账，库存管理，对冲录入，合约生命周期管理，日终结算处理</t>
+        </is>
+      </c>
+      <c r="F196" s="11" t="inlineStr">
+        <is>
           <t>功能完整/边界测试/集成冒烟/性能基线</t>
         </is>
       </c>
-      <c r="G195" s="23" t="inlineStr">
+      <c r="G196" s="23" t="inlineStr">
         <is>
           <t>高</t>
         </is>
       </c>
-      <c r="H195" s="13" t="n">
+      <c r="H196" s="13" t="n">
         <v>25</v>
       </c>
     </row>
-    <row r="196" ht="20" customHeight="1">
-      <c r="A196" s="29" t="inlineStr">
+    <row r="197" ht="28" customHeight="1">
+      <c r="A197" s="11" t="inlineStr">
+        <is>
+          <t>TRS收益互换</t>
+        </is>
+      </c>
+      <c r="B197" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="C197" s="10" t="inlineStr">
+        <is>
+          <t>F13-08</t>
+        </is>
+      </c>
+      <c r="D197" s="27" t="inlineStr">
+        <is>
+          <t>通知与文件生成</t>
+        </is>
+      </c>
+      <c r="E197" s="11" t="inlineStr">
+        <is>
+          <t>企微通知提醒，确认书/结算单/估值报告/出入金通知自动生成并通过邮箱发送</t>
+        </is>
+      </c>
+      <c r="F197" s="11" t="inlineStr">
+        <is>
+          <t>功能测试通过/正确率100%</t>
+        </is>
+      </c>
+      <c r="G197" s="24" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="H197" s="13" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="198" ht="28" customHeight="1">
+      <c r="A198" s="11" t="inlineStr">
+        <is>
+          <t>TRS收益互换</t>
+        </is>
+      </c>
+      <c r="B198" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="C198" s="10" t="inlineStr">
+        <is>
+          <t>F13-09</t>
+        </is>
+      </c>
+      <c r="D198" s="27" t="inlineStr">
+        <is>
+          <t>外部系统集成</t>
+        </is>
+      </c>
+      <c r="E198" s="11" t="inlineStr">
+        <is>
+          <t>衡泰系统客户信息同步，QTrade聊天记录同步，银行流水对接，公司邮箱系统集成</t>
+        </is>
+      </c>
+      <c r="F198" s="11" t="inlineStr">
+        <is>
+          <t>功能完整/边界测试/集成冒烟/性能基线</t>
+        </is>
+      </c>
+      <c r="G198" s="23" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="H198" s="13" t="n">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="199" ht="28" customHeight="1">
+      <c r="A199" s="11" t="inlineStr">
+        <is>
+          <t>TRS收益互换</t>
+        </is>
+      </c>
+      <c r="B199" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="C199" s="10" t="inlineStr">
+        <is>
+          <t>F13-10</t>
+        </is>
+      </c>
+      <c r="D199" s="27" t="inlineStr">
+        <is>
+          <t>内部系统集成</t>
+        </is>
+      </c>
+      <c r="E199" s="11" t="inlineStr">
+        <is>
+          <t>现券交易系统（对冲交易执行），IBOR（持仓记录），定价平台（估值报告），事前风控（合规校验）</t>
+        </is>
+      </c>
+      <c r="F199" s="11" t="inlineStr">
+        <is>
+          <t>功能完整/边界测试/集成冒烟/性能基线</t>
+        </is>
+      </c>
+      <c r="G199" s="23" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="H199" s="13" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="200" ht="20" customHeight="1">
+      <c r="A200" s="29" t="inlineStr">
         <is>
           <t>【P3】 做市商系统  (Market Making)</t>
         </is>
-      </c>
-    </row>
-    <row r="197" ht="28" customHeight="1">
-      <c r="A197" s="16" t="inlineStr">
-        <is>
-          <t>做市商系统</t>
-        </is>
-      </c>
-      <c r="B197" s="15" t="inlineStr">
-        <is>
-          <t>P3</t>
-        </is>
-      </c>
-      <c r="C197" s="15" t="inlineStr">
-        <is>
-          <t>F15-01</t>
-        </is>
-      </c>
-      <c r="D197" s="30" t="inlineStr">
-        <is>
-          <t>双边报价引擎</t>
-        </is>
-      </c>
-      <c r="E197" s="16" t="inlineStr">
-        <is>
-          <t>多品种同时双边报价，延迟&lt;5ms，报价宽度动态优化</t>
-        </is>
-      </c>
-      <c r="F197" s="16" t="inlineStr">
-        <is>
-          <t>p99延迟/误差率/精度验证/压测10k TPS</t>
-        </is>
-      </c>
-      <c r="G197" s="28" t="inlineStr">
-        <is>
-          <t>极高</t>
-        </is>
-      </c>
-      <c r="H197" s="18" t="n">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="198" ht="28" customHeight="1">
-      <c r="A198" s="16" t="inlineStr">
-        <is>
-          <t>做市商系统</t>
-        </is>
-      </c>
-      <c r="B198" s="15" t="inlineStr">
-        <is>
-          <t>P3</t>
-        </is>
-      </c>
-      <c r="C198" s="15" t="inlineStr">
-        <is>
-          <t>F15-02</t>
-        </is>
-      </c>
-      <c r="D198" s="30" t="inlineStr">
-        <is>
-          <t>库存风险实时管理</t>
-        </is>
-      </c>
-      <c r="E198" s="16" t="inlineStr">
-        <is>
-          <t>做市库存PnL实时监控，Delta对冲自动触发</t>
-        </is>
-      </c>
-      <c r="F198" s="16" t="inlineStr">
-        <is>
-          <t>p99延迟/误差率/精度验证/压测10k TPS</t>
-        </is>
-      </c>
-      <c r="G198" s="28" t="inlineStr">
-        <is>
-          <t>极高</t>
-        </is>
-      </c>
-      <c r="H198" s="18" t="n">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="199" ht="28" customHeight="1">
-      <c r="A199" s="16" t="inlineStr">
-        <is>
-          <t>做市商系统</t>
-        </is>
-      </c>
-      <c r="B199" s="15" t="inlineStr">
-        <is>
-          <t>P3</t>
-        </is>
-      </c>
-      <c r="C199" s="15" t="inlineStr">
-        <is>
-          <t>F15-03</t>
-        </is>
-      </c>
-      <c r="D199" s="30" t="inlineStr">
-        <is>
-          <t>报价优化算法</t>
-        </is>
-      </c>
-      <c r="E199" s="16" t="inlineStr">
-        <is>
-          <t>基于市场微结构理论动态调整bid-ask spread</t>
-        </is>
-      </c>
-      <c r="F199" s="16" t="inlineStr">
-        <is>
-          <t>p99延迟/误差率/精度验证/压测10k TPS</t>
-        </is>
-      </c>
-      <c r="G199" s="28" t="inlineStr">
-        <is>
-          <t>极高</t>
-        </is>
-      </c>
-      <c r="H199" s="18" t="n">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="200" ht="28" customHeight="1">
-      <c r="A200" s="16" t="inlineStr">
-        <is>
-          <t>做市商系统</t>
-        </is>
-      </c>
-      <c r="B200" s="15" t="inlineStr">
-        <is>
-          <t>P3</t>
-        </is>
-      </c>
-      <c r="C200" s="15" t="inlineStr">
-        <is>
-          <t>F15-04</t>
-        </is>
-      </c>
-      <c r="D200" s="30" t="inlineStr">
-        <is>
-          <t>竞争力分析</t>
-        </is>
-      </c>
-      <c r="E200" s="16" t="inlineStr">
-        <is>
-          <t>与市场最优报价对比，中签率分析，策略调优</t>
-        </is>
-      </c>
-      <c r="F200" s="16" t="inlineStr">
-        <is>
-          <t>功能完整/边界测试/集成冒烟/性能基线</t>
-        </is>
-      </c>
-      <c r="G200" s="23" t="inlineStr">
-        <is>
-          <t>高</t>
-        </is>
-      </c>
-      <c r="H200" s="18" t="n">
-        <v>25</v>
       </c>
     </row>
     <row r="201" ht="28" customHeight="1">
@@ -13741,53 +14273,213 @@
       </c>
       <c r="C201" s="15" t="inlineStr">
         <is>
+          <t>F15-01</t>
+        </is>
+      </c>
+      <c r="D201" s="30" t="inlineStr">
+        <is>
+          <t>双边报价引擎</t>
+        </is>
+      </c>
+      <c r="E201" s="16" t="inlineStr">
+        <is>
+          <t>多品种同时双边报价，延迟&lt;5ms，报价宽度动态优化</t>
+        </is>
+      </c>
+      <c r="F201" s="16" t="inlineStr">
+        <is>
+          <t>p99延迟/误差率/精度验证/压测10k TPS</t>
+        </is>
+      </c>
+      <c r="G201" s="28" t="inlineStr">
+        <is>
+          <t>极高</t>
+        </is>
+      </c>
+      <c r="H201" s="18" t="n">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="202" ht="28" customHeight="1">
+      <c r="A202" s="16" t="inlineStr">
+        <is>
+          <t>做市商系统</t>
+        </is>
+      </c>
+      <c r="B202" s="15" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="C202" s="15" t="inlineStr">
+        <is>
+          <t>F15-02</t>
+        </is>
+      </c>
+      <c r="D202" s="30" t="inlineStr">
+        <is>
+          <t>库存风险实时管理</t>
+        </is>
+      </c>
+      <c r="E202" s="16" t="inlineStr">
+        <is>
+          <t>做市库存PnL实时监控，Delta对冲自动触发</t>
+        </is>
+      </c>
+      <c r="F202" s="16" t="inlineStr">
+        <is>
+          <t>p99延迟/误差率/精度验证/压测10k TPS</t>
+        </is>
+      </c>
+      <c r="G202" s="28" t="inlineStr">
+        <is>
+          <t>极高</t>
+        </is>
+      </c>
+      <c r="H202" s="18" t="n">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="203" ht="28" customHeight="1">
+      <c r="A203" s="16" t="inlineStr">
+        <is>
+          <t>做市商系统</t>
+        </is>
+      </c>
+      <c r="B203" s="15" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="C203" s="15" t="inlineStr">
+        <is>
+          <t>F15-03</t>
+        </is>
+      </c>
+      <c r="D203" s="30" t="inlineStr">
+        <is>
+          <t>报价优化算法</t>
+        </is>
+      </c>
+      <c r="E203" s="16" t="inlineStr">
+        <is>
+          <t>基于市场微结构理论动态调整bid-ask spread</t>
+        </is>
+      </c>
+      <c r="F203" s="16" t="inlineStr">
+        <is>
+          <t>p99延迟/误差率/精度验证/压测10k TPS</t>
+        </is>
+      </c>
+      <c r="G203" s="28" t="inlineStr">
+        <is>
+          <t>极高</t>
+        </is>
+      </c>
+      <c r="H203" s="18" t="n">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="204" ht="28" customHeight="1">
+      <c r="A204" s="16" t="inlineStr">
+        <is>
+          <t>做市商系统</t>
+        </is>
+      </c>
+      <c r="B204" s="15" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="C204" s="15" t="inlineStr">
+        <is>
+          <t>F15-04</t>
+        </is>
+      </c>
+      <c r="D204" s="30" t="inlineStr">
+        <is>
+          <t>竞争力分析</t>
+        </is>
+      </c>
+      <c r="E204" s="16" t="inlineStr">
+        <is>
+          <t>与市场最优报价对比，中签率分析，策略调优</t>
+        </is>
+      </c>
+      <c r="F204" s="16" t="inlineStr">
+        <is>
+          <t>功能完整/边界测试/集成冒烟/性能基线</t>
+        </is>
+      </c>
+      <c r="G204" s="23" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="H204" s="18" t="n">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="205" ht="28" customHeight="1">
+      <c r="A205" s="16" t="inlineStr">
+        <is>
+          <t>做市商系统</t>
+        </is>
+      </c>
+      <c r="B205" s="15" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="C205" s="15" t="inlineStr">
+        <is>
           <t>F15-05</t>
         </is>
       </c>
-      <c r="D201" s="30" t="inlineStr">
+      <c r="D205" s="30" t="inlineStr">
         <is>
           <t>交易对手管理集成</t>
         </is>
       </c>
-      <c r="E201" s="16" t="inlineStr">
+      <c r="E205" s="16" t="inlineStr">
         <is>
           <t>做市交易对手信用实时检查，额度占用同步更新</t>
         </is>
       </c>
-      <c r="F201" s="16" t="inlineStr">
+      <c r="F205" s="16" t="inlineStr">
         <is>
           <t>功能测试通过/正确率100%</t>
         </is>
       </c>
-      <c r="G201" s="24" t="inlineStr">
+      <c r="G205" s="24" t="inlineStr">
         <is>
           <t>中</t>
         </is>
       </c>
-      <c r="H201" s="18" t="n">
+      <c r="H205" s="18" t="n">
         <v>20</v>
       </c>
     </row>
-    <row r="202">
-      <c r="A202" s="19" t="inlineStr">
+    <row r="206">
+      <c r="A206" s="19" t="inlineStr">
         <is>
           <t>总计功能数 / Total Function Points</t>
         </is>
       </c>
-      <c r="H202" s="20">
-        <f>SUM(H3:H201)</f>
+      <c r="H206" s="20">
+        <f>SUM(H3:H205)</f>
         <v/>
       </c>
     </row>
   </sheetData>
   <mergeCells count="16">
     <mergeCell ref="A143:H143"/>
-    <mergeCell ref="A202:G202"/>
     <mergeCell ref="A3:H3"/>
     <mergeCell ref="A101:H101"/>
     <mergeCell ref="A130:H130"/>
+    <mergeCell ref="A200:H200"/>
     <mergeCell ref="A180:H180"/>
-    <mergeCell ref="A196:H196"/>
+    <mergeCell ref="A206:G206"/>
     <mergeCell ref="A60:H60"/>
     <mergeCell ref="A112:H112"/>
     <mergeCell ref="A68:H68"/>

</xml_diff>

<commit_message>
Expand module 15 (做市商系统) to full function_domains + tech_design
Completes the full expansion of all 14 PPT-backed modules. Module 15
now has 12 functions across 4 domains covering 双边/TRS/RFQ/API做市
模式, 报价策略管理, 做市义务监控, 订单与库存风险管理. Duration updated
to 14m/140pm per Slide 53-54.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Feasibility_analysis/FICC_Gap_Analysis.xlsx
+++ b/Feasibility_analysis/FICC_Gap_Analysis.xlsx
@@ -24,6 +24,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="详情_信用债_信用衍生品" sheetId="15" state="visible" r:id="rId15"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="详情_投顾服务" sheetId="16" state="visible" r:id="rId16"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="详情_TRS收益互换" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="详情_做市商系统" sheetId="18" state="visible" r:id="rId18"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Area" localSheetId="0">'差距分析总表'!$A$1:$P$17</definedName>
@@ -1876,17 +1877,17 @@
         </is>
       </c>
       <c r="M16" s="15" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="N16" s="15" t="n">
         <v>12</v>
       </c>
       <c r="O16" s="18" t="n">
-        <v>120</v>
+        <v>140</v>
       </c>
       <c r="P16" s="16" t="inlineStr">
         <is>
-          <t>双边报价引擎，需深度市场经验</t>
+          <t>双边报价引擎，做市义务监控，报价策略自动优化，支持双边/TRS/RFQ/API四种做市模式；对应PPT Slide 53-54</t>
         </is>
       </c>
     </row>
@@ -6734,13 +6735,620 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J21"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="48" customWidth="1" min="4" max="4"/>
+    <col width="26" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="6" max="6"/>
+    <col width="8" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="8" max="8"/>
+    <col width="7" customWidth="1" min="9" max="9"/>
+    <col width="18" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="24" customHeight="1">
+      <c r="A1" s="38" t="inlineStr">
+        <is>
+          <t>系统详情：做市商系统  |  Market Making</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="36" customHeight="1">
+      <c r="A2" s="39" t="inlineStr">
+        <is>
+          <t>战略定位：双边报价引擎，做市义务监控，报价策略自动优化，支持双边/TRS/RFQ/API四种做市模式；对应PPT Slide 53-54   |   来源：Slide 53</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="28" customHeight="1">
+      <c r="A3" s="40" t="inlineStr">
+        <is>
+          <t>模块：做市商系统  (Market Making)  |  优先级：P3  |  竞品：Murex/专项  |  华锐基础：ATP报价接口  |  工期：14月  团队：12人</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="28" customHeight="1">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>功能域</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>编号</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>功能名称</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>功能描述</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>验收标准</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>集成依赖</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>复杂度</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>预估(人天)</t>
+        </is>
+      </c>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t>优先级</t>
+        </is>
+      </c>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>备注</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="18" customHeight="1">
+      <c r="A5" s="22" t="inlineStr">
+        <is>
+          <t>D1. 做市模式管理</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="48" customHeight="1">
+      <c r="A6" s="11" t="inlineStr">
+        <is>
+          <t>D1. 做市模式管理</t>
+        </is>
+      </c>
+      <c r="B6" s="10" t="inlineStr">
+        <is>
+          <t>F15-01</t>
+        </is>
+      </c>
+      <c r="C6" s="27" t="inlineStr">
+        <is>
+          <t>双边报价做市</t>
+        </is>
+      </c>
+      <c r="D6" s="11" t="inlineStr">
+        <is>
+          <t>多品种同时双边报价，延迟&lt;5ms，报价宽度动态优化，支持国债/信用债/利率互换多品种做市</t>
+        </is>
+      </c>
+      <c r="E6" s="11" t="inlineStr"/>
+      <c r="F6" s="11" t="inlineStr"/>
+      <c r="G6" s="28" t="inlineStr">
+        <is>
+          <t>极高</t>
+        </is>
+      </c>
+      <c r="H6" s="13" t="n">
+        <v>70</v>
+      </c>
+      <c r="I6" s="12" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="J6" s="11" t="inlineStr"/>
+    </row>
+    <row r="7" ht="48" customHeight="1">
+      <c r="A7" s="11" t="inlineStr">
+        <is>
+          <t>D1. 做市模式管理</t>
+        </is>
+      </c>
+      <c r="B7" s="10" t="inlineStr">
+        <is>
+          <t>F15-02</t>
+        </is>
+      </c>
+      <c r="C7" s="27" t="inlineStr">
+        <is>
+          <t>TRS做市服务</t>
+        </is>
+      </c>
+      <c r="D7" s="11" t="inlineStr">
+        <is>
+          <t>TRS产品双边报价，与TRS收益互换系统深度集成，对冲报价敞口，支持客户TRS交易</t>
+        </is>
+      </c>
+      <c r="E7" s="11" t="inlineStr"/>
+      <c r="F7" s="11" t="inlineStr"/>
+      <c r="G7" s="28" t="inlineStr">
+        <is>
+          <t>极高</t>
+        </is>
+      </c>
+      <c r="H7" s="13" t="n">
+        <v>40</v>
+      </c>
+      <c r="I7" s="12" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="J7" s="11" t="inlineStr"/>
+    </row>
+    <row r="8" ht="48" customHeight="1">
+      <c r="A8" s="11" t="inlineStr">
+        <is>
+          <t>D1. 做市模式管理</t>
+        </is>
+      </c>
+      <c r="B8" s="10" t="inlineStr">
+        <is>
+          <t>F15-03</t>
+        </is>
+      </c>
+      <c r="C8" s="27" t="inlineStr">
+        <is>
+          <t>RFQ询价响应</t>
+        </is>
+      </c>
+      <c r="D8" s="11" t="inlineStr">
+        <is>
+          <t>接收客户询价请求，自动生成报价，报价有效期管理，成交确认，询价历史记录</t>
+        </is>
+      </c>
+      <c r="E8" s="11" t="inlineStr"/>
+      <c r="F8" s="11" t="inlineStr"/>
+      <c r="G8" s="41" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="H8" s="13" t="n">
+        <v>25</v>
+      </c>
+      <c r="I8" s="12" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="J8" s="11" t="inlineStr"/>
+    </row>
+    <row r="9" ht="48" customHeight="1">
+      <c r="A9" s="11" t="inlineStr">
+        <is>
+          <t>D1. 做市模式管理</t>
+        </is>
+      </c>
+      <c r="B9" s="10" t="inlineStr">
+        <is>
+          <t>F15-04</t>
+        </is>
+      </c>
+      <c r="C9" s="27" t="inlineStr">
+        <is>
+          <t>API程序化做市</t>
+        </is>
+      </c>
+      <c r="D9" s="11" t="inlineStr">
+        <is>
+          <t>对外提供做市API接口，支持程序化交易对手接入，流式报价推送，API鉴权与频率限制</t>
+        </is>
+      </c>
+      <c r="E9" s="11" t="inlineStr"/>
+      <c r="F9" s="11" t="inlineStr"/>
+      <c r="G9" s="41" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="H9" s="13" t="n">
+        <v>25</v>
+      </c>
+      <c r="I9" s="12" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="J9" s="11" t="inlineStr"/>
+    </row>
+    <row r="10" ht="18" customHeight="1">
+      <c r="A10" s="40" t="inlineStr">
+        <is>
+          <t>D2. 报价策略管理</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="48" customHeight="1">
+      <c r="A11" s="11" t="inlineStr">
+        <is>
+          <t>D2. 报价策略管理</t>
+        </is>
+      </c>
+      <c r="B11" s="10" t="inlineStr">
+        <is>
+          <t>F15-05</t>
+        </is>
+      </c>
+      <c r="C11" s="27" t="inlineStr">
+        <is>
+          <t>报价策略配置</t>
+        </is>
+      </c>
+      <c r="D11" s="11" t="inlineStr">
+        <is>
+          <t>各品种做市参数配置（报价宽度/报价量/报价频率），分时段策略，按交易对手差异化报价</t>
+        </is>
+      </c>
+      <c r="E11" s="11" t="inlineStr"/>
+      <c r="F11" s="11" t="inlineStr"/>
+      <c r="G11" s="42" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="H11" s="13" t="n">
+        <v>20</v>
+      </c>
+      <c r="I11" s="12" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="J11" s="11" t="inlineStr"/>
+    </row>
+    <row r="12" ht="48" customHeight="1">
+      <c r="A12" s="11" t="inlineStr">
+        <is>
+          <t>D2. 报价策略管理</t>
+        </is>
+      </c>
+      <c r="B12" s="10" t="inlineStr">
+        <is>
+          <t>F15-06</t>
+        </is>
+      </c>
+      <c r="C12" s="27" t="inlineStr">
+        <is>
+          <t>报价优化算法</t>
+        </is>
+      </c>
+      <c r="D12" s="11" t="inlineStr">
+        <is>
+          <t>基于市场微结构理论动态调整bid-ask spread，流动性自适应调节，机器学习辅助报价优化</t>
+        </is>
+      </c>
+      <c r="E12" s="11" t="inlineStr"/>
+      <c r="F12" s="11" t="inlineStr"/>
+      <c r="G12" s="28" t="inlineStr">
+        <is>
+          <t>极高</t>
+        </is>
+      </c>
+      <c r="H12" s="13" t="n">
+        <v>50</v>
+      </c>
+      <c r="I12" s="12" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="J12" s="11" t="inlineStr"/>
+    </row>
+    <row r="13" ht="48" customHeight="1">
+      <c r="A13" s="11" t="inlineStr">
+        <is>
+          <t>D2. 报价策略管理</t>
+        </is>
+      </c>
+      <c r="B13" s="10" t="inlineStr">
+        <is>
+          <t>F15-07</t>
+        </is>
+      </c>
+      <c r="C13" s="27" t="inlineStr">
+        <is>
+          <t>债券过滤与筛选</t>
+        </is>
+      </c>
+      <c r="D13" s="11" t="inlineStr">
+        <is>
+          <t>做市标的券池管理，流动性分级筛选，黑名单管理，临时暂停做市规则</t>
+        </is>
+      </c>
+      <c r="E13" s="11" t="inlineStr"/>
+      <c r="F13" s="11" t="inlineStr"/>
+      <c r="G13" s="42" t="inlineStr">
+        <is>
+          <t>低</t>
+        </is>
+      </c>
+      <c r="H13" s="13" t="n">
+        <v>10</v>
+      </c>
+      <c r="I13" s="12" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="J13" s="11" t="inlineStr"/>
+    </row>
+    <row r="14" ht="18" customHeight="1">
+      <c r="A14" s="43" t="inlineStr">
+        <is>
+          <t>D3. 做市义务监控</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="48" customHeight="1">
+      <c r="A15" s="11" t="inlineStr">
+        <is>
+          <t>D3. 做市义务监控</t>
+        </is>
+      </c>
+      <c r="B15" s="10" t="inlineStr">
+        <is>
+          <t>F15-08</t>
+        </is>
+      </c>
+      <c r="C15" s="27" t="inlineStr">
+        <is>
+          <t>做市义务实时监控</t>
+        </is>
+      </c>
+      <c r="D15" s="11" t="inlineStr">
+        <is>
+          <t>实时监控做市义务完成情况（报价连续性/报价宽度/报价量达标），义务违规预警，监管报告生成</t>
+        </is>
+      </c>
+      <c r="E15" s="11" t="inlineStr"/>
+      <c r="F15" s="11" t="inlineStr"/>
+      <c r="G15" s="41" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="H15" s="13" t="n">
+        <v>30</v>
+      </c>
+      <c r="I15" s="12" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="J15" s="11" t="inlineStr"/>
+    </row>
+    <row r="16" ht="48" customHeight="1">
+      <c r="A16" s="11" t="inlineStr">
+        <is>
+          <t>D3. 做市义务监控</t>
+        </is>
+      </c>
+      <c r="B16" s="10" t="inlineStr">
+        <is>
+          <t>F15-09</t>
+        </is>
+      </c>
+      <c r="C16" s="27" t="inlineStr">
+        <is>
+          <t>做市行情展示</t>
+        </is>
+      </c>
+      <c r="D16" s="11" t="inlineStr">
+        <is>
+          <t>做市报价行情矩阵，实时价格展示，报价历史回放，市场最优报价对比，中签率统计</t>
+        </is>
+      </c>
+      <c r="E16" s="11" t="inlineStr"/>
+      <c r="F16" s="11" t="inlineStr"/>
+      <c r="G16" s="42" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="H16" s="13" t="n">
+        <v>20</v>
+      </c>
+      <c r="I16" s="12" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="J16" s="11" t="inlineStr"/>
+    </row>
+    <row r="17" ht="18" customHeight="1">
+      <c r="A17" s="43" t="inlineStr">
+        <is>
+          <t>D4. 订单与风险管理</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="48" customHeight="1">
+      <c r="A18" s="11" t="inlineStr">
+        <is>
+          <t>D4. 订单与风险管理</t>
+        </is>
+      </c>
+      <c r="B18" s="10" t="inlineStr">
+        <is>
+          <t>F15-10</t>
+        </is>
+      </c>
+      <c r="C18" s="27" t="inlineStr">
+        <is>
+          <t>做市订单管理</t>
+        </is>
+      </c>
+      <c r="D18" s="11" t="inlineStr">
+        <is>
+          <t>做市委托生成、撤改、成交回报处理，订单状态实时跟踪，批量撤单，做市台账</t>
+        </is>
+      </c>
+      <c r="E18" s="11" t="inlineStr"/>
+      <c r="F18" s="11" t="inlineStr"/>
+      <c r="G18" s="41" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="H18" s="13" t="n">
+        <v>30</v>
+      </c>
+      <c r="I18" s="12" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="J18" s="11" t="inlineStr"/>
+    </row>
+    <row r="19" ht="48" customHeight="1">
+      <c r="A19" s="11" t="inlineStr">
+        <is>
+          <t>D4. 订单与风险管理</t>
+        </is>
+      </c>
+      <c r="B19" s="10" t="inlineStr">
+        <is>
+          <t>F15-11</t>
+        </is>
+      </c>
+      <c r="C19" s="27" t="inlineStr">
+        <is>
+          <t>库存风险实时管理</t>
+        </is>
+      </c>
+      <c r="D19" s="11" t="inlineStr">
+        <is>
+          <t>做市库存PnL实时监控，Delta对冲自动触发，库存敞口上限控制，实时盯市损益</t>
+        </is>
+      </c>
+      <c r="E19" s="11" t="inlineStr"/>
+      <c r="F19" s="11" t="inlineStr"/>
+      <c r="G19" s="28" t="inlineStr">
+        <is>
+          <t>极高</t>
+        </is>
+      </c>
+      <c r="H19" s="13" t="n">
+        <v>60</v>
+      </c>
+      <c r="I19" s="12" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="J19" s="11" t="inlineStr"/>
+    </row>
+    <row r="20" ht="48" customHeight="1">
+      <c r="A20" s="11" t="inlineStr">
+        <is>
+          <t>D4. 订单与风险管理</t>
+        </is>
+      </c>
+      <c r="B20" s="10" t="inlineStr">
+        <is>
+          <t>F15-12</t>
+        </is>
+      </c>
+      <c r="C20" s="27" t="inlineStr">
+        <is>
+          <t>竞争力分析</t>
+        </is>
+      </c>
+      <c r="D20" s="11" t="inlineStr">
+        <is>
+          <t>与市场最优报价对比，中签率分析，报价表现统计，策略调优建议，竞争对手报价分析</t>
+        </is>
+      </c>
+      <c r="E20" s="11" t="inlineStr"/>
+      <c r="F20" s="11" t="inlineStr"/>
+      <c r="G20" s="41" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="H20" s="13" t="n">
+        <v>25</v>
+      </c>
+      <c r="I20" s="12" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="J20" s="11" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="40" t="inlineStr">
+        <is>
+          <t>合计 12项功能  |  P1: 0项  |  P2: 12项</t>
+        </is>
+      </c>
+      <c r="H21" s="20">
+        <f>SUM(H5:H20)</f>
+        <v/>
+      </c>
+      <c r="I21" s="34" t="inlineStr"/>
+      <c r="J21" s="34" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <mergeCells count="8">
+    <mergeCell ref="A1:J1"/>
+    <mergeCell ref="A5:J5"/>
+    <mergeCell ref="A14:J14"/>
+    <mergeCell ref="A17:J17"/>
+    <mergeCell ref="A21:G21"/>
+    <mergeCell ref="A3:J3"/>
+    <mergeCell ref="A2:J2"/>
+    <mergeCell ref="A10:J10"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" fitToWidth="1"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H206"/>
+  <dimension ref="A1:H213"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -14278,12 +14886,12 @@
       </c>
       <c r="D201" s="30" t="inlineStr">
         <is>
-          <t>双边报价引擎</t>
+          <t>双边报价做市</t>
         </is>
       </c>
       <c r="E201" s="16" t="inlineStr">
         <is>
-          <t>多品种同时双边报价，延迟&lt;5ms，报价宽度动态优化</t>
+          <t>多品种同时双边报价，延迟&lt;5ms，报价宽度动态优化，支持国债/信用债/利率互换多品种做市</t>
         </is>
       </c>
       <c r="F201" s="16" t="inlineStr">
@@ -14318,12 +14926,12 @@
       </c>
       <c r="D202" s="30" t="inlineStr">
         <is>
-          <t>库存风险实时管理</t>
+          <t>TRS做市服务</t>
         </is>
       </c>
       <c r="E202" s="16" t="inlineStr">
         <is>
-          <t>做市库存PnL实时监控，Delta对冲自动触发</t>
+          <t>TRS产品双边报价，与TRS收益互换系统深度集成，对冲报价敞口，支持客户TRS交易</t>
         </is>
       </c>
       <c r="F202" s="16" t="inlineStr">
@@ -14337,7 +14945,7 @@
         </is>
       </c>
       <c r="H202" s="18" t="n">
-        <v>60</v>
+        <v>40</v>
       </c>
     </row>
     <row r="203" ht="28" customHeight="1">
@@ -14358,26 +14966,26 @@
       </c>
       <c r="D203" s="30" t="inlineStr">
         <is>
-          <t>报价优化算法</t>
+          <t>RFQ询价响应</t>
         </is>
       </c>
       <c r="E203" s="16" t="inlineStr">
         <is>
-          <t>基于市场微结构理论动态调整bid-ask spread</t>
+          <t>接收客户询价请求，自动生成报价，报价有效期管理，成交确认，询价历史记录</t>
         </is>
       </c>
       <c r="F203" s="16" t="inlineStr">
         <is>
-          <t>p99延迟/误差率/精度验证/压测10k TPS</t>
-        </is>
-      </c>
-      <c r="G203" s="28" t="inlineStr">
-        <is>
-          <t>极高</t>
+          <t>功能完整/边界测试/集成冒烟/性能基线</t>
+        </is>
+      </c>
+      <c r="G203" s="23" t="inlineStr">
+        <is>
+          <t>高</t>
         </is>
       </c>
       <c r="H203" s="18" t="n">
-        <v>50</v>
+        <v>25</v>
       </c>
     </row>
     <row r="204" ht="28" customHeight="1">
@@ -14398,12 +15006,12 @@
       </c>
       <c r="D204" s="30" t="inlineStr">
         <is>
-          <t>竞争力分析</t>
+          <t>API程序化做市</t>
         </is>
       </c>
       <c r="E204" s="16" t="inlineStr">
         <is>
-          <t>与市场最优报价对比，中签率分析，策略调优</t>
+          <t>对外提供做市API接口，支持程序化交易对手接入，流式报价推送，API鉴权与频率限制</t>
         </is>
       </c>
       <c r="F204" s="16" t="inlineStr">
@@ -14438,12 +15046,12 @@
       </c>
       <c r="D205" s="30" t="inlineStr">
         <is>
-          <t>交易对手管理集成</t>
+          <t>报价策略配置</t>
         </is>
       </c>
       <c r="E205" s="16" t="inlineStr">
         <is>
-          <t>做市交易对手信用实时检查，额度占用同步更新</t>
+          <t>各品种做市参数配置（报价宽度/报价量/报价频率），分时段策略，按交易对手差异化报价</t>
         </is>
       </c>
       <c r="F205" s="16" t="inlineStr">
@@ -14460,14 +15068,294 @@
         <v>20</v>
       </c>
     </row>
-    <row r="206">
-      <c r="A206" s="19" t="inlineStr">
+    <row r="206" ht="28" customHeight="1">
+      <c r="A206" s="16" t="inlineStr">
+        <is>
+          <t>做市商系统</t>
+        </is>
+      </c>
+      <c r="B206" s="15" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="C206" s="15" t="inlineStr">
+        <is>
+          <t>F15-06</t>
+        </is>
+      </c>
+      <c r="D206" s="30" t="inlineStr">
+        <is>
+          <t>报价优化算法</t>
+        </is>
+      </c>
+      <c r="E206" s="16" t="inlineStr">
+        <is>
+          <t>基于市场微结构理论动态调整bid-ask spread，流动性自适应调节，机器学习辅助报价优化</t>
+        </is>
+      </c>
+      <c r="F206" s="16" t="inlineStr">
+        <is>
+          <t>p99延迟/误差率/精度验证/压测10k TPS</t>
+        </is>
+      </c>
+      <c r="G206" s="28" t="inlineStr">
+        <is>
+          <t>极高</t>
+        </is>
+      </c>
+      <c r="H206" s="18" t="n">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="207" ht="28" customHeight="1">
+      <c r="A207" s="16" t="inlineStr">
+        <is>
+          <t>做市商系统</t>
+        </is>
+      </c>
+      <c r="B207" s="15" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="C207" s="15" t="inlineStr">
+        <is>
+          <t>F15-07</t>
+        </is>
+      </c>
+      <c r="D207" s="30" t="inlineStr">
+        <is>
+          <t>债券过滤与筛选</t>
+        </is>
+      </c>
+      <c r="E207" s="16" t="inlineStr">
+        <is>
+          <t>做市标的券池管理，流动性分级筛选，黑名单管理，临时暂停做市规则</t>
+        </is>
+      </c>
+      <c r="F207" s="16" t="inlineStr">
+        <is>
+          <t>功能测试通过</t>
+        </is>
+      </c>
+      <c r="G207" s="25" t="inlineStr">
+        <is>
+          <t>低</t>
+        </is>
+      </c>
+      <c r="H207" s="18" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="208" ht="28" customHeight="1">
+      <c r="A208" s="16" t="inlineStr">
+        <is>
+          <t>做市商系统</t>
+        </is>
+      </c>
+      <c r="B208" s="15" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="C208" s="15" t="inlineStr">
+        <is>
+          <t>F15-08</t>
+        </is>
+      </c>
+      <c r="D208" s="30" t="inlineStr">
+        <is>
+          <t>做市义务实时监控</t>
+        </is>
+      </c>
+      <c r="E208" s="16" t="inlineStr">
+        <is>
+          <t>实时监控做市义务完成情况（报价连续性/报价宽度/报价量达标），义务违规预警，监管报告生成</t>
+        </is>
+      </c>
+      <c r="F208" s="16" t="inlineStr">
+        <is>
+          <t>功能完整/边界测试/集成冒烟/性能基线</t>
+        </is>
+      </c>
+      <c r="G208" s="23" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="H208" s="18" t="n">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="209" ht="28" customHeight="1">
+      <c r="A209" s="16" t="inlineStr">
+        <is>
+          <t>做市商系统</t>
+        </is>
+      </c>
+      <c r="B209" s="15" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="C209" s="15" t="inlineStr">
+        <is>
+          <t>F15-09</t>
+        </is>
+      </c>
+      <c r="D209" s="30" t="inlineStr">
+        <is>
+          <t>做市行情展示</t>
+        </is>
+      </c>
+      <c r="E209" s="16" t="inlineStr">
+        <is>
+          <t>做市报价行情矩阵，实时价格展示，报价历史回放，市场最优报价对比，中签率统计</t>
+        </is>
+      </c>
+      <c r="F209" s="16" t="inlineStr">
+        <is>
+          <t>功能测试通过/正确率100%</t>
+        </is>
+      </c>
+      <c r="G209" s="24" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="H209" s="18" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="210" ht="28" customHeight="1">
+      <c r="A210" s="16" t="inlineStr">
+        <is>
+          <t>做市商系统</t>
+        </is>
+      </c>
+      <c r="B210" s="15" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="C210" s="15" t="inlineStr">
+        <is>
+          <t>F15-10</t>
+        </is>
+      </c>
+      <c r="D210" s="30" t="inlineStr">
+        <is>
+          <t>做市订单管理</t>
+        </is>
+      </c>
+      <c r="E210" s="16" t="inlineStr">
+        <is>
+          <t>做市委托生成、撤改、成交回报处理，订单状态实时跟踪，批量撤单，做市台账</t>
+        </is>
+      </c>
+      <c r="F210" s="16" t="inlineStr">
+        <is>
+          <t>功能完整/边界测试/集成冒烟/性能基线</t>
+        </is>
+      </c>
+      <c r="G210" s="23" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="H210" s="18" t="n">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="211" ht="28" customHeight="1">
+      <c r="A211" s="16" t="inlineStr">
+        <is>
+          <t>做市商系统</t>
+        </is>
+      </c>
+      <c r="B211" s="15" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="C211" s="15" t="inlineStr">
+        <is>
+          <t>F15-11</t>
+        </is>
+      </c>
+      <c r="D211" s="30" t="inlineStr">
+        <is>
+          <t>库存风险实时管理</t>
+        </is>
+      </c>
+      <c r="E211" s="16" t="inlineStr">
+        <is>
+          <t>做市库存PnL实时监控，Delta对冲自动触发，库存敞口上限控制，实时盯市损益</t>
+        </is>
+      </c>
+      <c r="F211" s="16" t="inlineStr">
+        <is>
+          <t>p99延迟/误差率/精度验证/压测10k TPS</t>
+        </is>
+      </c>
+      <c r="G211" s="28" t="inlineStr">
+        <is>
+          <t>极高</t>
+        </is>
+      </c>
+      <c r="H211" s="18" t="n">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="212" ht="28" customHeight="1">
+      <c r="A212" s="16" t="inlineStr">
+        <is>
+          <t>做市商系统</t>
+        </is>
+      </c>
+      <c r="B212" s="15" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="C212" s="15" t="inlineStr">
+        <is>
+          <t>F15-12</t>
+        </is>
+      </c>
+      <c r="D212" s="30" t="inlineStr">
+        <is>
+          <t>竞争力分析</t>
+        </is>
+      </c>
+      <c r="E212" s="16" t="inlineStr">
+        <is>
+          <t>与市场最优报价对比，中签率分析，报价表现统计，策略调优建议，竞争对手报价分析</t>
+        </is>
+      </c>
+      <c r="F212" s="16" t="inlineStr">
+        <is>
+          <t>功能完整/边界测试/集成冒烟/性能基线</t>
+        </is>
+      </c>
+      <c r="G212" s="23" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="H212" s="18" t="n">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213" s="19" t="inlineStr">
         <is>
           <t>总计功能数 / Total Function Points</t>
         </is>
       </c>
-      <c r="H206" s="20">
-        <f>SUM(H3:H205)</f>
+      <c r="H213" s="20">
+        <f>SUM(H3:H212)</f>
         <v/>
       </c>
     </row>
@@ -14477,9 +15365,9 @@
     <mergeCell ref="A3:H3"/>
     <mergeCell ref="A101:H101"/>
     <mergeCell ref="A130:H130"/>
+    <mergeCell ref="A213:G213"/>
     <mergeCell ref="A200:H200"/>
     <mergeCell ref="A180:H180"/>
-    <mergeCell ref="A206:G206"/>
     <mergeCell ref="A60:H60"/>
     <mergeCell ref="A112:H112"/>
     <mergeCell ref="A68:H68"/>

</xml_diff>

<commit_message>
Expand module 07 (组合管理+绩效归因) to 18 functions per gy_solution 4.4.1
Deep analysis from gy_solution.md section 4.4.1 added 3 new functions:
- F07-07 Campisi 2.0 固收绩效归因 (五效应: 收入/国债平移斜率曲率/利差/交易/残差)
- F07-10 因子风险分解+MCTR边际风险贡献 (2200+因子, 风险大户排名)
- F07-11 Component VaR四层穿透 (资产类/行业/评级/发行人, 三方法互验)
- F07-15 衍生品对冲决策引擎 (七类工具矩阵, 系统推荐最优对冲方案)
Duration updated to 14m/160pm.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Feasibility_analysis/FICC_Gap_Analysis.xlsx
+++ b/Feasibility_analysis/FICC_Gap_Analysis.xlsx
@@ -1359,17 +1359,17 @@
         </is>
       </c>
       <c r="M9" s="3" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="N9" s="3" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="O9" s="8" t="n">
-        <v>120</v>
+        <v>160</v>
       </c>
       <c r="P9" s="5" t="inlineStr">
         <is>
-          <t>17项功能含量化底座集成；Slide44全景展开</t>
+          <t>全资产组合管理驾驶舱，十大核心能力：全资产持仓模型/QP优化/Shadow Portfolio/Campisi 2.0固收归因/Brinson归因/因子风险分解+MCTR/Component VaR/敏感度/情景压测/流动性；对应PPT Slide 44 + gy_solution 4.4.1</t>
         </is>
       </c>
     </row>
@@ -2454,7 +2454,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J28"/>
+  <dimension ref="A1:J29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -2479,14 +2479,14 @@
     <row r="2" ht="36" customHeight="1">
       <c r="A2" s="39" t="inlineStr">
         <is>
-          <t>战略定位：17项功能含量化底座集成；Slide44全景展开   |   来源：Slide 44   |   数据输入：交易数据 / 头寸数据 / 行情数据 / 估值数据   |   量化底座：定价计算 · 利率曲线 · 因子模型</t>
+          <t>战略定位：全资产组合管理驾驶舱，十大核心能力：全资产持仓模型/QP优化/Shadow Portfolio/Campisi 2.0固收归因/Brinson归因/因子风险分解+MCTR/Component VaR/敏感度/情景压测/流动性；对应PPT Slide 44 + gy_solution 4.4.1   |   来源：Slide 44   |   数据输入：交易数据 / 头寸数据 / 行情数据 / 估值数据   |   量化底座：定价计算 · 利率曲线 · 因子模型(2200+风险因子)</t>
         </is>
       </c>
     </row>
     <row r="3" ht="28" customHeight="1">
       <c r="A3" s="40" t="inlineStr">
         <is>
-          <t>模块：组合管理+绩效归因  (Portfolio Mgmt &amp; Perf)  |  优先级：P1  |  竞品：SimCorp/衡泰  |  华锐基础：M9 PMS模块  |  工期：12月  团队：12人</t>
+          <t>模块：组合管理+绩效归因  (Portfolio Mgmt &amp; Perf)  |  优先级：P1  |  竞品：SimCorp/衡泰  |  华锐基础：M9 PMS模块  |  工期：14月  团队：14人</t>
         </is>
       </c>
     </row>
@@ -2545,14 +2545,14 @@
     <row r="5" ht="18" customHeight="1">
       <c r="A5" s="22" t="inlineStr">
         <is>
-          <t>A. 组合分析</t>
+          <t>A. 全资产持仓管理</t>
         </is>
       </c>
     </row>
     <row r="6" ht="48" customHeight="1">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>A. 组合分析</t>
+          <t>A. 全资产持仓管理</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
@@ -2562,22 +2562,22 @@
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>债券横截面与时序分析</t>
+          <t>全资产统一持仓模型</t>
         </is>
       </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
-          <t>跨品种横截面信号挖掘（利差/久期偏差），历史时序趋势与均值回归分析</t>
+          <t>八类资产（利率债/信用债/权益/基金/黄金/商品/衍生品/非标）实时T+0持仓，多层组合树（公司→部门→策略→子组合→投资经理），穿透式敞口展示（品种/久期/评级/行业/地区分布），真实组合+Shadow Portfolio并行展示</t>
         </is>
       </c>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t>横截面信号与实际收益相关性&gt;0.3</t>
+          <t>T+0持仓实时刷新，穿透层级≥5层，数据与IBOR差异&lt;0.01%</t>
         </is>
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>AMD行情平台/估值数据</t>
+          <t>IBOR持仓账薄/AMD行情</t>
         </is>
       </c>
       <c r="G6" s="41" t="inlineStr">
@@ -2586,7 +2586,7 @@
         </is>
       </c>
       <c r="H6" s="8" t="n">
-        <v>35</v>
+        <v>40</v>
       </c>
       <c r="I6" s="6" t="inlineStr">
         <is>
@@ -2598,7 +2598,7 @@
     <row r="7" ht="48" customHeight="1">
       <c r="A7" s="5" t="inlineStr">
         <is>
-          <t>A. 组合分析</t>
+          <t>A. 全资产持仓管理</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
@@ -2608,22 +2608,22 @@
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>相对价值分析</t>
+          <t>跨资产相关性分析</t>
         </is>
       </c>
       <c r="D7" s="5" t="inlineStr">
         <is>
-          <t>利差/Z-spread/OAS相对价值计算，历史分位数定位，跨品种套利信号识别</t>
+          <t>全持仓跨资产相关矩阵（股/债/商品/衍生品/基金），多窗口滚动（20/60/252日），压力情景相关性vs历史相关性对比，动态相关性漂移预警，分散化比率(Diversification Ratio)计算，低相关候选资产推荐</t>
         </is>
       </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t>OAS计算误差&lt;1bps，分位数覆盖5年历史</t>
+          <t>相关矩阵计算&lt;30s（500券组合），动态漂移预警阈值可配</t>
         </is>
       </c>
       <c r="F7" s="5" t="inlineStr">
         <is>
-          <t>量化定价引擎/AMD行情</t>
+          <t>IBOR头寸/AMD历史行情</t>
         </is>
       </c>
       <c r="G7" s="41" t="inlineStr">
@@ -2644,7 +2644,7 @@
     <row r="8" ht="48" customHeight="1">
       <c r="A8" s="5" t="inlineStr">
         <is>
-          <t>A. 组合分析</t>
+          <t>A. 全资产持仓管理</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
@@ -2654,31 +2654,31 @@
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>组合相关度分析</t>
+          <t>相对价值分析</t>
         </is>
       </c>
       <c r="D8" s="5" t="inlineStr">
         <is>
-          <t>资产间收益相关矩阵计算（滚动60/120/250日），组合集中度风险识别，分散化系数监控</t>
+          <t>利差/Z-spread/OAS相对价值计算，历史分位数定位（覆盖5年），跨品种套利信号识别，债券横截面信号挖掘（利差/久期偏差），时序均值回归分析</t>
         </is>
       </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
-          <t>相关矩阵计算&lt;30s（500券组合）</t>
+          <t>OAS计算误差&lt;1bps，历史分位数覆盖5年，横截面信号与实际收益相关性&gt;0.3</t>
         </is>
       </c>
       <c r="F8" s="5" t="inlineStr">
         <is>
-          <t>IBOR头寸/AMD历史行情</t>
-        </is>
-      </c>
-      <c r="G8" s="42" t="inlineStr">
-        <is>
-          <t>中</t>
+          <t>定价平台/AMD行情</t>
+        </is>
+      </c>
+      <c r="G8" s="41" t="inlineStr">
+        <is>
+          <t>高</t>
         </is>
       </c>
       <c r="H8" s="8" t="n">
-        <v>25</v>
+        <v>30</v>
       </c>
       <c r="I8" s="6" t="inlineStr">
         <is>
@@ -2690,14 +2690,14 @@
     <row r="9" ht="18" customHeight="1">
       <c r="A9" s="40" t="inlineStr">
         <is>
-          <t>B. 风险计量</t>
+          <t>B. 组合优化与再平衡</t>
         </is>
       </c>
     </row>
     <row r="10" ht="48" customHeight="1">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>B. 风险计量</t>
+          <t>B. 组合优化与再平衡</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr">
@@ -2707,22 +2707,22 @@
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>情景分析</t>
+          <t>QP智能再平衡引擎</t>
         </is>
       </c>
       <c r="D10" s="5" t="inlineStr">
         <is>
-          <t>利率/信用/流动性三类自定义情景，组合P&amp;L影响量化，多情景并行对比</t>
+          <t>二次规划多目标优化（最小化跟踪误差+交易摩擦+融资成本+IFRS9波动），500+约束（合规/风险预算/流动性/IFRS9），2000+持仓毫秒级求解，支持整数规划（面值/手数取整），多期优化（含到期券），三种触发（定时/事件/手动），一键生成交易指令</t>
         </is>
       </c>
       <c r="E10" s="5" t="inlineStr">
         <is>
-          <t>情景P&amp;L与手工核算误差&lt;0.5%，支持≥20情景并行</t>
+          <t>QP求解2000持仓&lt;200ms，约束满足率100%，调仓前后TE对比即时输出</t>
         </is>
       </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
-          <t>FICC风险计量平台/量化定价引擎</t>
+          <t>事前风控/合规/IBOR/现券系统/定价平台</t>
         </is>
       </c>
       <c r="G10" s="41" t="inlineStr">
@@ -2731,7 +2731,7 @@
         </is>
       </c>
       <c r="H10" s="8" t="n">
-        <v>35</v>
+        <v>40</v>
       </c>
       <c r="I10" s="6" t="inlineStr">
         <is>
@@ -2743,7 +2743,7 @@
     <row r="11" ht="48" customHeight="1">
       <c r="A11" s="5" t="inlineStr">
         <is>
-          <t>B. 风险计量</t>
+          <t>B. 组合优化与再平衡</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
@@ -2753,22 +2753,22 @@
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>敏感度分析</t>
+          <t>Shadow Portfolio虚拟试算</t>
         </is>
       </c>
       <c r="D11" s="5" t="inlineStr">
         <is>
-          <t>久期/DV01/凸度/利差/Vega敏感度多因子并行计算，组合对冲比率建议</t>
+          <t>100+虚拟组合与真实组合并行运行，多维试算（增减仓/换仓/加杠杆/新资产类别），即时显示试算后风险指标/归因/相关性/预期收益，真实vs虚拟所有指标差异对比视图，冲击成本预估</t>
         </is>
       </c>
       <c r="E11" s="5" t="inlineStr">
         <is>
-          <t>DV01与Bloomberg基准误差&lt;0.5bps</t>
+          <t>虚拟组合模拟与真实执行偏差&lt;0.3%，秒级响应</t>
         </is>
       </c>
       <c r="F11" s="5" t="inlineStr">
         <is>
-          <t>量化定价引擎Greeks接口</t>
+          <t>IBOR/定价平台/现券交易系统</t>
         </is>
       </c>
       <c r="G11" s="41" t="inlineStr">
@@ -2777,7 +2777,7 @@
         </is>
       </c>
       <c r="H11" s="8" t="n">
-        <v>25</v>
+        <v>30</v>
       </c>
       <c r="I11" s="6" t="inlineStr">
         <is>
@@ -2787,34 +2787,34 @@
       <c r="J11" s="5" t="inlineStr"/>
     </row>
     <row r="12" ht="48" customHeight="1">
-      <c r="A12" s="5" t="inlineStr">
-        <is>
-          <t>B. 风险计量</t>
-        </is>
-      </c>
-      <c r="B12" s="3" t="inlineStr">
+      <c r="A12" s="11" t="inlineStr">
+        <is>
+          <t>B. 组合优化与再平衡</t>
+        </is>
+      </c>
+      <c r="B12" s="10" t="inlineStr">
         <is>
           <t>F07-06</t>
         </is>
       </c>
-      <c r="C12" s="4" t="inlineStr">
-        <is>
-          <t>极端事件分析</t>
-        </is>
-      </c>
-      <c r="D12" s="5" t="inlineStr">
-        <is>
-          <t>历史极端情景（924行情/2015股灾/2020疫情等8+情景），组合尾部损失分布，ES(99%)计算</t>
-        </is>
-      </c>
-      <c r="E12" s="5" t="inlineStr">
-        <is>
-          <t>历史情景复现误差&lt;1%</t>
-        </is>
-      </c>
-      <c r="F12" s="5" t="inlineStr">
-        <is>
-          <t>FICC风险计量平台</t>
+      <c r="C12" s="27" t="inlineStr">
+        <is>
+          <t>资产配置策略分析</t>
+        </is>
+      </c>
+      <c r="D12" s="11" t="inlineStr">
+        <is>
+          <t>SAA战略→TAA战术精准联动（投委会指令直接转化为因子约束输入QP引擎），宏观因子（利率/信用/流动性周期）驱动大类资产配置模型，动态权重优化，历史回测验证（≥5年），固收+策略P&amp;L归因（债券底仓+衍生品增强）</t>
+        </is>
+      </c>
+      <c r="E12" s="11" t="inlineStr">
+        <is>
+          <t>回测期≥5年，预测方向胜率&gt;55%，SAA→TAA指令转化全程无人工干预</t>
+        </is>
+      </c>
+      <c r="F12" s="11" t="inlineStr">
+        <is>
+          <t>AMD宏观数据/因子模型/IBOR</t>
         </is>
       </c>
       <c r="G12" s="41" t="inlineStr">
@@ -2822,15 +2822,15 @@
           <t>高</t>
         </is>
       </c>
-      <c r="H12" s="8" t="n">
-        <v>30</v>
-      </c>
-      <c r="I12" s="6" t="inlineStr">
-        <is>
-          <t>P1</t>
-        </is>
-      </c>
-      <c r="J12" s="5" t="inlineStr"/>
+      <c r="H12" s="13" t="n">
+        <v>40</v>
+      </c>
+      <c r="I12" s="12" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="J12" s="11" t="inlineStr"/>
     </row>
     <row r="13" ht="18" customHeight="1">
       <c r="A13" s="43" t="inlineStr">
@@ -2852,31 +2852,31 @@
       </c>
       <c r="C14" s="4" t="inlineStr">
         <is>
-          <t>指数比较分析</t>
+          <t>Campisi 2.0 固收绩效归因</t>
         </is>
       </c>
       <c r="D14" s="5" t="inlineStr">
         <is>
-          <t>对标中债综合/信用/政策行等指数，跟踪误差（TE）日频监控，超额Alpha三因子分解</t>
+          <t>固定收益五效应完整拆解：①收入效应（票息+摊销），②国债效应（利率平移/曲线斜率/曲率三效应分离，用Key Rate Duration精确映射），③利差效应（DTS贡献/行业配置效应/个券选择效应），④交易效应（择时Alpha或损耗量化），⑤残差校验（&lt;5bp合格）；日/周/月/季多维度报告自动生成</t>
         </is>
       </c>
       <c r="E14" s="5" t="inlineStr">
         <is>
-          <t>TE计算误差&lt;1bps，支持≥10基准指数</t>
+          <t>五效应合计与实际收益残差&lt;5bps，T+1 9:00前自动报告</t>
         </is>
       </c>
       <c r="F14" s="5" t="inlineStr">
         <is>
-          <t>AMD中债估值/IBOR持仓</t>
-        </is>
-      </c>
-      <c r="G14" s="42" t="inlineStr">
-        <is>
-          <t>中</t>
+          <t>IBOR持仓/AMD行情/定价平台</t>
+        </is>
+      </c>
+      <c r="G14" s="41" t="inlineStr">
+        <is>
+          <t>高</t>
         </is>
       </c>
       <c r="H14" s="8" t="n">
-        <v>25</v>
+        <v>40</v>
       </c>
       <c r="I14" s="6" t="inlineStr">
         <is>
@@ -2898,17 +2898,17 @@
       </c>
       <c r="C15" s="4" t="inlineStr">
         <is>
-          <t>绩效归因（Brinson）</t>
+          <t>Brinson 资产组合绩效归因</t>
         </is>
       </c>
       <c r="D15" s="5" t="inlineStr">
         <is>
-          <t>BHB三效应：资产配置/个券选择/交互效应，日/周/月/季多维度，报告PDF自动生成</t>
+          <t>三效应：大类资产配置效应（超/低配决策贡献）/个券选择效应（同类标的选择Alpha）/交互效应，支持多层穿透（资产大类→行业→子行业→个股/个基），FOF基金穿透底层持仓，日/月/季/年累计归因趋势，投资经理能力量化排名</t>
         </is>
       </c>
       <c r="E15" s="5" t="inlineStr">
         <is>
-          <t>Brinson结果与Bloomberg AIM误差&lt;0.1%，T+1 9:00前自动报告</t>
+          <t>Brinson结果与Bloomberg AIM误差&lt;0.1%，穿透层级≥4层</t>
         </is>
       </c>
       <c r="F15" s="5" t="inlineStr">
@@ -2922,7 +2922,7 @@
         </is>
       </c>
       <c r="H15" s="8" t="n">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="I15" s="6" t="inlineStr">
         <is>
@@ -2931,63 +2931,63 @@
       </c>
       <c r="J15" s="5" t="inlineStr"/>
     </row>
-    <row r="16" ht="18" customHeight="1">
-      <c r="A16" s="43" t="inlineStr">
-        <is>
-          <t>D. 组合优化与再平衡</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="48" customHeight="1">
-      <c r="A17" s="5" t="inlineStr">
-        <is>
-          <t>D. 组合优化与再平衡</t>
-        </is>
-      </c>
-      <c r="B17" s="3" t="inlineStr">
+    <row r="16" ht="48" customHeight="1">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>C. 绩效归因</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="inlineStr">
         <is>
           <t>F07-09</t>
         </is>
       </c>
-      <c r="C17" s="4" t="inlineStr">
-        <is>
-          <t>虚拟组合分析</t>
-        </is>
-      </c>
-      <c r="D17" s="5" t="inlineStr">
-        <is>
-          <t>组合调整前后净值/风险/收益效果模拟（纸面交易），冲击成本预估，多方案对比</t>
-        </is>
-      </c>
-      <c r="E17" s="5" t="inlineStr">
-        <is>
-          <t>虚拟组合模拟与真实执行偏差&lt;0.3%</t>
-        </is>
-      </c>
-      <c r="F17" s="5" t="inlineStr">
-        <is>
-          <t>IBOR/现券交易系统</t>
-        </is>
-      </c>
-      <c r="G17" s="41" t="inlineStr">
-        <is>
-          <t>高</t>
-        </is>
-      </c>
-      <c r="H17" s="8" t="n">
-        <v>20</v>
-      </c>
-      <c r="I17" s="6" t="inlineStr">
-        <is>
-          <t>P1</t>
-        </is>
-      </c>
-      <c r="J17" s="5" t="inlineStr"/>
+      <c r="C16" s="4" t="inlineStr">
+        <is>
+          <t>指数跟踪误差与主动风险归因</t>
+        </is>
+      </c>
+      <c r="D16" s="5" t="inlineStr">
+        <is>
+          <t>对标中债综合/信用/政策行等基准指数，跟踪误差（TE）日频监控，TE分解（配置效应TE+选券效应TE+协方差），信息比率（IR）实时监控（目标IR&gt;0.5，预警IR连续3月&lt;0），超额Alpha三因子分解</t>
+        </is>
+      </c>
+      <c r="E16" s="5" t="inlineStr">
+        <is>
+          <t>TE计算误差&lt;1bps，支持≥10基准指数，IR预警自动推送</t>
+        </is>
+      </c>
+      <c r="F16" s="5" t="inlineStr">
+        <is>
+          <t>AMD中债估值/IBOR持仓/因子模型</t>
+        </is>
+      </c>
+      <c r="G16" s="42" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="H16" s="8" t="n">
+        <v>25</v>
+      </c>
+      <c r="I16" s="6" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="J16" s="5" t="inlineStr"/>
+    </row>
+    <row r="17" ht="18" customHeight="1">
+      <c r="A17" s="43" t="inlineStr">
+        <is>
+          <t>D. 风险计量</t>
+        </is>
+      </c>
     </row>
     <row r="18" ht="48" customHeight="1">
       <c r="A18" s="5" t="inlineStr">
         <is>
-          <t>D. 组合优化与再平衡</t>
+          <t>D. 风险计量</t>
         </is>
       </c>
       <c r="B18" s="3" t="inlineStr">
@@ -2997,22 +2997,22 @@
       </c>
       <c r="C18" s="4" t="inlineStr">
         <is>
-          <t>再平衡方案试算与比较</t>
+          <t>因子风险分解 + MCTR边际风险贡献</t>
         </is>
       </c>
       <c r="D18" s="5" t="inlineStr">
         <is>
-          <t>久期/集中度/流动性/合规约束联合优化（二次规划QP），多方案并行试算，最优路径推荐</t>
+          <t>全持仓分解为2200+风险因子（利率/信用/权益/商品/汇率），系统性风险+特异性风险分离；MCTR边际风险贡献（∂组合波动率/∂持仓权重），风险消耗排名（识别"风险大户"），减仓/加仓优先级引导，风险预算仪表盘（已用/剩余/预警线三档）</t>
         </is>
       </c>
       <c r="E18" s="5" t="inlineStr">
         <is>
-          <t>QP求解100券组合&lt;5s，约束满足率100%</t>
+          <t>因子模型解释方差&gt;80%，MCTR实时更新延迟&lt;5s，Alpha IC均值&gt;0.05</t>
         </is>
       </c>
       <c r="F18" s="5" t="inlineStr">
         <is>
-          <t>事前风控/合规/IBOR/现券系统</t>
+          <t>AMD历史行情/IBOR持仓/定价平台</t>
         </is>
       </c>
       <c r="G18" s="41" t="inlineStr">
@@ -3021,164 +3021,164 @@
         </is>
       </c>
       <c r="H18" s="8" t="n">
+        <v>40</v>
+      </c>
+      <c r="I18" s="6" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="J18" s="5" t="inlineStr"/>
+    </row>
+    <row r="19" ht="48" customHeight="1">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t>D. 风险计量</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>F07-11</t>
+        </is>
+      </c>
+      <c r="C19" s="4" t="inlineStr">
+        <is>
+          <t>Component VaR 四层穿透分析</t>
+        </is>
+      </c>
+      <c r="D19" s="5" t="inlineStr">
+        <is>
+          <t>VaR四层穿透：资产类别VaR→行业/子市场VaR→评级/信用质量VaR→单一发行人Component VaR，含跨类分散化收益量化；三种方法互验（历史模拟500日99%置信度/Monte Carlo 10000次/参数解析法），方法差异超阈值自动预警</t>
+        </is>
+      </c>
+      <c r="E19" s="5" t="inlineStr">
+        <is>
+          <t>三方法VaR差异&lt;10%，穿透至发行人层，全量计算&lt;1min</t>
+        </is>
+      </c>
+      <c r="F19" s="5" t="inlineStr">
+        <is>
+          <t>FICC风险计量平台/定价平台/IBOR</t>
+        </is>
+      </c>
+      <c r="G19" s="41" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="H19" s="8" t="n">
         <v>35</v>
       </c>
-      <c r="I18" s="6" t="inlineStr">
-        <is>
-          <t>P1</t>
-        </is>
-      </c>
-      <c r="J18" s="5" t="inlineStr"/>
-    </row>
-    <row r="19" ht="48" customHeight="1">
-      <c r="A19" s="11" t="inlineStr">
-        <is>
-          <t>D. 组合优化与再平衡</t>
-        </is>
-      </c>
-      <c r="B19" s="10" t="inlineStr">
-        <is>
-          <t>F07-11</t>
-        </is>
-      </c>
-      <c r="C19" s="27" t="inlineStr">
-        <is>
-          <t>资产配置策略分析</t>
-        </is>
-      </c>
-      <c r="D19" s="11" t="inlineStr">
-        <is>
-          <t>宏观因子（利率/信用/流动性周期）驱动大类资产配置模型，动态权重优化，历史回测验证</t>
-        </is>
-      </c>
-      <c r="E19" s="11" t="inlineStr">
-        <is>
-          <t>回测期≥5年，预测方向胜率&gt;55%</t>
-        </is>
-      </c>
-      <c r="F19" s="11" t="inlineStr">
-        <is>
-          <t>AMD宏观数据/因子模型</t>
-        </is>
-      </c>
-      <c r="G19" s="41" t="inlineStr">
+      <c r="I19" s="6" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="J19" s="5" t="inlineStr"/>
+    </row>
+    <row r="20" ht="48" customHeight="1">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>D. 风险计量</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>F07-12</t>
+        </is>
+      </c>
+      <c r="C20" s="4" t="inlineStr">
+        <is>
+          <t>敏感度分析（多维Shock Grid）</t>
+        </is>
+      </c>
+      <c r="D20" s="5" t="inlineStr">
+        <is>
+          <t>利率敏感度（DV01/关键期限点KRD/凸性），信用敏感度（CS01/DTS分评级/分行业），权益敏感度（Delta/Beta/行业Beta），商品汇率敏感度；利率×信用利差二维冲击矩阵（Shock Grid），识别最脆弱组合方向，对冲比率建议</t>
+        </is>
+      </c>
+      <c r="E20" s="5" t="inlineStr">
+        <is>
+          <t>DV01与Bloomberg基准误差&lt;0.5bps，Shock Grid 5×5矩阵实时刷新</t>
+        </is>
+      </c>
+      <c r="F20" s="5" t="inlineStr">
+        <is>
+          <t>定价平台Greeks接口/IBOR</t>
+        </is>
+      </c>
+      <c r="G20" s="41" t="inlineStr">
         <is>
           <t>高</t>
         </is>
       </c>
-      <c r="H19" s="13" t="n">
-        <v>40</v>
-      </c>
-      <c r="I19" s="12" t="inlineStr">
-        <is>
-          <t>P2</t>
-        </is>
-      </c>
-      <c r="J19" s="11" t="inlineStr"/>
-    </row>
-    <row r="20" ht="48" customHeight="1">
-      <c r="A20" s="11" t="inlineStr">
-        <is>
-          <t>D. 组合优化与再平衡</t>
-        </is>
-      </c>
-      <c r="B20" s="10" t="inlineStr">
-        <is>
-          <t>F07-12</t>
-        </is>
-      </c>
-      <c r="C20" s="27" t="inlineStr">
-        <is>
-          <t>固收+策略分析</t>
-        </is>
-      </c>
-      <c r="D20" s="11" t="inlineStr">
-        <is>
-          <t>债券底仓+衍生品增强策略P&amp;L归因，风险分解（利率/信用/期权贡献），固收+净值模拟</t>
-        </is>
-      </c>
-      <c r="E20" s="11" t="inlineStr">
-        <is>
-          <t>固收+净值模拟与实际偏差&lt;0.5%</t>
-        </is>
-      </c>
-      <c r="F20" s="11" t="inlineStr">
-        <is>
-          <t>IBOR/利率衍生品系统</t>
-        </is>
-      </c>
-      <c r="G20" s="41" t="inlineStr">
+      <c r="H20" s="8" t="n">
+        <v>30</v>
+      </c>
+      <c r="I20" s="6" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="J20" s="5" t="inlineStr"/>
+    </row>
+    <row r="21" ht="48" customHeight="1">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t>D. 风险计量</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>F07-13</t>
+        </is>
+      </c>
+      <c r="C21" s="4" t="inlineStr">
+        <is>
+          <t>情景分析与压力测试</t>
+        </is>
+      </c>
+      <c r="D21" s="5" t="inlineStr">
+        <is>
+          <t>三层：①历史情景重演（924行情/2019包商/2013钱荒/2015股灾等8+事件，含冲击参数还原），②假设情景模拟（自定义任意冲击组合，即时P&amp;L输出+应急对冲建议），③反向压力测试（倒推触发止损线的临界市场情景+历史发生频率），≥20情景并行</t>
+        </is>
+      </c>
+      <c r="E21" s="5" t="inlineStr">
+        <is>
+          <t>历史情景复现误差&lt;1%，情景P&amp;L误差&lt;0.5%，支持≥20情景并行</t>
+        </is>
+      </c>
+      <c r="F21" s="5" t="inlineStr">
+        <is>
+          <t>FICC风险计量平台/定价平台</t>
+        </is>
+      </c>
+      <c r="G21" s="41" t="inlineStr">
         <is>
           <t>高</t>
         </is>
       </c>
-      <c r="H20" s="13" t="n">
-        <v>30</v>
-      </c>
-      <c r="I20" s="12" t="inlineStr">
-        <is>
-          <t>P2</t>
-        </is>
-      </c>
-      <c r="J20" s="11" t="inlineStr"/>
-    </row>
-    <row r="21" ht="48" customHeight="1">
-      <c r="A21" s="11" t="inlineStr">
-        <is>
-          <t>D. 组合优化与再平衡</t>
-        </is>
-      </c>
-      <c r="B21" s="10" t="inlineStr">
-        <is>
-          <t>F07-13</t>
-        </is>
-      </c>
-      <c r="C21" s="27" t="inlineStr">
-        <is>
-          <t>量化策略组合分析</t>
-        </is>
-      </c>
-      <c r="D21" s="11" t="inlineStr">
-        <is>
-          <t>多策略组合叠加容量约束，策略相关性管理，Sharpe/最大回撤/Calmar实时监控</t>
-        </is>
-      </c>
-      <c r="E21" s="11" t="inlineStr">
-        <is>
-          <t>策略容量计算误差&lt;5%</t>
-        </is>
-      </c>
-      <c r="F21" s="11" t="inlineStr">
-        <is>
-          <t>策略投资/量化系统</t>
-        </is>
-      </c>
-      <c r="G21" s="41" t="inlineStr">
-        <is>
-          <t>高</t>
-        </is>
-      </c>
-      <c r="H21" s="13" t="n">
+      <c r="H21" s="8" t="n">
         <v>35</v>
       </c>
-      <c r="I21" s="12" t="inlineStr">
-        <is>
-          <t>P2</t>
-        </is>
-      </c>
-      <c r="J21" s="11" t="inlineStr"/>
+      <c r="I21" s="6" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="J21" s="5" t="inlineStr"/>
     </row>
     <row r="22" ht="18" customHeight="1">
       <c r="A22" s="29" t="inlineStr">
         <is>
-          <t>E. 流动性管理</t>
+          <t>E. 流动性与对冲管理</t>
         </is>
       </c>
     </row>
     <row r="23" ht="48" customHeight="1">
       <c r="A23" s="5" t="inlineStr">
         <is>
-          <t>E. 流动性管理</t>
+          <t>E. 流动性与对冲管理</t>
         </is>
       </c>
       <c r="B23" s="3" t="inlineStr">
@@ -3188,17 +3188,17 @@
       </c>
       <c r="C23" s="4" t="inlineStr">
         <is>
-          <t>流动性分析</t>
+          <t>流动性风险管理（LVaR）</t>
         </is>
       </c>
       <c r="D23" s="5" t="inlineStr">
         <is>
-          <t>逐券换手率/市场深度评估，组合变现能力分析，流动性压力下变现损失（LVaR）估算</t>
+          <t>逐持仓变现能力评估（规模/日均成交量→变现天数），Almgren-Chriss市场冲击成本模型，流动性压力测试（X天内变现Y亿最优路径+成本），流动性调整VaR（LVaR=传统VaR+流动性溢价），流动性覆盖率/缓冲监控（1/3/5/10日分层），回购到期日历</t>
         </is>
       </c>
       <c r="E23" s="5" t="inlineStr">
         <is>
-          <t>LVaR与市场基准误差&lt;5%，日均成交量覆盖≥95%持仓</t>
+          <t>LVaR与市场基准误差&lt;5%，日均成交量覆盖≥95%持仓，变现路径建议&lt;3s</t>
         </is>
       </c>
       <c r="F23" s="5" t="inlineStr">
@@ -3212,113 +3212,113 @@
         </is>
       </c>
       <c r="H23" s="8" t="n">
+        <v>25</v>
+      </c>
+      <c r="I23" s="6" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="J23" s="5" t="inlineStr"/>
+    </row>
+    <row r="24" ht="48" customHeight="1">
+      <c r="A24" s="11" t="inlineStr">
+        <is>
+          <t>E. 流动性与对冲管理</t>
+        </is>
+      </c>
+      <c r="B24" s="10" t="inlineStr">
+        <is>
+          <t>F07-15</t>
+        </is>
+      </c>
+      <c r="C24" s="27" t="inlineStr">
+        <is>
+          <t>衍生品对冲决策引擎</t>
+        </is>
+      </c>
+      <c r="D24" s="11" t="inlineStr">
+        <is>
+          <t>七类工具矩阵（国债期货2/5/10/30Y/IRS/CDS/股指期货IF/IH/IC/IM/股指期权/黄金期货/外汇远掉期），系统推荐最优对冲方案（成本最小约束），一键生成对冲指令，对冲效果追踪（前后风险指标对比/效率/执行滑点）；支持快速/精细/尾部/跨资产四种场景</t>
+        </is>
+      </c>
+      <c r="E24" s="11" t="inlineStr">
+        <is>
+          <t>对冲方案推荐&lt;5s，DV01对冲误差&lt;5%，指令自动流转执行引擎</t>
+        </is>
+      </c>
+      <c r="F24" s="11" t="inlineStr">
+        <is>
+          <t>衍生品交易系统/IBOR/定价平台/事前风控</t>
+        </is>
+      </c>
+      <c r="G24" s="41" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="H24" s="13" t="n">
+        <v>30</v>
+      </c>
+      <c r="I24" s="12" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="J24" s="11" t="inlineStr"/>
+    </row>
+    <row r="25" ht="18" customHeight="1">
+      <c r="A25" s="44" t="inlineStr">
+        <is>
+          <t>F. 量化底座集成</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="48" customHeight="1">
+      <c r="A26" s="11" t="inlineStr">
+        <is>
+          <t>F. 量化底座集成</t>
+        </is>
+      </c>
+      <c r="B26" s="10" t="inlineStr">
+        <is>
+          <t>F07-16</t>
+        </is>
+      </c>
+      <c r="C26" s="27" t="inlineStr">
+        <is>
+          <t>定价计算集成</t>
+        </is>
+      </c>
+      <c r="D26" s="11" t="inlineStr">
+        <is>
+          <t>调用定价平台实时估值与Greeks（含权债/可转债/IRS），Redis缓存结果，Kafka推送持仓+估值变化事件，日终全量估值批处理</t>
+        </is>
+      </c>
+      <c r="E26" s="11" t="inlineStr">
+        <is>
+          <t>定价API p99&lt;200ms，日终全量估值&lt;30min（10万券）</t>
+        </is>
+      </c>
+      <c r="F26" s="11" t="inlineStr">
+        <is>
+          <t>定价平台</t>
+        </is>
+      </c>
+      <c r="G26" s="41" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="H26" s="13" t="n">
         <v>20</v>
       </c>
-      <c r="I23" s="6" t="inlineStr">
-        <is>
-          <t>P1</t>
-        </is>
-      </c>
-      <c r="J23" s="5" t="inlineStr"/>
-    </row>
-    <row r="24" ht="18" customHeight="1">
-      <c r="A24" s="44" t="inlineStr">
-        <is>
-          <t>F. 量化底座集成</t>
-        </is>
-      </c>
-    </row>
-    <row r="25" ht="48" customHeight="1">
-      <c r="A25" s="11" t="inlineStr">
-        <is>
-          <t>F. 量化底座集成</t>
-        </is>
-      </c>
-      <c r="B25" s="10" t="inlineStr">
-        <is>
-          <t>F07-15</t>
-        </is>
-      </c>
-      <c r="C25" s="27" t="inlineStr">
-        <is>
-          <t>定价计算集成</t>
-        </is>
-      </c>
-      <c r="D25" s="11" t="inlineStr">
-        <is>
-          <t>调用量化定价引擎实时估值与Greeks，含权债/可转债/IRS，结果缓存（Redis）与Kafka推送</t>
-        </is>
-      </c>
-      <c r="E25" s="11" t="inlineStr">
-        <is>
-          <t>定价API p99&lt;200ms，日终全量估值&lt;30min（10万券）</t>
-        </is>
-      </c>
-      <c r="F25" s="11" t="inlineStr">
-        <is>
-          <t>量化定价引擎</t>
-        </is>
-      </c>
-      <c r="G25" s="41" t="inlineStr">
-        <is>
-          <t>高</t>
-        </is>
-      </c>
-      <c r="H25" s="13" t="n">
-        <v>20</v>
-      </c>
-      <c r="I25" s="12" t="inlineStr">
+      <c r="I26" s="12" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
       </c>
-      <c r="J25" s="11" t="inlineStr"/>
-    </row>
-    <row r="26" ht="48" customHeight="1">
-      <c r="A26" s="5" t="inlineStr">
-        <is>
-          <t>F. 量化底座集成</t>
-        </is>
-      </c>
-      <c r="B26" s="3" t="inlineStr">
-        <is>
-          <t>F07-16</t>
-        </is>
-      </c>
-      <c r="C26" s="4" t="inlineStr">
-        <is>
-          <t>利率曲线集成</t>
-        </is>
-      </c>
-      <c r="D26" s="5" t="inlineStr">
-        <is>
-          <t>多曲线实时消费（国债/政策行/AAA信用/OIS），NS参数提取（水平/斜率/曲率），敏感度映射</t>
-        </is>
-      </c>
-      <c r="E26" s="5" t="inlineStr">
-        <is>
-          <t>曲线更新延迟&lt;1s，NS拟合R²&gt;0.999</t>
-        </is>
-      </c>
-      <c r="F26" s="5" t="inlineStr">
-        <is>
-          <t>AMD行情平台/量化定价引擎</t>
-        </is>
-      </c>
-      <c r="G26" s="42" t="inlineStr">
-        <is>
-          <t>中</t>
-        </is>
-      </c>
-      <c r="H26" s="8" t="n">
-        <v>15</v>
-      </c>
-      <c r="I26" s="6" t="inlineStr">
-        <is>
-          <t>P1</t>
-        </is>
-      </c>
-      <c r="J26" s="5" t="inlineStr"/>
+      <c r="J26" s="11" t="inlineStr"/>
     </row>
     <row r="27" ht="48" customHeight="1">
       <c r="A27" s="5" t="inlineStr">
@@ -3333,63 +3333,109 @@
       </c>
       <c r="C27" s="4" t="inlineStr">
         <is>
+          <t>利率曲线集成</t>
+        </is>
+      </c>
+      <c r="D27" s="5" t="inlineStr">
+        <is>
+          <t>多曲线实时消费（国债/政策行/AAA信用/OIS），NS参数提取（水平/斜率/曲率），关键期限点敏感度映射，曲线版本快照（供归因历史复现）</t>
+        </is>
+      </c>
+      <c r="E27" s="5" t="inlineStr">
+        <is>
+          <t>曲线更新延迟&lt;1s，NS拟合R²&gt;0.999</t>
+        </is>
+      </c>
+      <c r="F27" s="5" t="inlineStr">
+        <is>
+          <t>AMD行情平台/定价平台</t>
+        </is>
+      </c>
+      <c r="G27" s="42" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="H27" s="8" t="n">
+        <v>15</v>
+      </c>
+      <c r="I27" s="6" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="J27" s="5" t="inlineStr"/>
+    </row>
+    <row r="28" ht="48" customHeight="1">
+      <c r="A28" s="5" t="inlineStr">
+        <is>
+          <t>F. 量化底座集成</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="inlineStr">
+        <is>
+          <t>F07-18</t>
+        </is>
+      </c>
+      <c r="C28" s="4" t="inlineStr">
+        <is>
           <t>因子模型</t>
         </is>
       </c>
-      <c r="D27" s="5" t="inlineStr">
-        <is>
-          <t>多因子风险模型（利率/信用/流动性/行业因子），Alpha因子库（≥20因子），因子暴露实时计算</t>
-        </is>
-      </c>
-      <c r="E27" s="5" t="inlineStr">
-        <is>
-          <t>因子模型解释方差&gt;80%，Alpha IC均值&gt;0.05</t>
-        </is>
-      </c>
-      <c r="F27" s="5" t="inlineStr">
+      <c r="D28" s="5" t="inlineStr">
+        <is>
+          <t>多因子风险模型（2200+风险因子：利率/信用/流动性/权益Beta/行业/风格/商品/汇率），Alpha因子库（≥20因子，IC均值&gt;0.05），因子暴露实时计算与历史追踪，因子风险贡献预算管理</t>
+        </is>
+      </c>
+      <c r="E28" s="5" t="inlineStr">
+        <is>
+          <t>因子模型解释方差&gt;80%，因子暴露更新延迟&lt;10s</t>
+        </is>
+      </c>
+      <c r="F28" s="5" t="inlineStr">
         <is>
           <t>AMD历史行情/IBOR持仓</t>
         </is>
       </c>
-      <c r="G27" s="41" t="inlineStr">
+      <c r="G28" s="41" t="inlineStr">
         <is>
           <t>高</t>
         </is>
       </c>
-      <c r="H27" s="8" t="n">
+      <c r="H28" s="8" t="n">
         <v>40</v>
       </c>
-      <c r="I27" s="6" t="inlineStr">
-        <is>
-          <t>P1</t>
-        </is>
-      </c>
-      <c r="J27" s="5" t="inlineStr"/>
-    </row>
-    <row r="28">
-      <c r="A28" s="40" t="inlineStr">
-        <is>
-          <t>合计 17项功能  |  P1: 13项  |  P2: 4项</t>
-        </is>
-      </c>
-      <c r="H28" s="20">
-        <f>SUM(H5:H27)</f>
+      <c r="I28" s="6" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="J28" s="5" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="40" t="inlineStr">
+        <is>
+          <t>合计 18项功能  |  P1: 15项  |  P2: 3项</t>
+        </is>
+      </c>
+      <c r="H29" s="20">
+        <f>SUM(H5:H28)</f>
         <v/>
       </c>
-      <c r="I28" s="34" t="inlineStr"/>
-      <c r="J28" s="34" t="inlineStr"/>
+      <c r="I29" s="34" t="inlineStr"/>
+      <c r="J29" s="34" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="10">
     <mergeCell ref="A1:J1"/>
     <mergeCell ref="A5:J5"/>
     <mergeCell ref="A22:J22"/>
-    <mergeCell ref="A16:J16"/>
+    <mergeCell ref="A17:J17"/>
     <mergeCell ref="A9:J9"/>
-    <mergeCell ref="A28:G28"/>
     <mergeCell ref="A3:J3"/>
-    <mergeCell ref="A24:J24"/>
+    <mergeCell ref="A29:G29"/>
     <mergeCell ref="A2:J2"/>
+    <mergeCell ref="A25:J25"/>
     <mergeCell ref="A13:J13"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -7348,7 +7394,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H213"/>
+  <dimension ref="A1:H214"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -7435,7 +7481,7 @@
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>跨资产实时头寸</t>
+          <t>全资产实时头寸</t>
         </is>
       </c>
       <c r="E4" s="5" t="inlineStr">
@@ -11597,17 +11643,17 @@
       </c>
       <c r="D113" s="4" t="inlineStr">
         <is>
-          <t>债券横截面与时序分析</t>
+          <t>全资产统一持仓模型</t>
         </is>
       </c>
       <c r="E113" s="5" t="inlineStr">
         <is>
-          <t>跨品种横截面信号挖掘（利差/久期偏差），历史时序趋势与均值回归分析</t>
+          <t>八类资产（利率债/信用债/权益/基金/黄金/商品/衍生品/非标）实时T+0持仓，多层组合树（公司→部门→策略→子组合→投资经理），穿透式敞口展示（品种/久期/评级/行业/地区分布），真实组合+Shadow Portfolio并行展示</t>
         </is>
       </c>
       <c r="F113" s="5" t="inlineStr">
         <is>
-          <t>横截面信号与实际收益相关性&gt;0.3</t>
+          <t>T+0持仓实时刷新，穿透层级≥5层，数据与IBOR差异&lt;0.01%</t>
         </is>
       </c>
       <c r="G113" s="23" t="inlineStr">
@@ -11616,7 +11662,7 @@
         </is>
       </c>
       <c r="H113" s="8" t="n">
-        <v>35</v>
+        <v>40</v>
       </c>
     </row>
     <row r="114" ht="28" customHeight="1">
@@ -11637,17 +11683,17 @@
       </c>
       <c r="D114" s="4" t="inlineStr">
         <is>
-          <t>相对价值分析</t>
+          <t>跨资产相关性分析</t>
         </is>
       </c>
       <c r="E114" s="5" t="inlineStr">
         <is>
-          <t>利差/Z-spread/OAS相对价值计算，历史分位数定位，跨品种套利信号识别</t>
+          <t>全持仓跨资产相关矩阵（股/债/商品/衍生品/基金），多窗口滚动（20/60/252日），压力情景相关性vs历史相关性对比，动态相关性漂移预警，分散化比率(Diversification Ratio)计算，低相关候选资产推荐</t>
         </is>
       </c>
       <c r="F114" s="5" t="inlineStr">
         <is>
-          <t>OAS计算误差&lt;1bps，分位数覆盖5年历史</t>
+          <t>相关矩阵计算&lt;30s（500券组合），动态漂移预警阈值可配</t>
         </is>
       </c>
       <c r="G114" s="23" t="inlineStr">
@@ -11677,26 +11723,26 @@
       </c>
       <c r="D115" s="4" t="inlineStr">
         <is>
-          <t>组合相关度分析</t>
+          <t>相对价值分析</t>
         </is>
       </c>
       <c r="E115" s="5" t="inlineStr">
         <is>
-          <t>资产间收益相关矩阵计算（滚动60/120/250日），组合集中度风险识别，分散化系数监控</t>
+          <t>利差/Z-spread/OAS相对价值计算，历史分位数定位（覆盖5年），跨品种套利信号识别，债券横截面信号挖掘（利差/久期偏差），时序均值回归分析</t>
         </is>
       </c>
       <c r="F115" s="5" t="inlineStr">
         <is>
-          <t>相关矩阵计算&lt;30s（500券组合）</t>
-        </is>
-      </c>
-      <c r="G115" s="24" t="inlineStr">
-        <is>
-          <t>中</t>
+          <t>OAS计算误差&lt;1bps，历史分位数覆盖5年，横截面信号与实际收益相关性&gt;0.3</t>
+        </is>
+      </c>
+      <c r="G115" s="23" t="inlineStr">
+        <is>
+          <t>高</t>
         </is>
       </c>
       <c r="H115" s="8" t="n">
-        <v>25</v>
+        <v>30</v>
       </c>
     </row>
     <row r="116" ht="28" customHeight="1">
@@ -11717,17 +11763,17 @@
       </c>
       <c r="D116" s="4" t="inlineStr">
         <is>
-          <t>情景分析</t>
+          <t>QP智能再平衡引擎</t>
         </is>
       </c>
       <c r="E116" s="5" t="inlineStr">
         <is>
-          <t>利率/信用/流动性三类自定义情景，组合P&amp;L影响量化，多情景并行对比</t>
+          <t>二次规划多目标优化（最小化跟踪误差+交易摩擦+融资成本+IFRS9波动），500+约束（合规/风险预算/流动性/IFRS9），2000+持仓毫秒级求解，支持整数规划（面值/手数取整），多期优化（含到期券），三种触发（定时/事件/手动），一键生成交易指令</t>
         </is>
       </c>
       <c r="F116" s="5" t="inlineStr">
         <is>
-          <t>情景P&amp;L与手工核算误差&lt;0.5%，支持≥20情景并行</t>
+          <t>QP求解2000持仓&lt;200ms，约束满足率100%，调仓前后TE对比即时输出</t>
         </is>
       </c>
       <c r="G116" s="23" t="inlineStr">
@@ -11736,7 +11782,7 @@
         </is>
       </c>
       <c r="H116" s="8" t="n">
-        <v>35</v>
+        <v>40</v>
       </c>
     </row>
     <row r="117" ht="28" customHeight="1">
@@ -11757,17 +11803,17 @@
       </c>
       <c r="D117" s="4" t="inlineStr">
         <is>
-          <t>敏感度分析</t>
+          <t>Shadow Portfolio虚拟试算</t>
         </is>
       </c>
       <c r="E117" s="5" t="inlineStr">
         <is>
-          <t>久期/DV01/凸度/利差/Vega敏感度多因子并行计算，组合对冲比率建议</t>
+          <t>100+虚拟组合与真实组合并行运行，多维试算（增减仓/换仓/加杠杆/新资产类别），即时显示试算后风险指标/归因/相关性/预期收益，真实vs虚拟所有指标差异对比视图，冲击成本预估</t>
         </is>
       </c>
       <c r="F117" s="5" t="inlineStr">
         <is>
-          <t>DV01与Bloomberg基准误差&lt;0.5bps</t>
+          <t>虚拟组合模拟与真实执行偏差&lt;0.3%，秒级响应</t>
         </is>
       </c>
       <c r="G117" s="23" t="inlineStr">
@@ -11776,7 +11822,7 @@
         </is>
       </c>
       <c r="H117" s="8" t="n">
-        <v>25</v>
+        <v>30</v>
       </c>
     </row>
     <row r="118" ht="28" customHeight="1">
@@ -11797,17 +11843,17 @@
       </c>
       <c r="D118" s="4" t="inlineStr">
         <is>
-          <t>极端事件分析</t>
+          <t>资产配置策略分析</t>
         </is>
       </c>
       <c r="E118" s="5" t="inlineStr">
         <is>
-          <t>历史极端情景（924行情/2015股灾/2020疫情等8+情景），组合尾部损失分布，ES(99%)计算</t>
+          <t>SAA战略→TAA战术精准联动（投委会指令直接转化为因子约束输入QP引擎），宏观因子（利率/信用/流动性周期）驱动大类资产配置模型，动态权重优化，历史回测验证（≥5年），固收+策略P&amp;L归因（债券底仓+衍生品增强）</t>
         </is>
       </c>
       <c r="F118" s="5" t="inlineStr">
         <is>
-          <t>历史情景复现误差&lt;1%</t>
+          <t>回测期≥5年，预测方向胜率&gt;55%，SAA→TAA指令转化全程无人工干预</t>
         </is>
       </c>
       <c r="G118" s="23" t="inlineStr">
@@ -11816,7 +11862,7 @@
         </is>
       </c>
       <c r="H118" s="8" t="n">
-        <v>30</v>
+        <v>40</v>
       </c>
     </row>
     <row r="119" ht="28" customHeight="1">
@@ -11837,26 +11883,26 @@
       </c>
       <c r="D119" s="4" t="inlineStr">
         <is>
-          <t>指数比较分析</t>
+          <t>Campisi 2.0 固收绩效归因</t>
         </is>
       </c>
       <c r="E119" s="5" t="inlineStr">
         <is>
-          <t>对标中债综合/信用/政策行等指数，跟踪误差（TE）日频监控，超额Alpha三因子分解</t>
+          <t>固定收益五效应完整拆解：①收入效应（票息+摊销），②国债效应（利率平移/曲线斜率/曲率三效应分离，用Key Rate Duration精确映射），③利差效应（DTS贡献/行业配置效应/个券选择效应），④交易效应（择时Alpha或损耗量化），⑤残差校验（&lt;5bp合格）；日/周/月/季多维度报告自动生成</t>
         </is>
       </c>
       <c r="F119" s="5" t="inlineStr">
         <is>
-          <t>TE计算误差&lt;1bps，支持≥10基准指数</t>
-        </is>
-      </c>
-      <c r="G119" s="24" t="inlineStr">
-        <is>
-          <t>中</t>
+          <t>五效应合计与实际收益残差&lt;5bps，T+1 9:00前自动报告</t>
+        </is>
+      </c>
+      <c r="G119" s="23" t="inlineStr">
+        <is>
+          <t>高</t>
         </is>
       </c>
       <c r="H119" s="8" t="n">
-        <v>25</v>
+        <v>40</v>
       </c>
     </row>
     <row r="120" ht="28" customHeight="1">
@@ -11877,17 +11923,17 @@
       </c>
       <c r="D120" s="4" t="inlineStr">
         <is>
-          <t>绩效归因（Brinson）</t>
+          <t>Brinson 资产组合绩效归因</t>
         </is>
       </c>
       <c r="E120" s="5" t="inlineStr">
         <is>
-          <t>BHB三效应：资产配置/个券选择/交互效应，日/周/月/季多维度，报告PDF自动生成</t>
+          <t>三效应：大类资产配置效应（超/低配决策贡献）/个券选择效应（同类标的选择Alpha）/交互效应，支持多层穿透（资产大类→行业→子行业→个股/个基），FOF基金穿透底层持仓，日/月/季/年累计归因趋势，投资经理能力量化排名</t>
         </is>
       </c>
       <c r="F120" s="5" t="inlineStr">
         <is>
-          <t>Brinson结果与Bloomberg AIM误差&lt;0.1%，T+1 9:00前自动报告</t>
+          <t>Brinson结果与Bloomberg AIM误差&lt;0.1%，穿透层级≥4层</t>
         </is>
       </c>
       <c r="G120" s="23" t="inlineStr">
@@ -11896,7 +11942,7 @@
         </is>
       </c>
       <c r="H120" s="8" t="n">
-        <v>40</v>
+        <v>35</v>
       </c>
     </row>
     <row r="121" ht="28" customHeight="1">
@@ -11917,26 +11963,26 @@
       </c>
       <c r="D121" s="4" t="inlineStr">
         <is>
-          <t>虚拟组合分析</t>
+          <t>指数跟踪误差与主动风险归因</t>
         </is>
       </c>
       <c r="E121" s="5" t="inlineStr">
         <is>
-          <t>组合调整前后净值/风险/收益效果模拟（纸面交易），冲击成本预估，多方案对比</t>
+          <t>对标中债综合/信用/政策行等基准指数，跟踪误差（TE）日频监控，TE分解（配置效应TE+选券效应TE+协方差），信息比率（IR）实时监控（目标IR&gt;0.5，预警IR连续3月&lt;0），超额Alpha三因子分解</t>
         </is>
       </c>
       <c r="F121" s="5" t="inlineStr">
         <is>
-          <t>虚拟组合模拟与真实执行偏差&lt;0.3%</t>
-        </is>
-      </c>
-      <c r="G121" s="23" t="inlineStr">
-        <is>
-          <t>高</t>
+          <t>TE计算误差&lt;1bps，支持≥10基准指数，IR预警自动推送</t>
+        </is>
+      </c>
+      <c r="G121" s="24" t="inlineStr">
+        <is>
+          <t>中</t>
         </is>
       </c>
       <c r="H121" s="8" t="n">
-        <v>20</v>
+        <v>25</v>
       </c>
     </row>
     <row r="122" ht="28" customHeight="1">
@@ -11957,17 +12003,17 @@
       </c>
       <c r="D122" s="4" t="inlineStr">
         <is>
-          <t>再平衡方案试算与比较</t>
+          <t>因子风险分解 + MCTR边际风险贡献</t>
         </is>
       </c>
       <c r="E122" s="5" t="inlineStr">
         <is>
-          <t>久期/集中度/流动性/合规约束联合优化（二次规划QP），多方案并行试算，最优路径推荐</t>
+          <t>全持仓分解为2200+风险因子（利率/信用/权益/商品/汇率），系统性风险+特异性风险分离；MCTR边际风险贡献（∂组合波动率/∂持仓权重），风险消耗排名（识别"风险大户"），减仓/加仓优先级引导，风险预算仪表盘（已用/剩余/预警线三档）</t>
         </is>
       </c>
       <c r="F122" s="5" t="inlineStr">
         <is>
-          <t>QP求解100券组合&lt;5s，约束满足率100%</t>
+          <t>因子模型解释方差&gt;80%，MCTR实时更新延迟&lt;5s，Alpha IC均值&gt;0.05</t>
         </is>
       </c>
       <c r="G122" s="23" t="inlineStr">
@@ -11976,7 +12022,7 @@
         </is>
       </c>
       <c r="H122" s="8" t="n">
-        <v>35</v>
+        <v>40</v>
       </c>
     </row>
     <row r="123" ht="28" customHeight="1">
@@ -11997,17 +12043,17 @@
       </c>
       <c r="D123" s="4" t="inlineStr">
         <is>
-          <t>资产配置策略分析</t>
+          <t>Component VaR 四层穿透分析</t>
         </is>
       </c>
       <c r="E123" s="5" t="inlineStr">
         <is>
-          <t>宏观因子（利率/信用/流动性周期）驱动大类资产配置模型，动态权重优化，历史回测验证</t>
+          <t>VaR四层穿透：资产类别VaR→行业/子市场VaR→评级/信用质量VaR→单一发行人Component VaR，含跨类分散化收益量化；三种方法互验（历史模拟500日99%置信度/Monte Carlo 10000次/参数解析法），方法差异超阈值自动预警</t>
         </is>
       </c>
       <c r="F123" s="5" t="inlineStr">
         <is>
-          <t>回测期≥5年，预测方向胜率&gt;55%</t>
+          <t>三方法VaR差异&lt;10%，穿透至发行人层，全量计算&lt;1min</t>
         </is>
       </c>
       <c r="G123" s="23" t="inlineStr">
@@ -12016,7 +12062,7 @@
         </is>
       </c>
       <c r="H123" s="8" t="n">
-        <v>40</v>
+        <v>35</v>
       </c>
     </row>
     <row r="124" ht="28" customHeight="1">
@@ -12037,17 +12083,17 @@
       </c>
       <c r="D124" s="4" t="inlineStr">
         <is>
-          <t>固收+策略分析</t>
+          <t>敏感度分析（多维Shock Grid）</t>
         </is>
       </c>
       <c r="E124" s="5" t="inlineStr">
         <is>
-          <t>债券底仓+衍生品增强策略P&amp;L归因，风险分解（利率/信用/期权贡献），固收+净值模拟</t>
+          <t>利率敏感度（DV01/关键期限点KRD/凸性），信用敏感度（CS01/DTS分评级/分行业），权益敏感度（Delta/Beta/行业Beta），商品汇率敏感度；利率×信用利差二维冲击矩阵（Shock Grid），识别最脆弱组合方向，对冲比率建议</t>
         </is>
       </c>
       <c r="F124" s="5" t="inlineStr">
         <is>
-          <t>固收+净值模拟与实际偏差&lt;0.5%</t>
+          <t>DV01与Bloomberg基准误差&lt;0.5bps，Shock Grid 5×5矩阵实时刷新</t>
         </is>
       </c>
       <c r="G124" s="23" t="inlineStr">
@@ -12077,17 +12123,17 @@
       </c>
       <c r="D125" s="4" t="inlineStr">
         <is>
-          <t>量化策略组合分析</t>
+          <t>情景分析与压力测试</t>
         </is>
       </c>
       <c r="E125" s="5" t="inlineStr">
         <is>
-          <t>多策略组合叠加容量约束，策略相关性管理，Sharpe/最大回撤/Calmar实时监控</t>
+          <t>三层：①历史情景重演（924行情/2019包商/2013钱荒/2015股灾等8+事件，含冲击参数还原），②假设情景模拟（自定义任意冲击组合，即时P&amp;L输出+应急对冲建议），③反向压力测试（倒推触发止损线的临界市场情景+历史发生频率），≥20情景并行</t>
         </is>
       </c>
       <c r="F125" s="5" t="inlineStr">
         <is>
-          <t>策略容量计算误差&lt;5%</t>
+          <t>历史情景复现误差&lt;1%，情景P&amp;L误差&lt;0.5%，支持≥20情景并行</t>
         </is>
       </c>
       <c r="G125" s="23" t="inlineStr">
@@ -12117,17 +12163,17 @@
       </c>
       <c r="D126" s="4" t="inlineStr">
         <is>
-          <t>流动性分析</t>
+          <t>流动性风险管理（LVaR）</t>
         </is>
       </c>
       <c r="E126" s="5" t="inlineStr">
         <is>
-          <t>逐券换手率/市场深度评估，组合变现能力分析，流动性压力下变现损失（LVaR）估算</t>
+          <t>逐持仓变现能力评估（规模/日均成交量→变现天数），Almgren-Chriss市场冲击成本模型，流动性压力测试（X天内变现Y亿最优路径+成本），流动性调整VaR（LVaR=传统VaR+流动性溢价），流动性覆盖率/缓冲监控（1/3/5/10日分层），回购到期日历</t>
         </is>
       </c>
       <c r="F126" s="5" t="inlineStr">
         <is>
-          <t>LVaR与市场基准误差&lt;5%，日均成交量覆盖≥95%持仓</t>
+          <t>LVaR与市场基准误差&lt;5%，日均成交量覆盖≥95%持仓，变现路径建议&lt;3s</t>
         </is>
       </c>
       <c r="G126" s="24" t="inlineStr">
@@ -12136,7 +12182,7 @@
         </is>
       </c>
       <c r="H126" s="8" t="n">
-        <v>20</v>
+        <v>25</v>
       </c>
     </row>
     <row r="127" ht="28" customHeight="1">
@@ -12157,17 +12203,17 @@
       </c>
       <c r="D127" s="4" t="inlineStr">
         <is>
-          <t>定价计算集成</t>
+          <t>衍生品对冲决策引擎</t>
         </is>
       </c>
       <c r="E127" s="5" t="inlineStr">
         <is>
-          <t>调用量化定价引擎实时估值与Greeks，含权债/可转债/IRS，结果缓存（Redis）与Kafka推送</t>
+          <t>七类工具矩阵（国债期货2/5/10/30Y/IRS/CDS/股指期货IF/IH/IC/IM/股指期权/黄金期货/外汇远掉期），系统推荐最优对冲方案（成本最小约束），一键生成对冲指令，对冲效果追踪（前后风险指标对比/效率/执行滑点）；支持快速/精细/尾部/跨资产四种场景</t>
         </is>
       </c>
       <c r="F127" s="5" t="inlineStr">
         <is>
-          <t>定价API p99&lt;200ms，日终全量估值&lt;30min（10万券）</t>
+          <t>对冲方案推荐&lt;5s，DV01对冲误差&lt;5%，指令自动流转执行引擎</t>
         </is>
       </c>
       <c r="G127" s="23" t="inlineStr">
@@ -12176,7 +12222,7 @@
         </is>
       </c>
       <c r="H127" s="8" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
     </row>
     <row r="128" ht="28" customHeight="1">
@@ -12197,26 +12243,26 @@
       </c>
       <c r="D128" s="4" t="inlineStr">
         <is>
-          <t>利率曲线集成</t>
+          <t>定价计算集成</t>
         </is>
       </c>
       <c r="E128" s="5" t="inlineStr">
         <is>
-          <t>多曲线实时消费（国债/政策行/AAA信用/OIS），NS参数提取（水平/斜率/曲率），敏感度映射</t>
+          <t>调用定价平台实时估值与Greeks（含权债/可转债/IRS），Redis缓存结果，Kafka推送持仓+估值变化事件，日终全量估值批处理</t>
         </is>
       </c>
       <c r="F128" s="5" t="inlineStr">
         <is>
-          <t>曲线更新延迟&lt;1s，NS拟合R²&gt;0.999</t>
-        </is>
-      </c>
-      <c r="G128" s="24" t="inlineStr">
-        <is>
-          <t>中</t>
+          <t>定价API p99&lt;200ms，日终全量估值&lt;30min（10万券）</t>
+        </is>
+      </c>
+      <c r="G128" s="23" t="inlineStr">
+        <is>
+          <t>高</t>
         </is>
       </c>
       <c r="H128" s="8" t="n">
-        <v>15</v>
+        <v>20</v>
       </c>
     </row>
     <row r="129" ht="28" customHeight="1">
@@ -12237,73 +12283,73 @@
       </c>
       <c r="D129" s="4" t="inlineStr">
         <is>
+          <t>利率曲线集成</t>
+        </is>
+      </c>
+      <c r="E129" s="5" t="inlineStr">
+        <is>
+          <t>多曲线实时消费（国债/政策行/AAA信用/OIS），NS参数提取（水平/斜率/曲率），关键期限点敏感度映射，曲线版本快照（供归因历史复现）</t>
+        </is>
+      </c>
+      <c r="F129" s="5" t="inlineStr">
+        <is>
+          <t>曲线更新延迟&lt;1s，NS拟合R²&gt;0.999</t>
+        </is>
+      </c>
+      <c r="G129" s="24" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="H129" s="8" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="130" ht="28" customHeight="1">
+      <c r="A130" s="5" t="inlineStr">
+        <is>
+          <t>组合管理+绩效归因</t>
+        </is>
+      </c>
+      <c r="B130" s="3" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="C130" s="3" t="inlineStr">
+        <is>
+          <t>F07-18</t>
+        </is>
+      </c>
+      <c r="D130" s="4" t="inlineStr">
+        <is>
           <t>因子模型</t>
         </is>
       </c>
-      <c r="E129" s="5" t="inlineStr">
-        <is>
-          <t>多因子风险模型（利率/信用/流动性/行业因子），Alpha因子库（≥20因子），因子暴露实时计算</t>
-        </is>
-      </c>
-      <c r="F129" s="5" t="inlineStr">
-        <is>
-          <t>因子模型解释方差&gt;80%，Alpha IC均值&gt;0.05</t>
-        </is>
-      </c>
-      <c r="G129" s="23" t="inlineStr">
+      <c r="E130" s="5" t="inlineStr">
+        <is>
+          <t>多因子风险模型（2200+风险因子：利率/信用/流动性/权益Beta/行业/风格/商品/汇率），Alpha因子库（≥20因子，IC均值&gt;0.05），因子暴露实时计算与历史追踪，因子风险贡献预算管理</t>
+        </is>
+      </c>
+      <c r="F130" s="5" t="inlineStr">
+        <is>
+          <t>因子模型解释方差&gt;80%，因子暴露更新延迟&lt;10s</t>
+        </is>
+      </c>
+      <c r="G130" s="23" t="inlineStr">
         <is>
           <t>高</t>
         </is>
       </c>
-      <c r="H129" s="8" t="n">
+      <c r="H130" s="8" t="n">
         <v>40</v>
       </c>
     </row>
-    <row r="130" ht="20" customHeight="1">
-      <c r="A130" s="22" t="inlineStr">
+    <row r="131" ht="20" customHeight="1">
+      <c r="A131" s="22" t="inlineStr">
         <is>
           <t>【P1】 策略投资/量化  (Quant Strategy)</t>
         </is>
-      </c>
-    </row>
-    <row r="131" ht="28" customHeight="1">
-      <c r="A131" s="5" t="inlineStr">
-        <is>
-          <t>策略投资/量化</t>
-        </is>
-      </c>
-      <c r="B131" s="3" t="inlineStr">
-        <is>
-          <t>P1</t>
-        </is>
-      </c>
-      <c r="C131" s="3" t="inlineStr">
-        <is>
-          <t>F08-01</t>
-        </is>
-      </c>
-      <c r="D131" s="4" t="inlineStr">
-        <is>
-          <t>策略编写与版本管理</t>
-        </is>
-      </c>
-      <c r="E131" s="5" t="inlineStr">
-        <is>
-          <t>Python/C++策略脚本编写，沙箱隔离运行，策略版本管理，策略库分类管理（利差/基差/跨市场套利/网格/固收/量价）</t>
-        </is>
-      </c>
-      <c r="F131" s="5" t="inlineStr">
-        <is>
-          <t>功能完整/边界测试/集成冒烟/性能基线</t>
-        </is>
-      </c>
-      <c r="G131" s="23" t="inlineStr">
-        <is>
-          <t>高</t>
-        </is>
-      </c>
-      <c r="H131" s="8" t="n">
-        <v>40</v>
       </c>
     </row>
     <row r="132" ht="28" customHeight="1">
@@ -12319,17 +12365,17 @@
       </c>
       <c r="C132" s="3" t="inlineStr">
         <is>
-          <t>F08-02</t>
+          <t>F08-01</t>
         </is>
       </c>
       <c r="D132" s="4" t="inlineStr">
         <is>
-          <t>AI辅助策略开发</t>
+          <t>策略编写与版本管理</t>
         </is>
       </c>
       <c r="E132" s="5" t="inlineStr">
         <is>
-          <t>AI代码生成辅助，AI因子生成，AI参数优化建议，自然语言描述策略逻辑转代码</t>
+          <t>Python/C++策略脚本编写，沙箱隔离运行，策略版本管理，策略库分类管理（利差/基差/跨市场套利/网格/固收/量价）</t>
         </is>
       </c>
       <c r="F132" s="5" t="inlineStr">
@@ -12343,7 +12389,7 @@
         </is>
       </c>
       <c r="H132" s="8" t="n">
-        <v>35</v>
+        <v>40</v>
       </c>
     </row>
     <row r="133" ht="28" customHeight="1">
@@ -12359,17 +12405,17 @@
       </c>
       <c r="C133" s="3" t="inlineStr">
         <is>
-          <t>F08-03</t>
+          <t>F08-02</t>
         </is>
       </c>
       <c r="D133" s="4" t="inlineStr">
         <is>
-          <t>因子挖掘与管理</t>
+          <t>AI辅助策略开发</t>
         </is>
       </c>
       <c r="E133" s="5" t="inlineStr">
         <is>
-          <t>因子编写，信号生成，因子库管理，AlphaLens因子有效性分析，量化模型库，宏观/技术/基本面因子</t>
+          <t>AI代码生成辅助，AI因子生成，AI参数优化建议，自然语言描述策略逻辑转代码</t>
         </is>
       </c>
       <c r="F133" s="5" t="inlineStr">
@@ -12383,7 +12429,7 @@
         </is>
       </c>
       <c r="H133" s="8" t="n">
-        <v>40</v>
+        <v>35</v>
       </c>
     </row>
     <row r="134" ht="28" customHeight="1">
@@ -12399,31 +12445,31 @@
       </c>
       <c r="C134" s="3" t="inlineStr">
         <is>
-          <t>F08-04</t>
+          <t>F08-03</t>
         </is>
       </c>
       <c r="D134" s="4" t="inlineStr">
         <is>
-          <t>Tick级回测引擎</t>
+          <t>因子挖掘与管理</t>
         </is>
       </c>
       <c r="E134" s="5" t="inlineStr">
         <is>
-          <t>Tick数据驱动回测，真实滑点/冲击模型，批量参数优化，风险计量，绩效归因，AlphaLens分析集成</t>
+          <t>因子编写，信号生成，因子库管理，AlphaLens因子有效性分析，量化模型库，宏观/技术/基本面因子</t>
         </is>
       </c>
       <c r="F134" s="5" t="inlineStr">
         <is>
-          <t>p99延迟/误差率/精度验证/压测10k TPS</t>
-        </is>
-      </c>
-      <c r="G134" s="28" t="inlineStr">
-        <is>
-          <t>极高</t>
+          <t>功能完整/边界测试/集成冒烟/性能基线</t>
+        </is>
+      </c>
+      <c r="G134" s="23" t="inlineStr">
+        <is>
+          <t>高</t>
         </is>
       </c>
       <c r="H134" s="8" t="n">
-        <v>60</v>
+        <v>40</v>
       </c>
     </row>
     <row r="135" ht="28" customHeight="1">
@@ -12439,31 +12485,31 @@
       </c>
       <c r="C135" s="3" t="inlineStr">
         <is>
-          <t>F08-05</t>
+          <t>F08-04</t>
         </is>
       </c>
       <c r="D135" s="4" t="inlineStr">
         <is>
-          <t>模拟盘验证</t>
+          <t>Tick级回测引擎</t>
         </is>
       </c>
       <c r="E135" s="5" t="inlineStr">
         <is>
-          <t>情景模拟，敏感度模拟，极端场景模拟，性能测试，模拟盘与实盘结果对比分析</t>
+          <t>Tick数据驱动回测，真实滑点/冲击模型，批量参数优化，风险计量，绩效归因，AlphaLens分析集成</t>
         </is>
       </c>
       <c r="F135" s="5" t="inlineStr">
         <is>
-          <t>功能完整/边界测试/集成冒烟/性能基线</t>
-        </is>
-      </c>
-      <c r="G135" s="23" t="inlineStr">
-        <is>
-          <t>高</t>
+          <t>p99延迟/误差率/精度验证/压测10k TPS</t>
+        </is>
+      </c>
+      <c r="G135" s="28" t="inlineStr">
+        <is>
+          <t>极高</t>
         </is>
       </c>
       <c r="H135" s="8" t="n">
-        <v>30</v>
+        <v>60</v>
       </c>
     </row>
     <row r="136" ht="28" customHeight="1">
@@ -12479,31 +12525,31 @@
       </c>
       <c r="C136" s="3" t="inlineStr">
         <is>
-          <t>F08-06</t>
+          <t>F08-05</t>
         </is>
       </c>
       <c r="D136" s="4" t="inlineStr">
         <is>
-          <t>策略上线审批</t>
+          <t>模拟盘验证</t>
         </is>
       </c>
       <c r="E136" s="5" t="inlineStr">
         <is>
-          <t>模拟盘通过后触发上线审批流程，多级合规审核，审批留痕，参数锁定后方可实盘运行</t>
+          <t>情景模拟，敏感度模拟，极端场景模拟，性能测试，模拟盘与实盘结果对比分析</t>
         </is>
       </c>
       <c r="F136" s="5" t="inlineStr">
         <is>
-          <t>功能测试通过/正确率100%</t>
-        </is>
-      </c>
-      <c r="G136" s="24" t="inlineStr">
-        <is>
-          <t>中</t>
+          <t>功能完整/边界测试/集成冒烟/性能基线</t>
+        </is>
+      </c>
+      <c r="G136" s="23" t="inlineStr">
+        <is>
+          <t>高</t>
         </is>
       </c>
       <c r="H136" s="8" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
     </row>
     <row r="137" ht="28" customHeight="1">
@@ -12519,31 +12565,31 @@
       </c>
       <c r="C137" s="3" t="inlineStr">
         <is>
-          <t>F08-07</t>
+          <t>F08-06</t>
         </is>
       </c>
       <c r="D137" s="4" t="inlineStr">
         <is>
-          <t>策略运行管理</t>
+          <t>策略上线审批</t>
         </is>
       </c>
       <c r="E137" s="5" t="inlineStr">
         <is>
-          <t>实盘策略启停管理，策略状态实时监控，支持手动干预和自动触发停止，多策略并发调度</t>
+          <t>模拟盘通过后触发上线审批流程，多级合规审核，审批留痕，参数锁定后方可实盘运行</t>
         </is>
       </c>
       <c r="F137" s="5" t="inlineStr">
         <is>
-          <t>功能完整/边界测试/集成冒烟/性能基线</t>
-        </is>
-      </c>
-      <c r="G137" s="23" t="inlineStr">
-        <is>
-          <t>高</t>
+          <t>功能测试通过/正确率100%</t>
+        </is>
+      </c>
+      <c r="G137" s="24" t="inlineStr">
+        <is>
+          <t>中</t>
         </is>
       </c>
       <c r="H137" s="8" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
     </row>
     <row r="138" ht="28" customHeight="1">
@@ -12559,31 +12605,31 @@
       </c>
       <c r="C138" s="3" t="inlineStr">
         <is>
-          <t>F08-08</t>
+          <t>F08-07</t>
         </is>
       </c>
       <c r="D138" s="4" t="inlineStr">
         <is>
-          <t>策略绩效分析</t>
+          <t>策略运行管理</t>
         </is>
       </c>
       <c r="E138" s="5" t="inlineStr">
         <is>
-          <t>实时PnL/持仓/回撤/Sharpe看板，策略归因分析，与基准对比，风险触发自动平仓</t>
+          <t>实盘策略启停管理，策略状态实时监控，支持手动干预和自动触发停止，多策略并发调度</t>
         </is>
       </c>
       <c r="F138" s="5" t="inlineStr">
         <is>
-          <t>功能测试通过/正确率100%</t>
-        </is>
-      </c>
-      <c r="G138" s="24" t="inlineStr">
-        <is>
-          <t>中</t>
+          <t>功能完整/边界测试/集成冒烟/性能基线</t>
+        </is>
+      </c>
+      <c r="G138" s="23" t="inlineStr">
+        <is>
+          <t>高</t>
         </is>
       </c>
       <c r="H138" s="8" t="n">
-        <v>25</v>
+        <v>30</v>
       </c>
     </row>
     <row r="139" ht="28" customHeight="1">
@@ -12599,17 +12645,17 @@
       </c>
       <c r="C139" s="3" t="inlineStr">
         <is>
-          <t>F08-09</t>
+          <t>F08-08</t>
         </is>
       </c>
       <c r="D139" s="4" t="inlineStr">
         <is>
-          <t>实时多市场行情</t>
+          <t>策略绩效分析</t>
         </is>
       </c>
       <c r="E139" s="5" t="inlineStr">
         <is>
-          <t>现券/国债期货/股票/商品实时行情聚合展示，实时利差分析，跨市场价差监控，行情小窗</t>
+          <t>实时PnL/持仓/回撤/Sharpe看板，策略归因分析，与基准对比，风险触发自动平仓</t>
         </is>
       </c>
       <c r="F139" s="5" t="inlineStr">
@@ -12623,7 +12669,7 @@
         </is>
       </c>
       <c r="H139" s="8" t="n">
-        <v>20</v>
+        <v>25</v>
       </c>
     </row>
     <row r="140" ht="28" customHeight="1">
@@ -12639,17 +12685,17 @@
       </c>
       <c r="C140" s="3" t="inlineStr">
         <is>
-          <t>F08-10</t>
+          <t>F08-09</t>
         </is>
       </c>
       <c r="D140" s="4" t="inlineStr">
         <is>
-          <t>历史行情回放</t>
+          <t>实时多市场行情</t>
         </is>
       </c>
       <c r="E140" s="5" t="inlineStr">
         <is>
-          <t>现券/国债期货/股票/商品历史行情回放，支持任意时间点快照，用于回测验证和策略复盘</t>
+          <t>现券/国债期货/股票/商品实时行情聚合展示，实时利差分析，跨市场价差监控，行情小窗</t>
         </is>
       </c>
       <c r="F140" s="5" t="inlineStr">
@@ -12679,31 +12725,31 @@
       </c>
       <c r="C141" s="3" t="inlineStr">
         <is>
-          <t>F08-11</t>
+          <t>F08-10</t>
         </is>
       </c>
       <c r="D141" s="4" t="inlineStr">
         <is>
-          <t>CEP流引擎与信号调度</t>
+          <t>历史行情回放</t>
         </is>
       </c>
       <c r="E141" s="5" t="inlineStr">
         <is>
-          <t>复杂事件处理引擎，策略信号实时计算与调度，低延迟执行接口对接ATP超低延迟执行层</t>
+          <t>现券/国债期货/股票/商品历史行情回放，支持任意时间点快照，用于回测验证和策略复盘</t>
         </is>
       </c>
       <c r="F141" s="5" t="inlineStr">
         <is>
-          <t>p99延迟/误差率/精度验证/压测10k TPS</t>
-        </is>
-      </c>
-      <c r="G141" s="28" t="inlineStr">
-        <is>
-          <t>极高</t>
+          <t>功能测试通过/正确率100%</t>
+        </is>
+      </c>
+      <c r="G141" s="24" t="inlineStr">
+        <is>
+          <t>中</t>
         </is>
       </c>
       <c r="H141" s="8" t="n">
-        <v>45</v>
+        <v>20</v>
       </c>
     </row>
     <row r="142" ht="28" customHeight="1">
@@ -12719,78 +12765,78 @@
       </c>
       <c r="C142" s="3" t="inlineStr">
         <is>
+          <t>F08-11</t>
+        </is>
+      </c>
+      <c r="D142" s="4" t="inlineStr">
+        <is>
+          <t>CEP流引擎与信号调度</t>
+        </is>
+      </c>
+      <c r="E142" s="5" t="inlineStr">
+        <is>
+          <t>复杂事件处理引擎，策略信号实时计算与调度，低延迟执行接口对接ATP超低延迟执行层</t>
+        </is>
+      </c>
+      <c r="F142" s="5" t="inlineStr">
+        <is>
+          <t>p99延迟/误差率/精度验证/压测10k TPS</t>
+        </is>
+      </c>
+      <c r="G142" s="28" t="inlineStr">
+        <is>
+          <t>极高</t>
+        </is>
+      </c>
+      <c r="H142" s="8" t="n">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="143" ht="28" customHeight="1">
+      <c r="A143" s="5" t="inlineStr">
+        <is>
+          <t>策略投资/量化</t>
+        </is>
+      </c>
+      <c r="B143" s="3" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="C143" s="3" t="inlineStr">
+        <is>
           <t>F08-12</t>
         </is>
       </c>
-      <c r="D142" s="4" t="inlineStr">
+      <c r="D143" s="4" t="inlineStr">
         <is>
           <t>基础数据与模型底座</t>
         </is>
       </c>
-      <c r="E142" s="5" t="inlineStr">
+      <c r="E143" s="5" t="inlineStr">
         <is>
           <t>宏观因子库，债券曲线模型，估值数据接入，账户权限管理，AI引擎集成接口</t>
         </is>
       </c>
-      <c r="F142" s="5" t="inlineStr">
+      <c r="F143" s="5" t="inlineStr">
         <is>
           <t>功能完整/边界测试/集成冒烟/性能基线</t>
         </is>
       </c>
-      <c r="G142" s="23" t="inlineStr">
+      <c r="G143" s="23" t="inlineStr">
         <is>
           <t>高</t>
         </is>
       </c>
-      <c r="H142" s="8" t="n">
+      <c r="H143" s="8" t="n">
         <v>30</v>
       </c>
     </row>
-    <row r="143" ht="20" customHeight="1">
-      <c r="A143" s="26" t="inlineStr">
+    <row r="144" ht="20" customHeight="1">
+      <c r="A144" s="26" t="inlineStr">
         <is>
           <t>【P2】 定价平台  (Pricing Platform)</t>
         </is>
-      </c>
-    </row>
-    <row r="144" ht="28" customHeight="1">
-      <c r="A144" s="11" t="inlineStr">
-        <is>
-          <t>定价平台</t>
-        </is>
-      </c>
-      <c r="B144" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
-        </is>
-      </c>
-      <c r="C144" s="10" t="inlineStr">
-        <is>
-          <t>F09-01</t>
-        </is>
-      </c>
-      <c r="D144" s="27" t="inlineStr">
-        <is>
-          <t>期权收益结构定价</t>
-        </is>
-      </c>
-      <c r="E144" s="11" t="inlineStr">
-        <is>
-          <t>香草期权/价差期权/欧式/美式/雪球/自定义期权定价，挂钩标的覆盖国债/期货/股票/指数/商品</t>
-        </is>
-      </c>
-      <c r="F144" s="11" t="inlineStr">
-        <is>
-          <t>p99延迟/误差率/精度验证/压测10k TPS</t>
-        </is>
-      </c>
-      <c r="G144" s="28" t="inlineStr">
-        <is>
-          <t>极高</t>
-        </is>
-      </c>
-      <c r="H144" s="13" t="n">
-        <v>60</v>
       </c>
     </row>
     <row r="145" ht="28" customHeight="1">
@@ -12806,17 +12852,17 @@
       </c>
       <c r="C145" s="10" t="inlineStr">
         <is>
-          <t>F09-02</t>
+          <t>F09-01</t>
         </is>
       </c>
       <c r="D145" s="27" t="inlineStr">
         <is>
-          <t>结构化产品定价</t>
+          <t>期权收益结构定价</t>
         </is>
       </c>
       <c r="E145" s="11" t="inlineStr">
         <is>
-          <t>场外期权/远期/收益凭证/收益互换/融资融券/合约型互换定价，支持自定义结构化产品</t>
+          <t>香草期权/价差期权/欧式/美式/雪球/自定义期权定价，挂钩标的覆盖国债/期货/股票/指数/商品</t>
         </is>
       </c>
       <c r="F145" s="11" t="inlineStr">
@@ -12830,7 +12876,7 @@
         </is>
       </c>
       <c r="H145" s="13" t="n">
-        <v>50</v>
+        <v>60</v>
       </c>
     </row>
     <row r="146" ht="28" customHeight="1">
@@ -12846,31 +12892,31 @@
       </c>
       <c r="C146" s="10" t="inlineStr">
         <is>
-          <t>F09-03</t>
+          <t>F09-02</t>
         </is>
       </c>
       <c r="D146" s="27" t="inlineStr">
         <is>
-          <t>固收品种定价</t>
+          <t>结构化产品定价</t>
         </is>
       </c>
       <c r="E146" s="11" t="inlineStr">
         <is>
-          <t>固息/浮息国债，含权债，可转债精确定价，信用债估值，ABS定价</t>
+          <t>场外期权/远期/收益凭证/收益互换/融资融券/合约型互换定价，支持自定义结构化产品</t>
         </is>
       </c>
       <c r="F146" s="11" t="inlineStr">
         <is>
-          <t>功能完整/边界测试/集成冒烟/性能基线</t>
-        </is>
-      </c>
-      <c r="G146" s="23" t="inlineStr">
-        <is>
-          <t>高</t>
+          <t>p99延迟/误差率/精度验证/压测10k TPS</t>
+        </is>
+      </c>
+      <c r="G146" s="28" t="inlineStr">
+        <is>
+          <t>极高</t>
         </is>
       </c>
       <c r="H146" s="13" t="n">
-        <v>40</v>
+        <v>50</v>
       </c>
     </row>
     <row r="147" ht="28" customHeight="1">
@@ -12886,31 +12932,31 @@
       </c>
       <c r="C147" s="10" t="inlineStr">
         <is>
-          <t>F09-04</t>
+          <t>F09-03</t>
         </is>
       </c>
       <c r="D147" s="27" t="inlineStr">
         <is>
-          <t>利率与信用曲线构建</t>
+          <t>固收品种定价</t>
         </is>
       </c>
       <c r="E147" s="11" t="inlineStr">
         <is>
-          <t>利率曲线（多插值方法），信用利差曲线，利差曲线，违约曲线，全品种统一曲线服务</t>
+          <t>固息/浮息国债，含权债，可转债精确定价，信用债估值，ABS定价</t>
         </is>
       </c>
       <c r="F147" s="11" t="inlineStr">
         <is>
-          <t>p99延迟/误差率/精度验证/压测10k TPS</t>
-        </is>
-      </c>
-      <c r="G147" s="28" t="inlineStr">
-        <is>
-          <t>极高</t>
+          <t>功能完整/边界测试/集成冒烟/性能基线</t>
+        </is>
+      </c>
+      <c r="G147" s="23" t="inlineStr">
+        <is>
+          <t>高</t>
         </is>
       </c>
       <c r="H147" s="13" t="n">
-        <v>60</v>
+        <v>40</v>
       </c>
     </row>
     <row r="148" ht="28" customHeight="1">
@@ -12926,17 +12972,17 @@
       </c>
       <c r="C148" s="10" t="inlineStr">
         <is>
-          <t>F09-05</t>
+          <t>F09-04</t>
         </is>
       </c>
       <c r="D148" s="27" t="inlineStr">
         <is>
-          <t>波动率曲面构建</t>
+          <t>利率与信用曲线构建</t>
         </is>
       </c>
       <c r="E148" s="11" t="inlineStr">
         <is>
-          <t>隐含波动率曲面，红利曲线，汇率曲线，Local Volatility曲面，波动率微笑校准</t>
+          <t>利率曲线（多插值方法），信用利差曲线，利差曲线，违约曲线，全品种统一曲线服务</t>
         </is>
       </c>
       <c r="F148" s="11" t="inlineStr">
@@ -12950,7 +12996,7 @@
         </is>
       </c>
       <c r="H148" s="13" t="n">
-        <v>50</v>
+        <v>60</v>
       </c>
     </row>
     <row r="149" ht="28" customHeight="1">
@@ -12966,31 +13012,31 @@
       </c>
       <c r="C149" s="10" t="inlineStr">
         <is>
-          <t>F09-06</t>
+          <t>F09-05</t>
         </is>
       </c>
       <c r="D149" s="27" t="inlineStr">
         <is>
-          <t>市场数据管理</t>
+          <t>波动率曲面构建</t>
         </is>
       </c>
       <c r="E149" s="11" t="inlineStr">
         <is>
-          <t>境内外权益/债券/外汇/商品资讯统一接入，数据清洗，异常值处理，数据质量监控</t>
+          <t>隐含波动率曲面，红利曲线，汇率曲线，Local Volatility曲面，波动率微笑校准</t>
         </is>
       </c>
       <c r="F149" s="11" t="inlineStr">
         <is>
-          <t>功能完整/边界测试/集成冒烟/性能基线</t>
-        </is>
-      </c>
-      <c r="G149" s="23" t="inlineStr">
-        <is>
-          <t>高</t>
+          <t>p99延迟/误差率/精度验证/压测10k TPS</t>
+        </is>
+      </c>
+      <c r="G149" s="28" t="inlineStr">
+        <is>
+          <t>极高</t>
         </is>
       </c>
       <c r="H149" s="13" t="n">
-        <v>30</v>
+        <v>50</v>
       </c>
     </row>
     <row r="150" ht="28" customHeight="1">
@@ -13006,31 +13052,31 @@
       </c>
       <c r="C150" s="10" t="inlineStr">
         <is>
-          <t>F09-07</t>
+          <t>F09-06</t>
         </is>
       </c>
       <c r="D150" s="27" t="inlineStr">
         <is>
-          <t>蒙特卡洛求解器</t>
+          <t>市场数据管理</t>
         </is>
       </c>
       <c r="E150" s="11" t="inlineStr">
         <is>
-          <t>GPU加速MC，QMC低差异序列，支持路径相关期权定价，并行情景模拟</t>
+          <t>境内外权益/债券/外汇/商品资讯统一接入，数据清洗，异常值处理，数据质量监控</t>
         </is>
       </c>
       <c r="F150" s="11" t="inlineStr">
         <is>
-          <t>p99延迟/误差率/精度验证/压测10k TPS</t>
-        </is>
-      </c>
-      <c r="G150" s="28" t="inlineStr">
-        <is>
-          <t>极高</t>
+          <t>功能完整/边界测试/集成冒烟/性能基线</t>
+        </is>
+      </c>
+      <c r="G150" s="23" t="inlineStr">
+        <is>
+          <t>高</t>
         </is>
       </c>
       <c r="H150" s="13" t="n">
-        <v>70</v>
+        <v>30</v>
       </c>
     </row>
     <row r="151" ht="28" customHeight="1">
@@ -13046,17 +13092,17 @@
       </c>
       <c r="C151" s="10" t="inlineStr">
         <is>
-          <t>F09-08</t>
+          <t>F09-07</t>
         </is>
       </c>
       <c r="D151" s="27" t="inlineStr">
         <is>
-          <t>解析解与数值解</t>
+          <t>蒙特卡洛求解器</t>
         </is>
       </c>
       <c r="E151" s="11" t="inlineStr">
         <is>
-          <t>Black-Scholes解析解，Hull-White利率模型，SABR波动率模型，二叉树/三叉树数值解</t>
+          <t>GPU加速MC，QMC低差异序列，支持路径相关期权定价，并行情景模拟</t>
         </is>
       </c>
       <c r="F151" s="11" t="inlineStr">
@@ -13070,7 +13116,7 @@
         </is>
       </c>
       <c r="H151" s="13" t="n">
-        <v>60</v>
+        <v>70</v>
       </c>
     </row>
     <row r="152" ht="28" customHeight="1">
@@ -13086,17 +13132,17 @@
       </c>
       <c r="C152" s="10" t="inlineStr">
         <is>
-          <t>F09-09</t>
+          <t>F09-08</t>
         </is>
       </c>
       <c r="D152" s="27" t="inlineStr">
         <is>
-          <t>有限差分（PDE）</t>
+          <t>解析解与数值解</t>
         </is>
       </c>
       <c r="E152" s="11" t="inlineStr">
         <is>
-          <t>Crank-Nicolson/ADI方法，含权债/可转债精确定价，局部波动率模型数值解</t>
+          <t>Black-Scholes解析解，Hull-White利率模型，SABR波动率模型，二叉树/三叉树数值解</t>
         </is>
       </c>
       <c r="F152" s="11" t="inlineStr">
@@ -13126,31 +13172,31 @@
       </c>
       <c r="C153" s="10" t="inlineStr">
         <is>
-          <t>F09-10</t>
+          <t>F09-09</t>
         </is>
       </c>
       <c r="D153" s="27" t="inlineStr">
         <is>
-          <t>实时Greeks计算</t>
+          <t>有限差分（PDE）</t>
         </is>
       </c>
       <c r="E153" s="11" t="inlineStr">
         <is>
-          <t>Delta/Gamma/Vega/Theta/Rho分布式实时计算，DV01/CS01，分桶敏感度</t>
+          <t>Crank-Nicolson/ADI方法，含权债/可转债精确定价，局部波动率模型数值解</t>
         </is>
       </c>
       <c r="F153" s="11" t="inlineStr">
         <is>
-          <t>功能完整/边界测试/集成冒烟/性能基线</t>
-        </is>
-      </c>
-      <c r="G153" s="23" t="inlineStr">
-        <is>
-          <t>高</t>
+          <t>p99延迟/误差率/精度验证/压测10k TPS</t>
+        </is>
+      </c>
+      <c r="G153" s="28" t="inlineStr">
+        <is>
+          <t>极高</t>
         </is>
       </c>
       <c r="H153" s="13" t="n">
-        <v>40</v>
+        <v>60</v>
       </c>
     </row>
     <row r="154" ht="28" customHeight="1">
@@ -13166,17 +13212,17 @@
       </c>
       <c r="C154" s="10" t="inlineStr">
         <is>
-          <t>F09-11</t>
+          <t>F09-10</t>
         </is>
       </c>
       <c r="D154" s="27" t="inlineStr">
         <is>
-          <t>估值与结算计算</t>
+          <t>实时Greeks计算</t>
         </is>
       </c>
       <c r="E154" s="11" t="inlineStr">
         <is>
-          <t>日终估值，盯市计算，保证金计算，结算价格，历史估值回测与误差分析</t>
+          <t>Delta/Gamma/Vega/Theta/Rho分布式实时计算，DV01/CS01，分桶敏感度</t>
         </is>
       </c>
       <c r="F154" s="11" t="inlineStr">
@@ -13206,17 +13252,17 @@
       </c>
       <c r="C155" s="10" t="inlineStr">
         <is>
-          <t>F09-12</t>
+          <t>F09-11</t>
         </is>
       </c>
       <c r="D155" s="27" t="inlineStr">
         <is>
-          <t>风控与情景计算</t>
+          <t>估值与结算计算</t>
         </is>
       </c>
       <c r="E155" s="11" t="inlineStr">
         <is>
-          <t>风险计量（VaR/压力测试）调用，情景分析，保证金计算，为风控平台提供统一定价接口</t>
+          <t>日终估值，盯市计算，保证金计算，结算价格，历史估值回测与误差分析</t>
         </is>
       </c>
       <c r="F155" s="11" t="inlineStr">
@@ -13230,7 +13276,7 @@
         </is>
       </c>
       <c r="H155" s="13" t="n">
-        <v>35</v>
+        <v>40</v>
       </c>
     </row>
     <row r="156" ht="28" customHeight="1">
@@ -13246,17 +13292,17 @@
       </c>
       <c r="C156" s="10" t="inlineStr">
         <is>
-          <t>F09-13</t>
+          <t>F09-12</t>
         </is>
       </c>
       <c r="D156" s="27" t="inlineStr">
         <is>
-          <t>客需报价服务</t>
+          <t>风控与情景计算</t>
         </is>
       </c>
       <c r="E156" s="11" t="inlineStr">
         <is>
-          <t>为销售交易/TRS系统提供实时报价，一站式报价接口，支持结构化产品定制化快速报价</t>
+          <t>风险计量（VaR/压力测试）调用，情景分析，保证金计算，为风控平台提供统一定价接口</t>
         </is>
       </c>
       <c r="F156" s="11" t="inlineStr">
@@ -13286,17 +13332,17 @@
       </c>
       <c r="C157" s="10" t="inlineStr">
         <is>
-          <t>F09-14</t>
+          <t>F09-13</t>
         </is>
       </c>
       <c r="D157" s="27" t="inlineStr">
         <is>
-          <t>定价微服务架构</t>
+          <t>客需报价服务</t>
         </is>
       </c>
       <c r="E157" s="11" t="inlineStr">
         <is>
-          <t>REST/gRPC定价API，横向弹性扩容，p99&lt;100ms，模型插件化注册，版本管理</t>
+          <t>为销售交易/TRS系统提供实时报价，一站式报价接口，支持结构化产品定制化快速报价</t>
         </is>
       </c>
       <c r="F157" s="11" t="inlineStr">
@@ -13310,7 +13356,7 @@
         </is>
       </c>
       <c r="H157" s="13" t="n">
-        <v>40</v>
+        <v>35</v>
       </c>
     </row>
     <row r="158" ht="28" customHeight="1">
@@ -13326,78 +13372,78 @@
       </c>
       <c r="C158" s="10" t="inlineStr">
         <is>
+          <t>F09-14</t>
+        </is>
+      </c>
+      <c r="D158" s="27" t="inlineStr">
+        <is>
+          <t>定价微服务架构</t>
+        </is>
+      </c>
+      <c r="E158" s="11" t="inlineStr">
+        <is>
+          <t>REST/gRPC定价API，横向弹性扩容，p99&lt;100ms，模型插件化注册，版本管理</t>
+        </is>
+      </c>
+      <c r="F158" s="11" t="inlineStr">
+        <is>
+          <t>功能完整/边界测试/集成冒烟/性能基线</t>
+        </is>
+      </c>
+      <c r="G158" s="23" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="H158" s="13" t="n">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="159" ht="28" customHeight="1">
+      <c r="A159" s="11" t="inlineStr">
+        <is>
+          <t>定价平台</t>
+        </is>
+      </c>
+      <c r="B159" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="C159" s="10" t="inlineStr">
+        <is>
           <t>F09-15</t>
         </is>
       </c>
-      <c r="D158" s="27" t="inlineStr">
+      <c r="D159" s="27" t="inlineStr">
         <is>
           <t>灵活二次开发能力</t>
         </is>
       </c>
-      <c r="E158" s="11" t="inlineStr">
+      <c r="E159" s="11" t="inlineStr">
         <is>
           <t>全平台级/单功能模块级/系统框架级可扩展，支持自定义模型接入，策略团队自助扩展</t>
         </is>
       </c>
-      <c r="F158" s="11" t="inlineStr">
+      <c r="F159" s="11" t="inlineStr">
         <is>
           <t>功能完整/边界测试/集成冒烟/性能基线</t>
         </is>
       </c>
-      <c r="G158" s="23" t="inlineStr">
+      <c r="G159" s="23" t="inlineStr">
         <is>
           <t>高</t>
         </is>
       </c>
-      <c r="H158" s="13" t="n">
+      <c r="H159" s="13" t="n">
         <v>30</v>
       </c>
     </row>
-    <row r="159" ht="20" customHeight="1">
-      <c r="A159" s="26" t="inlineStr">
+    <row r="160" ht="20" customHeight="1">
+      <c r="A160" s="26" t="inlineStr">
         <is>
           <t>【P2】 销售交易  (Sales Trading)</t>
         </is>
-      </c>
-    </row>
-    <row r="160" ht="28" customHeight="1">
-      <c r="A160" s="11" t="inlineStr">
-        <is>
-          <t>销售交易</t>
-        </is>
-      </c>
-      <c r="B160" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
-        </is>
-      </c>
-      <c r="C160" s="10" t="inlineStr">
-        <is>
-          <t>F10-01</t>
-        </is>
-      </c>
-      <c r="D160" s="27" t="inlineStr">
-        <is>
-          <t>报价工作台</t>
-        </is>
-      </c>
-      <c r="E160" s="11" t="inlineStr">
-        <is>
-          <t>历史报价管理，当日报价快捷操作，导入/导出报价，一键unrefer，报价提醒功能</t>
-        </is>
-      </c>
-      <c r="F160" s="11" t="inlineStr">
-        <is>
-          <t>功能测试通过/正确率100%</t>
-        </is>
-      </c>
-      <c r="G160" s="24" t="inlineStr">
-        <is>
-          <t>中</t>
-        </is>
-      </c>
-      <c r="H160" s="13" t="n">
-        <v>20</v>
       </c>
     </row>
     <row r="161" ht="28" customHeight="1">
@@ -13413,31 +13459,31 @@
       </c>
       <c r="C161" s="10" t="inlineStr">
         <is>
-          <t>F10-02</t>
+          <t>F10-01</t>
         </is>
       </c>
       <c r="D161" s="27" t="inlineStr">
         <is>
-          <t>债券过滤与筛选</t>
+          <t>报价工作台</t>
         </is>
       </c>
       <c r="E161" s="11" t="inlineStr">
         <is>
-          <t>信用债全品种过滤，利率债（国债/证金债/地方债）过滤，精确识别与模糊识别双模式</t>
+          <t>历史报价管理，当日报价快捷操作，导入/导出报价，一键unrefer，报价提醒功能</t>
         </is>
       </c>
       <c r="F161" s="11" t="inlineStr">
         <is>
-          <t>功能测试通过</t>
-        </is>
-      </c>
-      <c r="G161" s="25" t="inlineStr">
-        <is>
-          <t>低</t>
+          <t>功能测试通过/正确率100%</t>
+        </is>
+      </c>
+      <c r="G161" s="24" t="inlineStr">
+        <is>
+          <t>中</t>
         </is>
       </c>
       <c r="H161" s="13" t="n">
-        <v>10</v>
+        <v>20</v>
       </c>
     </row>
     <row r="162" ht="28" customHeight="1">
@@ -13453,31 +13499,31 @@
       </c>
       <c r="C162" s="10" t="inlineStr">
         <is>
-          <t>F10-03</t>
+          <t>F10-02</t>
         </is>
       </c>
       <c r="D162" s="27" t="inlineStr">
         <is>
-          <t>报价撮合与对价</t>
+          <t>债券过滤与筛选</t>
         </is>
       </c>
       <c r="E162" s="11" t="inlineStr">
         <is>
-          <t>对价/最优报价聚合展示，撮合对价，交易包管理，报价成交确认，一键成交</t>
+          <t>信用债全品种过滤，利率债（国债/证金债/地方债）过滤，精确识别与模糊识别双模式</t>
         </is>
       </c>
       <c r="F162" s="11" t="inlineStr">
         <is>
-          <t>功能测试通过/正确率100%</t>
-        </is>
-      </c>
-      <c r="G162" s="24" t="inlineStr">
-        <is>
-          <t>中</t>
+          <t>功能测试通过</t>
+        </is>
+      </c>
+      <c r="G162" s="25" t="inlineStr">
+        <is>
+          <t>低</t>
         </is>
       </c>
       <c r="H162" s="13" t="n">
-        <v>20</v>
+        <v>10</v>
       </c>
     </row>
     <row r="163" ht="28" customHeight="1">
@@ -13493,17 +13539,17 @@
       </c>
       <c r="C163" s="10" t="inlineStr">
         <is>
-          <t>F10-04</t>
+          <t>F10-03</t>
         </is>
       </c>
       <c r="D163" s="27" t="inlineStr">
         <is>
-          <t>交易执行与要素校验</t>
+          <t>报价撮合与对价</t>
         </is>
       </c>
       <c r="E163" s="11" t="inlineStr">
         <is>
-          <t>意向达成，交易要素自动校验，手工价录入，业务审批流程，交易记录管理</t>
+          <t>对价/最优报价聚合展示，撮合对价，交易包管理，报价成交确认，一键成交</t>
         </is>
       </c>
       <c r="F163" s="11" t="inlineStr">
@@ -13517,7 +13563,7 @@
         </is>
       </c>
       <c r="H163" s="13" t="n">
-        <v>15</v>
+        <v>20</v>
       </c>
     </row>
     <row r="164" ht="28" customHeight="1">
@@ -13533,17 +13579,17 @@
       </c>
       <c r="C164" s="10" t="inlineStr">
         <is>
-          <t>F10-05</t>
+          <t>F10-04</t>
         </is>
       </c>
       <c r="D164" s="27" t="inlineStr">
         <is>
-          <t>风控检查</t>
+          <t>交易执行与要素校验</t>
         </is>
       </c>
       <c r="E164" s="11" t="inlineStr">
         <is>
-          <t>交易前风控规则同步校验，限额检查，合规拦截，风控记录留痕，不通过自动拦截</t>
+          <t>意向达成，交易要素自动校验，手工价录入，业务审批流程，交易记录管理</t>
         </is>
       </c>
       <c r="F164" s="11" t="inlineStr">
@@ -13573,31 +13619,31 @@
       </c>
       <c r="C165" s="10" t="inlineStr">
         <is>
-          <t>F10-06</t>
+          <t>F10-05</t>
         </is>
       </c>
       <c r="D165" s="27" t="inlineStr">
         <is>
-          <t>智能推荐系统</t>
+          <t>风控检查</t>
         </is>
       </c>
       <c r="E165" s="11" t="inlineStr">
         <is>
-          <t>基于客户画像与历史交易数据主动推荐券种，从被动服务转向主动服务，提升客户响应效率</t>
+          <t>交易前风控规则同步校验，限额检查，合规拦截，风控记录留痕，不通过自动拦截</t>
         </is>
       </c>
       <c r="F165" s="11" t="inlineStr">
         <is>
-          <t>功能完整/边界测试/集成冒烟/性能基线</t>
-        </is>
-      </c>
-      <c r="G165" s="23" t="inlineStr">
-        <is>
-          <t>高</t>
+          <t>功能测试通过/正确率100%</t>
+        </is>
+      </c>
+      <c r="G165" s="24" t="inlineStr">
+        <is>
+          <t>中</t>
         </is>
       </c>
       <c r="H165" s="13" t="n">
-        <v>25</v>
+        <v>15</v>
       </c>
     </row>
     <row r="166" ht="28" customHeight="1">
@@ -13613,78 +13659,78 @@
       </c>
       <c r="C166" s="10" t="inlineStr">
         <is>
+          <t>F10-06</t>
+        </is>
+      </c>
+      <c r="D166" s="27" t="inlineStr">
+        <is>
+          <t>智能推荐系统</t>
+        </is>
+      </c>
+      <c r="E166" s="11" t="inlineStr">
+        <is>
+          <t>基于客户画像与历史交易数据主动推荐券种，从被动服务转向主动服务，提升客户响应效率</t>
+        </is>
+      </c>
+      <c r="F166" s="11" t="inlineStr">
+        <is>
+          <t>功能完整/边界测试/集成冒烟/性能基线</t>
+        </is>
+      </c>
+      <c r="G166" s="23" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="H166" s="13" t="n">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="167" ht="28" customHeight="1">
+      <c r="A167" s="11" t="inlineStr">
+        <is>
+          <t>销售交易</t>
+        </is>
+      </c>
+      <c r="B167" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="C167" s="10" t="inlineStr">
+        <is>
           <t>F10-07</t>
         </is>
       </c>
-      <c r="D166" s="27" t="inlineStr">
+      <c r="D167" s="27" t="inlineStr">
         <is>
           <t>综合业务平台</t>
         </is>
       </c>
-      <c r="E166" s="11" t="inlineStr">
+      <c r="E167" s="11" t="inlineStr">
         <is>
           <t>解决交易员分散办公与客户交易信息共享问题，报价聚合展示，客户快速服务，多地协同</t>
         </is>
       </c>
-      <c r="F166" s="11" t="inlineStr">
+      <c r="F167" s="11" t="inlineStr">
         <is>
           <t>功能测试通过/正确率100%</t>
         </is>
       </c>
-      <c r="G166" s="24" t="inlineStr">
+      <c r="G167" s="24" t="inlineStr">
         <is>
           <t>中</t>
         </is>
       </c>
-      <c r="H166" s="13" t="n">
+      <c r="H167" s="13" t="n">
         <v>15</v>
       </c>
     </row>
-    <row r="167" ht="20" customHeight="1">
-      <c r="A167" s="26" t="inlineStr">
+    <row r="168" ht="20" customHeight="1">
+      <c r="A168" s="26" t="inlineStr">
         <is>
           <t>【P2】 信用债/信用衍生品  (Credit Bond &amp; CDS)</t>
         </is>
-      </c>
-    </row>
-    <row r="168" ht="28" customHeight="1">
-      <c r="A168" s="11" t="inlineStr">
-        <is>
-          <t>信用债/信用衍生品</t>
-        </is>
-      </c>
-      <c r="B168" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
-        </is>
-      </c>
-      <c r="C168" s="10" t="inlineStr">
-        <is>
-          <t>F11-01</t>
-        </is>
-      </c>
-      <c r="D168" s="27" t="inlineStr">
-        <is>
-          <t>信用风险数据接入</t>
-        </is>
-      </c>
-      <c r="E168" s="11" t="inlineStr">
-        <is>
-          <t>外部信用数据服务接入（Wind/中诚信/联合评级等），内部数据整合，数据质量检查，信用风险数据集市</t>
-        </is>
-      </c>
-      <c r="F168" s="11" t="inlineStr">
-        <is>
-          <t>功能完整/边界测试/集成冒烟/性能基线</t>
-        </is>
-      </c>
-      <c r="G168" s="23" t="inlineStr">
-        <is>
-          <t>高</t>
-        </is>
-      </c>
-      <c r="H168" s="13" t="n">
-        <v>30</v>
       </c>
     </row>
     <row r="169" ht="28" customHeight="1">
@@ -13700,31 +13746,31 @@
       </c>
       <c r="C169" s="10" t="inlineStr">
         <is>
-          <t>F11-02</t>
+          <t>F11-01</t>
         </is>
       </c>
       <c r="D169" s="27" t="inlineStr">
         <is>
-          <t>信用评估引擎</t>
+          <t>信用风险数据接入</t>
         </is>
       </c>
       <c r="E169" s="11" t="inlineStr">
         <is>
-          <t>持续迭代信用评价引擎，资产证券化评价，交易对手评价，违约概率（PD）建模，信用评分</t>
+          <t>外部信用数据服务接入（Wind/中诚信/联合评级等），内部数据整合，数据质量检查，信用风险数据集市</t>
         </is>
       </c>
       <c r="F169" s="11" t="inlineStr">
         <is>
-          <t>p99延迟/误差率/精度验证/压测10k TPS</t>
-        </is>
-      </c>
-      <c r="G169" s="28" t="inlineStr">
-        <is>
-          <t>极高</t>
+          <t>功能完整/边界测试/集成冒烟/性能基线</t>
+        </is>
+      </c>
+      <c r="G169" s="23" t="inlineStr">
+        <is>
+          <t>高</t>
         </is>
       </c>
       <c r="H169" s="13" t="n">
-        <v>40</v>
+        <v>30</v>
       </c>
     </row>
     <row r="170" ht="28" customHeight="1">
@@ -13740,31 +13786,31 @@
       </c>
       <c r="C170" s="10" t="inlineStr">
         <is>
-          <t>F11-03</t>
+          <t>F11-02</t>
         </is>
       </c>
       <c r="D170" s="27" t="inlineStr">
         <is>
-          <t>信用预警系统</t>
+          <t>信用评估引擎</t>
         </is>
       </c>
       <c r="E170" s="11" t="inlineStr">
         <is>
-          <t>市场数据自动触发预警，评级下调动态预警，投后预警跟踪与信号处理，预警规则配置</t>
+          <t>持续迭代信用评价引擎，资产证券化评价，交易对手评价，违约概率（PD）建模，信用评分</t>
         </is>
       </c>
       <c r="F170" s="11" t="inlineStr">
         <is>
-          <t>功能完整/边界测试/集成冒烟/性能基线</t>
-        </is>
-      </c>
-      <c r="G170" s="23" t="inlineStr">
-        <is>
-          <t>高</t>
+          <t>p99延迟/误差率/精度验证/压测10k TPS</t>
+        </is>
+      </c>
+      <c r="G170" s="28" t="inlineStr">
+        <is>
+          <t>极高</t>
         </is>
       </c>
       <c r="H170" s="13" t="n">
-        <v>30</v>
+        <v>40</v>
       </c>
     </row>
     <row r="171" ht="28" customHeight="1">
@@ -13780,31 +13826,31 @@
       </c>
       <c r="C171" s="10" t="inlineStr">
         <is>
-          <t>F11-04</t>
+          <t>F11-03</t>
         </is>
       </c>
       <c r="D171" s="27" t="inlineStr">
         <is>
-          <t>投资池管理</t>
+          <t>信用预警系统</t>
         </is>
       </c>
       <c r="E171" s="11" t="inlineStr">
         <is>
-          <t>债券池配置与维护，债券准入/退出规则，白名单/黑名单管理，池状态实时更新</t>
+          <t>市场数据自动触发预警，评级下调动态预警，投后预警跟踪与信号处理，预警规则配置</t>
         </is>
       </c>
       <c r="F171" s="11" t="inlineStr">
         <is>
-          <t>功能测试通过/正确率100%</t>
-        </is>
-      </c>
-      <c r="G171" s="24" t="inlineStr">
-        <is>
-          <t>中</t>
+          <t>功能完整/边界测试/集成冒烟/性能基线</t>
+        </is>
+      </c>
+      <c r="G171" s="23" t="inlineStr">
+        <is>
+          <t>高</t>
         </is>
       </c>
       <c r="H171" s="13" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
     </row>
     <row r="172" ht="28" customHeight="1">
@@ -13820,17 +13866,17 @@
       </c>
       <c r="C172" s="10" t="inlineStr">
         <is>
-          <t>F11-05</t>
+          <t>F11-04</t>
         </is>
       </c>
       <c r="D172" s="27" t="inlineStr">
         <is>
-          <t>评级管理</t>
+          <t>投资池管理</t>
         </is>
       </c>
       <c r="E172" s="11" t="inlineStr">
         <is>
-          <t>内部评级录入与更新，外部评级同步（中诚信/联合/大公），评级变更历史追踪，评级模型管理</t>
+          <t>债券池配置与维护，债券准入/退出规则，白名单/黑名单管理，池状态实时更新</t>
         </is>
       </c>
       <c r="F172" s="11" t="inlineStr">
@@ -13860,17 +13906,17 @@
       </c>
       <c r="C173" s="10" t="inlineStr">
         <is>
-          <t>F11-06</t>
+          <t>F11-05</t>
         </is>
       </c>
       <c r="D173" s="27" t="inlineStr">
         <is>
-          <t>投前审批管理</t>
+          <t>评级管理</t>
         </is>
       </c>
       <c r="E173" s="11" t="inlineStr">
         <is>
-          <t>新券投资准入审批流程，信用额度申请，投资决策材料生成，审批记录留痕</t>
+          <t>内部评级录入与更新，外部评级同步（中诚信/联合/大公），评级变更历史追踪，评级模型管理</t>
         </is>
       </c>
       <c r="F173" s="11" t="inlineStr">
@@ -13900,17 +13946,17 @@
       </c>
       <c r="C174" s="10" t="inlineStr">
         <is>
-          <t>F11-07</t>
+          <t>F11-06</t>
         </is>
       </c>
       <c r="D174" s="27" t="inlineStr">
         <is>
-          <t>持仓与敞口管理</t>
+          <t>投前审批管理</t>
         </is>
       </c>
       <c r="E174" s="11" t="inlineStr">
         <is>
-          <t>信用债持仓实时查询，敞口管理，集中度分析（行业/评级/发行人），到期提醒</t>
+          <t>新券投资准入审批流程，信用额度申请，投资决策材料生成，审批记录留痕</t>
         </is>
       </c>
       <c r="F174" s="11" t="inlineStr">
@@ -13940,31 +13986,31 @@
       </c>
       <c r="C175" s="10" t="inlineStr">
         <is>
-          <t>F11-08</t>
+          <t>F11-07</t>
         </is>
       </c>
       <c r="D175" s="27" t="inlineStr">
         <is>
-          <t>信用风险监控看板</t>
+          <t>持仓与敞口管理</t>
         </is>
       </c>
       <c r="E175" s="11" t="inlineStr">
         <is>
-          <t>多维度风险指标实时监控，信用利差走势，主体信用事件推送，指标监控与查询统计</t>
+          <t>信用债持仓实时查询，敞口管理，集中度分析（行业/评级/发行人），到期提醒</t>
         </is>
       </c>
       <c r="F175" s="11" t="inlineStr">
         <is>
-          <t>功能完整/边界测试/集成冒烟/性能基线</t>
-        </is>
-      </c>
-      <c r="G175" s="23" t="inlineStr">
-        <is>
-          <t>高</t>
+          <t>功能测试通过/正确率100%</t>
+        </is>
+      </c>
+      <c r="G175" s="24" t="inlineStr">
+        <is>
+          <t>中</t>
         </is>
       </c>
       <c r="H175" s="13" t="n">
-        <v>25</v>
+        <v>20</v>
       </c>
     </row>
     <row r="176" ht="28" customHeight="1">
@@ -13980,17 +14026,17 @@
       </c>
       <c r="C176" s="10" t="inlineStr">
         <is>
-          <t>F11-09</t>
+          <t>F11-08</t>
         </is>
       </c>
       <c r="D176" s="27" t="inlineStr">
         <is>
-          <t>违约管理</t>
+          <t>信用风险监控看板</t>
         </is>
       </c>
       <c r="E176" s="11" t="inlineStr">
         <is>
-          <t>违约事件记录，违约债券处置跟踪，损失估算，监管报送，违约主体黑名单自动更新</t>
+          <t>多维度风险指标实时监控，信用利差走势，主体信用事件推送，指标监控与查询统计</t>
         </is>
       </c>
       <c r="F176" s="11" t="inlineStr">
@@ -14020,17 +14066,17 @@
       </c>
       <c r="C177" s="10" t="inlineStr">
         <is>
-          <t>F11-10</t>
+          <t>F11-09</t>
         </is>
       </c>
       <c r="D177" s="27" t="inlineStr">
         <is>
-          <t>信用利差分析</t>
+          <t>违约管理</t>
         </is>
       </c>
       <c r="E177" s="11" t="inlineStr">
         <is>
-          <t>行业/评级/期限信用利差曲线实时计算，历史分位数分析，利差走势，相对价值分析</t>
+          <t>违约事件记录，违约债券处置跟踪，损失估算，监管报送，违约主体黑名单自动更新</t>
         </is>
       </c>
       <c r="F177" s="11" t="inlineStr">
@@ -14044,7 +14090,7 @@
         </is>
       </c>
       <c r="H177" s="13" t="n">
-        <v>30</v>
+        <v>25</v>
       </c>
     </row>
     <row r="178" ht="28" customHeight="1">
@@ -14060,31 +14106,31 @@
       </c>
       <c r="C178" s="10" t="inlineStr">
         <is>
-          <t>F11-11</t>
+          <t>F11-10</t>
         </is>
       </c>
       <c r="D178" s="27" t="inlineStr">
         <is>
-          <t>CDS定价与管理</t>
+          <t>信用利差分析</t>
         </is>
       </c>
       <c r="E178" s="11" t="inlineStr">
         <is>
-          <t>信用违约互换定价（ISDA标准），生存概率曲线校准，CDS交易录入与持仓管理</t>
+          <t>行业/评级/期限信用利差曲线实时计算，历史分位数分析，利差走势，相对价值分析</t>
         </is>
       </c>
       <c r="F178" s="11" t="inlineStr">
         <is>
-          <t>p99延迟/误差率/精度验证/压测10k TPS</t>
-        </is>
-      </c>
-      <c r="G178" s="28" t="inlineStr">
-        <is>
-          <t>极高</t>
+          <t>功能完整/边界测试/集成冒烟/性能基线</t>
+        </is>
+      </c>
+      <c r="G178" s="23" t="inlineStr">
+        <is>
+          <t>高</t>
         </is>
       </c>
       <c r="H178" s="13" t="n">
-        <v>40</v>
+        <v>30</v>
       </c>
     </row>
     <row r="179" ht="28" customHeight="1">
@@ -14100,78 +14146,78 @@
       </c>
       <c r="C179" s="10" t="inlineStr">
         <is>
+          <t>F11-11</t>
+        </is>
+      </c>
+      <c r="D179" s="27" t="inlineStr">
+        <is>
+          <t>CDS定价与管理</t>
+        </is>
+      </c>
+      <c r="E179" s="11" t="inlineStr">
+        <is>
+          <t>信用违约互换定价（ISDA标准），生存概率曲线校准，CDS交易录入与持仓管理</t>
+        </is>
+      </c>
+      <c r="F179" s="11" t="inlineStr">
+        <is>
+          <t>p99延迟/误差率/精度验证/压测10k TPS</t>
+        </is>
+      </c>
+      <c r="G179" s="28" t="inlineStr">
+        <is>
+          <t>极高</t>
+        </is>
+      </c>
+      <c r="H179" s="13" t="n">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="180" ht="28" customHeight="1">
+      <c r="A180" s="11" t="inlineStr">
+        <is>
+          <t>信用债/信用衍生品</t>
+        </is>
+      </c>
+      <c r="B180" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="C180" s="10" t="inlineStr">
+        <is>
           <t>F11-12</t>
         </is>
       </c>
-      <c r="D179" s="27" t="inlineStr">
+      <c r="D180" s="27" t="inlineStr">
         <is>
           <t>配置与权限管理</t>
         </is>
       </c>
-      <c r="E179" s="11" t="inlineStr">
+      <c r="E180" s="11" t="inlineStr">
         <is>
           <t>预警规则配置，指标库管理，评级模型管理，用户权限管理，债券池配置管理</t>
         </is>
       </c>
-      <c r="F179" s="11" t="inlineStr">
+      <c r="F180" s="11" t="inlineStr">
         <is>
           <t>功能测试通过</t>
         </is>
       </c>
-      <c r="G179" s="25" t="inlineStr">
+      <c r="G180" s="25" t="inlineStr">
         <is>
           <t>低</t>
         </is>
       </c>
-      <c r="H179" s="13" t="n">
+      <c r="H180" s="13" t="n">
         <v>15</v>
       </c>
     </row>
-    <row r="180" ht="20" customHeight="1">
-      <c r="A180" s="26" t="inlineStr">
+    <row r="181" ht="20" customHeight="1">
+      <c r="A181" s="26" t="inlineStr">
         <is>
           <t>【P2】 投顾服务  (Investment Advisory)</t>
         </is>
-      </c>
-    </row>
-    <row r="181" ht="28" customHeight="1">
-      <c r="A181" s="11" t="inlineStr">
-        <is>
-          <t>投顾服务</t>
-        </is>
-      </c>
-      <c r="B181" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
-        </is>
-      </c>
-      <c r="C181" s="10" t="inlineStr">
-        <is>
-          <t>F12-01</t>
-        </is>
-      </c>
-      <c r="D181" s="27" t="inlineStr">
-        <is>
-          <t>投顾操作工作台</t>
-        </is>
-      </c>
-      <c r="E181" s="11" t="inlineStr">
-        <is>
-          <t>投顾人员管理客户委托，上传研究报告，发送投资建议，查看客户反馈与确认状态</t>
-        </is>
-      </c>
-      <c r="F181" s="11" t="inlineStr">
-        <is>
-          <t>功能测试通过/正确率100%</t>
-        </is>
-      </c>
-      <c r="G181" s="24" t="inlineStr">
-        <is>
-          <t>中</t>
-        </is>
-      </c>
-      <c r="H181" s="13" t="n">
-        <v>20</v>
       </c>
     </row>
     <row r="182" ht="28" customHeight="1">
@@ -14187,17 +14233,17 @@
       </c>
       <c r="C182" s="10" t="inlineStr">
         <is>
-          <t>F12-02</t>
+          <t>F12-01</t>
         </is>
       </c>
       <c r="D182" s="27" t="inlineStr">
         <is>
-          <t>投资建议书管理</t>
+          <t>投顾操作工作台</t>
         </is>
       </c>
       <c r="E182" s="11" t="inlineStr">
         <is>
-          <t>投资建议书线上生成与审批，客户确认全流程，留痕追溯，电子签收，历史建议书归档</t>
+          <t>投顾人员管理客户委托，上传研究报告，发送投资建议，查看客户反馈与确认状态</t>
         </is>
       </c>
       <c r="F182" s="11" t="inlineStr">
@@ -14227,17 +14273,17 @@
       </c>
       <c r="C183" s="10" t="inlineStr">
         <is>
-          <t>F12-03</t>
+          <t>F12-02</t>
         </is>
       </c>
       <c r="D183" s="27" t="inlineStr">
         <is>
-          <t>投研报告服务</t>
+          <t>投资建议书管理</t>
         </is>
       </c>
       <c r="E183" s="11" t="inlineStr">
         <is>
-          <t>日/周/月研究报告上传与定向推送，RPA自动获取基础数据，报告分类管理与检索</t>
+          <t>投资建议书线上生成与审批，客户确认全流程，留痕追溯，电子签收，历史建议书归档</t>
         </is>
       </c>
       <c r="F183" s="11" t="inlineStr">
@@ -14251,7 +14297,7 @@
         </is>
       </c>
       <c r="H183" s="13" t="n">
-        <v>15</v>
+        <v>20</v>
       </c>
     </row>
     <row r="184" ht="28" customHeight="1">
@@ -14267,17 +14313,17 @@
       </c>
       <c r="C184" s="10" t="inlineStr">
         <is>
-          <t>F12-04</t>
+          <t>F12-03</t>
         </is>
       </c>
       <c r="D184" s="27" t="inlineStr">
         <is>
-          <t>客户投资服务界面</t>
+          <t>投研报告服务</t>
         </is>
       </c>
       <c r="E184" s="11" t="inlineStr">
         <is>
-          <t>客户查看投资建议与分析报告，发送确认，查看账户净值走势、持仓明细、交易明细</t>
+          <t>日/周/月研究报告上传与定向推送，RPA自动获取基础数据，报告分类管理与检索</t>
         </is>
       </c>
       <c r="F184" s="11" t="inlineStr">
@@ -14291,7 +14337,7 @@
         </is>
       </c>
       <c r="H184" s="13" t="n">
-        <v>20</v>
+        <v>15</v>
       </c>
     </row>
     <row r="185" ht="28" customHeight="1">
@@ -14307,31 +14353,31 @@
       </c>
       <c r="C185" s="10" t="inlineStr">
         <is>
-          <t>F12-05</t>
+          <t>F12-04</t>
         </is>
       </c>
       <c r="D185" s="27" t="inlineStr">
         <is>
-          <t>账户深度分析</t>
+          <t>客户投资服务界面</t>
         </is>
       </c>
       <c r="E185" s="11" t="inlineStr">
         <is>
-          <t>账户净值走势，久期走势，归因分析，估值台账，持仓明细，交易明细，定期分析报告生成</t>
+          <t>客户查看投资建议与分析报告，发送确认，查看账户净值走势、持仓明细、交易明细</t>
         </is>
       </c>
       <c r="F185" s="11" t="inlineStr">
         <is>
-          <t>功能完整/边界测试/集成冒烟/性能基线</t>
-        </is>
-      </c>
-      <c r="G185" s="23" t="inlineStr">
-        <is>
-          <t>高</t>
+          <t>功能测试通过/正确率100%</t>
+        </is>
+      </c>
+      <c r="G185" s="24" t="inlineStr">
+        <is>
+          <t>中</t>
         </is>
       </c>
       <c r="H185" s="13" t="n">
-        <v>25</v>
+        <v>20</v>
       </c>
     </row>
     <row r="186" ht="28" customHeight="1">
@@ -14347,31 +14393,31 @@
       </c>
       <c r="C186" s="10" t="inlineStr">
         <is>
-          <t>F12-06</t>
+          <t>F12-05</t>
         </is>
       </c>
       <c r="D186" s="27" t="inlineStr">
         <is>
-          <t>交易服务对接</t>
+          <t>账户深度分析</t>
         </is>
       </c>
       <c r="E186" s="11" t="inlineStr">
         <is>
-          <t>客户查看投资建议后直接触发交易委托，与销售交易系统对接，全程数字化交易确认</t>
+          <t>账户净值走势，久期走势，归因分析，估值台账，持仓明细，交易明细，定期分析报告生成</t>
         </is>
       </c>
       <c r="F186" s="11" t="inlineStr">
         <is>
-          <t>功能测试通过/正确率100%</t>
-        </is>
-      </c>
-      <c r="G186" s="24" t="inlineStr">
-        <is>
-          <t>中</t>
+          <t>功能完整/边界测试/集成冒烟/性能基线</t>
+        </is>
+      </c>
+      <c r="G186" s="23" t="inlineStr">
+        <is>
+          <t>高</t>
         </is>
       </c>
       <c r="H186" s="13" t="n">
-        <v>15</v>
+        <v>25</v>
       </c>
     </row>
     <row r="187" ht="28" customHeight="1">
@@ -14387,31 +14433,31 @@
       </c>
       <c r="C187" s="10" t="inlineStr">
         <is>
-          <t>F12-07</t>
+          <t>F12-06</t>
         </is>
       </c>
       <c r="D187" s="27" t="inlineStr">
         <is>
-          <t>客户服务中心</t>
+          <t>交易服务对接</t>
         </is>
       </c>
       <c r="E187" s="11" t="inlineStr">
         <is>
-          <t>服务中心，消息中心，常见问题，问卷系统，客户满意度管理</t>
+          <t>客户查看投资建议后直接触发交易委托，与销售交易系统对接，全程数字化交易确认</t>
         </is>
       </c>
       <c r="F187" s="11" t="inlineStr">
         <is>
-          <t>功能测试通过</t>
-        </is>
-      </c>
-      <c r="G187" s="25" t="inlineStr">
-        <is>
-          <t>低</t>
+          <t>功能测试通过/正确率100%</t>
+        </is>
+      </c>
+      <c r="G187" s="24" t="inlineStr">
+        <is>
+          <t>中</t>
         </is>
       </c>
       <c r="H187" s="13" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="188" ht="28" customHeight="1">
@@ -14427,17 +14473,17 @@
       </c>
       <c r="C188" s="10" t="inlineStr">
         <is>
-          <t>F12-08</t>
+          <t>F12-07</t>
         </is>
       </c>
       <c r="D188" s="27" t="inlineStr">
         <is>
-          <t>平台基础管理</t>
+          <t>客户服务中心</t>
         </is>
       </c>
       <c r="E188" s="11" t="inlineStr">
         <is>
-          <t>用户管理，账户管理，数据管理，消息群发，登录注册，权限控制</t>
+          <t>服务中心，消息中心，常见问题，问卷系统，客户满意度管理</t>
         </is>
       </c>
       <c r="F188" s="11" t="inlineStr">
@@ -14454,51 +14500,51 @@
         <v>10</v>
       </c>
     </row>
-    <row r="189" ht="20" customHeight="1">
-      <c r="A189" s="26" t="inlineStr">
+    <row r="189" ht="28" customHeight="1">
+      <c r="A189" s="11" t="inlineStr">
+        <is>
+          <t>投顾服务</t>
+        </is>
+      </c>
+      <c r="B189" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="C189" s="10" t="inlineStr">
+        <is>
+          <t>F12-08</t>
+        </is>
+      </c>
+      <c r="D189" s="27" t="inlineStr">
+        <is>
+          <t>平台基础管理</t>
+        </is>
+      </c>
+      <c r="E189" s="11" t="inlineStr">
+        <is>
+          <t>用户管理，账户管理，数据管理，消息群发，登录注册，权限控制</t>
+        </is>
+      </c>
+      <c r="F189" s="11" t="inlineStr">
+        <is>
+          <t>功能测试通过</t>
+        </is>
+      </c>
+      <c r="G189" s="25" t="inlineStr">
+        <is>
+          <t>低</t>
+        </is>
+      </c>
+      <c r="H189" s="13" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="190" ht="20" customHeight="1">
+      <c r="A190" s="26" t="inlineStr">
         <is>
           <t>【P2】 TRS收益互换  (Total Return Swap)</t>
         </is>
-      </c>
-    </row>
-    <row r="190" ht="28" customHeight="1">
-      <c r="A190" s="11" t="inlineStr">
-        <is>
-          <t>TRS收益互换</t>
-        </is>
-      </c>
-      <c r="B190" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
-        </is>
-      </c>
-      <c r="C190" s="10" t="inlineStr">
-        <is>
-          <t>F13-01</t>
-        </is>
-      </c>
-      <c r="D190" s="27" t="inlineStr">
-        <is>
-          <t>报价与成交管理</t>
-        </is>
-      </c>
-      <c r="E190" s="11" t="inlineStr">
-        <is>
-          <t>一站式报价（市场各渠道 + 内部自营），成交回报处理，请求报价（RFQ），历史确认查询</t>
-        </is>
-      </c>
-      <c r="F190" s="11" t="inlineStr">
-        <is>
-          <t>功能完整/边界测试/集成冒烟/性能基线</t>
-        </is>
-      </c>
-      <c r="G190" s="23" t="inlineStr">
-        <is>
-          <t>高</t>
-        </is>
-      </c>
-      <c r="H190" s="13" t="n">
-        <v>30</v>
       </c>
     </row>
     <row r="191" ht="28" customHeight="1">
@@ -14514,17 +14560,17 @@
       </c>
       <c r="C191" s="10" t="inlineStr">
         <is>
-          <t>F13-02</t>
+          <t>F13-01</t>
         </is>
       </c>
       <c r="D191" s="27" t="inlineStr">
         <is>
-          <t>自动对冲</t>
+          <t>报价与成交管理</t>
         </is>
       </c>
       <c r="E191" s="11" t="inlineStr">
         <is>
-          <t>对冲委托自动触发，对冲回报处理，风险校验，组合重叠分析，开平仓设置，对冲策略配置</t>
+          <t>一站式报价（市场各渠道 + 内部自营），成交回报处理，请求报价（RFQ），历史确认查询</t>
         </is>
       </c>
       <c r="F191" s="11" t="inlineStr">
@@ -14554,31 +14600,31 @@
       </c>
       <c r="C192" s="10" t="inlineStr">
         <is>
-          <t>F13-03</t>
+          <t>F13-02</t>
         </is>
       </c>
       <c r="D192" s="27" t="inlineStr">
         <is>
-          <t>行情与资讯</t>
+          <t>自动对冲</t>
         </is>
       </c>
       <c r="E192" s="11" t="inlineStr">
         <is>
-          <t>实时行情矩阵展示，债券行情，我的关注，历史行情，资讯推送</t>
+          <t>对冲委托自动触发，对冲回报处理，风险校验，组合重叠分析，开平仓设置，对冲策略配置</t>
         </is>
       </c>
       <c r="F192" s="11" t="inlineStr">
         <is>
-          <t>功能测试通过/正确率100%</t>
-        </is>
-      </c>
-      <c r="G192" s="24" t="inlineStr">
-        <is>
-          <t>中</t>
+          <t>功能完整/边界测试/集成冒烟/性能基线</t>
+        </is>
+      </c>
+      <c r="G192" s="23" t="inlineStr">
+        <is>
+          <t>高</t>
         </is>
       </c>
       <c r="H192" s="13" t="n">
-        <v>15</v>
+        <v>30</v>
       </c>
     </row>
     <row r="193" ht="28" customHeight="1">
@@ -14594,17 +14640,17 @@
       </c>
       <c r="C193" s="10" t="inlineStr">
         <is>
-          <t>F13-04</t>
+          <t>F13-03</t>
         </is>
       </c>
       <c r="D193" s="27" t="inlineStr">
         <is>
-          <t>开户与账户管理</t>
+          <t>行情与资讯</t>
         </is>
       </c>
       <c r="E193" s="11" t="inlineStr">
         <is>
-          <t>客户开户申请，账户信息管理，出入金申请，银行账号绑定，资金管理</t>
+          <t>实时行情矩阵展示，债券行情，我的关注，历史行情，资讯推送</t>
         </is>
       </c>
       <c r="F193" s="11" t="inlineStr">
@@ -14618,7 +14664,7 @@
         </is>
       </c>
       <c r="H193" s="13" t="n">
-        <v>20</v>
+        <v>15</v>
       </c>
     </row>
     <row r="194" ht="28" customHeight="1">
@@ -14634,31 +14680,31 @@
       </c>
       <c r="C194" s="10" t="inlineStr">
         <is>
-          <t>F13-05</t>
+          <t>F13-04</t>
         </is>
       </c>
       <c r="D194" s="27" t="inlineStr">
         <is>
-          <t>客户自主交易</t>
+          <t>开户与账户管理</t>
         </is>
       </c>
       <c r="E194" s="11" t="inlineStr">
         <is>
-          <t>客户委托下单，合约持仓查询，标的持仓查询，当日委托，行情矩阵，历史确认，开平仓设置</t>
+          <t>客户开户申请，账户信息管理，出入金申请，银行账号绑定，资金管理</t>
         </is>
       </c>
       <c r="F194" s="11" t="inlineStr">
         <is>
-          <t>功能完整/边界测试/集成冒烟/性能基线</t>
-        </is>
-      </c>
-      <c r="G194" s="23" t="inlineStr">
-        <is>
-          <t>高</t>
+          <t>功能测试通过/正确率100%</t>
+        </is>
+      </c>
+      <c r="G194" s="24" t="inlineStr">
+        <is>
+          <t>中</t>
         </is>
       </c>
       <c r="H194" s="13" t="n">
-        <v>25</v>
+        <v>20</v>
       </c>
     </row>
     <row r="195" ht="28" customHeight="1">
@@ -14674,31 +14720,31 @@
       </c>
       <c r="C195" s="10" t="inlineStr">
         <is>
-          <t>F13-06</t>
+          <t>F13-05</t>
         </is>
       </c>
       <c r="D195" s="27" t="inlineStr">
         <is>
-          <t>审批管理</t>
+          <t>客户自主交易</t>
         </is>
       </c>
       <c r="E195" s="11" t="inlineStr">
         <is>
-          <t>开户申请审批，出入金审批，合约成交审核，多级审批工作流，审批留痕</t>
+          <t>客户委托下单，合约持仓查询，标的持仓查询，当日委托，行情矩阵，历史确认，开平仓设置</t>
         </is>
       </c>
       <c r="F195" s="11" t="inlineStr">
         <is>
-          <t>功能测试通过/正确率100%</t>
-        </is>
-      </c>
-      <c r="G195" s="24" t="inlineStr">
-        <is>
-          <t>中</t>
+          <t>功能完整/边界测试/集成冒烟/性能基线</t>
+        </is>
+      </c>
+      <c r="G195" s="23" t="inlineStr">
+        <is>
+          <t>高</t>
         </is>
       </c>
       <c r="H195" s="13" t="n">
-        <v>20</v>
+        <v>25</v>
       </c>
     </row>
     <row r="196" ht="28" customHeight="1">
@@ -14714,31 +14760,31 @@
       </c>
       <c r="C196" s="10" t="inlineStr">
         <is>
-          <t>F13-07</t>
+          <t>F13-06</t>
         </is>
       </c>
       <c r="D196" s="27" t="inlineStr">
         <is>
-          <t>运营管理</t>
+          <t>审批管理</t>
         </is>
       </c>
       <c r="E196" s="11" t="inlineStr">
         <is>
-          <t>对账，库存管理，对冲录入，合约生命周期管理，日终结算处理</t>
+          <t>开户申请审批，出入金审批，合约成交审核，多级审批工作流，审批留痕</t>
         </is>
       </c>
       <c r="F196" s="11" t="inlineStr">
         <is>
-          <t>功能完整/边界测试/集成冒烟/性能基线</t>
-        </is>
-      </c>
-      <c r="G196" s="23" t="inlineStr">
-        <is>
-          <t>高</t>
+          <t>功能测试通过/正确率100%</t>
+        </is>
+      </c>
+      <c r="G196" s="24" t="inlineStr">
+        <is>
+          <t>中</t>
         </is>
       </c>
       <c r="H196" s="13" t="n">
-        <v>25</v>
+        <v>20</v>
       </c>
     </row>
     <row r="197" ht="28" customHeight="1">
@@ -14754,31 +14800,31 @@
       </c>
       <c r="C197" s="10" t="inlineStr">
         <is>
-          <t>F13-08</t>
+          <t>F13-07</t>
         </is>
       </c>
       <c r="D197" s="27" t="inlineStr">
         <is>
-          <t>通知与文件生成</t>
+          <t>运营管理</t>
         </is>
       </c>
       <c r="E197" s="11" t="inlineStr">
         <is>
-          <t>企微通知提醒，确认书/结算单/估值报告/出入金通知自动生成并通过邮箱发送</t>
+          <t>对账，库存管理，对冲录入，合约生命周期管理，日终结算处理</t>
         </is>
       </c>
       <c r="F197" s="11" t="inlineStr">
         <is>
-          <t>功能测试通过/正确率100%</t>
-        </is>
-      </c>
-      <c r="G197" s="24" t="inlineStr">
-        <is>
-          <t>中</t>
+          <t>功能完整/边界测试/集成冒烟/性能基线</t>
+        </is>
+      </c>
+      <c r="G197" s="23" t="inlineStr">
+        <is>
+          <t>高</t>
         </is>
       </c>
       <c r="H197" s="13" t="n">
-        <v>15</v>
+        <v>25</v>
       </c>
     </row>
     <row r="198" ht="28" customHeight="1">
@@ -14794,31 +14840,31 @@
       </c>
       <c r="C198" s="10" t="inlineStr">
         <is>
-          <t>F13-09</t>
+          <t>F13-08</t>
         </is>
       </c>
       <c r="D198" s="27" t="inlineStr">
         <is>
-          <t>外部系统集成</t>
+          <t>通知与文件生成</t>
         </is>
       </c>
       <c r="E198" s="11" t="inlineStr">
         <is>
-          <t>衡泰系统客户信息同步，QTrade聊天记录同步，银行流水对接，公司邮箱系统集成</t>
+          <t>企微通知提醒，确认书/结算单/估值报告/出入金通知自动生成并通过邮箱发送</t>
         </is>
       </c>
       <c r="F198" s="11" t="inlineStr">
         <is>
-          <t>功能完整/边界测试/集成冒烟/性能基线</t>
-        </is>
-      </c>
-      <c r="G198" s="23" t="inlineStr">
-        <is>
-          <t>高</t>
+          <t>功能测试通过/正确率100%</t>
+        </is>
+      </c>
+      <c r="G198" s="24" t="inlineStr">
+        <is>
+          <t>中</t>
         </is>
       </c>
       <c r="H198" s="13" t="n">
-        <v>25</v>
+        <v>15</v>
       </c>
     </row>
     <row r="199" ht="28" customHeight="1">
@@ -14834,78 +14880,78 @@
       </c>
       <c r="C199" s="10" t="inlineStr">
         <is>
+          <t>F13-09</t>
+        </is>
+      </c>
+      <c r="D199" s="27" t="inlineStr">
+        <is>
+          <t>外部系统集成</t>
+        </is>
+      </c>
+      <c r="E199" s="11" t="inlineStr">
+        <is>
+          <t>衡泰系统客户信息同步，QTrade聊天记录同步，银行流水对接，公司邮箱系统集成</t>
+        </is>
+      </c>
+      <c r="F199" s="11" t="inlineStr">
+        <is>
+          <t>功能完整/边界测试/集成冒烟/性能基线</t>
+        </is>
+      </c>
+      <c r="G199" s="23" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="H199" s="13" t="n">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="200" ht="28" customHeight="1">
+      <c r="A200" s="11" t="inlineStr">
+        <is>
+          <t>TRS收益互换</t>
+        </is>
+      </c>
+      <c r="B200" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="C200" s="10" t="inlineStr">
+        <is>
           <t>F13-10</t>
         </is>
       </c>
-      <c r="D199" s="27" t="inlineStr">
+      <c r="D200" s="27" t="inlineStr">
         <is>
           <t>内部系统集成</t>
         </is>
       </c>
-      <c r="E199" s="11" t="inlineStr">
+      <c r="E200" s="11" t="inlineStr">
         <is>
           <t>现券交易系统（对冲交易执行），IBOR（持仓记录），定价平台（估值报告），事前风控（合规校验）</t>
         </is>
       </c>
-      <c r="F199" s="11" t="inlineStr">
+      <c r="F200" s="11" t="inlineStr">
         <is>
           <t>功能完整/边界测试/集成冒烟/性能基线</t>
         </is>
       </c>
-      <c r="G199" s="23" t="inlineStr">
+      <c r="G200" s="23" t="inlineStr">
         <is>
           <t>高</t>
         </is>
       </c>
-      <c r="H199" s="13" t="n">
+      <c r="H200" s="13" t="n">
         <v>20</v>
       </c>
     </row>
-    <row r="200" ht="20" customHeight="1">
-      <c r="A200" s="29" t="inlineStr">
+    <row r="201" ht="20" customHeight="1">
+      <c r="A201" s="29" t="inlineStr">
         <is>
           <t>【P3】 做市商系统  (Market Making)</t>
         </is>
-      </c>
-    </row>
-    <row r="201" ht="28" customHeight="1">
-      <c r="A201" s="16" t="inlineStr">
-        <is>
-          <t>做市商系统</t>
-        </is>
-      </c>
-      <c r="B201" s="15" t="inlineStr">
-        <is>
-          <t>P3</t>
-        </is>
-      </c>
-      <c r="C201" s="15" t="inlineStr">
-        <is>
-          <t>F15-01</t>
-        </is>
-      </c>
-      <c r="D201" s="30" t="inlineStr">
-        <is>
-          <t>双边报价做市</t>
-        </is>
-      </c>
-      <c r="E201" s="16" t="inlineStr">
-        <is>
-          <t>多品种同时双边报价，延迟&lt;5ms，报价宽度动态优化，支持国债/信用债/利率互换多品种做市</t>
-        </is>
-      </c>
-      <c r="F201" s="16" t="inlineStr">
-        <is>
-          <t>p99延迟/误差率/精度验证/压测10k TPS</t>
-        </is>
-      </c>
-      <c r="G201" s="28" t="inlineStr">
-        <is>
-          <t>极高</t>
-        </is>
-      </c>
-      <c r="H201" s="18" t="n">
-        <v>70</v>
       </c>
     </row>
     <row r="202" ht="28" customHeight="1">
@@ -14921,17 +14967,17 @@
       </c>
       <c r="C202" s="15" t="inlineStr">
         <is>
-          <t>F15-02</t>
+          <t>F15-01</t>
         </is>
       </c>
       <c r="D202" s="30" t="inlineStr">
         <is>
-          <t>TRS做市服务</t>
+          <t>双边报价做市</t>
         </is>
       </c>
       <c r="E202" s="16" t="inlineStr">
         <is>
-          <t>TRS产品双边报价，与TRS收益互换系统深度集成，对冲报价敞口，支持客户TRS交易</t>
+          <t>多品种同时双边报价，延迟&lt;5ms，报价宽度动态优化，支持国债/信用债/利率互换多品种做市</t>
         </is>
       </c>
       <c r="F202" s="16" t="inlineStr">
@@ -14945,7 +14991,7 @@
         </is>
       </c>
       <c r="H202" s="18" t="n">
-        <v>40</v>
+        <v>70</v>
       </c>
     </row>
     <row r="203" ht="28" customHeight="1">
@@ -14961,31 +15007,31 @@
       </c>
       <c r="C203" s="15" t="inlineStr">
         <is>
-          <t>F15-03</t>
+          <t>F15-02</t>
         </is>
       </c>
       <c r="D203" s="30" t="inlineStr">
         <is>
-          <t>RFQ询价响应</t>
+          <t>TRS做市服务</t>
         </is>
       </c>
       <c r="E203" s="16" t="inlineStr">
         <is>
-          <t>接收客户询价请求，自动生成报价，报价有效期管理，成交确认，询价历史记录</t>
+          <t>TRS产品双边报价，与TRS收益互换系统深度集成，对冲报价敞口，支持客户TRS交易</t>
         </is>
       </c>
       <c r="F203" s="16" t="inlineStr">
         <is>
-          <t>功能完整/边界测试/集成冒烟/性能基线</t>
-        </is>
-      </c>
-      <c r="G203" s="23" t="inlineStr">
-        <is>
-          <t>高</t>
+          <t>p99延迟/误差率/精度验证/压测10k TPS</t>
+        </is>
+      </c>
+      <c r="G203" s="28" t="inlineStr">
+        <is>
+          <t>极高</t>
         </is>
       </c>
       <c r="H203" s="18" t="n">
-        <v>25</v>
+        <v>40</v>
       </c>
     </row>
     <row r="204" ht="28" customHeight="1">
@@ -15001,17 +15047,17 @@
       </c>
       <c r="C204" s="15" t="inlineStr">
         <is>
-          <t>F15-04</t>
+          <t>F15-03</t>
         </is>
       </c>
       <c r="D204" s="30" t="inlineStr">
         <is>
-          <t>API程序化做市</t>
+          <t>RFQ询价响应</t>
         </is>
       </c>
       <c r="E204" s="16" t="inlineStr">
         <is>
-          <t>对外提供做市API接口，支持程序化交易对手接入，流式报价推送，API鉴权与频率限制</t>
+          <t>接收客户询价请求，自动生成报价，报价有效期管理，成交确认，询价历史记录</t>
         </is>
       </c>
       <c r="F204" s="16" t="inlineStr">
@@ -15041,31 +15087,31 @@
       </c>
       <c r="C205" s="15" t="inlineStr">
         <is>
-          <t>F15-05</t>
+          <t>F15-04</t>
         </is>
       </c>
       <c r="D205" s="30" t="inlineStr">
         <is>
-          <t>报价策略配置</t>
+          <t>API程序化做市</t>
         </is>
       </c>
       <c r="E205" s="16" t="inlineStr">
         <is>
-          <t>各品种做市参数配置（报价宽度/报价量/报价频率），分时段策略，按交易对手差异化报价</t>
+          <t>对外提供做市API接口，支持程序化交易对手接入，流式报价推送，API鉴权与频率限制</t>
         </is>
       </c>
       <c r="F205" s="16" t="inlineStr">
         <is>
-          <t>功能测试通过/正确率100%</t>
-        </is>
-      </c>
-      <c r="G205" s="24" t="inlineStr">
-        <is>
-          <t>中</t>
+          <t>功能完整/边界测试/集成冒烟/性能基线</t>
+        </is>
+      </c>
+      <c r="G205" s="23" t="inlineStr">
+        <is>
+          <t>高</t>
         </is>
       </c>
       <c r="H205" s="18" t="n">
-        <v>20</v>
+        <v>25</v>
       </c>
     </row>
     <row r="206" ht="28" customHeight="1">
@@ -15081,31 +15127,31 @@
       </c>
       <c r="C206" s="15" t="inlineStr">
         <is>
-          <t>F15-06</t>
+          <t>F15-05</t>
         </is>
       </c>
       <c r="D206" s="30" t="inlineStr">
         <is>
-          <t>报价优化算法</t>
+          <t>报价策略配置</t>
         </is>
       </c>
       <c r="E206" s="16" t="inlineStr">
         <is>
-          <t>基于市场微结构理论动态调整bid-ask spread，流动性自适应调节，机器学习辅助报价优化</t>
+          <t>各品种做市参数配置（报价宽度/报价量/报价频率），分时段策略，按交易对手差异化报价</t>
         </is>
       </c>
       <c r="F206" s="16" t="inlineStr">
         <is>
-          <t>p99延迟/误差率/精度验证/压测10k TPS</t>
-        </is>
-      </c>
-      <c r="G206" s="28" t="inlineStr">
-        <is>
-          <t>极高</t>
+          <t>功能测试通过/正确率100%</t>
+        </is>
+      </c>
+      <c r="G206" s="24" t="inlineStr">
+        <is>
+          <t>中</t>
         </is>
       </c>
       <c r="H206" s="18" t="n">
-        <v>50</v>
+        <v>20</v>
       </c>
     </row>
     <row r="207" ht="28" customHeight="1">
@@ -15121,31 +15167,31 @@
       </c>
       <c r="C207" s="15" t="inlineStr">
         <is>
-          <t>F15-07</t>
+          <t>F15-06</t>
         </is>
       </c>
       <c r="D207" s="30" t="inlineStr">
         <is>
-          <t>债券过滤与筛选</t>
+          <t>报价优化算法</t>
         </is>
       </c>
       <c r="E207" s="16" t="inlineStr">
         <is>
-          <t>做市标的券池管理，流动性分级筛选，黑名单管理，临时暂停做市规则</t>
+          <t>基于市场微结构理论动态调整bid-ask spread，流动性自适应调节，机器学习辅助报价优化</t>
         </is>
       </c>
       <c r="F207" s="16" t="inlineStr">
         <is>
-          <t>功能测试通过</t>
-        </is>
-      </c>
-      <c r="G207" s="25" t="inlineStr">
-        <is>
-          <t>低</t>
+          <t>p99延迟/误差率/精度验证/压测10k TPS</t>
+        </is>
+      </c>
+      <c r="G207" s="28" t="inlineStr">
+        <is>
+          <t>极高</t>
         </is>
       </c>
       <c r="H207" s="18" t="n">
-        <v>10</v>
+        <v>50</v>
       </c>
     </row>
     <row r="208" ht="28" customHeight="1">
@@ -15161,31 +15207,31 @@
       </c>
       <c r="C208" s="15" t="inlineStr">
         <is>
-          <t>F15-08</t>
+          <t>F15-07</t>
         </is>
       </c>
       <c r="D208" s="30" t="inlineStr">
         <is>
-          <t>做市义务实时监控</t>
+          <t>债券过滤与筛选</t>
         </is>
       </c>
       <c r="E208" s="16" t="inlineStr">
         <is>
-          <t>实时监控做市义务完成情况（报价连续性/报价宽度/报价量达标），义务违规预警，监管报告生成</t>
+          <t>做市标的券池管理，流动性分级筛选，黑名单管理，临时暂停做市规则</t>
         </is>
       </c>
       <c r="F208" s="16" t="inlineStr">
         <is>
-          <t>功能完整/边界测试/集成冒烟/性能基线</t>
-        </is>
-      </c>
-      <c r="G208" s="23" t="inlineStr">
-        <is>
-          <t>高</t>
+          <t>功能测试通过</t>
+        </is>
+      </c>
+      <c r="G208" s="25" t="inlineStr">
+        <is>
+          <t>低</t>
         </is>
       </c>
       <c r="H208" s="18" t="n">
-        <v>30</v>
+        <v>10</v>
       </c>
     </row>
     <row r="209" ht="28" customHeight="1">
@@ -15201,31 +15247,31 @@
       </c>
       <c r="C209" s="15" t="inlineStr">
         <is>
-          <t>F15-09</t>
+          <t>F15-08</t>
         </is>
       </c>
       <c r="D209" s="30" t="inlineStr">
         <is>
-          <t>做市行情展示</t>
+          <t>做市义务实时监控</t>
         </is>
       </c>
       <c r="E209" s="16" t="inlineStr">
         <is>
-          <t>做市报价行情矩阵，实时价格展示，报价历史回放，市场最优报价对比，中签率统计</t>
+          <t>实时监控做市义务完成情况（报价连续性/报价宽度/报价量达标），义务违规预警，监管报告生成</t>
         </is>
       </c>
       <c r="F209" s="16" t="inlineStr">
         <is>
-          <t>功能测试通过/正确率100%</t>
-        </is>
-      </c>
-      <c r="G209" s="24" t="inlineStr">
-        <is>
-          <t>中</t>
+          <t>功能完整/边界测试/集成冒烟/性能基线</t>
+        </is>
+      </c>
+      <c r="G209" s="23" t="inlineStr">
+        <is>
+          <t>高</t>
         </is>
       </c>
       <c r="H209" s="18" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
     </row>
     <row r="210" ht="28" customHeight="1">
@@ -15241,31 +15287,31 @@
       </c>
       <c r="C210" s="15" t="inlineStr">
         <is>
-          <t>F15-10</t>
+          <t>F15-09</t>
         </is>
       </c>
       <c r="D210" s="30" t="inlineStr">
         <is>
-          <t>做市订单管理</t>
+          <t>做市行情展示</t>
         </is>
       </c>
       <c r="E210" s="16" t="inlineStr">
         <is>
-          <t>做市委托生成、撤改、成交回报处理，订单状态实时跟踪，批量撤单，做市台账</t>
+          <t>做市报价行情矩阵，实时价格展示，报价历史回放，市场最优报价对比，中签率统计</t>
         </is>
       </c>
       <c r="F210" s="16" t="inlineStr">
         <is>
-          <t>功能完整/边界测试/集成冒烟/性能基线</t>
-        </is>
-      </c>
-      <c r="G210" s="23" t="inlineStr">
-        <is>
-          <t>高</t>
+          <t>功能测试通过/正确率100%</t>
+        </is>
+      </c>
+      <c r="G210" s="24" t="inlineStr">
+        <is>
+          <t>中</t>
         </is>
       </c>
       <c r="H210" s="18" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
     </row>
     <row r="211" ht="28" customHeight="1">
@@ -15281,31 +15327,31 @@
       </c>
       <c r="C211" s="15" t="inlineStr">
         <is>
-          <t>F15-11</t>
+          <t>F15-10</t>
         </is>
       </c>
       <c r="D211" s="30" t="inlineStr">
         <is>
-          <t>库存风险实时管理</t>
+          <t>做市订单管理</t>
         </is>
       </c>
       <c r="E211" s="16" t="inlineStr">
         <is>
-          <t>做市库存PnL实时监控，Delta对冲自动触发，库存敞口上限控制，实时盯市损益</t>
+          <t>做市委托生成、撤改、成交回报处理，订单状态实时跟踪，批量撤单，做市台账</t>
         </is>
       </c>
       <c r="F211" s="16" t="inlineStr">
         <is>
-          <t>p99延迟/误差率/精度验证/压测10k TPS</t>
-        </is>
-      </c>
-      <c r="G211" s="28" t="inlineStr">
-        <is>
-          <t>极高</t>
+          <t>功能完整/边界测试/集成冒烟/性能基线</t>
+        </is>
+      </c>
+      <c r="G211" s="23" t="inlineStr">
+        <is>
+          <t>高</t>
         </is>
       </c>
       <c r="H211" s="18" t="n">
-        <v>60</v>
+        <v>30</v>
       </c>
     </row>
     <row r="212" ht="28" customHeight="1">
@@ -15321,62 +15367,102 @@
       </c>
       <c r="C212" s="15" t="inlineStr">
         <is>
+          <t>F15-11</t>
+        </is>
+      </c>
+      <c r="D212" s="30" t="inlineStr">
+        <is>
+          <t>库存风险实时管理</t>
+        </is>
+      </c>
+      <c r="E212" s="16" t="inlineStr">
+        <is>
+          <t>做市库存PnL实时监控，Delta对冲自动触发，库存敞口上限控制，实时盯市损益</t>
+        </is>
+      </c>
+      <c r="F212" s="16" t="inlineStr">
+        <is>
+          <t>p99延迟/误差率/精度验证/压测10k TPS</t>
+        </is>
+      </c>
+      <c r="G212" s="28" t="inlineStr">
+        <is>
+          <t>极高</t>
+        </is>
+      </c>
+      <c r="H212" s="18" t="n">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="213" ht="28" customHeight="1">
+      <c r="A213" s="16" t="inlineStr">
+        <is>
+          <t>做市商系统</t>
+        </is>
+      </c>
+      <c r="B213" s="15" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="C213" s="15" t="inlineStr">
+        <is>
           <t>F15-12</t>
         </is>
       </c>
-      <c r="D212" s="30" t="inlineStr">
+      <c r="D213" s="30" t="inlineStr">
         <is>
           <t>竞争力分析</t>
         </is>
       </c>
-      <c r="E212" s="16" t="inlineStr">
+      <c r="E213" s="16" t="inlineStr">
         <is>
           <t>与市场最优报价对比，中签率分析，报价表现统计，策略调优建议，竞争对手报价分析</t>
         </is>
       </c>
-      <c r="F212" s="16" t="inlineStr">
+      <c r="F213" s="16" t="inlineStr">
         <is>
           <t>功能完整/边界测试/集成冒烟/性能基线</t>
         </is>
       </c>
-      <c r="G212" s="23" t="inlineStr">
+      <c r="G213" s="23" t="inlineStr">
         <is>
           <t>高</t>
         </is>
       </c>
-      <c r="H212" s="18" t="n">
+      <c r="H213" s="18" t="n">
         <v>25</v>
       </c>
     </row>
-    <row r="213">
-      <c r="A213" s="19" t="inlineStr">
+    <row r="214">
+      <c r="A214" s="19" t="inlineStr">
         <is>
           <t>总计功能数 / Total Function Points</t>
         </is>
       </c>
-      <c r="H213" s="20">
-        <f>SUM(H3:H212)</f>
+      <c r="H214" s="20">
+        <f>SUM(H3:H213)</f>
         <v/>
       </c>
     </row>
   </sheetData>
   <mergeCells count="16">
-    <mergeCell ref="A143:H143"/>
+    <mergeCell ref="A131:H131"/>
+    <mergeCell ref="A144:H144"/>
     <mergeCell ref="A3:H3"/>
     <mergeCell ref="A101:H101"/>
-    <mergeCell ref="A130:H130"/>
-    <mergeCell ref="A213:G213"/>
-    <mergeCell ref="A200:H200"/>
-    <mergeCell ref="A180:H180"/>
+    <mergeCell ref="A201:H201"/>
+    <mergeCell ref="A190:H190"/>
+    <mergeCell ref="A214:G214"/>
+    <mergeCell ref="A160:H160"/>
     <mergeCell ref="A60:H60"/>
     <mergeCell ref="A112:H112"/>
     <mergeCell ref="A68:H68"/>
+    <mergeCell ref="A181:H181"/>
     <mergeCell ref="A1:H1"/>
-    <mergeCell ref="A189:H189"/>
     <mergeCell ref="A31:H31"/>
-    <mergeCell ref="A159:H159"/>
+    <mergeCell ref="A168:H168"/>
     <mergeCell ref="A88:H88"/>
-    <mergeCell ref="A167:H167"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -16327,10 +16413,10 @@
         </is>
       </c>
       <c r="H8" s="8" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="I8" s="8" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="J8" s="4" t="inlineStr">
         <is>
@@ -16516,7 +16602,7 @@
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>跨资产实时头寸</t>
+          <t>全资产实时头寸</t>
         </is>
       </c>
       <c r="D6" s="5" t="inlineStr">
@@ -16623,7 +16709,7 @@
       </c>
       <c r="F8" s="5" t="inlineStr">
         <is>
-          <t>中登/中债登结算接口</t>
+          <t>中登/中债登/上清结算接口</t>
         </is>
       </c>
       <c r="G8" s="42" t="inlineStr">

</xml_diff>

<commit_message>
Update resource estimates for M04 and M07 after boundary clarification
M04: 140 → 130 pm (removed F04-14, -30 days, ~5% effort reduction)
M07: 160 → 150 pm (F07-11/12/13 reframed as consumer layers, -35 days, ~6% reduction)
Both duration_m unchanged at 14m (critical paths unaffected)

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Feasibility_analysis/FICC_Gap_Analysis.xlsx
+++ b/Feasibility_analysis/FICC_Gap_Analysis.xlsx
@@ -1143,7 +1143,7 @@
         <v>12</v>
       </c>
       <c r="O6" s="8" t="n">
-        <v>140</v>
+        <v>130</v>
       </c>
       <c r="P6" s="5" t="inlineStr">
         <is>
@@ -1365,7 +1365,7 @@
         <v>14</v>
       </c>
       <c r="O9" s="8" t="n">
-        <v>160</v>
+        <v>150</v>
       </c>
       <c r="P9" s="5" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Fix M07 function ordering: move F07-20 (TCA) to domain C, reorder F07-22 in domain E
M07 domain reorganization (logical grouping by function type):
- Domain C (绩效归因): F07-07, F07-08, F07-09, F07-19, F07-20 (TCA), F07-21 (moved F07-20 from E)
- Domain D (风险计量): F07-10, F07-11, F07-12, F07-13
- Domain E (流动性与对冲管理): F07-14, F07-15, F07-22 (removed F07-20, reordered F07-22)
- Domain F (量化底座集成): F07-16, F07-17, F07-18

Function indices now sequential: F07-01 through F07-22 with no gaps in domain order.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Feasibility_analysis/FICC_Gap_Analysis.xlsx
+++ b/Feasibility_analysis/FICC_Gap_Analysis.xlsx
@@ -3070,103 +3070,103 @@
       <c r="J17" s="5" t="inlineStr"/>
     </row>
     <row r="18" ht="48" customHeight="1">
-      <c r="A18" s="5" t="inlineStr">
+      <c r="A18" s="11" t="inlineStr">
         <is>
           <t>C. 绩效归因</t>
         </is>
       </c>
-      <c r="B18" s="3" t="inlineStr">
+      <c r="B18" s="10" t="inlineStr">
+        <is>
+          <t>F07-20</t>
+        </is>
+      </c>
+      <c r="C18" s="27" t="inlineStr">
+        <is>
+          <t>交易成本分析TCA</t>
+        </is>
+      </c>
+      <c r="D18" s="11" t="inlineStr">
+        <is>
+          <t>事后TCA：实施成本差（Implementation Shortfall = 决策时盘中价−成交均价）、VWAP/TWAP基准偏差，滑点分解（市场冲击+时机成本+价差成本）；经纪商执行质量排名（月度），超额成本自动触发路由策略优化建议，逐交易TCA反馈循环（成本预测模型再训练输入）；TCA结果回写F07-07归因（提升交易效应精确度）；实时TCA反馈推送至F07-22盘中P&amp;L仪表盘</t>
+        </is>
+      </c>
+      <c r="E18" s="11" t="inlineStr">
+        <is>
+          <t>TCA报告T+1生成，经纪商排名覆盖≥90%成交量，实施成本差计算与外部TCA服务误差&lt;1bps，每日TCA反馈驱动&lt;100bps超额成本自动预警</t>
+        </is>
+      </c>
+      <c r="F18" s="11" t="inlineStr">
+        <is>
+          <t>IBOR交易记录/AMD实时行情（决策时间戳价格）/现券交易系统成交回报/F07-22盘中P&amp;L</t>
+        </is>
+      </c>
+      <c r="G18" s="42" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="H18" s="13" t="n">
+        <v>25</v>
+      </c>
+      <c r="I18" s="12" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="J18" s="11" t="inlineStr"/>
+    </row>
+    <row r="19" ht="48" customHeight="1">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t>C. 绩效归因</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="inlineStr">
         <is>
           <t>F07-21</t>
         </is>
       </c>
-      <c r="C18" s="4" t="inlineStr">
+      <c r="C19" s="4" t="inlineStr">
         <is>
           <t>绩效报告生成</t>
         </is>
       </c>
-      <c r="D18" s="5" t="inlineStr">
+      <c r="D19" s="5" t="inlineStr">
         <is>
           <t>TWR（时间加权收益率）/MWR（资金加权收益率）多期计算，Grap算法多期归因链接（月度→季度→年度），PM工作台标准化绩效仪表盘（夏普/IR/最大回撤/信息比率），自动生成投委会汇报材料（PDF/PPT），历史归因报告版本存档与对比</t>
         </is>
       </c>
-      <c r="E18" s="5" t="inlineStr">
+      <c r="E19" s="5" t="inlineStr">
         <is>
           <t>TWR/MWR与Bloomberg AIM误差&lt;0.1%，月度报告T+1 9:00前自动生成，支持≥12期累计归因</t>
         </is>
       </c>
-      <c r="F18" s="5" t="inlineStr">
+      <c r="F19" s="5" t="inlineStr">
         <is>
           <t>M07归因引擎（F07-07/F07-08）/IBOR持仓/AMD指数基准</t>
         </is>
       </c>
-      <c r="G18" s="42" t="inlineStr">
+      <c r="G19" s="42" t="inlineStr">
         <is>
           <t>中</t>
         </is>
       </c>
-      <c r="H18" s="8" t="n">
+      <c r="H19" s="8" t="n">
         <v>20</v>
       </c>
-      <c r="I18" s="6" t="inlineStr">
-        <is>
-          <t>P1</t>
-        </is>
-      </c>
-      <c r="J18" s="5" t="inlineStr"/>
-    </row>
-    <row r="19" ht="18" customHeight="1">
-      <c r="A19" s="43" t="inlineStr">
+      <c r="I19" s="6" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="J19" s="5" t="inlineStr"/>
+    </row>
+    <row r="20" ht="18" customHeight="1">
+      <c r="A20" s="43" t="inlineStr">
         <is>
           <t>D. 风险计量</t>
         </is>
       </c>
-    </row>
-    <row r="20" ht="48" customHeight="1">
-      <c r="A20" s="5" t="inlineStr">
-        <is>
-          <t>D. 风险计量</t>
-        </is>
-      </c>
-      <c r="B20" s="3" t="inlineStr">
-        <is>
-          <t>F07-10</t>
-        </is>
-      </c>
-      <c r="C20" s="4" t="inlineStr">
-        <is>
-          <t>因子风险分解 + MCTR边际风险贡献（消费M08因子暴露）</t>
-        </is>
-      </c>
-      <c r="D20" s="5" t="inlineStr">
-        <is>
-          <t>【消费M08因子暴露结果】将组合持仓分解为系统性风险（2200+因子，来自M08）+特异性风险；计算MCTR边际风险贡献（∂组合波动率/∂持仓权重，热路径用C++矩阵求导），输出风险消耗排名（识别「风险大户」），驱动减仓/加仓优先级；多周期因子归因分解（日/周/月级跨期间）：按宏观因子类别（利率水平/曲线斜率/曲率/信用利差/流动性溢价/汇率/商品/权益Beta）拆分组合收益来源，因子贡献追踪与漂移预警；提供QP再平衡的风险预算约束输入。本模块不计算因子协方差矩阵，协方差矩阵由M08维护</t>
-        </is>
-      </c>
-      <c r="E20" s="5" t="inlineStr">
-        <is>
-          <t>因子模型解释方差&gt;80%（由M08保证），MCTR实时更新延迟&lt;5s，多周期因子归因对账&lt;1bps，日度初步结果&lt;2h，风险预算仪表盘刷新延迟&lt;5s</t>
-        </is>
-      </c>
-      <c r="F20" s="5" t="inlineStr">
-        <is>
-          <t>M08因子暴露API（协方差矩阵）/IBOR持仓/定价平台</t>
-        </is>
-      </c>
-      <c r="G20" s="41" t="inlineStr">
-        <is>
-          <t>高</t>
-        </is>
-      </c>
-      <c r="H20" s="8" t="n">
-        <v>80</v>
-      </c>
-      <c r="I20" s="6" t="inlineStr">
-        <is>
-          <t>P1</t>
-        </is>
-      </c>
-      <c r="J20" s="5" t="inlineStr"/>
     </row>
     <row r="21" ht="48" customHeight="1">
       <c r="A21" s="5" t="inlineStr">
@@ -3176,36 +3176,36 @@
       </c>
       <c r="B21" s="3" t="inlineStr">
         <is>
-          <t>F07-11</t>
+          <t>F07-10</t>
         </is>
       </c>
       <c r="C21" s="4" t="inlineStr">
         <is>
-          <t>Component VaR 四层穿透展示（调用M04引擎）</t>
+          <t>因子风险分解 + MCTR边际风险贡献（消费M08因子暴露）</t>
         </is>
       </c>
       <c r="D21" s="5" t="inlineStr">
         <is>
-          <t>PM决策展示层——调用M04(F04-10)VaR计算引擎获取三方法结果，在本模块实现四层穿透钻取：资产类别VaR→行业/子市场VaR→评级/信用质量VaR→单一发行人Component VaR，含跨类分散化收益量化；本模块不重复实现VaR计算，专注投资决策视角的风险溯源与持仓优化引导</t>
+          <t>【消费M08因子暴露结果】将组合持仓分解为系统性风险（2200+因子，来自M08）+特异性风险；计算MCTR边际风险贡献（∂组合波动率/∂持仓权重，热路径用C++矩阵求导），输出风险消耗排名（识别「风险大户」），驱动减仓/加仓优先级；多周期因子归因分解（日/周/月级跨期间）：按宏观因子类别（利率水平/曲线斜率/曲率/信用利差/流动性溢价/汇率/商品/权益Beta）拆分组合收益来源，因子贡献追踪与漂移预警；提供QP再平衡的风险预算约束输入。本模块不计算因子协方差矩阵，协方差矩阵由M08维护</t>
         </is>
       </c>
       <c r="E21" s="5" t="inlineStr">
         <is>
-          <t>穿透至发行人层展示&lt;3s，三方法差异预警由M04提供，本模块直接透传</t>
+          <t>因子模型解释方差&gt;80%（由M08保证），MCTR实时更新延迟&lt;5s，多周期因子归因对账&lt;1bps，日度初步结果&lt;2h，风险预算仪表盘刷新延迟&lt;5s</t>
         </is>
       </c>
       <c r="F21" s="5" t="inlineStr">
         <is>
-          <t>FICC风险计量平台(M04 F04-10)/IBOR</t>
-        </is>
-      </c>
-      <c r="G21" s="42" t="inlineStr">
-        <is>
-          <t>中</t>
+          <t>M08因子暴露API（协方差矩阵）/IBOR持仓/定价平台</t>
+        </is>
+      </c>
+      <c r="G21" s="41" t="inlineStr">
+        <is>
+          <t>高</t>
         </is>
       </c>
       <c r="H21" s="8" t="n">
-        <v>40</v>
+        <v>80</v>
       </c>
       <c r="I21" s="6" t="inlineStr">
         <is>
@@ -3222,27 +3222,27 @@
       </c>
       <c r="B22" s="3" t="inlineStr">
         <is>
-          <t>F07-12</t>
+          <t>F07-11</t>
         </is>
       </c>
       <c r="C22" s="4" t="inlineStr">
         <is>
-          <t>敏感度展示（多维Shock Grid，调用M04引擎）</t>
+          <t>Component VaR 四层穿透展示（调用M04引擎）</t>
         </is>
       </c>
       <c r="D22" s="5" t="inlineStr">
         <is>
-          <t>PM决策展示层——M04(F04-08/09)计算DV01/CS01/Greeks，本模块负责：组合层面聚合（按资产类别/行业/评级汇总），构建利率×信用利差二维冲击矩阵（Shock Grid 5×5），识别最脆弱组合方向，输出对冲比率建议；本模块不重复实现敏感度计算</t>
+          <t>PM决策展示层——调用M04(F04-10)VaR计算引擎获取三方法结果，在本模块实现四层穿透钻取：资产类别VaR→行业/子市场VaR→评级/信用质量VaR→单一发行人Component VaR，含跨类分散化收益量化；本模块不重复实现VaR计算，专注投资决策视角的风险溯源与持仓优化引导</t>
         </is>
       </c>
       <c r="E22" s="5" t="inlineStr">
         <is>
-          <t>Shock Grid 5×5矩阵实时刷新，组合DV01聚合与M04单券结果误差&lt;0.1bps</t>
+          <t>穿透至发行人层展示&lt;3s，三方法差异预警由M04提供，本模块直接透传</t>
         </is>
       </c>
       <c r="F22" s="5" t="inlineStr">
         <is>
-          <t>FICC风险计量平台(M04 F04-08/09)/定价平台(M09 KRD)/IBOR</t>
+          <t>FICC风险计量平台(M04 F04-10)/IBOR</t>
         </is>
       </c>
       <c r="G22" s="42" t="inlineStr">
@@ -3268,142 +3268,142 @@
       </c>
       <c r="B23" s="3" t="inlineStr">
         <is>
+          <t>F07-12</t>
+        </is>
+      </c>
+      <c r="C23" s="4" t="inlineStr">
+        <is>
+          <t>敏感度展示（多维Shock Grid，调用M04引擎）</t>
+        </is>
+      </c>
+      <c r="D23" s="5" t="inlineStr">
+        <is>
+          <t>PM决策展示层——M04(F04-08/09)计算DV01/CS01/Greeks，本模块负责：组合层面聚合（按资产类别/行业/评级汇总），构建利率×信用利差二维冲击矩阵（Shock Grid 5×5），识别最脆弱组合方向，输出对冲比率建议；本模块不重复实现敏感度计算</t>
+        </is>
+      </c>
+      <c r="E23" s="5" t="inlineStr">
+        <is>
+          <t>Shock Grid 5×5矩阵实时刷新，组合DV01聚合与M04单券结果误差&lt;0.1bps</t>
+        </is>
+      </c>
+      <c r="F23" s="5" t="inlineStr">
+        <is>
+          <t>FICC风险计量平台(M04 F04-08/09)/定价平台(M09 KRD)/IBOR</t>
+        </is>
+      </c>
+      <c r="G23" s="42" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="H23" s="8" t="n">
+        <v>40</v>
+      </c>
+      <c r="I23" s="6" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="J23" s="5" t="inlineStr"/>
+    </row>
+    <row r="24" ht="48" customHeight="1">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t>D. 风险计量</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="inlineStr">
+        <is>
           <t>F07-13</t>
         </is>
       </c>
-      <c r="C23" s="4" t="inlineStr">
+      <c r="C24" s="4" t="inlineStr">
         <is>
           <t>情景分析PM决策层（调用M04场景库）</t>
         </is>
       </c>
-      <c r="D23" s="5" t="inlineStr">
+      <c r="D24" s="5" t="inlineStr">
         <is>
           <t>PM投资决策层——M04(F04-11)维护历史场景库并提供计算API，本模块负责：①调用M04获取场景P&amp;L结果（924行情/包商/钱荒/股灾等8+历史场景+自定义场景），②PM工作流：基于场景结果生成对冲建议、触发再平衡方案、输出持仓调整优先级，③反向压力测试（倒推临界情景→止损线设计依据）；场景库维护与全公司治理由M04负责</t>
         </is>
       </c>
-      <c r="E23" s="5" t="inlineStr">
+      <c r="E24" s="5" t="inlineStr">
         <is>
           <t>调用M04 API获取场景P&amp;L&lt;2s，PM决策输出（对冲建议）&lt;5s，≥20情景并行</t>
         </is>
       </c>
-      <c r="F23" s="5" t="inlineStr">
+      <c r="F24" s="5" t="inlineStr">
         <is>
           <t>FICC风险计量平台(M04 F04-11 场景API)/定价平台</t>
         </is>
       </c>
-      <c r="G23" s="42" t="inlineStr">
+      <c r="G24" s="42" t="inlineStr">
         <is>
           <t>中</t>
         </is>
       </c>
-      <c r="H23" s="8" t="n">
+      <c r="H24" s="8" t="n">
         <v>60</v>
       </c>
-      <c r="I23" s="6" t="inlineStr">
-        <is>
-          <t>P1</t>
-        </is>
-      </c>
-      <c r="J23" s="5" t="inlineStr"/>
-    </row>
-    <row r="24" ht="18" customHeight="1">
-      <c r="A24" s="29" t="inlineStr">
+      <c r="I24" s="6" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="J24" s="5" t="inlineStr"/>
+    </row>
+    <row r="25" ht="18" customHeight="1">
+      <c r="A25" s="29" t="inlineStr">
         <is>
           <t>E. 流动性与对冲管理</t>
         </is>
       </c>
     </row>
-    <row r="25" ht="48" customHeight="1">
-      <c r="A25" s="5" t="inlineStr">
+    <row r="26" ht="48" customHeight="1">
+      <c r="A26" s="5" t="inlineStr">
         <is>
           <t>E. 流动性与对冲管理</t>
         </is>
       </c>
-      <c r="B25" s="3" t="inlineStr">
+      <c r="B26" s="3" t="inlineStr">
         <is>
           <t>F07-14</t>
         </is>
       </c>
-      <c r="C25" s="4" t="inlineStr">
+      <c r="C26" s="4" t="inlineStr">
         <is>
           <t>流动性风险管理（LVaR）</t>
         </is>
       </c>
-      <c r="D25" s="5" t="inlineStr">
+      <c r="D26" s="5" t="inlineStr">
         <is>
           <t>逐持仓变现能力评估（规模/日均成交量→变现天数），Almgren-Chriss市场冲击成本模型，流动性压力测试（X天内变现Y亿最优路径+成本），流动性调整VaR（LVaR=传统VaR+流动性溢价），流动性覆盖率/缓冲监控（1/3/5/10日分层），回购到期日历</t>
         </is>
       </c>
-      <c r="E25" s="5" t="inlineStr">
+      <c r="E26" s="5" t="inlineStr">
         <is>
           <t>LVaR与市场基准误差&lt;5%，日均成交量覆盖≥95%持仓，变现路径建议&lt;3s</t>
         </is>
       </c>
-      <c r="F25" s="5" t="inlineStr">
+      <c r="F26" s="5" t="inlineStr">
         <is>
           <t>AMD行情/IBOR持仓</t>
         </is>
       </c>
-      <c r="G25" s="42" t="inlineStr">
+      <c r="G26" s="42" t="inlineStr">
         <is>
           <t>中</t>
         </is>
       </c>
-      <c r="H25" s="8" t="n">
+      <c r="H26" s="8" t="n">
         <v>50</v>
       </c>
-      <c r="I25" s="6" t="inlineStr">
-        <is>
-          <t>P1</t>
-        </is>
-      </c>
-      <c r="J25" s="5" t="inlineStr"/>
-    </row>
-    <row r="26" ht="48" customHeight="1">
-      <c r="A26" s="11" t="inlineStr">
-        <is>
-          <t>E. 流动性与对冲管理</t>
-        </is>
-      </c>
-      <c r="B26" s="10" t="inlineStr">
-        <is>
-          <t>F07-15</t>
-        </is>
-      </c>
-      <c r="C26" s="27" t="inlineStr">
-        <is>
-          <t>衍生品对冲决策引擎</t>
-        </is>
-      </c>
-      <c r="D26" s="11" t="inlineStr">
-        <is>
-          <t>七类工具矩阵（国债期货2/5/10/30Y/IRS/CDS/股指期货IF/IH/IC/IM/股指期权/黄金期货/外汇远掉期），系统推荐最优对冲方案（成本最小约束），一键生成对冲指令，对冲效果追踪（前后风险指标对比/效率/执行滑点）；支持快速/精细/尾部/跨资产四种场景</t>
-        </is>
-      </c>
-      <c r="E26" s="11" t="inlineStr">
-        <is>
-          <t>对冲方案推荐&lt;5s，DV01对冲误差&lt;5%，指令自动流转执行引擎</t>
-        </is>
-      </c>
-      <c r="F26" s="11" t="inlineStr">
-        <is>
-          <t>衍生品交易系统/IBOR/定价平台/事前风控</t>
-        </is>
-      </c>
-      <c r="G26" s="41" t="inlineStr">
-        <is>
-          <t>高</t>
-        </is>
-      </c>
-      <c r="H26" s="13" t="n">
-        <v>40</v>
-      </c>
-      <c r="I26" s="12" t="inlineStr">
-        <is>
-          <t>P2</t>
-        </is>
-      </c>
-      <c r="J26" s="11" t="inlineStr"/>
+      <c r="I26" s="6" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="J26" s="5" t="inlineStr"/>
     </row>
     <row r="27" ht="48" customHeight="1">
       <c r="A27" s="11" t="inlineStr">
@@ -3413,36 +3413,36 @@
       </c>
       <c r="B27" s="10" t="inlineStr">
         <is>
-          <t>F07-20</t>
+          <t>F07-15</t>
         </is>
       </c>
       <c r="C27" s="27" t="inlineStr">
         <is>
-          <t>交易成本分析TCA</t>
+          <t>衍生品对冲决策引擎</t>
         </is>
       </c>
       <c r="D27" s="11" t="inlineStr">
         <is>
-          <t>事后TCA：实施成本差（Implementation Shortfall = 决策时盘中价−成交均价）、VWAP/TWAP基准偏差，滑点分解（市场冲击+时机成本+价差成本）；经纪商执行质量排名（月度），超额成本自动触发路由策略优化建议，逐交易TCA反馈循环（成本预测模型再训练输入）；TCA结果回写F07-07归因（提升交易效应精确度）；实时TCA反馈推送至F07-22盘中P&amp;L仪表盘</t>
+          <t>七类工具矩阵（国债期货2/5/10/30Y/IRS/CDS/股指期货IF/IH/IC/IM/股指期权/黄金期货/外汇远掉期），系统推荐最优对冲方案（成本最小约束），一键生成对冲指令，对冲效果追踪（前后风险指标对比/效率/执行滑点）；支持快速/精细/尾部/跨资产四种场景</t>
         </is>
       </c>
       <c r="E27" s="11" t="inlineStr">
         <is>
-          <t>TCA报告T+1生成，经纪商排名覆盖≥90%成交量，实施成本差计算与外部TCA服务误差&lt;1bps，每日TCA反馈驱动&lt;100bps超额成本自动预警</t>
+          <t>对冲方案推荐&lt;5s，DV01对冲误差&lt;5%，指令自动流转执行引擎</t>
         </is>
       </c>
       <c r="F27" s="11" t="inlineStr">
         <is>
-          <t>IBOR交易记录/AMD实时行情（决策时间戳价格）/现券交易系统成交回报/F07-22盘中P&amp;L</t>
-        </is>
-      </c>
-      <c r="G27" s="42" t="inlineStr">
-        <is>
-          <t>中</t>
+          <t>衍生品交易系统/IBOR/定价平台/事前风控</t>
+        </is>
+      </c>
+      <c r="G27" s="41" t="inlineStr">
+        <is>
+          <t>高</t>
         </is>
       </c>
       <c r="H27" s="13" t="n">
-        <v>25</v>
+        <v>40</v>
       </c>
       <c r="I27" s="12" t="inlineStr">
         <is>
@@ -3662,10 +3662,10 @@
     <mergeCell ref="A9:J9"/>
     <mergeCell ref="A3:J3"/>
     <mergeCell ref="A29:J29"/>
-    <mergeCell ref="A19:J19"/>
-    <mergeCell ref="A24:J24"/>
+    <mergeCell ref="A20:J20"/>
     <mergeCell ref="A2:J2"/>
     <mergeCell ref="A33:G33"/>
+    <mergeCell ref="A25:J25"/>
     <mergeCell ref="A13:J13"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -12524,22 +12524,22 @@
       </c>
       <c r="C127" s="3" t="inlineStr">
         <is>
-          <t>F07-21</t>
+          <t>F07-20</t>
         </is>
       </c>
       <c r="D127" s="4" t="inlineStr">
         <is>
-          <t>绩效报告生成</t>
+          <t>交易成本分析TCA</t>
         </is>
       </c>
       <c r="E127" s="5" t="inlineStr">
         <is>
-          <t>TWR（时间加权收益率）/MWR（资金加权收益率）多期计算，Grap算法多期归因链接（月度→季度→年度），PM工作台标准化绩效仪表盘（夏普/IR/最大回撤/信息比率），自动生成投委会汇报材料（PDF/PPT），历史归因报告版本存档与对比</t>
+          <t>事后TCA：实施成本差（Implementation Shortfall = 决策时盘中价−成交均价）、VWAP/TWAP基准偏差，滑点分解（市场冲击+时机成本+价差成本）；经纪商执行质量排名（月度），超额成本自动触发路由策略优化建议，逐交易TCA反馈循环（成本预测模型再训练输入）；TCA结果回写F07-07归因（提升交易效应精确度）；实时TCA反馈推送至F07-22盘中P&amp;L仪表盘</t>
         </is>
       </c>
       <c r="F127" s="5" t="inlineStr">
         <is>
-          <t>TWR/MWR与Bloomberg AIM误差&lt;0.1%，月度报告T+1 9:00前自动生成，支持≥12期累计归因</t>
+          <t>TCA报告T+1生成，经纪商排名覆盖≥90%成交量，实施成本差计算与外部TCA服务误差&lt;1bps，每日TCA反馈驱动&lt;100bps超额成本自动预警</t>
         </is>
       </c>
       <c r="G127" s="24" t="inlineStr">
@@ -12548,7 +12548,7 @@
         </is>
       </c>
       <c r="H127" s="8" t="n">
-        <v>20</v>
+        <v>25</v>
       </c>
     </row>
     <row r="128" ht="28" customHeight="1">
@@ -12564,31 +12564,31 @@
       </c>
       <c r="C128" s="3" t="inlineStr">
         <is>
-          <t>F07-10</t>
+          <t>F07-21</t>
         </is>
       </c>
       <c r="D128" s="4" t="inlineStr">
         <is>
-          <t>因子风险分解 + MCTR边际风险贡献（消费M08因子暴露）</t>
+          <t>绩效报告生成</t>
         </is>
       </c>
       <c r="E128" s="5" t="inlineStr">
         <is>
-          <t>【消费M08因子暴露结果】将组合持仓分解为系统性风险（2200+因子，来自M08）+特异性风险；计算MCTR边际风险贡献（∂组合波动率/∂持仓权重，热路径用C++矩阵求导），输出风险消耗排名（识别「风险大户」），驱动减仓/加仓优先级；多周期因子归因分解（日/周/月级跨期间）：按宏观因子类别（利率水平/曲线斜率/曲率/信用利差/流动性溢价/汇率/商品/权益Beta）拆分组合收益来源，因子贡献追踪与漂移预警；提供QP再平衡的风险预算约束输入。本模块不计算因子协方差矩阵，协方差矩阵由M08维护</t>
+          <t>TWR（时间加权收益率）/MWR（资金加权收益率）多期计算，Grap算法多期归因链接（月度→季度→年度），PM工作台标准化绩效仪表盘（夏普/IR/最大回撤/信息比率），自动生成投委会汇报材料（PDF/PPT），历史归因报告版本存档与对比</t>
         </is>
       </c>
       <c r="F128" s="5" t="inlineStr">
         <is>
-          <t>因子模型解释方差&gt;80%（由M08保证），MCTR实时更新延迟&lt;5s，多周期因子归因对账&lt;1bps，日度初步结果&lt;2h，风险预算仪表盘刷新延迟&lt;5s</t>
-        </is>
-      </c>
-      <c r="G128" s="23" t="inlineStr">
-        <is>
-          <t>高</t>
+          <t>TWR/MWR与Bloomberg AIM误差&lt;0.1%，月度报告T+1 9:00前自动生成，支持≥12期累计归因</t>
+        </is>
+      </c>
+      <c r="G128" s="24" t="inlineStr">
+        <is>
+          <t>中</t>
         </is>
       </c>
       <c r="H128" s="8" t="n">
-        <v>80</v>
+        <v>20</v>
       </c>
     </row>
     <row r="129" ht="28" customHeight="1">
@@ -12604,31 +12604,31 @@
       </c>
       <c r="C129" s="3" t="inlineStr">
         <is>
-          <t>F07-11</t>
+          <t>F07-10</t>
         </is>
       </c>
       <c r="D129" s="4" t="inlineStr">
         <is>
-          <t>Component VaR 四层穿透展示（调用M04引擎）</t>
+          <t>因子风险分解 + MCTR边际风险贡献（消费M08因子暴露）</t>
         </is>
       </c>
       <c r="E129" s="5" t="inlineStr">
         <is>
-          <t>PM决策展示层——调用M04(F04-10)VaR计算引擎获取三方法结果，在本模块实现四层穿透钻取：资产类别VaR→行业/子市场VaR→评级/信用质量VaR→单一发行人Component VaR，含跨类分散化收益量化；本模块不重复实现VaR计算，专注投资决策视角的风险溯源与持仓优化引导</t>
+          <t>【消费M08因子暴露结果】将组合持仓分解为系统性风险（2200+因子，来自M08）+特异性风险；计算MCTR边际风险贡献（∂组合波动率/∂持仓权重，热路径用C++矩阵求导），输出风险消耗排名（识别「风险大户」），驱动减仓/加仓优先级；多周期因子归因分解（日/周/月级跨期间）：按宏观因子类别（利率水平/曲线斜率/曲率/信用利差/流动性溢价/汇率/商品/权益Beta）拆分组合收益来源，因子贡献追踪与漂移预警；提供QP再平衡的风险预算约束输入。本模块不计算因子协方差矩阵，协方差矩阵由M08维护</t>
         </is>
       </c>
       <c r="F129" s="5" t="inlineStr">
         <is>
-          <t>穿透至发行人层展示&lt;3s，三方法差异预警由M04提供，本模块直接透传</t>
-        </is>
-      </c>
-      <c r="G129" s="24" t="inlineStr">
-        <is>
-          <t>中</t>
+          <t>因子模型解释方差&gt;80%（由M08保证），MCTR实时更新延迟&lt;5s，多周期因子归因对账&lt;1bps，日度初步结果&lt;2h，风险预算仪表盘刷新延迟&lt;5s</t>
+        </is>
+      </c>
+      <c r="G129" s="23" t="inlineStr">
+        <is>
+          <t>高</t>
         </is>
       </c>
       <c r="H129" s="8" t="n">
-        <v>40</v>
+        <v>80</v>
       </c>
     </row>
     <row r="130" ht="28" customHeight="1">
@@ -12644,22 +12644,22 @@
       </c>
       <c r="C130" s="3" t="inlineStr">
         <is>
-          <t>F07-12</t>
+          <t>F07-11</t>
         </is>
       </c>
       <c r="D130" s="4" t="inlineStr">
         <is>
-          <t>敏感度展示（多维Shock Grid，调用M04引擎）</t>
+          <t>Component VaR 四层穿透展示（调用M04引擎）</t>
         </is>
       </c>
       <c r="E130" s="5" t="inlineStr">
         <is>
-          <t>PM决策展示层——M04(F04-08/09)计算DV01/CS01/Greeks，本模块负责：组合层面聚合（按资产类别/行业/评级汇总），构建利率×信用利差二维冲击矩阵（Shock Grid 5×5），识别最脆弱组合方向，输出对冲比率建议；本模块不重复实现敏感度计算</t>
+          <t>PM决策展示层——调用M04(F04-10)VaR计算引擎获取三方法结果，在本模块实现四层穿透钻取：资产类别VaR→行业/子市场VaR→评级/信用质量VaR→单一发行人Component VaR，含跨类分散化收益量化；本模块不重复实现VaR计算，专注投资决策视角的风险溯源与持仓优化引导</t>
         </is>
       </c>
       <c r="F130" s="5" t="inlineStr">
         <is>
-          <t>Shock Grid 5×5矩阵实时刷新，组合DV01聚合与M04单券结果误差&lt;0.1bps</t>
+          <t>穿透至发行人层展示&lt;3s，三方法差异预警由M04提供，本模块直接透传</t>
         </is>
       </c>
       <c r="G130" s="24" t="inlineStr">
@@ -12684,22 +12684,22 @@
       </c>
       <c r="C131" s="3" t="inlineStr">
         <is>
-          <t>F07-13</t>
+          <t>F07-12</t>
         </is>
       </c>
       <c r="D131" s="4" t="inlineStr">
         <is>
-          <t>情景分析PM决策层（调用M04场景库）</t>
+          <t>敏感度展示（多维Shock Grid，调用M04引擎）</t>
         </is>
       </c>
       <c r="E131" s="5" t="inlineStr">
         <is>
-          <t>PM投资决策层——M04(F04-11)维护历史场景库并提供计算API，本模块负责：①调用M04获取场景P&amp;L结果（924行情/包商/钱荒/股灾等8+历史场景+自定义场景），②PM工作流：基于场景结果生成对冲建议、触发再平衡方案、输出持仓调整优先级，③反向压力测试（倒推临界情景→止损线设计依据）；场景库维护与全公司治理由M04负责</t>
+          <t>PM决策展示层——M04(F04-08/09)计算DV01/CS01/Greeks，本模块负责：组合层面聚合（按资产类别/行业/评级汇总），构建利率×信用利差二维冲击矩阵（Shock Grid 5×5），识别最脆弱组合方向，输出对冲比率建议；本模块不重复实现敏感度计算</t>
         </is>
       </c>
       <c r="F131" s="5" t="inlineStr">
         <is>
-          <t>调用M04 API获取场景P&amp;L&lt;2s，PM决策输出（对冲建议）&lt;5s，≥20情景并行</t>
+          <t>Shock Grid 5×5矩阵实时刷新，组合DV01聚合与M04单券结果误差&lt;0.1bps</t>
         </is>
       </c>
       <c r="G131" s="24" t="inlineStr">
@@ -12708,7 +12708,7 @@
         </is>
       </c>
       <c r="H131" s="8" t="n">
-        <v>60</v>
+        <v>40</v>
       </c>
     </row>
     <row r="132" ht="28" customHeight="1">
@@ -12724,22 +12724,22 @@
       </c>
       <c r="C132" s="3" t="inlineStr">
         <is>
-          <t>F07-14</t>
+          <t>F07-13</t>
         </is>
       </c>
       <c r="D132" s="4" t="inlineStr">
         <is>
-          <t>流动性风险管理（LVaR）</t>
+          <t>情景分析PM决策层（调用M04场景库）</t>
         </is>
       </c>
       <c r="E132" s="5" t="inlineStr">
         <is>
-          <t>逐持仓变现能力评估（规模/日均成交量→变现天数），Almgren-Chriss市场冲击成本模型，流动性压力测试（X天内变现Y亿最优路径+成本），流动性调整VaR（LVaR=传统VaR+流动性溢价），流动性覆盖率/缓冲监控（1/3/5/10日分层），回购到期日历</t>
+          <t>PM投资决策层——M04(F04-11)维护历史场景库并提供计算API，本模块负责：①调用M04获取场景P&amp;L结果（924行情/包商/钱荒/股灾等8+历史场景+自定义场景），②PM工作流：基于场景结果生成对冲建议、触发再平衡方案、输出持仓调整优先级，③反向压力测试（倒推临界情景→止损线设计依据）；场景库维护与全公司治理由M04负责</t>
         </is>
       </c>
       <c r="F132" s="5" t="inlineStr">
         <is>
-          <t>LVaR与市场基准误差&lt;5%，日均成交量覆盖≥95%持仓，变现路径建议&lt;3s</t>
+          <t>调用M04 API获取场景P&amp;L&lt;2s，PM决策输出（对冲建议）&lt;5s，≥20情景并行</t>
         </is>
       </c>
       <c r="G132" s="24" t="inlineStr">
@@ -12748,7 +12748,7 @@
         </is>
       </c>
       <c r="H132" s="8" t="n">
-        <v>50</v>
+        <v>60</v>
       </c>
     </row>
     <row r="133" ht="28" customHeight="1">
@@ -12764,31 +12764,31 @@
       </c>
       <c r="C133" s="3" t="inlineStr">
         <is>
-          <t>F07-15</t>
+          <t>F07-14</t>
         </is>
       </c>
       <c r="D133" s="4" t="inlineStr">
         <is>
-          <t>衍生品对冲决策引擎</t>
+          <t>流动性风险管理（LVaR）</t>
         </is>
       </c>
       <c r="E133" s="5" t="inlineStr">
         <is>
-          <t>七类工具矩阵（国债期货2/5/10/30Y/IRS/CDS/股指期货IF/IH/IC/IM/股指期权/黄金期货/外汇远掉期），系统推荐最优对冲方案（成本最小约束），一键生成对冲指令，对冲效果追踪（前后风险指标对比/效率/执行滑点）；支持快速/精细/尾部/跨资产四种场景</t>
+          <t>逐持仓变现能力评估（规模/日均成交量→变现天数），Almgren-Chriss市场冲击成本模型，流动性压力测试（X天内变现Y亿最优路径+成本），流动性调整VaR（LVaR=传统VaR+流动性溢价），流动性覆盖率/缓冲监控（1/3/5/10日分层），回购到期日历</t>
         </is>
       </c>
       <c r="F133" s="5" t="inlineStr">
         <is>
-          <t>对冲方案推荐&lt;5s，DV01对冲误差&lt;5%，指令自动流转执行引擎</t>
-        </is>
-      </c>
-      <c r="G133" s="23" t="inlineStr">
-        <is>
-          <t>高</t>
+          <t>LVaR与市场基准误差&lt;5%，日均成交量覆盖≥95%持仓，变现路径建议&lt;3s</t>
+        </is>
+      </c>
+      <c r="G133" s="24" t="inlineStr">
+        <is>
+          <t>中</t>
         </is>
       </c>
       <c r="H133" s="8" t="n">
-        <v>40</v>
+        <v>50</v>
       </c>
     </row>
     <row r="134" ht="28" customHeight="1">
@@ -12804,31 +12804,31 @@
       </c>
       <c r="C134" s="3" t="inlineStr">
         <is>
-          <t>F07-20</t>
+          <t>F07-15</t>
         </is>
       </c>
       <c r="D134" s="4" t="inlineStr">
         <is>
-          <t>交易成本分析TCA</t>
+          <t>衍生品对冲决策引擎</t>
         </is>
       </c>
       <c r="E134" s="5" t="inlineStr">
         <is>
-          <t>事后TCA：实施成本差（Implementation Shortfall = 决策时盘中价−成交均价）、VWAP/TWAP基准偏差，滑点分解（市场冲击+时机成本+价差成本）；经纪商执行质量排名（月度），超额成本自动触发路由策略优化建议，逐交易TCA反馈循环（成本预测模型再训练输入）；TCA结果回写F07-07归因（提升交易效应精确度）；实时TCA反馈推送至F07-22盘中P&amp;L仪表盘</t>
+          <t>七类工具矩阵（国债期货2/5/10/30Y/IRS/CDS/股指期货IF/IH/IC/IM/股指期权/黄金期货/外汇远掉期），系统推荐最优对冲方案（成本最小约束），一键生成对冲指令，对冲效果追踪（前后风险指标对比/效率/执行滑点）；支持快速/精细/尾部/跨资产四种场景</t>
         </is>
       </c>
       <c r="F134" s="5" t="inlineStr">
         <is>
-          <t>TCA报告T+1生成，经纪商排名覆盖≥90%成交量，实施成本差计算与外部TCA服务误差&lt;1bps，每日TCA反馈驱动&lt;100bps超额成本自动预警</t>
-        </is>
-      </c>
-      <c r="G134" s="24" t="inlineStr">
-        <is>
-          <t>中</t>
+          <t>对冲方案推荐&lt;5s，DV01对冲误差&lt;5%，指令自动流转执行引擎</t>
+        </is>
+      </c>
+      <c r="G134" s="23" t="inlineStr">
+        <is>
+          <t>高</t>
         </is>
       </c>
       <c r="H134" s="8" t="n">
-        <v>25</v>
+        <v>40</v>
       </c>
     </row>
     <row r="135" ht="28" customHeight="1">

</xml_diff>